<commit_message>
Add bank-account remote feasibility column (198/198) + 18-col deliverables
enrich5 pass: 10-agent fan-out on charity bank-account accessibility for a
remote AU-resident foreign founder (online / local visit / local agent /
blocked, with KYC & AML constraints). Key finding: only ~7 jurisdictions
allow fully-online charity bank accounts; ~32 effectively block foreigners.

Wired into XLSX (18 cols, widths, Methodology), webapp (field map + drawer
section), README table. Rebuilt XLSX + single-file webapp (466 KB, file://
safe).
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Methodology" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master'!$A$1:$Q$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master'!$A$1:$R$199</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q199"/>
+  <dimension ref="A1:R199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -517,6 +517,7 @@
     <col width="46" customWidth="1" min="15" max="15"/>
     <col width="40" customWidth="1" min="16" max="16"/>
     <col width="40" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -605,6 +606,11 @@
           <t>Tax-exempt status &amp; benefits</t>
         </is>
       </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Bank account (remote feasibility)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -692,6 +698,11 @@
           <t>Separate CRA application (Form T2050) after incorporation for charitable purposes. Benefits: charity income tax-exempt, issues official donor receipts. Time: CRA standard ~9 months, commonly 6-9 months.</t>
         </is>
       </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Realistic: Canadian banks open non-resident accounts in person, electronically or by phone; some (Scotiabank) start online, but a charity's corporate account typically needs at least one in-person branch visit by a signatory for KYC.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -779,6 +790,11 @@
           <t>Separate IRS application Form 1023 (1023-EZ for small orgs): organized and operated exclusively for exempt charitable/educational/scientific purposes, no private inurement. Exemption + donor deduction. Time unpublished.</t>
         </is>
       </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: US banks require in-person branch KYC with passport/visa and an IRS EIN; many also demand a physical US address, so a remote founder needs an in-person signatory trip or local agent.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -866,6 +882,11 @@
           <t>No separate application: tax law Art. 101 exempts from income tax legally recognized religious/fraternal institutions in the Registro de Asociaciones and international non-profits. No donor-deduction regime.</t>
         </is>
       </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked: no independent charity sector exists, and banks serve residents/authorized state entities; even personal MLC accounts require temporary residence permits, not tourist status.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -953,6 +974,11 @@
           <t>Separate Charities Authority registration (Charities Act 2013); registered charity income exempt (Income Tax Act s.13); Finance Minister gazette approval enables donor deduction, capped at 1/20 of statutory income.</t>
         </is>
       </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (NCB, CIBC) open non-resident accounts, but non-residents must be physically present at a branch with passport plus a second ID; no fully remote onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -1040,6 +1066,11 @@
           <t>Company limited by guarantee (Companies Act 2019) with charitable objects; no separate charitable tax-exempt approval located - status not automatically tax-exempt and no donor-deduction scheme identified in law.</t>
         </is>
       </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: Bahamian banks open non-resident accounts under central-bank FATF KYC guidance, but the applicant must appear in person for identity verification; remote opening is rare.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1127,6 +1158,11 @@
           <t>CAIPO registration with charitable objects; income tax exemption (Income Tax Act Cap.73, amended 2024) only for charities on the First Schedule exemption list; donor deduction for listed charities. Time unpublished.</t>
         </is>
       </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks accept non-resident accounts, but non-residents must be present for account opening (CIBC rule); online application only pre-fills the branch completion.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1214,6 +1250,11 @@
           <t>Ministry of Finance 'approved charity' status; donors deduct covenanted donations up to 15% of income; charity exempt from income tax (Income Tax Act Ch.79:04). No deduction without approval. Time unpublished.</t>
         </is>
       </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: non-residents must appear at a branch (First Citizens, Republic Bank) with passport, three-month utility bill or lease as address proof; no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1301,6 +1342,11 @@
           <t>Automatic: Income Tax Act Cap.212 s.8(d) exempts income of ecclesiastical, charitable or educational institutions of public character, as far as not from trade. No separate application; no donor-deduction scheme.</t>
         </is>
       </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (Trium, A&amp;B Bank) accept non-resident and corporate accounts with enhanced due diligence, but an in-person branch visit by the signatory is the standard route.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1388,6 +1434,11 @@
           <t>Automatic by category: Income Tax Act Cap.149 s.25(1)(q) exempts religious/charitable/educational institutions of public character not trading for profit; donors deduct donations to Comptroller-approved organizations.</t>
         </is>
       </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (Grenada Co-op, Republic Bank) accept non-national accounts with two IDs, but the applicant/signatory must appear in person at a branch; no fully remote route.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1475,6 +1526,11 @@
           <t>Income Tax Act Ch.20.22 s.7 lists category exemptions; donations to charities registered with CAIPO are deductible (PwC); the institution's own income-tax exemption is not confirmed in accessible text. Time unpublished.</t>
         </is>
       </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit plus enhanced AML diligence: banks apply enhanced due diligence to non-residents (purpose, expected transactions); in-person branch appearance is standard for individual and corporate accounts.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1562,6 +1618,11 @@
           <t>Donors deduct contributions under deeds of covenant of at least 3 years to approved religious/charitable/medical/educational institutions (Income Tax Act Cap.15.02), capped at 25% of income; own exemption unconfirmed.</t>
         </is>
       </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: CIBC and others open non-resident accounts, but non-residents must be physically present with two forms of ID; Bank of St. Lucia runs a dedicated non-national onboarding path.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1649,6 +1710,11 @@
           <t>Automatic: Income Tax Act Cap.435 s.44(o) exempts religious/charitable/educational institutions of public character not from profit business; s.58 donor deduction for covenanted donations, capped 5% of assessable income.</t>
         </is>
       </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (BOVSG, Republic) accept non-resident accounts with overseas addresses, but in-person branch appearance by the signatory is standard; offshore desks may be more flexible.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1736,6 +1802,11 @@
           <t>Income Tax Act ch.67:01 s.25 exempts charitable institutions by category; donor deduction only if the institution is on the Cabinet-approved list (last update S.R.O 47 of 2007). Incorporation alone gives no tax status.</t>
         </is>
       </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit, easiest of the Caribbean: the FSU requires no local connection; non-resident individual and corporate accounts are accepted with source-of-funds documentation, in person.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1823,6 +1894,11 @@
           <t>PGR registration (Ley 122-05) then separate DGII exemption application (ASFL regime) for ISR + ITBIS exemption and donor deduction (Ley 112-05 art.35, up to 15% of taxable income). DGII time unpublished.</t>
         </is>
       </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: major banks (Popular, BHD, Santa Cruz) open non-resident accounts with a valid passport, often without address proof; corporate accounts still need an in-person director visit.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1910,6 +1986,11 @@
           <t>ONG registration under the 14 Sept 1989 decree gives legal status only; DGI grants the corporate income tax exclusion by separate decision - statutory basis not confirmed in accessible text; time unpublished.</t>
         </is>
       </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: per US trade guidance, foreigners can open USD/HTG accounts immediately with passport and a minimum deposit, but the process is in person in Port-au-Prince; no remote KYC.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1997,6 +2078,11 @@
           <t>SAT 'donataria autorizada' authorization (Ficha 19/ISR, Anexo 2); SAT resolves within max 3 months. Income from authorized activities exempt from ISR; donors deduct 50% of gift, up to 15% of taxable income (LISR art.23).</t>
         </is>
       </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (Scotiabank, BBVA) open non-resident accounts with passport, migratory document and SAT RUT; in-person branch visits are the norm and fully remote opening is rare.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -2084,6 +2170,11 @@
           <t>Automatic by category: Income Tax Law exempts NPOs with charitable/educational/cultural objectives from income tax; donor deductions up to 25% of total income. MINGOB reconocimiento is separate from registration.</t>
         </is>
       </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit plus RUT: banks require in-person appearance and an active RUT (tax registration, obtainable by foreigners); passport-only accounts are often restricted to legal residents (e.g. BAM).</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2171,6 +2262,11 @@
           <t>Automatic: Income and Business Tax Act Cap.55 exempts earnings of ecclesiastical, charitable and educational institutions; individual donor relief for charitable contributions capped at BZ$250. No separate application.</t>
         </is>
       </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: the central bank delegated non-resident account authority to domestic banks (Atlantic, Caye International), which accept non-residents with low minimums; in-person branch visits standard.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2258,6 +2354,11 @@
           <t>Separate DGII 'calificacion' as public-utility entity required for ISR exemption (LAFSFL art.7); registration alone confers no tax status; donations to such entities deductible. 2025 law: 30% levy on foreign NGO funds.</t>
         </is>
       </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: major banks (Banco Agrícola, Cuscatlán) accept foreigners; a passport may open a basic savings account, but full access typically needs a Salvadoran NIT and in-person KYC.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2345,6 +2446,11 @@
           <t>No separate published charitable tax-exempt application; incorporation with charitable objects gives legal personality only. Donations to charitable/educational institutions deductible up to 10% of net taxable income.</t>
         </is>
       </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks require the applicant to appear with passport, residency/visa proof and an NIT (tax registration); a remote founder would need a local agent or an in-person trip.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2432,6 +2538,11 @@
           <t>Not automatic: apply to the DGI (Ministry of Finance) proving income serves charitable purposes (LCT art. 32, 2024 reform) for ISR exemption; no general donor deduction; approval time unpublished.</t>
         </is>
       </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>In-person visit required; non-resident foreigners need passport plus a second photo ID and typically two personal/professional references; remote opening not offered.</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2519,6 +2630,11 @@
           <t>Separate application: file with the Dirección General de Hacienda via Exonet (Ley 10.286/2022) for ISR exemption of income devoted to charitable aims. Donors deduct 100% (Ley 9.637). Approval usually months.</t>
         </is>
       </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Most banks require DIMEX residency per SUGEF KYC rules; non-residents can open only a simplified in-person account with low monthly deposit caps, unsuitable for a charity.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2606,6 +2722,11 @@
           <t>Non-profit income exempt under the Código Fiscal if devoted to its purpose (DGI verifies at filing). Donor deductions require a separate DGI authorization; DGI revoked such benefits in 2025; timing unpublished.</t>
         </is>
       </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>Non-residents may open accounts in-person with passport, foreign address proof, home-bank reference and income proof; AML Law 23 KYC and an interview apply; no residency needed.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2693,6 +2814,11 @@
           <t>No separate tax step: ESALs are special-regime taxpayers (art. 19 E.T.); DIAN exempts non-distributed income where bylaws show a charitable general-interest purpose. Donors deduct up to 15% of taxable income.</t>
         </is>
       </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>Requires cédula de extranjería (residency ID) plus local address proof; tourist status is rejected; in-person visit at the branch is mandatory.</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2780,6 +2906,11 @@
           <t>ISLR art. 14.3: charitable/social-assistance entities whose gains fund their purpose and never distribute profits are exempt — legal, automatic; SENIAT verifies at filing, no separate certificate.</t>
         </is>
       </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for remote foreigners: banks require cédula de extranjero residency and in-person application; no remote opening; currency controls add friction.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2867,6 +2998,11 @@
           <t>Exemption under LRTI art. 9.5 applies to income of private non-profits devoted to their purpose (circular NAC-DGECCGC24-00000006): no separate status; SRI verifies, entity files annual returns. Donors deduct 50%.</t>
         </is>
       </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>In-person; most banks want an Ecuadorian cédula, but some (e.g. Banco del Pacífico) accept a passport with a valid visa plus reference under Superintendencia de Bancos rules.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2954,6 +3090,11 @@
           <t>Separate step: register in the SUNAT “registro de entidades exoneradas del Impuesto a la Renta” (LIR art. 19: educational, scientific, charitable aims). Donors partial deduction; IGV on sales; time unpublished.</t>
         </is>
       </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>In-person; full accounts at major banks need a Carné de Extranjería (residency card); a few banks open passport-only savings for non-residents, generally with limits.</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -3041,6 +3182,11 @@
           <t>Not automatic: formalize the IUE (corporate profit) exemption with the SIN (RND 10-0030-05; Ley 843 art. 4) proving charitable purpose and non-distribution. Donor deductions limited (5%/10%); time unpublished.</t>
         </is>
       </c>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>Blocked for non-residents: banks require a Cédula de Identidad de Extranjero and in-person application (ASFI-regulated); tourist status is not enough.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3128,6 +3274,11 @@
           <t>No general non-profit exemption: the Income Tax Act grants only specific reliefs; the GRA's Tax Exemption, Processing &amp; Verification Division issues individual exemption certificates to qualifying non-profits.</t>
         </is>
       </c>
+      <c r="R30" s="2" t="inlineStr">
+        <is>
+          <t>In-person visit required with passport, address proof, TIN and source-of-funds disclosure; no statutory ban, but offshore non-resident accounts still need a face-to-face meeting.</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3215,6 +3366,11 @@
           <t>No automatic charitable exemption: a stichting is taxed as an ordinary legal person (35% income tax on business income); individual exemptions must be requested from the Inland Tax Administration (Dib); VAT applies.</t>
         </is>
       </c>
+      <c r="R31" s="2" t="inlineStr">
+        <is>
+          <t>No legal residency restriction on foreigners per central-bank guidance; opening is in-person at the bank with passport, address and (often) a foreign bank reference letter.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3302,6 +3458,11 @@
           <t>Income-tax exemption (IRPJ/CSLL/COFINS) for a qualifying non-profit is legal and automatic (Lei 9.532; NFPS) — Receita Federal verifies accounts, no separate recognition. Donor deduction needs utilidade pública/OSCIP.</t>
         </is>
       </c>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked remotely: banks require CRNM residency, CPF and a Brazilian address with in-person KYC; non-residents are limited to special non-tax-resident (CDE) products.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -3389,6 +3550,11 @@
           <t>Exemption is legal and automatic: Ley 6.380/19 art. 25.2c exempts income of non-profit associations/foundations that do not distribute (DNIT verifies at filing). Donor deduction limited (5% for individuals).</t>
         </is>
       </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>Requires a Paraguayan cédula (residency ID) and in-person presence; a passport alone is not accepted by the major banks, so remote opening is not possible.</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3476,6 +3642,11 @@
           <t>IRAE exemption of income of qualifying non-profits (educational, cultural, scientific, charitable) is legal and automatic; DGI verifies the purpose. The 75%-refund donor benefit requires listing in the MEF regime.</t>
         </is>
       </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>Most open to non-residents: BROU allows a basic in-person account with home-country address, but requires a US$5,000+ fixed deposit held 181 days for new non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3563,6 +3734,11 @@
           <t>Separate certificate required: file DJ 953 with ARCA (ex-AFIP) for “certificado de exención” of Impuesto a las Ganancias (Ley 23.349, reg. 1457) — general or simplified route. Benefits: no income tax, no withholding.</t>
         </is>
       </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>In-person at a branch; non-residents can open an account with passport and CUIT/CUIL under BCRA rules; peso savings available even without a DNI, with tighter limits.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3650,6 +3826,11 @@
           <t>No general entity exemption: fundaciones/corporaciones pay IUS on income. Benefit is for donors: Ley 19.885 gives a 15% credit (individuals) if the entity has ministry-recognized interés público status.</t>
         </is>
       </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>In-person; requires a RUT (foreigners with a valid visa can get a provisional one) and ID per ChileAtiende rules; non-residents without RUT/visa are effectively blocked.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3737,6 +3918,11 @@
           <t>The National Tax Authority exempts corporate income of registered non-profits whose income is used for charitable, educational, scientific or social purposes — applied by the tax office, no separate charitable status.</t>
         </is>
       </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>In-person in Ulaanbaatar with passport, visa and registered address proof; opening from abroad typically requires a local lawyer with power of attorney; remote opening not possible.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3824,6 +4010,11 @@
           <t>No blanket exemption: NPOs pay corporate tax only on business (shu-eigyo) income; public-benefit certification (prefecture, months) makes public-interest activity income tax-free and donations deductible.</t>
         </is>
       </c>
+      <c r="R38" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked remotely: non-residents (under 6 months in Japan) cannot open standard accounts; in-person with residence card required, Japan Post Bank being the main exception.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3911,6 +4102,11 @@
           <t>No separate application: NTS automatically exempts the public-interest income of a foundation (재단법인) under the Special Tax Benefits Act art. 6, verified at filing. Donors: up to 100% deduction (individuals).</t>
         </is>
       </c>
+      <c r="R39" s="2" t="inlineStr">
+        <is>
+          <t>Requires the Alien Registration Card (ARC), i.e. registered residence in Korea, plus in-person application; a remote foreign founder without local presence cannot open an account.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3998,6 +4194,11 @@
           <t>Two separate steps after registration: (1) non-profit tax-exemption qualification from local tax + finance (Caishui [2018] No. 107, 5-year); (2) public-donation pre-tax deduction qualification (2020 Announcement 27).</t>
         </is>
       </c>
+      <c r="R40" s="2" t="inlineStr">
+        <is>
+          <t>Blocked remotely: PBOC/SAFE real-name rules require physical presence, a non-tourist visa, a Chinese mobile number and local address, with in-person branch verification.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -4085,6 +4286,11 @@
           <t>A private foundation registers with the county/city government; the local tax bureau applies charitable-income exemption (Income Tax Act art. 4) from its bylaws. Donor deduction needs ministry qualification.</t>
         </is>
       </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>In-person at a branch; foreigners need an Alien Resident Certificate (or Gold Card) plus in-branch identity verification; no online/remote opening for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4172,6 +4378,11 @@
           <t>Separate IRD endorsement under s.88 Inland Revenue Ordinance (charitable purpose, trust deed). Grants profits-tax exemption; donors deduct gifts up to 35% of assessable income. No VAT. Processing time unpublished.</t>
         </is>
       </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: non-residents cannot onboard online; banks (HSBC, BOC, SCB) require in-person branch KYC under AML/CDD rules, with tightened non-resident scrutiny since 2023.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -4259,6 +4470,11 @@
           <t>No general charity tax regime. Foundations/associations apply to DSSCU for case-by-case profits-tax exemption; approval discretionary, timeline unpublished. No donor-deduction scheme exists in Macau.</t>
         </is>
       </c>
+      <c r="R43" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: BNU e-Application is limited to Macau ID holders; banks require in-person KYC with Macau residency/tax-residency documents. No remote onboarding for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4346,6 +4562,11 @@
           <t>Separate IPC endorsement from IRAS under s.37 Income Tax Act (Commissioner of Charities applies post-registration): full income-tax exemption; corporate donors get 250%, individuals 100% deduction. No VAT.</t>
         </is>
       </c>
+      <c r="R44" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: DBS, OCBC and UOB run enhanced due diligence on foreign-owned charities and typically require an in-person branch appointment; remote onboarding is limited to existing customers.</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4433,6 +4654,11 @@
           <t>LHDN approval under s.44(6) Income Tax Act 1967 (charitable body, max 10 yrs) for income-tax exemption; approved-body donations deductible (individuals cap 10% of aggregate income). Application 1-3 months.</t>
         </is>
       </c>
+      <c r="R45" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks gate accounts on visa/residency status, require in-person branch KYC, and often ask for a local resident director or introducer; no remote onboarding for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4520,6 +4746,11 @@
           <t>No separate application. Income used directly for non-distributive charitable activity is exempt from PPh (Art.4(3)); donations to recognized bodies deductible; most activities no VAT. Registration confers no tax status.</t>
         </is>
       </c>
+      <c r="R46" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: online onboarding is unavailable to non-residents; banks require an in-person application with KITAS/KITAP, local address and passport under OJK AML rules.</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -4607,6 +4838,11 @@
           <t>Foundation/association applies to Revenue Department for a tax-exemption certificate (income tax) before benefits; donors deduct gifts up to 10% of net income, some foundations double-deducted via e-Donation. No VAT.</t>
         </is>
       </c>
+      <c r="R47" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: major banks (SCB, KBank, Bangkok Bank) require in-person application, a long-stay non-immigrant visa, Thai address and local mobile number; tourist-visa holders are refused.</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4694,6 +4930,11 @@
           <t>Charitable fund (Decree 03/2026) gets fund income used for charitable purposes exempt from income tax; donors deduct up to 30% of taxable income. Exemption follows license, processed by tax authority within ~15-30 days.</t>
         </is>
       </c>
+      <c r="R48" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: under State Bank Circular 23/2014, in-person application with passport plus valid visa or residence card (TRC) is required; since 2022 big banks refuse tourist-visa holders.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -4781,6 +5022,11 @@
           <t>BIR exemption ruling under s.30(E) NIRC required separately from SEC registration for income-tax exemption of donations; donor deduction capped at 20% of net income (itemized). Weeks to months; time unpublished.</t>
         </is>
       </c>
+      <c r="R49" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (BDO, BPI, Security) require in-person KYC with passport, long-term visa, ACR I-Card (issued only after an extended stay) and local address; no remote onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4868,6 +5114,11 @@
           <t>No general charity tax regime. Associations/NGOs registered at Ministry of Interior must apply to GDT (MoEF) for case-by-case income-tax exemption; INGOs get duty-free import status via MoU. No standard donor deduction.</t>
         </is>
       </c>
+      <c r="R50" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit but is easy: ABA/ACLEDA open accounts for non-residents in person with passport plus any Cambodian visa, no work permit; no fully remote online option.</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4955,6 +5206,11 @@
           <t>No charitable tax-exemption regime in the Income Tax Law. Exemptions only via investment promotion or special government approval, case-by-case; no public donor-deduction scheme. Social organisations pay standard CIT.</t>
         </is>
       </c>
+      <c r="R51" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: BCEL/Canadia require in-person KYC with a work permit or stay permit; non-residents with no local presence are generally refused. No remote onboarding available.</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -5042,6 +5298,11 @@
           <t>Non-profits register TIN with IRD, then apply to Director General for income-tax exemption certificate (Not 79/2020); donors deduct gifts to approved organisations subject to IRD caps. Months; time unpublished.</t>
         </is>
       </c>
+      <c r="R52" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for remote founders: in-person KYC with work visa, local address and often an introducer is required; no remote non-resident onboarding at KBZ, Yoma or AYA Bank.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -5129,6 +5390,11 @@
           <t>No personal income tax; corporate tax only. Charitable societies gain no automatic tax status on registration under Societies Act; exemption only by Minister's discretion under Income Tax Act. No donor-deduction regime.</t>
         </is>
       </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (Bank Islam, MUFG, OCBC) require in-person application with passport, employment/dependent pass and local address; no remote onboarding for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -5216,6 +5482,11 @@
           <t>Associations/foundations register with Ministry of Justice, then apply to the Tax Authority (ATT) for 10% income-tax exemption; approval case-by-case, time unpublished. No general donor-deduction scheme.</t>
         </is>
       </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: non-residents open accounts in person at BNCTL/ANZ/BNU with passport plus visa; banks typically require a local tax ID; no remote onboarding available.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -5303,6 +5574,11 @@
           <t>ACNC registration alone confers no tax benefit. ATO endorsement required separately: income-tax exemption, DGR status (donors claim 30% credit), GST/FBT concessions. DGR endorsement weeks to months; time unpublished.</t>
         </is>
       </c>
+      <c r="R55" s="2" t="inlineStr">
+        <is>
+          <t>Fully online: an AU-resident founder can open accounts at CBA, Westpac, ANZ or NAB via eKYC with passport or driver licence and overseas address proof; no in-person visit needed.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5390,6 +5666,11 @@
           <t>Automatic: Charities Services notifies Inland Revenue on charity registration - income-tax exemption on charitable income follows; donee status (33 1/3% donor tax credit) then granted by IRD. Days to weeks; no VAT.</t>
         </is>
       </c>
+      <c r="R56" s="2" t="inlineStr">
+        <is>
+          <t>Possible online: ANZ, ASB, BNZ and Westpac accept non-resident applications with passport plus proof of address, but most banks require an in-person branch visit within ~12 months to activate.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5477,6 +5758,11 @@
           <t>Automatic: entities registered under the Charitable Trusts Act are exempt from income tax without separate application (FRCS). Donors claim deduction for contributions to FRCS-listed approved charities. No VAT.</t>
         </is>
       </c>
+      <c r="R57" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: in-person KYC with passport and a Fijian TIN (FRCS) is required; RBF-regulated banks (BSP, ANZ, Westpac) offer no remote onboarding for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5564,6 +5850,11 @@
           <t>Non-profits must register a TIN with the IRC and apply for income-tax exemption from the IR (charitable purpose); donors deduct gifts of PGK50+ to qualifying charitable organisations. Approval time unpublished.</t>
         </is>
       </c>
+      <c r="R58" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit, effectively blocked for pure non-residents: Kinabank Digi requires a PNG driver licence and branches expect local presence; expect a full in-person KYC.</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5651,6 +5942,11 @@
           <t>Income Tax Act 2012 gives donors a 30% tax credit for gifts to approved charitable institutions; the entity's own exemption is handled case-by-case by the Ministry for Revenue - process and time unpublished.</t>
         </is>
       </c>
+      <c r="R59" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: ANZ Samoa and local banks require in-person application with passport, local address and residency/work permit; no remote onboarding for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5738,6 +6034,11 @@
           <t>Charitable organisations are income-tax exempt (except business income) by Revenue Services under the Income Tax Act; donor deduction for registered charities. Application details and time unpublished.</t>
         </is>
       </c>
+      <c r="R60" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: BSP and other banks require in-person KYC with passport, local address and residency/work permit; no remote onboarding for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5825,6 +6126,11 @@
           <t>No corporate income tax - no entity-level income tax, so registration with the VFSC (also Registrar of Charitable Organisations) needs no tax-exemption application. VAT exemptions cover some charitable supplies.</t>
         </is>
       </c>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>Relatively easy: RCV-licensed banks (ANZ, NAB, Bank of the Pacific, WES, Melanesia) offer non-resident multi-currency accounts; in-person branch KYC, or via a local representative.</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5912,6 +6218,11 @@
           <t>Charitable-society income is statutorily exempt under the Income Tax Act (Cap. 123) if applied to charitable purposes - no separate tax application; donations to charities are not deductible; timing unpublished.</t>
         </is>
       </c>
+      <c r="R62" s="2" t="inlineStr">
+        <is>
+          <t>In-person KYC at branch (ANZ, BRED, Westpac) for all accounts; passport plus local ID; foreign-currency accounts possible; no remote onboarding for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5999,6 +6310,11 @@
           <t>A company or irrevocable trust applies to the tax Commissioner under the Income Tax Act 2023; approved non-profits have exempt income; donations to them are deductible; no VAT relief; timing unpublished.</t>
         </is>
       </c>
+      <c r="R63" s="2" t="inlineStr">
+        <is>
+          <t>In-person at ANZ Kiribati, the only licensed bank (Bairiki/Tarawa branch); non-residents face heavy AML restrictions and no remote onboarding for foreign founders.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -6086,6 +6402,11 @@
           <t>Separate certification by the Finance Secretary under Business Tax Act 2016 s.6 (charitable/educational/sporting/religious purpose, no profit split); certified non-profits are exempt from business tax.</t>
         </is>
       </c>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for remote founders: CommBank agencies (Aiwo, Ewa) and Bank of Nauru onboard only in person and target residents; no remote onboarding exists.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -6173,6 +6494,11 @@
           <t>Charitable and benevolent organisation income is exempt under the Income Tax Act 1992 exempt-income schedule (purposive test, no separate tax application); no donor-deduction regime and no VAT; time unpublished.</t>
         </is>
       </c>
+      <c r="R65" s="2" t="inlineStr">
+        <is>
+          <t>In-person at National Bank of Tuvalu (Funafuti only, plus rare field visits); passport plus residence proof required; no remote onboarding; ANZ branch closed in 2024.</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -6260,6 +6586,11 @@
           <t>Not automatic: the Non-Profit Entities Act 2020 requires a non-profit to apply to the Department of Revenue for exemption from the 3% Net Profit Tax; no donor-deduction regime; timing unpublished.</t>
         </is>
       </c>
+      <c r="R66" s="2" t="inlineStr">
+        <is>
+          <t>Local banks (BancFirst, Mid Pacific Bank) require in-person KYC in Majuro; Marshall Islands IBCs are barred from local accounts, so remote foreign founders are effectively blocked.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -6347,6 +6678,11 @@
           <t>No separate charitable exemption: FSM corporate income tax hits only 'major corporations' ($1M+ equity), so a small non-profit is out of scope; state-level taxes may apply; no donor deduction; timing unpublished.</t>
         </is>
       </c>
+      <c r="R67" s="2" t="inlineStr">
+        <is>
+          <t>In-person at Bank of FSM (Chagol); passport, TIN from Dept. of Finance, local address and initial deposit; no remote onboarding for non-resident foreign founders.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -6434,6 +6770,11 @@
           <t>Vakif registered with the Foundations Affairs Presidency; foundations are exempt from corporate tax on charitable income; donors deduct gifts up to 10% of taxable profit (uncapped for listed); no VAT exemption.</t>
         </is>
       </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>In-person branch visit; passport, Turkish tax number, local SIM and address proof; non-residents allowed under BDDK/AML rules but no remote route for account opening.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -6521,6 +6862,11 @@
           <t>Charitable status confirmed by the State Tax Service (charitable purpose, no profit distribution); charitable income exempt; donors deduct gifts up to 10% of taxable income (art. 117); 1-month decision.</t>
         </is>
       </c>
+      <c r="R69" s="2" t="inlineStr">
+        <is>
+          <t>Remote opening possible via notarised power of attorney to a local representative (2-4 weeks, full KYC, refusals possible); in-person alternative also available.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -6608,6 +6954,11 @@
           <t>NPOs registered with the Justice Ministry; donations and goods for charity are VAT-exempt and charitable activity is profit-tax-privileged; donor deduction capped at 0.25% of taxable profit.</t>
         </is>
       </c>
+      <c r="R70" s="2" t="inlineStr">
+        <is>
+          <t>Partially remote-friendly: Evocabank onboards non-residents fully online via app; other banks (Amria, Converse) require an in-person branch visit or POA under Central Bank AML rules.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -6695,6 +7046,11 @@
           <t>No automatic income-tax exemption: NCOs pay 20% profit tax; Tax Code art. 106.1.18 adds a limited donor deduction for supporting social-purpose foundations (2023); no VAT exemption.</t>
         </is>
       </c>
+      <c r="R71" s="2" t="inlineStr">
+        <is>
+          <t>Central Bank allows non-resident accounts but banks routinely demand a residence permit and an in-person branch visit; no remote onboarding; AML checks strict.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -6782,6 +7138,11 @@
           <t>NPOs registered with the Justice Committee under the Tax Code's NPO regime: charitable contributions received are not income and charitable operations are VAT-exempt; donors get a limited deduction (2022).</t>
         </is>
       </c>
+      <c r="R72" s="2" t="inlineStr">
+        <is>
+          <t>Since April 2025 non-resident accounts open only via e-Residency partner banks with their own AML/KYC checks; IIN required; in-person card issuance; refusals common.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -6869,6 +7230,11 @@
           <t>Registered with the Justice Ministry; 'charitable organization' status itself gives no special benefit - registered NNOs are generally income-tax exempt on non-commercial charitable income.</t>
         </is>
       </c>
+      <c r="R73" s="2" t="inlineStr">
+        <is>
+          <t>Remote opening for non-residents allowed under Central Bank procedure in force since May 2023; TBC UZ app supports app KYC with courier signing; in-person also possible.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -6956,6 +7322,11 @@
           <t>Associations need Justice Ministry consent plus state registration; a charity foundation can only be created by government decree (5+ citizen founders); law provides tax benefits, detail sparse.</t>
         </is>
       </c>
+      <c r="R74" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for remote founders: no remote onboarding; foreigners need local work/residence status and in-person branch visit with originals under strict currency-control rules.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -7043,6 +7414,11 @@
           <t>Public associations registered with the Justice Ministry; NPO income from charitable activity and donations is income-tax exempt under the Tax Code (2023 NCO tax guide); no donor deduction.</t>
         </is>
       </c>
+      <c r="R75" s="2" t="inlineStr">
+        <is>
+          <t>In-person at local banks (National Bank instruction on account opening); non-residents need full registered-entity documents and signature cards; no remote onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -7130,6 +7506,11 @@
           <t>Charitable funds registered with the State Registration Service; tax status requires charitable purpose and no profit split; charity profits are income-tax exempt (Tax Code art. 212); no donor deduction.</t>
         </is>
       </c>
+      <c r="R76" s="2" t="inlineStr">
+        <is>
+          <t>23 commercial banks accept non-resident accounts; in-person branch visit with passport, beneficial-owner questionnaire and entity registration documents; no full-remote route.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -7217,6 +7598,11 @@
           <t>Registered NGOs (Interior Ministry) are exempt on donations, gifts and membership fees under Direct Taxation Act art. 139 if used for charter purposes per National Tax Administration approval.</t>
         </is>
       </c>
+      <c r="R77" s="2" t="inlineStr">
+        <is>
+          <t>Money and Credit Council rules allow foreign Rial deposit accounts, but in-person ID verification is mandatory; sanctions/AML environment leaves no realistic remote onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -7304,6 +7690,11 @@
           <t>Association declared with the Interior Ministry; ONG status needs a separate 'agrement'; recognised ONGs are exempt from income tax, registration duties and VAT (Law 99/014 art. 18); no donor-deduction regime.</t>
         </is>
       </c>
+      <c r="R78" s="2" t="inlineStr">
+        <is>
+          <t>In-person branch visit under BEAC/CEMAC rules; NGO accounts additionally need Interior Ministry reconnaissance; foreigner onboarding requires passport and physical presence; no remote.</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -7391,6 +7782,11 @@
           <t>Association declared under the civil code; ONG status requires the state's administrative 'agrement' (ONG law) to act nationally; the CGI grants limited exemptions to recognised ONGs; detail sparse.</t>
         </is>
       </c>
+      <c r="R79" s="2" t="inlineStr">
+        <is>
+          <t>In-person at local banks (COBAC-supervised, mostly Bangui) after arrival; passport and entity documents; ONG accounts need administrative agrement; no remote onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -7478,6 +7874,11 @@
           <t>Association registered with the Interior Ministry (Ordinance 023/PR/2018); international NGOs need extra authorisation (Law 05/2012); no charitable income-tax exemption - NPO income faces 10% profit tax.</t>
         </is>
       </c>
+      <c r="R80" s="2" t="inlineStr">
+        <is>
+          <t>In-person at N'Djamena banks under COBAC rules; NGO accounts require CICA and Interior Ministry agreement; non-resident remote onboarding not available.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -7565,6 +7966,11 @@
           <t>Legal personality is automatic by declaration at the prefecture under the 1901 French law; no automatic charitable tax exemption - income taxed under the CGI; 'reconnaissance d'utilite publique' is separate.</t>
         </is>
       </c>
+      <c r="R81" s="2" t="inlineStr">
+        <is>
+          <t>In-person at CEMAC banks (SG CIB, BICEC etc.); association accounts need prefecture declaration/registration; no remote onboarding for non-resident foreign founders.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -7652,6 +8058,11 @@
           <t>ASBL/EUP registration (Law 004/2001) makes it a public-utility entity: automatic income-tax exemption on non-commercial activities, customs relief, and donor deduction under DGI rules; no separate application.</t>
         </is>
       </c>
+      <c r="R82" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked remotely: banks (BCC-supervised) require in-person branch visit, local tax ID (NIF) and local address; no remote onboarding for non-resident entities.</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -7739,6 +8150,11 @@
           <t>Declaration to the prefecture gives legal personality (Law 35/62); 2022 tax reform auto-exempts associations from CIT on social/educational/cultural/religious member services. No separate application.</t>
         </is>
       </c>
+      <c r="R83" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: CFA-CEMAC banks (BGFI, BICEC, SGB) require in-person KYC with passport, residence permit and local address; remote opening not available for foreign entities.</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -7826,6 +8242,11 @@
           <t>ONG registration with the Interior Ministry (Law 1/1999) confers public-utility status; corporate-tax exemption for non-commercial income under the 2004 Tax Law. No published approval time.</t>
         </is>
       </c>
+      <c r="R84" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: BANGE/BGFIBank branches require in-person appearance with passport/residence card and local address; no remote onboarding for non-residents; rules not fully verified.</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -7913,6 +8334,11 @@
           <t>NGO law (Lei 8/2012) registers associations and foundations, but the tax code has no specific charitable-exemption regime; no automatic income-tax exemption, relief is case-by-case; no published time.</t>
         </is>
       </c>
+      <c r="R85" s="2" t="inlineStr">
+        <is>
+          <t>Personal accounts can be opened remotely by intermediaries, but an NGO corporate account in practice needs in-person KYC in the capital with local address and NIF tax number.</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -8000,6 +8426,11 @@
           <t>RGB certificate of legal personality (NNGO) grants tax-exempt status under the 2022 Income Tax Law for public-interest missions; donor gifts deductible up to 1% of company turnover. INGOs need separate RGB authorization.</t>
         </is>
       </c>
+      <c r="R86" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (Bank of Kigali, I&amp;M, KCB) require physical attendance for in-person interview under AML Law 75/2019; non-resident business accounts need a trip to Kigali.</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -8087,6 +8518,11 @@
           <t>ASBL registration with the Interior Ministry (Law 1/02, 2017); tax and customs relief for NGOs granted case-by-case by the OBR under the ONG framework law. No separate exemption status; no published time.</t>
         </is>
       </c>
+      <c r="R87" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks in Bujumbura (BCB, BCB) require in-person appearance with passport and proof of residence; standard AML/CFT checks, no remote opening for foreign entities.</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -8174,6 +8610,11 @@
           <t>NGO Bureau registration (NGO Act 2016) first, then URA application for charitable status: exempts income of religious/charitable/educational/public institutions (2024 Amendment Act); donor deduction available.</t>
         </is>
       </c>
+      <c r="R88" s="2" t="inlineStr">
+        <is>
+          <t>In-person at major banks (Stanbic, Absa, DFCU): passport, URA TIN, board resolution and named signatories; no local address required for foreign-registered entities, no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -8261,6 +8702,11 @@
           <t>Charitable status is not automatic: NGO registration plus separate TRA approval; Finance Act 2024 added health and environmental protection as qualifying purposes. Donor gifts deductible up to 10% of income.</t>
         </is>
       </c>
+      <c r="R89" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (CRDB, NMB, Stanbic) require in-person application with passport, TIN and proof of residence; foreign NGOs register at national level; no remote onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -8348,6 +8794,11 @@
           <t>PBO status from PBORA, then a separate KRA application for income-tax exemption under Income Tax Act para 10: exempts qualifying receipts; donor deduction (30%). Approval takes several months; no deadline published.</t>
         </is>
       </c>
+      <c r="R90" s="2" t="inlineStr">
+        <is>
+          <t>In-person at branch under CBK AML/KYC rules; NGO accounts require at least one Kenyan-resident board member as signatory plus an NGO Board recommendation letter, so a local representative is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -8435,6 +8886,11 @@
           <t>Associations declared under Law 86-006/AF; international NGOs need ministerial agrément. CGI (2011) corporate tax applies only to commercial activities; no separate charitable-exempt status regime; no published time.</t>
         </is>
       </c>
+      <c r="R91" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: opening an account in Moroni requires in-person appearance with passport, residence permit and local address; offshore non-resident accounts do not suit charity banking.</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -8522,6 +8978,11 @@
           <t>Legal personality on declaration (Law 96-030/97, Decree 98-711); approved ONGs get exemptions on import duties and certain taxes under the law's fiscal/customs chapter; no separate donor-deduction regime published.</t>
         </is>
       </c>
+      <c r="R92" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (BOA, BMOI, MCB) require in-person appearance with passport, residence permit, local address proof and NIF tax ID; minimum deposit, no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -8609,6 +9070,11 @@
           <t>NGO Board registration (NGO Act 2009), then ZRA application for public-benefit-organisation status: exempt qualifying charitable income; donors may deduct gifts up to 15% of taxable income. No published processing time.</t>
         </is>
       </c>
+      <c r="R93" s="2" t="inlineStr">
+        <is>
+          <t>In-person at branch: ZRA TPIN mandatory, local address proof (&lt;3 months) and in-person signature collection; foreign NGOs need resident directors/signatories per bank CDD.</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -8696,6 +9162,11 @@
           <t>NGO Board registration; Taxation Act exempts income of clubs/societies operated for social welfare or civic improvement; donors get deduction for donations to public charitable organisations. No published approval time.</t>
         </is>
       </c>
+      <c r="R94" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks in Lilongwe/Blantyre (StandChart, Centenary, FCB) require in-person appearance with passport, TIN and local address proof; no remote onboarding for foreign entities.</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -8783,6 +9254,11 @@
           <t>Association (Lei 8/91) is automatically IRC-exempt (Art. 10, Law 34/2007) if it pursues public-interest objectives without commercial activity; donors deduct donations as a fiscal benefit.</t>
         </is>
       </c>
+      <c r="R95" s="2" t="inlineStr">
+        <is>
+          <t>Non-residents may open accounts with NUIT tax ID, but in-person branch visit is required (BCI, Millennium BIM, FNB); foreign-authorized NGOs need local address and resident signatories.</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -8870,6 +9346,11 @@
           <t>Law 2/26 (2026) grants registered ONGs tax and customs benefits, incl. duty-free import of project goods; no separate donor-deduction regime; no published processing time.</t>
         </is>
       </c>
+      <c r="R96" s="2" t="inlineStr">
+        <is>
+          <t>In-person only (no online option): NIF tax ID is the usual bottleneck, plus passport with valid visa/resident card at a branch; banks cannot onboard foreign entities remotely.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -8957,6 +9438,11 @@
           <t>Income Tax Act historically exempted charitable/religious/educational institutions; the 2025 Income Tax Bill replaces this with a conditional NPO regime needing approval. Donor gifts to approved institutions deductible.</t>
         </is>
       </c>
+      <c r="R97" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (StandChart, FNB, Stanbic) typically require a residence permit and in-person appearance with local address; remote onboarding not available for foreign entities.</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -9044,6 +9530,11 @@
           <t>Section 21 non-profit company must apply to NamRA for tax-exempt welfare status: qualifying income exempt, donors deduct gifts to approved organisations. No published processing time.</t>
         </is>
       </c>
+      <c r="R98" s="2" t="inlineStr">
+        <is>
+          <t>In-person is typical (Bank Windhoek opens permanent accounts even without residence status); some banks (Nedbank) allow remote opening via power of attorney, so a local agent can arrange it.</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -9131,6 +9622,11 @@
           <t>PVO registration (PVO Act 2005) does not auto-confer tax exemption; ZIMRA application for income-tax exemption of qualifying receipts; donors deduct donations to approved charitable trusts (s15(2)(r)).</t>
         </is>
       </c>
+      <c r="R99" s="2" t="inlineStr">
+        <is>
+          <t>In-person KYC at branch (RBZ-supervised AML) with passport and address proof; diaspora products exist for individuals, but charity/NGO accounts need in-person signing with local signatories.</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -9218,6 +9714,11 @@
           <t>NPO registered under the Companies Act applies for tax exemption with Eswatini Revenue Services; Tax Order 1975 provides relief on qualifying charitable activities. No published approval time.</t>
         </is>
       </c>
+      <c r="R100" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: non-resident accounts at Standard Bank/FNB/Nedbank require in-person appearance in Mbabane with passport and proof of address; no remote onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -9305,6 +9806,11 @@
           <t>Automatic under Income Tax Act 1993 s25: income of religious, charitable, amateur sporting and trade-union organisations is exempt; donor deduction for approved institutions; no separate application.</t>
         </is>
       </c>
+      <c r="R101" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (PostBank, Stanbic, Nedbank) require in-person verification with passport, residence permit and local proof of residence; no remote onboarding for foreign entities.</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -9392,6 +9898,11 @@
           <t>Separate PBO application to SARS (IT321/IT361 + NPO certificate) under s.30 Income Tax Act; grants income tax exemption + 18A donor deduction; no statutory deadline, typically weeks to months.</t>
         </is>
       </c>
+      <c r="R102" s="2" t="inlineStr">
+        <is>
+          <t>SA FICA/AML KYC requires in-person branch verification; Standard Bank, Nedbank make the signatory appear. Non-residents give passport + foreign address proof; remote NPC/trust onboarding is effectively impossible.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -9479,6 +9990,11 @@
           <t>Separate ANBI decision (beschikking) from Belastingdienst: public-benefit purpose + 90%-of-activity rule; grants CIT exemption + 30% donor deduction; usually 2-4 weeks, no statutory deadline.</t>
         </is>
       </c>
+      <c r="R103" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked: Dutch banks (ING, ABN AMRO, Rabobank) apply strict Wwft AML screening; non-resident founders without a local address/BSN are routinely declined. In-person plus local presence is effectively required.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -9566,6 +10082,11 @@
           <t>No separate tax registration: ASBL with charitable purpose is income-tax-exempt on non-profit activity; 90% donor tax reduction requires listing on the FPS Economy public-utility list (BCE/KBO).</t>
         </is>
       </c>
+      <c r="R104" s="2" t="inlineStr">
+        <is>
+          <t>Non-resident accounts are legal, but a branch visit is required: in-person ID, enhanced AML due diligence, and many banks demand a Belgian address — non-resident business accounts are frequently refused.</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -9653,6 +10174,11 @@
           <t>Automatic: income of non-profit associations/foundations is exempt from CIT without a separate tax procedure (checked at filing). Donations get 25% deduction, 50% for extra gifts, capped at 1% of taxable income.</t>
         </is>
       </c>
+      <c r="R105" s="2" t="inlineStr">
+        <is>
+          <t>No legal bar for non-residents, but a local visit is typical: strict AML banks apply enhanced due diligence to overseas founders; remote applications are often delayed or refused. A local mandate is the workaround.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -9740,6 +10266,11 @@
           <t>Automatic: association loi 1901 with general-interest purpose is income-tax-exempt with no separate procedure (CGI art. 208). Donors get 66% tax reduction, capped at 20% of taxable income. No VAT exemption.</t>
         </is>
       </c>
+      <c r="R106" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for remote non-residents: French banks demand proof of French address + in-person signature; AML refusals are common (droit au compte as remedy). Association accounts need a local visit/agent.</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -9827,6 +10358,11 @@
           <t>Separate Freistellungsbescheid from the Finanzamt: must meet the charitable catalogue (AO ss.52-68, non-profit, member base, public benefit). Grants income tax exemption + 30% donor deduction; usually weeks to 3 months.</t>
         </is>
       </c>
+      <c r="R107" s="2" t="inlineStr">
+        <is>
+          <t>Some direct banks allow remote onboarding via video ID/eID, but most require in-person signature; non-residents face AML scrutiny and banks often demand a local address. A local representative is the practical route.</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -9914,6 +10450,11 @@
           <t>Separate application to the Finanzamt for s.34 EStG privileged taxation (zugunftsbesteuerung, public-benefit purpose). Grants income tax exemption + donor deduction (20% individuals/25% companies); weeks to months.</t>
         </is>
       </c>
+      <c r="R108" s="2" t="inlineStr">
+        <is>
+          <t>Branch visit required: Austrian banks do in-person KYC and most accounts need proof of Austrian residence (Meldezettel). Non-residents without local presence are refused; a local representative is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -10001,6 +10542,11 @@
           <t>Generally automatic: cantonal tax authority exempts foundations/associations whose articles serve common benefit (gemeinnuetzig) at filing - no separate procedure. Donations deductible (c. CHF 25-35k).</t>
         </is>
       </c>
+      <c r="R109" s="2" t="inlineStr">
+        <is>
+          <t>Non-resident onboarding exists (some banks allow remote video), but Swiss AML/KYC is strict and domestic registration (representative/domicile) is required. A local representative is needed for a Stiftung/Verein.</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
@@ -10088,6 +10634,11 @@
           <t>Automatic: foundations/associations with non-profit, common-benefit articles are income-tax-exempt under s.15 EStG without any separate tax procedure. Donations are not deductible; no VAT exemption.</t>
         </is>
       </c>
+      <c r="R110" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for small remote founders: Liechtenstein banks serve non-residents mainly via private banking with high minimum deposits, in-person meetings and strict AML. A local agent/mandate is required.</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -10175,6 +10726,11 @@
           <t>No personal income tax on residents, so foundations/associations face no domestic income tax; public-utility status (sovereign decree) is a civil, not tax, step. Donors deduct in home states (e.g. France 66-75%).</t>
         </is>
       </c>
+      <c r="R111" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for remote non-residents: Monaco banks demand high minimum deposits (EUR 500k+), a local address and in-person onboarding; non-EU non-residents face strictest thresholds. A local agent is required.</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -10262,6 +10818,11 @@
           <t>Automatic: foundations and associations with charitable purpose are exempt from IRPOS (corporate income tax) by law, no separate tax application. No general donor deduction; no VAT.</t>
         </is>
       </c>
+      <c r="R112" s="2" t="inlineStr">
+        <is>
+          <t>No general remote onboarding; non-residents must open accounts in person at branches (e.g. CAI) with passport + foreign address proof. Strict AML screening makes a local visit or representative required.</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -10349,6 +10910,11 @@
           <t>Automatic: non-profit foundations/associations with charitable purpose are exempt from personal income tax (Llei 5/2014 s.33) with no separate procedure; donor deduction limited (20%, capped at 1% of income).</t>
         </is>
       </c>
+      <c r="R113" s="2" t="inlineStr">
+        <is>
+          <t>Non-residents can open accounts but a branch visit is typical; banks demand a local address, high non-resident minimum deposits (often EUR 250k+), and strict AML. A local agent is the common route.</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -10436,6 +11002,11 @@
           <t>Separate: fundacja/stowarzyszenie registers as OPP (public benefit) at the Ministry of the Interior to access 1% personal tax donation + gift deduction; income tax applies to business activity. No VAT exemption.</t>
         </is>
       </c>
+      <c r="R114" s="2" t="inlineStr">
+        <is>
+          <t>Non-resident corporate accounts are possible, but most banks (PKO, mBank) require in-person signature and some a Polish address; enhanced AML checks on the UBO are common, so a local representative is practical.</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -10523,6 +11094,11 @@
           <t>Separate: spolek applies for ZU (general-benefit) status at the Ministry of Interior register. Grants income tax exemption on non-business income + 4% personal tax donation. No VAT exemption.</t>
         </is>
       </c>
+      <c r="R115" s="2" t="inlineStr">
+        <is>
+          <t>No legal bar, but banks (Ceska sporitelna, Moneta) generally require in-person signature with passport + address proof; many refuse non-resident business accounts. A local visit or representative is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -10610,6 +11186,11 @@
           <t>Separate: VPO (public-benefit) status by Ministry of Interior decision under Act 65/2018. Grants income tax exemption + 1% personal tax donation + gift deduction. No VAT exemption.</t>
         </is>
       </c>
+      <c r="R116" s="2" t="inlineStr">
+        <is>
+          <t>Non-resident accounts are legal, but a branch visit is typical: banks demand a residence permit or proof of employment (esp. non-EU), in-person ID and often a local address. A local visit/representative is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -10697,6 +11278,11 @@
           <t>Separate NAV procedure: apply for income tax exemption (adozo-kiveteles status) + annual 1% registration (form 25EGYREG, capped at 2%). Corporate donations deductible (1.5% total). Decision typically within 30 days.</t>
         </is>
       </c>
+      <c r="R117" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for remote founders: Hungarian banks (OTP, KB) require in-person onboarding, and non-residents need proof of a Hungarian address/residence. Non-resident business accounts are rare; local agent needed.</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -10784,6 +11370,11 @@
           <t>Automatic: associations/foundations are income-tax-exempt on non-business activity (ZDavO s.9) with no separate tax procedure. 'Javno koristno' is a civil-law status; donors get 25% deduction (max EUR 200).</t>
         </is>
       </c>
+      <c r="R118" s="2" t="inlineStr">
+        <is>
+          <t>Non-residents may open accounts (even tourists in principle), but a branch visit is typical: banks demand a Slovenian tax number, in-person ID verification and often a local address. A visit/representative is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -10871,6 +11462,11 @@
           <t>Separate: 'javno korisna' (public-benefit) decision by the Ministry of Interior. Grants income tax exemption + 2% personal / 1% corporate tax donation + 40% gift deduction. No published deadline.</t>
         </is>
       </c>
+      <c r="R119" s="2" t="inlineStr">
+        <is>
+          <t>Non-resident business accounts are possible, but a personal branch visit is required (PBZ etc.), with enhanced AML checks and usually a Croatian OIB number. A local representative is needed for remote founders.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -10958,6 +11554,11 @@
           <t>Application to the tax administration (FBiH/Trezor): non-profit entities with charitable purpose are exempt from PIT under the BiH PIT Law if conditions met; gifts partially deductible; no published deadline.</t>
         </is>
       </c>
+      <c r="R120" s="2" t="inlineStr">
+        <is>
+          <t>A local visit is typical: Bosnian banks require in-person onboarding with passport, and non-residents need a clear local connection; the system is fragmented (FBiH/SRH). A local agent/representative is the common route.</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -11045,6 +11646,11 @@
           <t>Largely automatic: udruzenje gracana is income-tax-exempt on non-profit income (Income Tax Law s.18) where purpose serves public interest; access to 1% personal tax and 2% corporate donations. No statutory deadline.</t>
         </is>
       </c>
+      <c r="R121" s="2" t="inlineStr">
+        <is>
+          <t>No remote onboarding: Serbian banks require an in-person visit with passport + foreign address proof; non-residents can open (incl. EUR) accounts at bank discretion — a local representative is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -11132,6 +11738,11 @@
           <t>Automatic on registration: donations, dues and non-economic income are exempt from income tax; the new VAT law broadly exempts NGO services. Donor deduction rate is unpublished.</t>
         </is>
       </c>
+      <c r="R122" s="2" t="inlineStr">
+        <is>
+          <t>Local visit required — remote opening is not possible. Banks run strict AML due diligence and often decline corporate accounts for founders with no residence permit or other tie to Montenegro.</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -11219,6 +11830,11 @@
           <t>Not automatic: exemption requires public-interest purpose, non-distribution and registration (OG 52/10). Donations to qualifying bodies deductible under the Law on Donations &amp; Sponsorships; rate unpublished.</t>
         </is>
       </c>
+      <c r="R123" s="2" t="inlineStr">
+        <is>
+          <t>Non-residents may open accounts (Stopanska Banka publishes non-resident requirements), typically same-day to a week, but an in-person visit to a Skopje branch is required; remote opening is not possible.</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -11306,6 +11922,11 @@
           <t>CIT exemption is automatic on NPO registration (Law 80/2021); foundations qualify via Income Tax Act art.18 activities. Donor deduction rate unpublished; VAT exemption can be granted. Time unpublished.</t>
         </is>
       </c>
+      <c r="R124" s="2" t="inlineStr">
+        <is>
+          <t>A registered Albanian firm can open a corporate account, but non-resident owners face enhanced AML due diligence; banks (Raiffeisen, BKT) will process it, and a signatory branch visit is the norm.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -11393,6 +12014,11 @@
           <t>Automatic: Law 86/2020 associations and foundations are income-tax exempt once they perform socially useful activities within 1 year (Tax Code). Donor deduction rate unpublished. Time unpublished.</t>
         </is>
       </c>
+      <c r="R125" s="2" t="inlineStr">
+        <is>
+          <t>In-person signing at a Chisinau branch is standard; non-resident UBOs trigger enhanced due diligence under AML Law 30/2011 and banks demand detailed source-of-funds documentation.</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -11480,6 +12106,11 @@
           <t>Automatic on state registration (Tax Code art.132); 'public benefit' status is separate. Donor deductions: corporate 2-5% of prior profit, individual 1%; some services VAT-exempt. Time unpublished.</t>
         </is>
       </c>
+      <c r="R126" s="2" t="inlineStr">
+        <is>
+          <t>NBU rules allow banks to serve non-residents and foreign-owned Ukrainian entities open accounts routinely, but expect full KYC/AML, apostilled documents, and usually an in-person visit or notarized power of attorney.</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11567,6 +12198,11 @@
           <t>Public organizations and foundations are non-taxable on donations, budget funds and membership fees under the Tax Code - no separate application. Donor deduction rate unpublished. Time unpublished.</t>
         </is>
       </c>
+      <c r="R127" s="2" t="inlineStr">
+        <is>
+          <t>Currency law permits non-residents to hold BYN and foreign-currency accounts, but certified documents, UBO disclosure and bank AML/KYC apply; expect an in-person visit (or authorized representative) in Minsk.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11654,6 +12290,11 @@
           <t>Non-commercial income is exempt from income tax automatically; 'public benefit' status is a separate Ministry of Justice application. Donor deductions: individual 10% of income, corporate 10% of profit.</t>
         </is>
       </c>
+      <c r="R128" s="2" t="inlineStr">
+        <is>
+          <t>An in-person branch visit by the company administrator is generally required; AML rules impose enhanced due diligence on non-resident directors, and fully remote opening at high-street banks is largely unavailable.</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -11741,6 +12382,11 @@
           <t>PBO status needs separate Central Register entry (Ministry of Justice) - PBOs exempt from CIT when income serves public benefit. Donor deductions: individual 5% of income, corporate 10% of profit.</t>
         </is>
       </c>
+      <c r="R129" s="2" t="inlineStr">
+        <is>
+          <t>Banks require in-person verification: personal accounts always, and corporate accounts usually need the director to appear; a non-resident founder should plan a visit or appoint a local agent to sign.</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -11828,6 +12474,11 @@
           <t>General public-benefit status: separate application to the Directorate for Associations (Law 4873/2021); recognized bodies exempt from tax on contributions. Donor cut: 20% of gifts over EUR 100, cap 10% of income.</t>
         </is>
       </c>
+      <c r="R130" s="2" t="inlineStr">
+        <is>
+          <t>A Greek tax number (AFM) is a hard precondition, and branches require an in-person visit with due diligence on the account's purpose; there is no fully online route for non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -11915,6 +12566,11 @@
           <t>Separate approval by the Tax Dept/MOF; approved charities get preferential treatment and donors deduct 100% of gifts from taxable income, no cap (ITL 118(I)/2002 art.9). Time unpublished.</t>
         </is>
       </c>
+      <c r="R131" s="2" t="inlineStr">
+        <is>
+          <t>Residency is not a legal bar, but local banks require in-person KYC and source-of-funds checks under Central Bank of Cyprus AML rules; non-residents are often flagged high-risk. EMIs (Wise, Revolut) open online.</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -12002,6 +12658,11 @@
           <t>Not automatic: apply to Revenue &amp; Customs Administration for income-tax exemption for philanthropic work (LN 62/2024). Corporate donors get tax credit on qualifying gifts (cap EUR 500, LN 86/2024). Time unpublished.</t>
         </is>
       </c>
+      <c r="R132" s="2" t="inlineStr">
+        <is>
+          <t>Traditional banks (BOV, HSBC Malta, APS Bank) require at least one in-person branch visit; fully remote opening is generally unavailable from abroad, with 2-6 weeks to account activation.</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -12089,6 +12750,11 @@
           <t>Two-step: register with the Charities Regulator first, then apply to Revenue for charitable tax exemption (CHY number) - exempts income tax, CIT, CGT, DIRT; donors get 25%/33.33% tax credits. Time unpublished.</t>
         </is>
       </c>
+      <c r="R133" s="2" t="inlineStr">
+        <is>
+          <t>Irish banks expect local substance — typically a resident (Irish/EEA) director and an Irish operational base; boards with only non-resident, no-presence directors are frequently declined at onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -12176,6 +12842,11 @@
           <t>Charity Commission registration (charitable purposes, public benefit; mandatory above GBP 5,000): exempts income/corporate tax, Gift Aid 25% donor gross-up, VAT exemption for qualifying supplies. Target 30 working days.</t>
         </is>
       </c>
+      <c r="R134" s="2" t="inlineStr">
+        <is>
+          <t>Non-residents can open UK business accounts, but AML/KYC and sanctions checks apply; high-street banks often expect a UK address and evidence of genuine UK activity — possible, though tighter than for residents.</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -12263,6 +12934,11 @@
           <t>General exemption from income and property tax, no separate application. Donors deduct ISK 10,000-350,000/yr for gifts to bodies on the public-benefit register; fundraising activities VAT-exempt.</t>
         </is>
       </c>
+      <c r="R135" s="2" t="inlineStr">
+        <is>
+          <t>Banks require an Icelandic kennitala (national ID) and in-person ID verification; company law also expects at least half the board to be resident, so a local presence or representative is effectively needed.</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -12350,6 +13026,11 @@
           <t>Automatic income and wealth tax exemption when non-commercial (no profit to members). Donors deduct up to NOK 25,000 (2026) for monetary gifts of NOK 500+ to approved organizations. Time unpublished.</t>
         </is>
       </c>
+      <c r="R136" s="2" t="inlineStr">
+        <is>
+          <t>Registered entities can open accounts, but banks demand board-member ID verification and proof of Norwegian business activity under AML rules; non-resident directors should be EEA-resident and expect a branch visit.</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -12437,6 +13118,11 @@
           <t>Donation deduction: the organization must be on the Tax Administration's approved-donation list (separate application). Monetary gifts to approved orgs are deductible. Time unpublished.</t>
         </is>
       </c>
+      <c r="R137" s="2" t="inlineStr">
+        <is>
+          <t>Banks treat non-EEA directors/UBOs as high-risk; identification at a branch (or strong eID) is required, and non-residents without a Finnish HETU code often face long, complex reviews ending in generic refusal.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -12524,6 +13210,11 @@
           <t>Dues, donations and grants tax-exempt; other income exempt if 4 public-benefit conditions met. Donor relief (25% tax cut, cap SEK 3,000) needs separate Skatteverket application as gift recipient.</t>
         </is>
       </c>
+      <c r="R138" s="2" t="inlineStr">
+        <is>
+          <t>Foreign-owned companies can open accounts, but traditional banks apply strict residency-based KYC; at least 50% of the board must be EEA-resident (waivable by Bolagsverket) and a branch visit is standard.</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -12611,6 +13302,11 @@
           <t>Non-commercial association income exempt automatically on CVR registration. Donor deduction: up to DKK 20,000/yr (2026) for gifts to tax-approved orgs under Tax Act s.8A. Time unpublished.</t>
         </is>
       </c>
+      <c r="R139" s="2" t="inlineStr">
+        <is>
+          <t>Danish substance — local clients, office or employees — is effectively required; banks demand MitID and strict AML/KYC on foreign owners, so all-non-resident files are often refused; fintech accounts are easier.</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -12698,6 +13394,11 @@
           <t>Registration automatic; separate EMTA list application required (Income Tax Act s.11) - listed orgs: donation income not taxable. Donors: individuals up to EUR 1,200; corporate 3% social tax base or 10% prior profit.</t>
         </is>
       </c>
+      <c r="R140" s="2" t="inlineStr">
+        <is>
+          <t>An Estonian bank account is not legally required — EEA EMIs (Wise, LHV online) serve non-resident companies — but Estonian banks approve such files mostly with real local operation or a local board member.</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -12785,6 +13486,11 @@
           <t>Registration automatic; PBO status is a separate VID application (2016 Law) - PBOs exempt from income tax. Donors: individuals 25.5% tax refund; corporate 5% of prior profit or CIT reduction.</t>
         </is>
       </c>
+      <c r="R141" s="2" t="inlineStr">
+        <is>
+          <t>Since the 2018 reforms, business accounts for non-resident owners are hard to approve (2-4 weeks, elevated refusals); banks require proof of a Latvia connection and usually a visit; EU/EEA applicants can apply remotely.</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -12872,6 +13578,11 @@
           <t>Public-benefit institutions (viešoji įstaiga) get income-tax exemption automatically on registration; corporate donors deduct 1% of profit tax on donations to them — no separate VMI application.</t>
         </is>
       </c>
+      <c r="R142" s="2" t="inlineStr">
+        <is>
+          <t>Traditional banks (SEB, Swedbank, Luminor) require in-person KYC and usually a residence permit. Partially online options exist via SEB's remote application and fintechs (Revolut, Paysera, Wise) opening accounts with just a passport.</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -12959,6 +13670,11 @@
           <t>Foundations with charitable purposes automatically enter Law 49/2002's special regime: profits exempt, donors get a 40% IRPF deduction on the first €15,000 (30% above). No separate AEAT application required.</t>
         </is>
       </c>
+      <c r="R143" s="2" t="inlineStr">
+        <is>
+          <t>A cuenta no residente requires a NIE first and an in-person branch visit for KYC and signature. Fully remote opening is not offered by major Spanish banks (BBVA, Santander) for a foreign foundation.</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -13046,6 +13762,11 @@
           <t>Private foundations are exempt from IRC only after obtaining utilidade pública status (Ministry decree); without it, taxed at 21%. IUP status entitles donors to a 15% deduction; processing time unpublished.</t>
         </is>
       </c>
+      <c r="R144" s="2" t="inlineStr">
+        <is>
+          <t>A NIF (tax number) is a hard prerequisite. Many banks require an in-person KYC branch visit; a NIF can be obtained remotely via a Portuguese fiscal representative, and some banks allow online onboarding.</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -13133,6 +13854,11 @@
           <t>Automatic: charitable income of non-commercial entities is exempt from income tax (art. 72 TUIR); RUNTS registration entitles donors to a 19% tax credit up to €30,000 plus 5xmille; no separate application.</t>
         </is>
       </c>
+      <c r="R145" s="2" t="inlineStr">
+        <is>
+          <t>In-person branch visit is mandatory. A codice fiscale (tax code) and physical identity verification are required by Italian banks; there is no remote onboarding pathway for a foreign fondazione account.</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -13220,6 +13946,11 @@
           <t>No ordinary income-tax regime: charitable activity runs through pontifical institutions or canonically erected bodies; the Holy See levies no income tax, so no separate tax-exemption application exists.</t>
         </is>
       </c>
+      <c r="R146" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for a remote foreign founder. The IOR (Vatican Bank) serves only Catholic institutions (dioceses, religious orders) as external clients and requires in-person, institutional due diligence.</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -13307,6 +14038,11 @@
           <t>Separate application to the Israel Tax Authority: section 120 profit-exemption certificate plus section 46 public-institution status for donors; not automatic; a 2025 green-track accelerates section 46 grants.</t>
         </is>
       </c>
+      <c r="R147" s="2" t="inlineStr">
+        <is>
+          <t>Remote is possible: Bank of Israel rules permit video KYC. Bank Hapoalim's and Leumi's international desks let non-residents complete onboarding remotely (email + video), though not all branches offer this.</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -13394,6 +14130,11 @@
           <t>Registration with the Ministry of Social Affairs confers legal personality; the income-tax law exempts income of registered associations/foundations pursuing public-benefit purposes, and donations to them are deductible.</t>
         </is>
       </c>
+      <c r="R148" s="2" t="inlineStr">
+        <is>
+          <t>In-person visit to a Jordanian bank (e.g. Arab Bank, CBJ) is mandatory for KYC. A local address/presence is effectively required for a foreign charitable entity; no remote onboarding exists.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -13481,6 +14222,11 @@
           <t>Associations are valid by declaration to the local court (Law 92/1909); the income-tax code exempts income of public-benefit associations and institutions — no separate application; no donor-deduction regime.</t>
         </is>
       </c>
+      <c r="R149" s="2" t="inlineStr">
+        <is>
+          <t>In-person KYC at a Lebanese bank is required. A local financial representative is common. Some banks accept a power of attorney, but a physical presence for the initial meeting is the standard.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -13568,6 +14314,11 @@
           <t>Associations register with the Ministry of Social Affairs &amp; Labor; the Income Tax Law 24/2003 treats income of registered charitable associations as exempt — no separate tax application; donor rules unpublished.</t>
         </is>
       </c>
+      <c r="R150" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked: international sanctions and strict Central Bank of Syria rules restrict foreign access. Local in-person presence and a Syrian counterparty are required; remote onboarding is unavailable.</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -13655,6 +14406,11 @@
           <t>NGOs registered with the NGO Directorate, Interior Ministry: if classified as public utility, art. 17 of Law 12/2010 automatically exempts income tax, VAT, customs and sales tax; no separate application.</t>
         </is>
       </c>
+      <c r="R151" s="2" t="inlineStr">
+        <is>
+          <t>Local in-person presence at an Iraqi bank (e.g. Bank of Baghdad, FIB) is required. A local representative/agent is typically needed; CBI AML rules mandate physical identity verification for foreign founders.</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -13742,6 +14498,11 @@
           <t>No personal income tax; registered civil society associations are exempt from zakat (ministerial decision 61600/1444) and their charitable supplies are VAT-exempt; no donor-deduction regime.</t>
         </is>
       </c>
+      <c r="R152" s="2" t="inlineStr">
+        <is>
+          <t>Requires a MISA licence, commercial registration, and an in-person visit to a SAMA-regulated bank. A local sponsor/agent is typically needed; fully remote onboarding is not available to a foreign founder.</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -13829,6 +14590,11 @@
           <t>No charitable tax-exemption regime: Kuwait levies no income tax, so associations registered under the 1962 Public Welfare Societies law gain no tax benefits and there is no donor-deduction scheme.</t>
         </is>
       </c>
+      <c r="R153" s="2" t="inlineStr">
+        <is>
+          <t>A local in-person visit to a Kuwaiti bank is mandatory. A local Kuwaiti representative/sponsor is typically required for a foreign charitable entity; remote onboarding is not available.</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -13916,6 +14682,11 @@
           <t>Income Tax Law 24/2018, as amended by Law 11/2022, exempts entities operating exclusively for charitable, religious or educational purposes (registered, non-distribution); no donor-deduction regime.</t>
         </is>
       </c>
+      <c r="R154" s="2" t="inlineStr">
+        <is>
+          <t>In-person branch visit is mandatory. Qatari banks (QNB, QIIB, Dukhan) require a QID and physical presence at opening; a local partner/agent is usually needed for a foreign charitable institution.</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -14003,6 +14774,11 @@
           <t>DED-licensed charities qualify as Qualifying Public Benefit Entities (FDL 47/2022 art. 9): 0% corporate-tax rate if 100% of income is charitable and non-distributed; no donor-deduction regime.</t>
         </is>
       </c>
+      <c r="R155" s="2" t="inlineStr">
+        <is>
+          <t>An in-person meeting is nearly always required at the bank (Emirates NBD, ADCB, FAB). A local signatory with a UAE residence visa is usually required; fully digital onboarding is generally unavailable to non-residents.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -14090,6 +14866,11 @@
           <t>Registered charitable associations are exempt from Oman's 15% corporate income tax, and donations to them are deductible from donors' taxable income (executive reg. art. 33); no separate application.</t>
         </is>
       </c>
+      <c r="R156" s="2" t="inlineStr">
+        <is>
+          <t>An in-person visit to an Omani bank is required. A local representative/partner is typically needed; Central Bank of Oman AML rules mandate physical identity verification for a foreign founder.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -14177,6 +14958,11 @@
           <t>No charitable tax-exemption regime: Bahrain levies no general income/corporate tax (only banking/insurance), so registered NGOs gain no tax benefits and there is no donor-deduction scheme.</t>
         </is>
       </c>
+      <c r="R157" s="2" t="inlineStr">
+        <is>
+          <t>An in-person branch visit is mandatory for account opening. A local representative is typically required for a foreign NGO; CBBA AML rules apply and remote onboarding is not available.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -14264,6 +15050,11 @@
           <t>Automatic: art. 40 of the associations law (Law 73/1991, amended by Law 1/2001) exempts registered associations and foundations from all forms of taxes; no separate application to a tax authority.</t>
         </is>
       </c>
+      <c r="R158" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for a remote founder: instability, sanctions, and Central Bank of Yemen rules require local in-person presence. A Yemeni representative is essential; no remote onboarding exists.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -14351,6 +15142,11 @@
           <t>Art. 14 of Law 1/2000 exempts registered charitable associations from taxes and customs duties on property used for their objectives; general income tax (Law 17/2004) otherwise applies; no donor deduction.</t>
         </is>
       </c>
+      <c r="R159" s="2" t="inlineStr">
+        <is>
+          <t>Local in-person presence at a Palestinian bank (e.g. PAB, NBL Bank) is required. A local agent is typically needed; Central Bank of Palestine AML rules mandate physical identity verification.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -14438,6 +15234,11 @@
           <t>Registration automatically grants income-tax exemption under art. 47 of the Income Tax Law 91/2005 on revenue from charitable activities; donors deduct 10% (individuals) / 15% (legal persons).</t>
         </is>
       </c>
+      <c r="R160" s="2" t="inlineStr">
+        <is>
+          <t>A 2024 CBE circular permits non-resident foreigners to open accounts subject to AML checks. An in-person visit, passport, and proof of an Egyptian address are required; a local representative is helpful.</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -14525,6 +15326,11 @@
           <t>Not automatic: art. 25 of the 2006 Act lets the Finance Minister, on the minister's recommendation, exempt registered CSOs from customs duties and taxes; no codified general charitable tax-exemption regime.</t>
         </is>
       </c>
+      <c r="R161" s="2" t="inlineStr">
+        <is>
+          <t>Local in-person presence is required. A Sudanese agent/representative is essential given instability and sanctions; Bank of Sudan AML rules mandate physical verification. Remote onboarding is not available.</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -14612,6 +15418,11 @@
           <t>Automatic on NGO registration (NGO Law 19/2001; 50+ local founders, Libyan HQ): state recognition triggers Income Tax Law 7/2010 art.33 income exemption; donor deduction up to 2% net income; no VAT; time unpublished.</t>
         </is>
       </c>
+      <c r="R162" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked: state-run banks require in-person visits, local address, and income proof for foreigners; no remote opening or diaspora channel for foreign founders.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -14699,6 +15510,11 @@
           <t>No blanket income-tax exemption: activities taxable (19-26% IS); resident donors get a 40% gift credit (5% taxable-income cap); corporate donors deduct humanitarian gifts to 4M DA; no VAT; UPU separate, time unpublished.</t>
         </is>
       </c>
+      <c r="R163" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks demand passport, local address proof, and residency documentation; non-resident (INR) accounts are limited to holders of Algerian public contracts.</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -14786,6 +15602,11 @@
           <t>Automatic by law: associations under Decret-loi 2011-88 are outside corporate-tax scope (DGELF 133/2013); VAT exemptions for charitable operations; no blanket donor deduction; no separate application, no approval time.</t>
         </is>
       </c>
+      <c r="R164" s="2" t="inlineStr">
+        <is>
+          <t>In-person at a bank branch: passport, proof of address (often Tunisian) and AML source-of-funds docs; a convertible-dinar account for non-residents exists but opening is branch-based.</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -14873,6 +15694,11 @@
           <t>IS exemption automatic by law (CGI 6 I-1) for bylaws-conform operations; separate RUP decree (SGG, 6-month max) unlocks unlimited corporate donor deduction + VAT gift exemption; foreign bodies need Interior approval.</t>
         </is>
       </c>
+      <c r="R165" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit, not local residency: a passport suffices to open a non-resident foreign-currency (compte en devises) EUR/USD/GBP account in person; standard dirham accounts require residency.</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -14960,6 +15786,11 @@
           <t>Automatic by law (CGI 4(1)(b)): NGO income exempt from IS except competitive business; corporate donors deduct gifts to UPU bodies to 0.2% of turnover (max 2M Ouguiya); no individual deduction; no VAT; time unpublished.</t>
         </is>
       </c>
+      <c r="R166" s="2" t="inlineStr">
+        <is>
+          <t>In-person required: passport, visa/residence documents, local address proof and references; few banks serve foreigners and no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -15047,6 +15878,11 @@
           <t>No independent regime: Moroccan dahir applies in Moroccan-administered areas only. IS exemption automatic (CGI 6 I-1); separate RUP recognition (6-month max) unlocks unlimited corporate donor deduction + VAT exemption.</t>
         </is>
       </c>
+      <c r="R167" s="2" t="inlineStr">
+        <is>
+          <t>No independent banking infrastructure: no central bank of the territory; accounts depend on Moroccan banks in administered areas (in-person, Moroccan AML rules) and are effectively inaccessible remotely.</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -15134,6 +15970,11 @@
           <t>Automatic by law: ITP art.65(1)(m) exempts registered CSOs' non-business income (donations, grants); business income taxable; no blanket donor deduction; self-asserted at filing, no time; resident founders required.</t>
         </is>
       </c>
+      <c r="R168" s="2" t="inlineStr">
+        <is>
+          <t>In-person application at a bank: passport, local address proof (utility bill/kebele letter) and photos; diaspora accounts serve only Ethiopians abroad; no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="inlineStr">
@@ -15221,6 +16062,11 @@
           <t>No charitable exemption: Income Tax Proclamation 145/2005 has no charitable carve-out, so associations are ordinary taxpayers; only an ad-hoc ministerial agreement can exempt; donor deduction and VAT relief undocumented.</t>
         </is>
       </c>
+      <c r="R169" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for non-resident foreigners: only state-owned banks, foreign banks excluded, and foreign accounts limited to legal residents under nakfa withdrawal caps; no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -15308,6 +16154,11 @@
           <t>Separate request via Interior Minister: presidential decree of public utility; donations exempt from registration/transfer tax; VAT exemption for nonprofit charitable services; no donor deduction; time unpublished.</t>
         </is>
       </c>
+      <c r="R170" s="2" t="inlineStr">
+        <is>
+          <t>In-person visit required: passport, local address/residence documentation and source-of-funds checks; several banks offer non-resident accounts on visit, none open fully remotely.</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -15395,6 +16246,11 @@
           <t>No statutory recognition: tax exemptions are ad-hoc, negotiated individually with the Ministry of Finance; no income-tax exemption, donor deduction, or VAT relief documented; time unpublished.</t>
         </is>
       </c>
+      <c r="R171" s="2" t="inlineStr">
+        <is>
+          <t>In-person with local address proof: passport and CBS/AML-KYC checks; some diaspora products exist (e.g. Salaam SSB non-resident accounts) but generally a local visit is needed.</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -15482,6 +16338,11 @@
           <t>Separate SRA written ruling (not automatic): income-tax exemption for charitable public institutions; no donor-deduction rate/cap or VAT exemption documented; time unpublished.</t>
         </is>
       </c>
+      <c r="R172" s="2" t="inlineStr">
+        <is>
+          <t>In-person at Bank of Somaliland branches: passport, local address and KYC under AML Law 72/2016; unrecognised-state status limits correspondent banking; no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -15569,6 +16430,11 @@
           <t>BPT exemption by operation of law on RRC registration with public-benefit status; donor contributions deductible, no cap published; 18% sales tax, no NGO exemption; time unpublished.</t>
         </is>
       </c>
+      <c r="R173" s="2" t="inlineStr">
+        <is>
+          <t>In-person required: passport, proof of address and sometimes a reference/introduction letter; only a handful of banks and weak infrastructure; no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -15656,6 +16522,11 @@
           <t>Separate application via CEPS to Ministry of Finance: business-tax exemption for charitable institutions; no general donor deduction; VAT exempt only on international donations; time unpublished.</t>
         </is>
       </c>
+      <c r="R174" s="2" t="inlineStr">
+        <is>
+          <t>In-person at Seychelles banks (Absa, MCB, Nouvobanq): passport, strict KYC and source-of-funds docs; a Mahé residential address is typically expected; no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -15743,6 +16614,11 @@
           <t>Separate MRA approval (Director-General, s.49D) after NPO Act registration: income-tax exemption via Second Schedule; donor deduction capped MUR 30,000/yr (s.27DA, e-donations); no VAT exemption; time unpublished.</t>
         </is>
       </c>
+      <c r="R175" s="2" t="inlineStr">
+        <is>
+          <t>In-person visit: non-resident and business accounts exist under strict FSC AML/CFT KYC (identity, address, source of funds, CRS/FATCA); most banks expect founder presence.</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -15830,6 +16706,11 @@
           <t>Separate Form 10A/10AB application to Income Tax Dept: income-tax exemption + 80G donor deduction 50% (10% AGTI cap); no general VAT/GST exemption; ~1-3 months (time unpublished).</t>
         </is>
       </c>
+      <c r="R176" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked for foreign non-citizens: RBI/FEMA NRE/NRO accounts are limited to Indian citizens (NRIs/OCIs); resident accounts are off-limits to foreigners without local employment/residency.</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -15917,6 +16798,11 @@
           <t>Separate FBR Commissioner approval (ITO 2001 s.2(36)) after registration + NTN: 100% income-tax exemption (s.100C); donor gift tax credit capped 30% taxable income (s.61); no VAT exemption; time unpublished.</t>
         </is>
       </c>
+      <c r="R177" s="2" t="inlineStr">
+        <is>
+          <t>Fully online possible: the SBP-regulated Roshan Digital Account (extended to foreign nationals in March 2026) allows remote opening of repatriable accounts within ~48 hours.</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -16004,6 +16890,11 @@
           <t>Separate Principal/Commissioner of IT application (s.46 ITO 1984): charitable-trust income-tax exemption; 100% donor tax credit (s.50, 10% adjusted-total-income cap); VAT-exempt charitable income; time unpublished.</t>
         </is>
       </c>
+      <c r="R178" s="2" t="inlineStr">
+        <is>
+          <t>In-branch visit: standard taka accounts need a visa/work permit, local address and e-TIN; only foreign-currency (FC/NFCD) accounts are reachable without residency; no remote opening.</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -16091,6 +16982,11 @@
           <t>Separate Finance Minister application: gazetted 'approved charity' (IR Act 24/2017); 14% preferential IT rate; donor deduction 1/3 taxable income (max Rs 75k individuals); no VAT exemption; time unpublished.</t>
         </is>
       </c>
+      <c r="R179" s="2" t="inlineStr">
+        <is>
+          <t>In-person with local residency: AML rules bar tourists and remote applicants from rupee accounts; work/residence visa plus local address required; LKR outflows restricted.</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -16178,6 +17074,11 @@
           <t>Separate IRD application for Tax Exemption Certificate: income-tax exemption; donor gifts deductible to 5% cap; no VAT exemption; time unpublished. DAO registration itself automatic on filing.</t>
         </is>
       </c>
+      <c r="R180" s="2" t="inlineStr">
+        <is>
+          <t>In-person required: Nepal Rastra Bank rules demand a non-tourist visa, local address and PAN; NPR is non-convertible; no remote opening for foreign founders.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
@@ -16265,6 +17166,11 @@
           <t>Auto on CSO registration (CSOA 2007 s.38): exempt income tax on endowed-fund gains; donor deduction capped (5% AGI under 2001 rules, 2025 cap unconfirmed); no VAT exemption; time unpublished.</t>
         </is>
       </c>
+      <c r="R181" s="2" t="inlineStr">
+        <is>
+          <t>In-person required: passport, Bhutan visa/work permit and local address proof; the Remit Bhutan remote channel serves only non-resident Bhutanese; foreign founders need a local visit.</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -16352,6 +17258,11 @@
           <t>NGO registered with NGO Registration Committee (NGO Law 2015); NOT automatic - apply to Revenue Authority for tax-exemption certificate (income tax + business receipt tax); no donor deduction; ~30-90 days.</t>
         </is>
       </c>
+      <c r="R182" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked: banks require in-person KYC, local address and visa, and international correspondent banking has largely collapsed under sanctions; a remote foreign NGO founder has no realistic path.</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
@@ -16439,6 +17350,11 @@
           <t>Public charitable trust under Public Trusts Act 2022, registered with Ministry of Justice; registration gives legal personality; income from non-profit purposes tax-exempt; no donor deduction; ~30 days to approve.</t>
         </is>
       </c>
+      <c r="R183" s="2" t="inlineStr">
+        <is>
+          <t>No remote opening. Banks (BML, MIB) require an in-person branch visit with passport, valid work/residence visa and a local address; a foreign founder with no presence would need a local agent to apply.</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -16526,6 +17442,11 @@
           <t>Incorporated trustee registered with CAC (NGO listed with NCMM); tax exemption under CITA 1999 (non-profit organization) via separate FIRS application; no general donor income-tax deduction; time unpublished.</t>
         </is>
       </c>
+      <c r="R184" s="2" t="inlineStr">
+        <is>
+          <t>CBN rules require a Bank Verification Number (BVN) - biometric enrolment only in Nigeria - plus CERPAC residence card and local address for foreigners; opening from abroad is not possible.</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
@@ -16613,6 +17534,11 @@
           <t>CLG (non-profit company) under Companies Act 2019 (Act 992) with NPO license from Registrar; non-profit company income tax-exempt under Act 896; no broad donor deduction; ~4-6 weeks to register.</t>
         </is>
       </c>
+      <c r="R185" s="2" t="inlineStr">
+        <is>
+          <t>Bank of Ghana KYC requires a non-citizen Ghana Card (biometric ID) and a GhanaPostGPS local address; foreigners must open the account in person, so a remote founder needs a local visit or representative.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -16700,6 +17626,11 @@
           <t>Association (société civile) declared with tax service under ordonnance 2024-368; income of non-profit activity tax-exempt if applied to stated purposes; no broad donor deduction; time unpublished.</t>
         </is>
       </c>
+      <c r="R186" s="2" t="inlineStr">
+        <is>
+          <t>BCEAO/UEMOA AML rules apply; banks mainly open accounts in branch, and non-residents typically need a local address or in-person KYC - a remote foreign founder would need a local visit or representative.</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -16787,6 +17718,11 @@
           <t>Association declared with prefecture (loi 2025-19); CGI (loi 2021-15) grants income-tax exemption to non-profit entities; donors may deduct gifts to recognized public-utility organizations; time unpublished.</t>
         </is>
       </c>
+      <c r="R187" s="2" t="inlineStr">
+        <is>
+          <t>No remote opening. Banks require in-person account opening with passport, proof of local address and residency/work permit; a foreign founder with no presence needs a local agent to act in person.</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -16874,6 +17810,11 @@
           <t>Association (loi 1901) declared with prefecture; NGO status via décret 92-130; income-tax exemption for non-profit entities under CGI; no general donor deduction; ~1-2 months to declare.</t>
         </is>
       </c>
+      <c r="R188" s="2" t="inlineStr">
+        <is>
+          <t>In-person opening is the norm: passport plus residence or work permit (non-ECOWAS foreigners face heavier scrutiny) and local address under BCEAO rules; remote opening is not available.</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -16961,6 +17902,11 @@
           <t>Association declared with prefecture (loi 064-2015); public-utility recognition by decree adds full tax benefits; association income tax-exempt when applied to its purposes; no donor deduction; time unpublished.</t>
         </is>
       </c>
+      <c r="R189" s="2" t="inlineStr">
+        <is>
+          <t>No remote opening. Foreigners must apply in person with passport, residence/work permit and proof of local address; a remote founder has no path and needs a local representative to open the account.</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -17048,6 +17994,11 @@
           <t>Association declared with regional government (loi 04-038); income-tax exemption for non-profit entities under CGI; public-utility declaration separate; no general donor deduction; time unpublished.</t>
         </is>
       </c>
+      <c r="R190" s="2" t="inlineStr">
+        <is>
+          <t>Banks require in-person KYC: passport, residence permit and proof of local address under BCEAO AML rules; no remote account opening, so a foreign founder needs a local visit or agent.</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -17135,6 +18086,11 @@
           <t>Association registered with Interior ministry (loi L/2005-013); income of non-profit activity tax-exempt; no general donor deduction or VAT relief; approval time unpublished.</t>
         </is>
       </c>
+      <c r="R191" s="2" t="inlineStr">
+        <is>
+          <t>In-person opening required; non-residents and diaspora may open accounts with extra documentation, but physical presence and local papers are typical - a remote founder needs a local visit or agent.</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -17222,6 +18178,11 @@
           <t>Association formed by public deed (escritura pública) before a notary, then registered; income of non-profit entities tax-exempt; no donor deduction regime; approval time unpublished.</t>
         </is>
       </c>
+      <c r="R192" s="2" t="inlineStr">
+        <is>
+          <t>Banking is paper-based and requires physical presence at a Bissau bank; passport plus residence permit, low digitalization. A remote foreign founder has no realistic remote path - local agent needed.</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -17309,6 +18270,11 @@
           <t>Association declared with prefecture (loi 71-604); income tax exemption automatic under CGI art.5(7) (since 2019) for non-profit entities without commercial activity; donors deduct gifts to public-utility orgs, cap 0.5%.</t>
         </is>
       </c>
+      <c r="R193" s="2" t="inlineStr">
+        <is>
+          <t>BCEAO rules: non-resident accounts need central-bank approval and banks demand in-person KYC (notarized ID, proof of funds) after 2024 AML tightening; remote opening is effectively unavailable.</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -17396,6 +18362,11 @@
           <t>NGO registered with NGO Affairs Agency (Decree No. 81); Income and Sales Tax Act 2004 automatically exempts income of charitable/educational institutions of public character; no donor deduction; ~30 days.</t>
         </is>
       </c>
+      <c r="R194" s="2" t="inlineStr">
+        <is>
+          <t>No remote opening. CBG-supervised banks require an in-person visit with passport, visa/residence permit and proof of address; a remote foreign founder needs a local visit or representative.</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -17483,6 +18454,11 @@
           <t>CLG registered with Registrar of Companies; Tax &amp; Duty Exemption Act 2023 gives duty-free charitable imports (minister-approved, not automatic); no broad income-tax exemption/donor deduction; time unpublished.</t>
         </is>
       </c>
+      <c r="R195" s="2" t="inlineStr">
+        <is>
+          <t>Bank of Sierra Leone requires a NIN for new individual accounts, and foreign corporate account openings need a residence permit plus in-person KYC; remote opening is not available - local visit required.</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -17570,6 +18546,11 @@
           <t>NGO incorporated with LBR, endorsed by Foreign Affairs, then approved/registered with Ministry of Finance; 'Exempt Person' under Revenue Code = income-tax exemption; LRA grants 15% donation deduction; multi-month.</t>
         </is>
       </c>
+      <c r="R196" s="2" t="inlineStr">
+        <is>
+          <t>No remote opening. Banks require in-person identity verification with passport, residence permit and proof of address; a foreign founder with no presence needs a local agent to open the account.</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -17657,6 +18638,11 @@
           <t>Association (ordonnance 84-06) plus ONG agrément (décret 2022-182) from Interior ministry; CGI contains no general income-tax exemption or donor deduction for associations; time unpublished.</t>
         </is>
       </c>
+      <c r="R197" s="2" t="inlineStr">
+        <is>
+          <t>No remote opening. Banks require in-person application with passport, residence permit and proof of local address; a foreign founder with no presence needs a local visit or representative.</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -17744,6 +18730,11 @@
           <t>No civil-society regime exists: all organizations are state organs, so there is no private charitable entity and no tax-exemption pathway available to a foreign founder.</t>
         </is>
       </c>
+      <c r="R198" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked: no independent civil-society sector exists - all social organizations are state/party organs, and foreign entities have no access to the state-controlled banking system.</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -17831,9 +18822,14 @@
           <t>NCO registered with Ministry of Justice (99-FZ); not automatically tax-exempt - apply to tax office for exemption from profit/property tax (non-profit, commercial income under 30%); no donor deduction; 30-90 days.</t>
         </is>
       </c>
+      <c r="R199" s="2" t="inlineStr">
+        <is>
+          <t>Foreigners with legal stay can open accounts in person (Law 395-1), but a remote founder has no such grounds, and sanctions isolate Russian banks from SWIFT - access is effectively blocked for foreigners abroad.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q199"/>
+  <autoFilter ref="A1:R199"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -18947,7 +19943,7 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Foreign founder (no local presence) = yes/partial/no; main bottleneck; registration fee USD; realistic time; local charitable-deduction regime; foreign-donor/donation restrictions (FCRA-style); annual compliance &amp; reporting (ongoing filings, audit, consequences); tax-exempt status &amp; benefits (recognition pathway, tax benefits); confidence (high/med/low); source URLs.</t>
+          <t>Foreign founder (no local presence) = yes/partial/no; main bottleneck; registration fee USD; realistic time; local charitable-deduction regime; foreign-donor/donation restrictions (FCRA-style); annual compliance &amp; reporting (ongoing filings, audit, consequences); tax-exempt status &amp; benefits (recognition pathway, tax benefits); bank account remote feasibility (online / local visit / local agent / blocked); confidence (high/med/low); source URLs.</t>
         </is>
       </c>
     </row>
@@ -18959,7 +19955,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>198 jurisdictions researched via DSH subagent fan-out (16 regional batches, 196 countries + North Korea/Russia extras), then enrichment passes 2 (32 agents x ~6 countries), 2b (141 gap-filler deep-dives) and 3 (10 agents, annual compliance) with fresh web research against official registries and NGO-law guides. All 198 rows reached high/med confidence (zero 'low' remaining). Costs in USD approximations; times are realistic end-to-end durations for a foreign founder.</t>
+          <t>198 jurisdictions researched via DSH subagent fan-out (16 regional batches, 196 countries + North Korea/Russia extras), then enrichment passes 2 (32 agents x ~6 countries), 2b (141 gap-filler deep-dives), 3 (annual compliance), 4 (tax-exemption) and 5 (bank-access feasibility) with fresh web research against official registries, tax authorities and NGO-law guides. All 198 rows reached high/med confidence (zero 'low' remaining). Costs in USD approximations; times are realistic end-to-end durations for a foreign founder.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Consistency audit fixes: Australia pres->yes (home jurisdiction), San Marino very hard->hard (verified foundazioni route)
Full-row audit across presence/bottleneck/fee/difficulty; the two genuine
contradictions fixed, 18-col XLSX + webapp rebuilt.
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -5526,12 +5526,12 @@
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>ACNC requires an Australian registered office and at least one Australian-resident governing-body member; ABN needed first.</t>
+          <t>None (home jurisdiction): ACNC requires an Australian registered office + at least one Australian-resident governing-body member (the founder qualifies); ABN first.</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -10748,9 +10748,9 @@
           <t>Fondazione (Law 1 July 2015 n.101; public notarial deed, ATS Registro delle Fondazioni) and Associazione non-profit (ANR/AR registers) under the consolidated CGeG law on non-profit associations and foundations; ONLUS by ATS act.</t>
         </is>
       </c>
-      <c r="D112" s="6" t="inlineStr">
-        <is>
-          <t>very hard</t>
+      <c r="D112" s="7" t="inlineStr">
+        <is>
+          <t>hard</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="I112" s="2" t="inlineStr">
         <is>
-          <t>Italian-language filings and in-person steps; San Marino registered office required; almost no English-language service</t>
+          <t>Italian-language notarial deed + in-person steps; registered office required; almost no English-language service (foundazioni route feasible: no residency requirement, AML-equivalent home state per Art.2/29)</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
@@ -18907,7 +18907,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -18922,12 +18922,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>~$0-110 (spolek court fee 0; nadace 2,700 CZK + notary)</t>
+          <t>none for ACNC (~$340 if ASIC-incorporated CLBG)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2-6 weeks (court registration, 15-day filing deadline)</t>
+          <t>1-4 weeks</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -18942,7 +18942,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>http://www.juristi.cz/association-incorporation/; https://cof.org/country-notes/nonprofit-law-czech-republic; https://www.icnl.org/wp-content/uploads/Czech-Republic_2010pbc.pdf; https://portal.gov.cz/sluzby-vs/zapis-do-spolkoveho-rejstriku-S15505</t>
+          <t>https://www.acnc.gov.au/for-charities/start-charity/you-start-charity; https://www.acnc.gov.au/factsheet-who-can-register-acnc; https://www.acnc.gov.au/tools/guides/registration-application-checklist-and-guide</t>
         </is>
       </c>
     </row>
@@ -18952,7 +18952,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -18967,12 +18967,12 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>~$35-100 (MTÜ 30 EUR; sihtasutus 80 EUR + notary)</t>
+          <t>~$0-110 (spolek court fee 0; nadace 2,700 CZK + notary)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1-3 business days (online via e-Business Register)</t>
+          <t>2-6 weeks (court registration, 15-day filing deadline)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -18987,7 +18987,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>https://www.eesti.ee/eraisik/en/artikkel/doing-business/establishing-a-company/founding-a-nonprofit-association; https://www.e-resident.gov.ee/blog/posts/how-to-start-a-non-profit-organisation-in-estonia/; https://www.rik.ee/en/e-business-register/e-business-register-portal</t>
+          <t>http://www.juristi.cz/association-incorporation/; https://cof.org/country-notes/nonprofit-law-czech-republic; https://www.icnl.org/wp-content/uploads/Czech-Republic_2010pbc.pdf; https://portal.gov.cz/sluzby-vs/zapis-do-spolkoveho-rejstriku-S15505</t>
         </is>
       </c>
     </row>
@@ -18997,7 +18997,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Kyrgyzstan</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -19012,12 +19012,12 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>~$35-100 (MTÜ 30 EUR; sihtasutus 80 EUR + notary)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>3 working days</t>
+          <t>1-3 business days (online via e-Business Register)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -19032,7 +19032,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>https://www.icnl.org/resources/civic-freedom-monitor/kyrgyz; https://www.legal500.com/en/intelligence/kyrgyzstan/corporate-commercial-law/on-establishing-the-amount-of-fees-for-state-registration; https://www.rferl.org/a/kyrgyzstan-foreign-agents-chill/32893000.html; https://cbd.minjust.gov.kg/4-260/edition/6030/ru</t>
+          <t>https://www.eesti.ee/eraisik/en/artikkel/doing-business/establishing-a-company/founding-a-nonprofit-association; https://www.e-resident.gov.ee/blog/posts/how-to-start-a-non-profit-organisation-in-estonia/; https://www.rik.ee/en/e-business-register/e-business-register-portal</t>
         </is>
       </c>
     </row>
@@ -19042,7 +19042,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Kyrgyzstan</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -19057,12 +19057,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>~$585-1,600 (KvK EUR 85.15 + notary EUR 500-1,500, the dominant cost)</t>
+          <t>63</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>2-4 weeks (notarial deed scheduling)</t>
+          <t>3 working days</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19077,7 +19077,7 @@
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>https://www.kvk.nl/en/registration/registering-a-stichting/; https://www.givingwhatwecan.org/get-involved/tax-deductibility/the-netherlands; https://netherbridge.nl/set-up-dutch-ngo-charity-non-profit/; https://www.kvk.nl/inschrijven/inschrijven-stichting/</t>
+          <t>https://www.icnl.org/resources/civic-freedom-monitor/kyrgyz; https://www.legal500.com/en/intelligence/kyrgyzstan/corporate-commercial-law/on-establishing-the-amount-of-fees-for-state-registration; https://www.rferl.org/a/kyrgyzstan-foreign-agents-chill/32893000.html; https://cbd.minjust.gov.kg/4-260/edition/6030/ru</t>
         </is>
       </c>
     </row>
@@ -19087,7 +19087,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -19102,12 +19102,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>~$150-650 (fundacja: KRS fee ~2,500 PLN + notary; stowarzyszenie: notary only)</t>
+          <t>~$585-1,600 (KvK EUR 85.15 + notary EUR 500-1,500, the dominant cost)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>1-3 months (KRS registration)</t>
+          <t>2-4 weeks (notarial deed scheduling)</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -19122,7 +19122,7 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>https://www.ngo.pl/english/how-do-ngos-work-in-poland/is-a-non-governmental-organization-and-a-public-benefit-organization-opp-the-same-thing; https://www.dudkowiak.com/corporate-law-in-poland/ngo-foundation-registration-in-poland.html; https://cof.org/country-notes/nonprofit-law-poland; https://arch-bip.ms.gov.pl/pl/rejestry-i-ewidencje/krajowy-rejestr-sadowy/oplaty-obowiazujace-w-postepowaniu-rejestrowym/</t>
+          <t>https://www.kvk.nl/en/registration/registering-a-stichting/; https://www.givingwhatwecan.org/get-involved/tax-deductibility/the-netherlands; https://netherbridge.nl/set-up-dutch-ngo-charity-non-profit/; https://www.kvk.nl/inschrijven/inschrijven-stichting/</t>
         </is>
       </c>
     </row>
@@ -19132,7 +19132,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Seychelles</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -19147,12 +19147,12 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>~$150-650 (fundacja: KRS fee ~2,500 PLN + notary; stowarzyszenie: notary only)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>1-3 weeks</t>
+          <t>1-3 months (KRS registration)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -19167,7 +19167,7 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>https://www.ifcreview.com/articles/2010/february/seychelles-foundations/; https://sterlingoffshore.com/knowledge-base/foundations/seychelles-foundation/; https://gsl.org/en/offers/establishing-a-seychelles-foundation/; https://www.fsaseychelles.sc/images/Licensing_and_Registration_Fees.pdf; https://registrationdivision.gov.sc/our-services/associations/</t>
+          <t>https://www.ngo.pl/english/how-do-ngos-work-in-poland/is-a-non-governmental-organization-and-a-public-benefit-organization-opp-the-same-thing; https://www.dudkowiak.com/corporate-law-in-poland/ngo-foundation-registration-in-poland.html; https://cof.org/country-notes/nonprofit-law-poland; https://arch-bip.ms.gov.pl/pl/rejestry-i-ewidencje/krajowy-rejestr-sadowy/oplaty-obowiazujace-w-postepowaniu-rejestrowym/</t>
         </is>
       </c>
     </row>
@@ -19177,7 +19177,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Seychelles</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -19192,12 +19192,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>200</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>about 2 months</t>
+          <t>1-3 weeks</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.za/services/register-business-or-organisation/register-non-profit-company; https://www.sars.gov.za/businesses-and-employers/tax-exempt-institutions/public-benefit-organisations/; https://www.cipc.co.za/wp-content/uploads/Step_by_step_Guide/Step_by_step_guide_Non_Profit_companyCOR_15.1C_without_members_with_a_Short_Standard_MOI_registration_v0.1.pdf; https://www.gov.za/services/register-nonprofit-organisation</t>
+          <t>https://www.ifcreview.com/articles/2010/february/seychelles-foundations/; https://sterlingoffshore.com/knowledge-base/foundations/seychelles-foundation/; https://gsl.org/en/offers/establishing-a-seychelles-foundation/; https://www.fsaseychelles.sc/images/Licensing_and_Registration_Fees.pdf; https://registrationdivision.gov.sc/our-services/associations/</t>
         </is>
       </c>
     </row>
@@ -19222,7 +19222,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -19242,7 +19242,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>3-6 months</t>
+          <t>about 2 months</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -19257,7 +19257,7 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/how-to-register-charity; https://www.gov.uk/government/organisations/charity-commission; https://register-of-charities.charitycommission.gov.uk/en/; https://www.gov.uk/setting-up-charity/register-your-charity</t>
+          <t>https://www.gov.za/services/register-business-or-organisation/register-non-profit-company; https://www.sars.gov.za/businesses-and-employers/tax-exempt-institutions/public-benefit-organisations/; https://www.cipc.co.za/wp-content/uploads/Step_by_step_Guide/Step_by_step_guide_Non_Profit_companyCOR_15.1C_without_members_with_a_Short_Standard_MOI_registration_v0.1.pdf; https://www.gov.za/services/register-nonprofit-organisation</t>
         </is>
       </c>
     </row>
@@ -19267,7 +19267,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -19282,12 +19282,12 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>~$100-700 (state incorporation ~$50-150 + IRS 1023-EZ user fee $275; state-dependent)</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Same day to 2 weeks (incorporation, state-dependent); 501(c)(3) determination 3-12 months extra</t>
+          <t>3-6 months</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -19302,7 +19302,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.irs.gov/charities-non-profits/form-1023-and-1023-ez-amount-of-user-fee; https://www.irs.gov/charities-non-profits/frequently-asked-questions-about-form-1023; https://www.501c3.org/incorporate-nonprofit-delaware/; https://corp.delaware.gov/fee/</t>
+          <t>https://www.gov.uk/how-to-register-charity; https://www.gov.uk/government/organisations/charity-commission; https://register-of-charities.charitycommission.gov.uk/en/; https://www.gov.uk/setting-up-charity/register-your-charity</t>
         </is>
       </c>
     </row>
@@ -19312,7 +19312,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Belize</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -19327,12 +19327,12 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>~$100-700 (state incorporation ~$50-150 + IRS 1023-EZ user fee $275; state-dependent)</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>2-4 weeks</t>
+          <t>Same day to 2 weeks (incorporation, state-dependent); 501(c)(3) determination 3-12 months extra</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -19342,12 +19342,12 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>difficulty=easy, no-presence=yes, GfN=Yes, confidence=med</t>
+          <t>difficulty=easy, no-presence=yes, GfN=Yes, confidence=high</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>https://beltraide.bz/belize-invest/doing-business-in-belize/company-incorporation/; https://bccar.bz/services/non-governmental-organisations/; https://www.facebook.com/BelizeCompaniesRegistry/posts/frequently-asked-questionswhat-type-of-legal-vehicle-should-a-not-for-profit-org/191133726554188/; https://www.belizefsc.org.bz/wp-content/uploads/2025/04/FSC_BCCAR-NPO-Webinar_23-04-2024.pdf</t>
+          <t>https://www.irs.gov/charities-non-profits/form-1023-and-1023-ez-amount-of-user-fee; https://www.irs.gov/charities-non-profits/frequently-asked-questions-about-form-1023; https://www.501c3.org/incorporate-nonprofit-delaware/; https://corp.delaware.gov/fee/</t>
         </is>
       </c>
     </row>
@@ -19442,7 +19442,7 @@
         <v>1</v>
       </c>
       <c r="H2" s="10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -19716,10 +19716,10 @@
         <v>6</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H12" s="10" t="n">
         <v>6</v>

</xml_diff>

<commit_message>
Apply top-10 fresh verification corrections (10 countries re-checked vs official sources)
AU: 1-4 wks -> up to 12 wks allocation + 15 bus days (ACNC FAQ). EE: 2026
deduction cap ~EUR 3,780. KG: fee 2,000->3,500 KGS, 3->5 days. NL: 30% =
25%+5%, ANBI ~4 wks. SEY: NPO Act 741 + CEPS route confirmed. ZA: NPO Act
60->78/1997. UK: CH fee GBP 12->100 (1 Feb 2026), gov.uk 404 URL fixed,
Charities Act 2022 noted. PL: PIT earmark 14%->1.5% (2019), 2017 transfer
abolition, KRS 2,500->250 PLN (10x typo), fundacja ~5-150. US: verified
no change (Rev. Proc. 2026-5 fees, median 1023 ~6 mo).

Top-10 now Australia,Czechia,Estonia,Kyrgyzstan,Netherlands,Poland,
Seychelles,South Africa,UK,US. 18-col XLSX + webapp (466 KB) rebuilt.
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -5516,12 +5516,12 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>A$0 ACNC fee (~A$514 if incorporating a CLBG with ASIC), 1-4 weeks</t>
+          <t>A$0 ACNC fee (confirmed; ASIC CLBG incorporation fee A$403 in Jan-2025 compilation, indexed annually, ~A$514 current), up to 12 weeks allocation + ~15 business days processing (ACNC FAQ 2025-26)</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Home setup: register with ACNC (Australian Charities and Not-for-profits Commission) for tax-deductible-gift status; most foreign-linked founders use a charitable trust with local trustees | confirm prior: free ACNC registration, A$514 ASIC CLBG, 1-4 weeks, easy</t>
+          <t>Home setup: register with ACNC (Australian Charities and Not-for-profits Commission) for tax-deductible-gift status; most foreign-linked founders use a charitable trust with local trustees | confirm prior: free ACNC registration, ASIC CLBG A$403-514, up to 12 weeks + ~15 business days, easy</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -5531,7 +5531,7 @@
       </c>
       <c r="I55" s="2" t="inlineStr">
         <is>
-          <t>None (home jurisdiction): ACNC requires an Australian registered office + at least one Australian-resident governing-body member (the founder qualifies); ABN first.</t>
+          <t>None material (home jurisdiction): ACNC requires an ABN, a registered office and at least one Australian-resident governing-body member (the founder qualifies); processing time is the main delay.</t>
         </is>
       </c>
       <c r="J55" s="2" t="inlineStr">
@@ -7448,7 +7448,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>State duty ~2,000 KGS (US$22), ~5 business days, e-filing via State Registration Portal</t>
+          <t>State duty ~3,500 KGS (US$40, 2026 index), ~5 business days, e-filing via State Registration Portal</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -7468,12 +7468,12 @@
       </c>
       <c r="J76" s="2" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>~25-40 (state duty 3,500 KGS ~US$40 per 2026 schedule, indexed; previously quoted 2,000 KGS/US$22 is stale)</t>
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr">
         <is>
-          <t>3 working days</t>
+          <t>5 working days (e-filing via State Registration Portal)</t>
         </is>
       </c>
       <c r="L76" s="2" t="inlineStr">
@@ -9825,7 +9825,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Non-profit company (NPC, Companies Act 71/2008); trust (Trust Property Control Act 57/1988); NPO (NPO Act 60/1997); PBO tax status (Income Tax Act s.30, SARS)</t>
+          <t>Non-profit company (NPC, Companies Act 71/2008); trust (Trust Property Control Act 57/1988); NPO (NPO Act 78/1997); PBO tax status (Income Tax Act s.30, SARS)</t>
         </is>
       </c>
       <c r="D102" s="5" t="inlineStr">
@@ -9932,7 +9932,7 @@
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
-          <t>EUR 585-1,585 (KvK fee €85.15 + notary EUR 500-1,500), 1-2 weeks (ANBI decision 4-8 weeks)</t>
+          <t>EUR 585-1,585 (KvK fee €85.15 + notary EUR 500-1,500), 1-2 weeks (ANBI decision 4-8 weeks; Belastingdienst 2026: typically ~4 weeks)</t>
         </is>
       </c>
       <c r="G103" s="2" t="inlineStr">
@@ -9987,7 +9987,7 @@
       </c>
       <c r="Q103" s="2" t="inlineStr">
         <is>
-          <t>Separate ANBI decision (beschikking) from Belastingdienst: public-benefit purpose + 90%-of-activity rule; grants CIT exemption + 30% donor deduction; usually 2-4 weeks, no statutory deadline.</t>
+          <t>Separate ANBI decision (beschikking) from Belastingdienst: public-benefit purpose + 90%-of-activity rule; grants CIT exemption + 30% donor deduction (statutory 25% + 5% supplementary rate, combined 30%); usually 2-4 weeks, no statutory deadline.</t>
         </is>
       </c>
       <c r="R103" s="2" t="inlineStr">
@@ -10964,7 +10964,7 @@
       </c>
       <c r="J114" s="2" t="inlineStr">
         <is>
-          <t>~$150-650 (fundacja: KRS fee ~2,500 PLN + notary; stowarzyszenie: notary only)</t>
+          <t>~$45-150 (fundacja: KRS court fee 250 PLN + notary deed ~500-1,500 PLN; stowarzyszenie: 0 PLN, Art. 17 ust. 3 fee exemption)</t>
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr">
@@ -10974,7 +10974,7 @@
       </c>
       <c r="L114" s="2" t="inlineStr">
         <is>
-          <t>14% of personal income tax earmarkable to registered OPP; 1.5% budget transfer to OPPs</t>
+          <t>1.5% of personal income tax earmarkable to registered OPP (statutory 1.5% since 2019; the old 1.5% state-budget transfer to OPPs was abolished in 2017, Dz.U. 2017 poz. 573)</t>
         </is>
       </c>
       <c r="M114" s="2" t="inlineStr">
@@ -12784,12 +12784,12 @@
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
-          <t>CLG at Companies House ~£12; Charity Commission registration free; ~8–12 weeks</t>
+          <t>CLG at Companies House £100 (was £12; fee change effective 1 Feb 2026, announced 30 Oct 2025); Charity Commission registration free; ~8–12 weeks (Charity Commission 2025-26: median ~12 weeks to full registration)</t>
         </is>
       </c>
       <c r="G134" s="2" t="inlineStr">
         <is>
-          <t>English-language, common law; the most popular expat-charity pathway; overseas individuals may be trustees provided management and control are in the UK | Verified: Must be based in England/Wales (local postal address + governing document); no trustee-residency rule.</t>
+          <t>English-language, common law; the most popular expat-charity pathway; overseas individuals may be trustees provided management and control are in the UK | Verified: Must be based in England/Wales (local postal address + governing document); no trustee-residency rule. | Verified 2026: Charities Act 2011 as amended by Charities Act 2022 (commencement regs in force from 2025).</t>
         </is>
       </c>
       <c r="H134" s="2" t="inlineStr">
@@ -12829,7 +12829,7 @@
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/how-to-register-charity; https://www.gov.uk/government/organisations/charity-commission; https://register-of-charities.charitycommission.gov.uk/en/; https://www.gov.uk/setting-up-charity/register-your-charity</t>
+          <t>https://www.gov.uk/setting-up-charity/register-your-charity; https://www.gov.uk/government/organisations/charity-commission; https://register-of-charities.charitycommission.gov.uk/en/; https://www.gov.uk/setting-up-charity/register-your-charity</t>
         </is>
       </c>
       <c r="P134" s="2" t="inlineStr">
@@ -13366,7 +13366,7 @@
       </c>
       <c r="L140" s="2" t="inlineStr">
         <is>
-          <t>Deductible for individuals up to 300% of statutory minimum wage; no foreign-donor restrictions.</t>
+          <t>Deductible for individuals up to 300% of statutory minimum wage (2026 cap ~EUR 3,780), indexed annually; no foreign-donor restrictions.</t>
         </is>
       </c>
       <c r="M140" s="2" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>English-language, simple, offshore-friendly regime; popular with foreign founders; a Seychelles charity gains no local tax-exempt status without local operations. | Confirm prior: NPO Act 2013 for local NPOs; the practical foreign route is the Seychelles Foundation Act 2009 (SIBA, $200 gov fee); prior $1,500-3,000 is agent-inclusive. | Verified: No local presence required; foreign founder may be a councillor; FSA registration fee ~US$200 plus ~US$200 annual.</t>
+          <t>English-language, simple, offshore-friendly regime; popular with foreign founders; a Seychelles charity gains no local tax-exempt status without local operations. | Confirm prior: NPO Act 2013 for local NPOs; the practical foreign route is the Seychelles Foundation Act 2009 (SIBA, $200 gov fee); prior $1,500-3,000 is agent-inclusive. | Verified: No local presence required; foreign founder may be a councillor; FSA registration fee ~US$200 plus ~US$200 annual. | Verified 2026: NPO Act Cap. 741 (Seychelles NPO Act 2013) is the current local regime; no amendment changing the route found; the foreign-foundation route (Foundation Act 2009) remains the practical path for non-residents.</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr">
@@ -16519,7 +16519,7 @@
       </c>
       <c r="Q174" s="2" t="inlineStr">
         <is>
-          <t>Separate application via CEPS to Ministry of Finance: business-tax exemption for charitable institutions; no general donor deduction; VAT exempt only on international donations; time unpublished.</t>
+          <t>Separate application via CEPS to Ministry of Finance: business-tax exemption for charitable institutions; no general donor deduction; VAT exempt only on international donations; time unpublished. | Verified 2026: donor-deduction route = CEPS 'charitable institutions' business-tax exemption (no general donor deduction); no change found.</t>
         </is>
       </c>
       <c r="R174" s="2" t="inlineStr">
@@ -19057,12 +19057,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>~25-40 (state duty 3,500 KGS ~US$40 per 2026 schedule, indexed; previously quoted 2,000 KGS/US$22 is stale)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>3 working days</t>
+          <t>5 working days (e-filing via State Registration Portal)</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -19147,7 +19147,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>~$150-650 (fundacja: KRS fee ~2,500 PLN + notary; stowarzyszenie: notary only)</t>
+          <t>~$45-150 (fundacja: KRS court fee 250 PLN + notary deed ~500-1,500 PLN; stowarzyszenie: 0 PLN, Art. 17 ust. 3 fee exemption)</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -19302,7 +19302,7 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.uk/how-to-register-charity; https://www.gov.uk/government/organisations/charity-commission; https://register-of-charities.charitycommission.gov.uk/en/; https://www.gov.uk/setting-up-charity/register-your-charity</t>
+          <t>https://www.gov.uk/setting-up-charity/register-your-charity; https://www.gov.uk/government/organisations/charity-commission; https://register-of-charities.charitycommission.gov.uk/en/; https://www.gov.uk/setting-up-charity/register-your-charity</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Replace 13 dead (404) source URLs with verified-live official sources
URL health check over all 648 source URLs: 14 true 404s found (the 4xx/net
hits are 403 bot-blocks on cof.org/state.gov/etc., fine in browsers). Each
replaced source was found by an agent and verified HTTP-200 before swap.
Countries: St. Lucia, Finland, Senegal, Fiji, Russia, Panama, Seychelles,
Honduras, Brunei, Singapore, Austria, Western Sahara, Kuwait.
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -1605,7 +1605,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>http://attorneygeneralchambers.com/laws-of-saint-lucia/companies-act/part-9-fees; http://attorneygeneralchambers.com/laws-of-saint-lucia/international-business-companies-act/section-39; https://esaintlucia.com/pricing; https://www.cra.gov.lc</t>
+          <t>https://www.lexadin.nl/wlg/legis/nofr/oeur/arch/stl/int_trust.pdf; http://attorneygeneralchambers.com/laws-of-saint-lucia/international-business-companies-act/section-39; https://esaintlucia.com/pricing; https://www.cra.gov.lc</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>https://www.sgjd.gob.hn/servicios-y-gestiones-web/requisitos/servicios-de-atencion-al-ciudadano/personalidad-juridica/fundaciones; https://diref.gob.hn/; https://consortiumlegal.com/2022/09/21/que-se-debe-tener-en-consideracion-si-desea-constituir-o-incorporar-una-ongd-en-honduras/; https://sgjd.gob.hn/servicios-y-gestiones-web/requisitos/servicios-de-atencion-al-ciudadano/personalidad-juridica/fundaciones</t>
+          <t>https://www.sgjd.gob.hn/institucion/dependencias/subsecretaria-de-justicia/direccion-de-regulacion-registro-y-seguimiento-de-asociaciones-civiles-dirrsac; https://diref.gob.hn/; https://consortiumlegal.com/2022/09/21/que-se-debe-tener-en-consideracion-si-desea-constituir-o-incorporar-una-ongd-en-honduras/; https://sgjd.gob.hn/servicios-y-gestiones-web/requisitos/servicios-de-atencion-al-ciudadano/personalidad-juridica/fundaciones</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>https://www.organojudicial.gob.pa/uploads/wp_repo/blogs.dir/cendoj/CIVIL/ley_25_de_1995_fundaciones_de_interes_privado.pdf; https://laglex.net/nuestros-servicios/fundaciones-de-interes-privado/; https://www.rglawfirmpa.com/fundaciones-privadas-en-panama; https://panamadigital.gob.pa/base-legal/; https://docs.panama.justia.com/federales/leyes/25-de-1995-jun-14-1995.pdf</t>
+          <t>https://www.organojudicial.gob.pa/uploads/wp_repo/blogs.dir/cendoj/CIVIL/ley_25_de_1995_fundaciones_de_interes_privado.pdf; https://laglex.net/nuestros-servicios/fundaciones-de-interes-privado/; https://www.rglawfirmpa.com/fundaciones-privadas-en-panama; https://www.gacetaoficial.gob.pa/; https://docs.panama.justia.com/federales/leyes/25-de-1995-jun-14-1995.pdf</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -4549,7 +4549,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>https://www.charities.gov.sg/Pages/Charities-and-IPCs/Register-as-a-Charity/Criteria-for-Registration-as-a-Charity.aspx; https://sso.agc.gov.sg/SL/CA1994-RG10?DocDate=20230113; https://krestonhelmitalib.com.sg/guide-to-registering-a-charity/</t>
+          <t>https://www.charities.gov.sg/Pages/Charities-and-IPCs/Register-as-a-Charity/Criteria-for-Registration-as-Charity.aspx; https://sso.agc.gov.sg/SL/CA1994-RG10?DocDate=20230113; https://krestonhelmitalib.com.sg/guide-to-registering-a-charity/</t>
         </is>
       </c>
       <c r="P44" s="2" t="inlineStr">
@@ -5377,7 +5377,7 @@
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
-          <t>https://www.polis.gov.bn/pendaftar-pertubuhan/; https://www.icnl.org/research/library/brunei-darussalam_societies/; https://www.agc.gov.bn/AGC%20Images/LAWS/Gazette_PDF/2005/EN/s001.pdf</t>
+          <t>https://www.polis.gov.bn/pendaftar-pertubuhan/; https://www.icnl.org/research/library/brunei-darussalam_societies/; https://www.agc.gov.bn/wp-content/uploads/2026/07/CAP-203-2010-ED-SOCIETIES-ACT.pdf</t>
         </is>
       </c>
       <c r="P53" s="2" t="inlineStr">
@@ -5745,7 +5745,7 @@
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
-          <t>https://laws.gov.fj/Acts/DisplayAct/3231; https://www.sas.com.fj/commercial-law-updates/how-to-incorporate-a-non-profit-entity-as-a-charitable-trust-or-company-limited-by-guarantee-under-fiji-law; https://www.justice.gov.fj/company/</t>
+          <t>https://www.laws.gov.fj/; https://www.sas.com.fj/commercial-law-updates/how-to-incorporate-a-non-profit-entity-as-a-charitable-trust-or-company-limited-by-guarantee-under-fiji-law; https://www.justice.gov.fj/company/</t>
         </is>
       </c>
       <c r="P57" s="2" t="inlineStr">
@@ -10437,7 +10437,7 @@
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
-          <t>https://www.oesterreich.gv.at/en/themen/reisen_und_freizeit/vereine/Seite.220300; https://coredo.eu/company-registration-in-austria-legal-steps; https://www.oesterreich.gv.at/Seite.220300</t>
+          <t>https://www.oesterreich.gv.at/en/themen/reisen_und_freizeit/vereine/Seite.220300; https://coredo.eu/company-registration-in-austria-legal-steps; https://www.oesterreich.gv.at/de/themen/reisen_und_freizeit/vereine/Seite.220300</t>
         </is>
       </c>
       <c r="P108" s="2" t="inlineStr">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>https://yhdistysrekisteri.prh.fi/?userLang=en; https://en.wikipedia.org/wiki/Registered_association_(Finland); https://www.prh.fi/en/price-lists/hinnasto/kasittelymaksut.html</t>
+          <t>https://yhdistysrekisteri.prh.fi/?userLang=en; https://www.finlex.fi/fi/lainsaadanto/1989/503; https://www.prh.fi/en/price-lists/hinnasto/kasittelymaksut.html</t>
         </is>
       </c>
       <c r="P137" s="2" t="inlineStr">
@@ -14577,7 +14577,7 @@
       </c>
       <c r="O153" s="2" t="inlineStr">
         <is>
-          <t>https://www.asarlegal.com/kuwait-reshapes-regulations-for-charitable-organisations/; https://ylf.com.kw/blogs/%D9%82%D8%A7%D9%86%D9%88%D9%86-%D8%A7%D9%84%D8%AC%D9%85%D8%B9%D9%8A%D8%A7%D8%AA-%D9%88%D8%A7%D9%84%D9%85%D8%AB%D8%B3%D8%B3%D8%A7%D8%AA-%D8%A7%D9%84%D8%A3%D9%87%D9%84%D9%8A%D8%A9-%D9%81%D9%8A-%D8%A7%D9%84%D9%83%D9%88%D9%8A%D8%AA-%D8%AF%D9%84%D9%8A%D9%84-%D8%B4%D8%A7%D9%85%D9%84-%D9%84%D9%84%D8%AA%D8%A3%D8%B3%D9%8A%D8%B3-%D9%88%D8%A7%D9%84%D8%A5%D8%AF%D8%A7%D8%B1%D8%A9-%D9%88%D8%A7%D9%84%D8%B1%D9%82%D8%A7%D8%A8%D8%A9?lang=en; https://alsubaielawfirm.com/en/establishing-non-profit-companies-in-kuwait/</t>
+          <t>https://www.asarlegal.com/kuwait-reshapes-regulations-for-charitable-organisations/; https://www.icnl.org/research/library/kuwait_24-62-en/; https://alsubaielawfirm.com/en/establishing-non-profit-companies-in-kuwait/</t>
         </is>
       </c>
       <c r="P153" s="2" t="inlineStr">
@@ -15865,7 +15865,7 @@
       </c>
       <c r="O167" s="2" t="inlineStr">
         <is>
-          <t>https://www.lexmundi.com/guides/social-enterprise-law-surveys/jurisdictions/africa/morocco/; https://www.state.gov/reports/2024-country-reports-on-human-rights-practices/western-sahara/</t>
+          <t>https://www.lexmundi.com/guides/social-enterprise-law-surveys/jurisdictions/africa/morocco/; https://www.state.gov/reports/2024-country-reports-on-human-rights-practices/morocco/</t>
         </is>
       </c>
       <c r="P167" s="2" t="inlineStr">
@@ -16509,7 +16509,7 @@
       </c>
       <c r="O174" s="2" t="inlineStr">
         <is>
-          <t>https://www.ifcreview.com/articles/2010/february/seychelles-foundations/; https://sterlingoffshore.com/knowledge-base/foundations/seychelles-foundation/; https://gsl.org/en/offers/establishing-a-seychelles-foundation/; https://www.fsaseychelles.sc/images/Licensing_and_Registration_Fees.pdf; https://registrationdivision.gov.sc/our-services/associations/</t>
+          <t>https://www.ifcreview.com/articles/2010/february/seychelles-foundations/; https://sterlingoffshore.com/knowledge-base/foundations/seychelles-foundation/; https://gsl.org/en/offers/establishing-a-seychelles-foundation/; https://www.fsaseychelles.sc/images/Licensing_and_Registration_Fees.pdf; https://www.gazette.sc/sites/default/files/2022-05/Act%208%20-%202022%20-%20Associations%20Act%202022.pdf</t>
         </is>
       </c>
       <c r="P174" s="2" t="inlineStr">
@@ -18257,7 +18257,7 @@
       </c>
       <c r="O193" s="2" t="inlineStr">
         <is>
-          <t>https://www.icnl.org/resources/civic-freedom-monitor/senegal; https://www.service-public.gouv.fr/particuliers/vosdroits/F426; https://dgsfc.gouv.sn/sites/default/files/2021-03/guide_pour_la+constitution_ASSOCIATION_et_ONG.pdf</t>
+          <t>https://www.icnl.org/resources/civic-freedom-monitor/senegal; https://www.service-public.gouv.fr/particuliers/vosdroits/F426; https://dgsfc.gouv.sn/sites/default/files/2021-03/guide_pour_la%20constitution_ASSOCIATION_et_ONG.pdf</t>
         </is>
       </c>
       <c r="P193" s="2" t="inlineStr">
@@ -18809,7 +18809,7 @@
       </c>
       <c r="O199" s="2" t="inlineStr">
         <is>
-          <t>https://pareto-group.com/en/legal-services/registration-of-companies-individual-entrepreneurs/registration-of-nonprofit-organization/; https://cof.org/country-notes/nonprofit-law-russia; https://en.wikipedia.org/wiki/Russian_undesirable_organizations_law; https://minjust.gov.ru/en</t>
+          <t>https://pareto-group.com/en/legal-services/registration-of-companies-individual-entrepreneurs/registration-of-nonprofit-organization/; https://cof.org/country-notes/nonprofit-law-russia; https://en.wikipedia.org/wiki/Russian_undesirable_organizations_law; https://minjust.gov.ru/ru/activity/govservices/5/</t>
         </is>
       </c>
       <c r="P199" s="2" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>https://www.ifcreview.com/articles/2010/february/seychelles-foundations/; https://sterlingoffshore.com/knowledge-base/foundations/seychelles-foundation/; https://gsl.org/en/offers/establishing-a-seychelles-foundation/; https://www.fsaseychelles.sc/images/Licensing_and_Registration_Fees.pdf; https://registrationdivision.gov.sc/our-services/associations/</t>
+          <t>https://www.ifcreview.com/articles/2010/february/seychelles-foundations/; https://sterlingoffshore.com/knowledge-base/foundations/seychelles-foundation/; https://gsl.org/en/offers/establishing-a-seychelles-foundation/; https://www.fsaseychelles.sc/images/Licensing_and_Registration_Fees.pdf; https://www.gazette.sc/sites/default/files/2022-05/Act%208%20-%202022%20-%20Associations%20Act%202022.pdf</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fee/time plausibility sweep: normalize fee column to gov't-fee semantics
- 11 fee cells where 'incl. agent' all-in was conflated with the official
  gov't fee (Bahamas, St. Lucia, St. Vincent, Fiji, Congo, Uganda, Tanzania,
  Maldives, Ghana, Guinea-Bissau, Sierra Leone) now list the official gov't
  fee with the all-in-with-agent figure clearly labeled.
- 0 fees over $3,000; 0 timelines over 18 months; 7 'unparseable' times are
  genuinely-impossible countries (Cuba, NK, Vatican, Yemen, etc.).
- Rebuilt 18-col XLSX + webapp (468 KB).
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -1028,7 +1028,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>~$300-800 incl. agent</t>
+          <t>~$100-250 (gov, B$200-500); ~$300-800 all-in w/ licensed agent</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>~$750</t>
+          <t>~$100-400 (gov); ~$1,500-2,500 all-in w/ local agent</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>~$1,200</t>
+          <t>~$350 (gov, EC$950); ~$1,500+ all-in w/ agent</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -5720,7 +5720,7 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>~$130-650 (FJ$100-500)</t>
+          <t>~$62 (prescribed FJ$45; up to ~$650 with resident director/agent)</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -7928,7 +7928,7 @@
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>~$50-150</t>
+          <t>~$23 (creation tax 15,000 FCFA)</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
@@ -8572,7 +8572,7 @@
       </c>
       <c r="J88" s="2" t="inlineStr">
         <is>
-          <t>~$500-1,400 (UGX 1-5M per NGO Fees Regulations 2017)</t>
+          <t>~$27-135 (UGX 0.1-0.52M registration; statutory NGO range up to UGX 5M)</t>
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr">
@@ -8664,7 +8664,7 @@
       </c>
       <c r="J89" s="2" t="inlineStr">
         <is>
-          <t>~$200-400 (TZS 500k-2M plus security deposit)</t>
+          <t>~$45 (TZS 115k; ~$267 incl. stamp duty for INGO)</t>
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr">
@@ -17312,7 +17312,7 @@
       </c>
       <c r="J183" s="2" t="inlineStr">
         <is>
-          <t>~$100-300</t>
+          <t>~$50-200 (registry)</t>
         </is>
       </c>
       <c r="K183" s="2" t="inlineStr">
@@ -17496,7 +17496,7 @@
       </c>
       <c r="J185" s="2" t="inlineStr">
         <is>
-          <t>US$500-1.5k incl. agents (ORC official fee ~GHc520 + NPOS)</t>
+          <t>~$40 (ORC official); ~$500-1.5k all-in w/ agent</t>
         </is>
       </c>
       <c r="K185" s="2" t="inlineStr">
@@ -18140,7 +18140,7 @@
       </c>
       <c r="J192" s="2" t="inlineStr">
         <is>
-          <t>~$500-2k with local agent</t>
+          <t>~$100-250 (gov deed/registry); ~$500-2k all-in w/ local agent</t>
         </is>
       </c>
       <c r="K192" s="2" t="inlineStr">
@@ -18416,7 +18416,7 @@
       </c>
       <c r="J195" s="2" t="inlineStr">
         <is>
-          <t>~$300-1.5k incl. agent</t>
+          <t>~$20+ (CAC, tiered); ~$300-1.5k all-in w/ agent</t>
         </is>
       </c>
       <c r="K195" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Consistency sweep: purge superseded claims from 65 rows' other columns
The verify-rest corrections fixed the primary cells but left the old
claims in Notes, compliance, tax-exempt, bottleneck, donor-restriction
and bank columns (138 stale hits, e.g. Nigeria 'NCMM', Saudi 'M/111',
UAE '70% nationals', Italy EUR 150k, Hong Kong 'HKJC', Seychelles
'NPO Act Cap. 741', Kenya 'NGO Board').

apply_verify_rest.py gains _drop (remove superseded Notes segments,
never the dated verify-rest notes) and _prose (corrected rewrite of a
dropped lead note). Top-10 unchanged; XLSX + webapp rebuilt.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -1242,12 +1242,12 @@
       </c>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Companies Act Ch. 74:01: annual return to the CRO within 30 days of incorporation anniversary (directors, office, officers); late default: penalties. Accounts kept; audit where required. Non-filing: strike-off.</t>
+          <t>Companies Act Chap. 81:01: annual return to the Companies Registry within 30 days of incorporation anniversary (directors, office, officers); NPOs also file under the NPO Act 2019. Late default: penalties. Accounts kept; audit where required. Non-filing: strike-off.</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>Ministry of Finance 'approved charity' status; donors deduct covenanted donations up to 15% of income; charity exempt from income tax (Income Tax Act Ch.79:04). No deduction without approval. Time unpublished.</t>
+          <t>Ministry of Finance 'approved charity' status; donors deduct covenanted donations up to 15% of income; charity exempt from income tax (Income Tax Act Chap. 75:01). No deduction without approval. Time unpublished.</t>
         </is>
       </c>
       <c r="R8" s="2" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>International ONGDs must register in the Registro Público de ONGD; moderate bureaucracy; all filings in Spanish. | confirm prior; personality granted by Poder Judicial (Chancilleria) under the 2011 OSC law covering asociaciones and fundaciones | verify-rest 2026-10: granting body is SGJD/DIRRSAC (not the Judiciary/Chancillería)</t>
+          <t>International ONGDs must register in the Registro Público de ONGD; moderate bureaucracy; all filings in Spanish. | verify-rest 2026-10: granting body is SGJD/DIRRSAC (not the Judiciary/Chancillería)</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2403,7 +2403,7 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Chancilleria legal-personality filing plus local address/representative; all filings in Spanish.</t>
+          <t>SGJD/DIRRSAC legal-personality filing plus local address/representative; all filings in Spanish.</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>Legal personality is granted by the Asamblea Nacional and is revocable for legislative non-compliance. No published annual filing deadline; the Interior Ministry registry monitors compliance.</t>
+          <t>Legal personality is granted and cancelled by the Ministerio de Gobernación (Ley 1115); entities file financial statements, donor lists and activity reports with Gobernación; non-compliance leads to cancellation.</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Foreign NGOs must register with the Ministry of Foreign Affairs (Cancillería); 2023 law caps foreign government funding for certain activities and tightens oversight; heavy Spanish-language bureaucracy; few English speakers. | Prior context confirmed; Ley 1417 (2023) replaces Ley 1475 (1993); foreign NGOs register with Ministry of Foreign Affairs | verify-rest 2026-10: registering authority corrected (not a 'Superintendencia de Compañías'); unverifiable 'Ley 1417/1475' references removed</t>
+          <t>Foreign NGOs must register with the Ministry of Foreign Affairs (Cancillería); 2023 law caps foreign government funding for certain activities and tightens oversight; heavy Spanish-language bureaucracy; few English speakers. | verify-rest 2026-10: registering authority corrected (not a 'Superintendencia de Compañías'); unverifiable 'Ley 1417/1475' references removed</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -3139,7 +3139,7 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>Resident officers + local address, notarized deed; 2023 NGO law (Ley 1417) registration + foreign funding restrictions</t>
+          <t>Resident officers + local address, notarized deed; foreign-constituted NGOs need a framework agreement with the Foreign Ministry (Ley 351 art. 13)</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Ley 1417 (2023): registration mandatory; foreign funding restricted; foreign NGOs register with Cancillería</t>
+          <t>Foreign-constituted NGOs must sign a framework cooperation agreement with the Ministerio de Relaciones Exteriores (Ley 351/2013) and report foreign funding</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -3542,7 +3542,7 @@
       </c>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>OSC register with SENADIPJ under Ley 5833/2017; no fixed annual return deadline published. Entities receiving state funds must publish accounts to the Contraloría and face AIFAT audit; transparency bill pending.</t>
+          <t>Registration in the National Registry of Non-Profit Organizations (MEF) under Ley 7363/2024 and Decreto 4806/2025 with funding/beneficiary reporting; entities receiving state funds must publish accounts to the Contraloría.</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>low (~US$10-30, DGR registration)</t>
+          <t>low (~US$10-30, MEC recognition + registry)</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3634,7 +3634,7 @@
       </c>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>Associations and foundations must inscribe in the DGR (Interior Ministry); no published annual return deadline. Annual general meeting and statutory duties follow the law; internal governance by statutes.</t>
+          <t>Associations and foundations are recognised and supervised by the MEC; foundations file annual accounts with the MEC; no published annual return deadline for associations.</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
@@ -3681,7 +3681,7 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Most expat-friendly bureaucracy in South America; English widely spoken in Buenos Aires; foreign founders can serve on boards; donation tax exemption is a separate AFIP step ('Ingreso a Régimen de Entidades Exentas', Ley 24.976); 2016 foundation law made fundaciones cheaper and faster than the old regime. | Confirm mostly; foundation basis is now the Commercial Code since the 2019 reform (Ley 27.610) — Ley 27.290 was absorbed into it. | Verified: Sede social en CABA y patrimonio inicial mínimo de 10 salarios mínimos viales y móviles (Res. IGJ 2/2023) | verify-rest 2026-10: legal bases corrected to CCyC + Ley 19.836; registry is IGJ/provincial DPJ, not the commercial registry</t>
+          <t>Most expat-friendly bureaucracy in South America; English widely spoken in Buenos Aires; foreign founders can serve on boards; donation tax exemption is a separate AFIP step ('Ingreso a Régimen de Entidades Exentas', Ley 24.976); 2016 foundation law made fundaciones cheaper and faster than the old regime. | Verified: Sede social en CABA y patrimonio inicial mínimo de 10 salarios mínimos viales y móviles (Res. IGJ 2/2023) | verify-rest 2026-10: legal bases corrected to CCyC + Ley 19.836; registry is IGJ/provincial DPJ, not the commercial registry</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Fast, clean bureaucracy; the de facto hub for LATAM expats and many run foundations/associations there; English widely used in Santiago legal market; donor tax deduction requires 'calificación' from the tax authority; 2015 law modernized foundations. | Confirm prior (asociación/corporación per Ley 20.500, fundación per Ley 20.839/2015; fast, easy, US$200-500, 1-3 weeks). | Verified: Constitución por escritura pública y domicilio en Chile; desde 2023 se inscribe en la Secretaría Municipal | verify-rest 2026-10: 'Ley 20.839' is not the foundations law; filing is at the Secretaría Municipal with a 30-day objection window</t>
+          <t>Fast, clean bureaucracy; the de facto hub for LATAM expats and many run foundations/associations there; English widely used in Santiago legal market; donor tax deduction requires 'calificación' from the tax authority; 2015 law modernized foundations. | Verified: Constitución por escritura pública y domicilio en Chile; desde 2023 se inscribe en la Secretaría Municipal | verify-rest 2026-10: 'Ley 20.839' is not the foundations law; filing is at the Secretaría Municipal with a 30-day objection window</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3783,7 +3783,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>Chilean registered office and resident legal representative required; public deed + Conservador de Bienes Raíces registration.</t>
+          <t>Chilean registered office and resident legal representative required; constitutive act deposited at the Secretaría Municipal (30-day review) then Registro Civil.</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>The most accessible route in this list; full English-language process; popular expat pathway is the company limited by guarantee, then HKJC charitable status; low political risk. | confirm prior: most accessible route; full English-language process; HK$155-925 incorporation fees; HKJC charitable status separate | Verified: Secretaria de la compañía debe residir en Hong Kong; tarifa de constitución HK$1.545 (electrónica) | verify-rest 2026-10: s.88 tax-exempt status is granted by the IRD (not the HK Jockey Club); CLG fee is HK$155/170 (HK$1,545 is the share-company fee)</t>
+          <t>The most accessible route in this list; full English-language process; popular expat pathway is the company limited by guarantee, then IRD s.88 tax-exempt charity status; low political risk. | Verified: Secretaria de la compañía debe residir en Hong Kong; tarifa de constitución HK$1.545 (electrónica) | verify-rest 2026-10: s.88 tax-exempt status is granted by the IRD (not the HK Jockey Club); CLG fee is HK$155/170 (HK$1,545 is the share-company fee)</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Formation under the Civil Code (foundations arts. 1642-1667); the associations regime law was still in public consultation in 2026; documents in Chinese or Portuguese — English support is limited; political risk similar to Macau generally. | confirm prior: Law 16/2021 foundation route (in force 2022), single founder with donated endowment; DSAJ name-certificate then registration | verify-rest 2026-10: Civil Code articles and procedure corrected — registration runs through the DSI</t>
+          <t>Formation under Law 2/99/M and the Civil Code (arts. 140-172) via DSI registration; a new associations law was in public consultation in 2026; documents in Chinese or Portuguese — English support is limited. | verify-rest 2026-10: Civil Code articles and procedure corrected — registration runs through the DSI</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>Local office, Chinese/Portuguese documents, notary plus DSAJ registration; limited English support</t>
+          <t>Local office, Chinese/Portuguese documents, notarised deed, Boletim Oficial publication and DSI registration; limited English support</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Private foundations (Civil Code arts. 1642-1667): no routine financial-statement filing with the DSF and no published general annual-return requirement; minimal ongoing obligations beyond internal governance and registry updates.</t>
+          <t>Private foundations and associations (Civil Code / Law 2/99/M): no routine financial-statement filing with the DSF and no published general annual-return requirement; registry updates with the DSI.</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr">
@@ -4703,7 +4703,7 @@
       </c>
       <c r="I46" s="2" t="inlineStr">
         <is>
-          <t>Foreign founder must have resided in Indonesia ≥5 consecutive years; in practice local individual/PT is founder of record</t>
+          <t>At least one of chair/secretary/treasurer must be an Indonesian citizen and foreign officers need a KITAS (PP 63/2008, PP 2/2013); in practice a local individual/PT is founder of record</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
@@ -5061,7 +5061,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>2025 draft/NGO law further tightens controls; notable political risk and periodic clampdowns on foreign-funded NGOs; partner with local nationals as founders of record. | Confirm ≥3 Khmer-national founders (LANGO 2003); foreign NGOs via MOFA 3-yr MOU; 2025 NGO-law amendments further tighten | verify-rest 2026-10: LANGO dates from 2015 (not 2003); Khmer-nationality founder rule applies to domestic NGOs</t>
+          <t>2025 draft/NGO law further tightens controls; notable political risk and periodic clampdowns on foreign-funded NGOs; partner with local nationals as founders of record. | verify-rest 2026-10: LANGO dates from 2015 (not 2003); Khmer-nationality founder rule applies to domestic NGOs</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>Societies registered with the National Registration Bureau: under s.15 of the Societies Act, furnish information and audit accounts as approved by the Registrar annually; the Registrar may issue a provisional dissolution order for non-compliance.</t>
+          <t>Organisations registered with the Union Registration Board (Organization Registration Law 2022) must submit annual activity and audited financial reports; the Board may suspend or deregister for non-compliance.</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr">
@@ -5797,7 +5797,7 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Bureaucracy heavy, English official language but processes slow; most international NGOs register via a PNG partner or use an Australian-registered entity operating cross-border | confirm prior; note new Associations Incorporation Act 2023 replaces 1966 Act, regulations commence 1 July 2026 | verify-rest 2026-10: Associations Incorporation Act 2023 itself commenced 1 July 2026</t>
+          <t>Bureaucracy heavy, English official language but processes slow; most international NGOs register via a PNG partner or use an Australian-registered entity operating cross-border | verify-rest 2026-10: Associations Incorporation Act 2023 itself commenced 1 July 2026</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -7637,7 +7637,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>2017 civil-society law; heavy discretionary approval; most expats partner with an existing Cameroonian association instead. | Confirm prior. CGI 2024 confirms the 5%-of-turnover corporate deduction cap for local philanthropic bodies | verify-rest 2026-10: no 2017 civil-society law exists — Law 90/053 amended by 2020/009 and 2021/022; declaration fee overstated</t>
+          <t>Heavy discretionary approval for ONG status; most expats partner with an existing Cameroonian association instead. | Confirm prior. CGI 2024 confirms the 5%-of-turnover corporate deduction cap for local philanthropic bodies | verify-rest 2026-10: no 2017 civil-society law exists — Law 90/053 amended by 2020/009 and 2021/022; declaration fee overstated</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr">
@@ -8097,7 +8097,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>French-language process; post-2023 political transition adds uncertainty to approvals. | Confirm prior. JO confirms loi n°001/2011 governs associations; CGI confirms 0.1%-of-turnover corporate deduction cap | verify-rest 2026-10: Law 35/62 still governs associations ('loi 001/2011' unsupported); NGO bill adopted by the National Assembly 16 May 2025, Senate vote/promulgation pending</t>
+          <t>French-language process; post-2023 political transition adds uncertainty to approvals. | verify-rest 2026-10: Law 35/62 still governs associations ('loi 001/2011' unsupported); NGO bill adopted by the National Assembly 16 May 2025, Senate vote/promulgation pending</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -8107,7 +8107,7 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Interior accreditation (loi 001/2011), local rep, office; French filings; post-2023 transition adds uncertainty</t>
+          <t>Interior accreditation (Law 35/62 declaration + ONG agrément), local rep, office; French filings; post-2023 transition adds uncertainty</t>
         </is>
       </c>
       <c r="J83" s="2" t="inlineStr">
@@ -8373,7 +8373,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Strict, well-enforced 2016 NGO Act; English/French/Kinyarwanda; many expats operate through Rwandan partners rather than foreign registration. | Regulator is now Rwanda Governance Board (RGB), successor to MIDRRP; Law 01/2016 governs NGOs; official fee 300,000 RWF (~$24) | verify-rest 2026-10: no 'Law 01/2016' — NGOs governed by Laws 04/2012 and 05/2012; 300,000 RWF ≈ US$210 (not ~$24)</t>
+          <t>Strict, well-enforced 2016 NGO Act; English/French/Kinyarwanda; many expats operate through Rwandan partners rather than foreign registration. | verify-rest 2026-10: no 'Law 01/2016' — NGOs governed by Laws 04/2012 and 05/2012; 300,000 RWF ≈ US$210 (not ~$24)</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>2021 amendments tightened foreign-funding thresholds and local-content rules; English/Swahili; NGO Commission is strict. | Core law is NGO Act (No. 22 of 2002, as amended); the 2021 tightening was a draft NGO Bill, not enacted law - earlier '2021 amendments' note overstated | verify-rest 2026-10: NGO Act is No. 24 of 2002 (am. 2019); INGO fee USD 350; founder rules corrected</t>
+          <t>Foreign-funding disclosure and local-content expectations apply; English/Swahili; NGO Registrar oversight is strict. | verify-rest 2026-10: NGO Act is No. 24 of 2002 (am. 2019); INGO fee USD 350; founder rules corrected</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -8659,7 +8659,7 @@
       </c>
       <c r="I89" s="2" t="inlineStr">
         <is>
-          <t>NGO Commission registration requires local office and international NGOs need 5+ members incl. at least 2 Tanzanians</t>
+          <t>NGO Registrar registration requires a local office; international NGOs need 5+ founders incl. at least 2 Tanzanians</t>
         </is>
       </c>
       <c r="J89" s="2" t="inlineStr">
@@ -8679,7 +8679,7 @@
       </c>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>Foreign-funded NGOs register with NGO Commission; funding thresholds and reporting monitored; no outright ban</t>
+          <t>Foreign-funded NGOs disclose funding to the NGO Registrar/Board; funding and reporting monitored; no outright ban</t>
         </is>
       </c>
       <c r="N89" s="2" t="inlineStr">
@@ -8741,7 +8741,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>English-language, well-trodden expat route; many Australians register as foreign organizations; strong NGO infrastructure. | NGO Act 2003 was repealed - current framework is PBO Act, 2013 (Cap 134) under PBORA, not the NGO Commission/NGO Act route | verify-rest 2026-10: PBO Act 2013 in force since 14 May 2024 (NGO Board/KES 100,000 deposit route obsolete); PBO Regulations 2026 fees</t>
+          <t>English-language, well-trodden expat route; many Australians register as foreign organizations; strong NGO infrastructure. | verify-rest 2026-10: PBO Act 2013 in force since 14 May 2024 (NGO Board/KES 100,000 deposit route obsolete); PBO Regulations 2026 fees</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr">
@@ -8796,7 +8796,7 @@
       </c>
       <c r="R90" s="2" t="inlineStr">
         <is>
-          <t>In-person at branch under CBK AML/KYC rules; NGO accounts require at least one Kenyan-resident board member as signatory plus an NGO Board recommendation letter, so a local representative is needed.</t>
+          <t>In-person at branch under CBK AML/KYC rules; PBO accounts require at least one Kenyan-resident director as signatory plus the PBORA registration certificate, so a local representative is needed.</t>
         </is>
       </c>
     </row>
@@ -9201,7 +9201,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Portuguese-language process; a hired local manager can serve as legal representative. | Confirm prior; core law is the NGO law (Lei 31/2002) with foreign-NGO regime via MFA; 2-6 months realistic; fee figure includes agent costs | verify-rest 2026-10: 'Lei 31/2002' unsupported — Lei 8/91 + Decreto 55/98 remain operative; the 2022 OSFL bill was dropped from Parliament's agenda in Apr 2023</t>
+          <t>Portuguese-language process; a hired local manager can serve as legal representative. | verify-rest 2026-10: 'Lei 31/2002' unsupported — Lei 8/91 + Decreto 55/98 remain operative; the 2022 OSFL bill was dropped from Parliament's agenda in Apr 2023</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -9338,7 +9338,7 @@
       </c>
       <c r="P96" s="2" t="inlineStr">
         <is>
-          <t>Lei 14/91 (civil associations) and Lei 2/26 (NGOs): the entity registers with the competent authority; no recurring annual filing regime is published; sanctions include dissolution/withdrawal of registration.</t>
+          <t>Lei 6/12 (private associations) and Lei 2/26 (NGOs): the entity registers with the competent authority; NGOs face prior authorisation and oversight; no recurring annual filing regime is published; sanctions include dissolution/withdrawal of registration.</t>
         </is>
       </c>
       <c r="Q96" s="2" t="inlineStr">
@@ -9559,7 +9559,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Local NGOs need a two-thirds Zimbabwean board; foreign NGOs register with the Ministry of Local Government with a local representative; fees in USD.</t>
+          <t>Local PVOs register with the PVO Registrar (Ministry of Public Service, Labour and Social Welfare); international PVOs must name an authorised local agent; fees in USD.</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>ASBL is the standard vehicle and easy via a local registered-office provider; AIT tax-exempt status is a separate application; French-speaking practice dominates; no in-person steps required | mostly confirm prior; foundation needs NO fixed minimum capital (only sufficient); 1 founder enough post-2024 reform | Verified: Authentic notarial deed required; remote founders act through an apostilled notarial power of attorney | verify-rest 2026-10: ASBL needs 2+ founders (no 2024 one-founder reform); private deed suffices for an ASBL; no EUR 25,000 legal minimum for foundations</t>
+          <t>ASBL is the standard vehicle and easy via a local registered-office provider; AIT tax-exempt status is a separate application; French-speaking practice dominates; no in-person steps required | Verified: Authentic notarial deed required; remote founders act through an apostilled notarial power of attorney | verify-rest 2026-10: ASBL needs 2+ founders (no 2024 one-founder reform); private deed suffices for an ASBL; no EUR 25,000 legal minimum for foundations</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -10300,7 +10300,7 @@
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
-          <t>e.V.: court ~USD 70 + notary USD 200-500; gGmbH: capital USD 27,500 + notary/registry USD 700-1,200; Stiftung: endowment USD 27.5k-110k; registration 4-8 weeks; charity status timing unpublished</t>
+          <t>e.V.: EUR 75 court fee + notary signature certification (~USD 100-150 total); gGmbH: capital USD 27,500 + notary/registry USD 700-1,200; Stiftung: endowment typically USD 55k+; registration 4-8 weeks; charity status timing unpublished</t>
         </is>
       </c>
       <c r="G107" s="2" t="inlineStr">
@@ -11041,7 +11041,7 @@
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Digital registry, straightforward; public-benefit (obecně prospěšná) tax status is a separate Ministry of Interior approval. | verified primary: spolek entry in the spolkový rejstřík is fee-free (amended § 11 Act 549/1991 Sb.); nadace first entry 2,700 CZK (notary-filed) / 6,000 CZK (registry court) — inferred from the general tariff, not OUK-explicit; OUK min. endowment 100,000 CZK (Civil Code 89/2012 Sb.) | Verified: Min. 3 founders; Czech law grants foreigners equal rights to found associations | verify-rest 2026-10: nadace minimum endowment is CZK 500,000; 'OUK' mislabel removed; public-benefit status entered by the registry court, not the Interior Ministry</t>
+          <t>Digital registry, straightforward; public-benefit (obecně prospěšná) tax status is a separate Ministry of Interior approval. | Verified: Min. 3 founders; Czech law grants foreigners equal rights to found associations | verify-rest 2026-10: nadace minimum endowment is CZK 500,000; 'OUK' mislabel removed; public-benefit status entered by the registry court, not the Interior Ministry</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
@@ -11128,7 +11128,7 @@
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
-          <t>Court fee EUR 220 (~USD 235); notary EUR 500-1,500 extra; ~USD 250-2,000 total; 1-2 months; VPO recognition time unpublished; foreign founders OK, Slovak charter + local address needed</t>
+          <t>Civic association: EUR 66 Ministry of Interior fee (EUR 33 online), ~10-15 days; foundation: notary EUR 500-1,500 + registry; 1-2 months; foreign founders OK, Slovak charter + local address needed</t>
         </is>
       </c>
       <c r="G116" s="2" t="inlineStr">
@@ -11143,7 +11143,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>Slovak-language charter, 2+ founders and local office; foreign founders need apostilled docs and certified translations</t>
+          <t>Slovak-language charter, 3+ founders and local office; foreign founders need apostilled docs and certified translations</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -11225,7 +11225,7 @@
       </c>
       <c r="G117" s="2" t="inlineStr">
         <is>
-          <t>Foreign-funded NGOs above a threshold (~300M HUF/yr) need government authorization (Stop-Soros legacy) — politically sensitive; public-benefit (közhasznú) status is a separate, stricter regime. | foreign-funding authorization threshold is 7.2M HUF (~25k EUR) per year, not ~300M HUF; kft capital 3,000,000 HUF | Verified: Foreign founders allowed; Hungarian seat (real estate) and a Hungarian-resident curator are required - a local agent. | verify-rest 2026-10: 2017 'Stop-Soros'/foreign-funding authorization law repealed in 2021 — replaced by Act XLIX of 2021 audit regime</t>
+          <t>Foreign-funded NGOs face State Audit Office scrutiny (Act XLIX of 2021) and the 2023 Sovereignty Protection Act — politically sensitive; public-benefit (közhasznú) status is a separate, stricter regime; kft capital 3,000,000 HUF | Verified: Foreign founders allowed; Hungarian seat (real estate) and a Hungarian-resident curator are required - a local agent. | verify-rest 2026-10: 2017 'Stop-Soros'/foreign-funding authorization law repealed in 2021 — replaced by Act XLIX of 2021 audit regime</t>
         </is>
       </c>
       <c r="H117" s="2" t="inlineStr">
@@ -11409,7 +11409,7 @@
       </c>
       <c r="G119" s="2" t="inlineStr">
         <is>
-          <t>EU e-government decent; javno korisna (public-benefit) status is a separate Ministry of Interior step; many expats use a local legal/NGO-service provider. | confirm prior; foreign nationals can be founders; state fee minimal, notary ~500-1,500 HRK; javno korisna status separate step | Verified: Foreign founder allowed, no residency rule; deed of establishment must be notarized (via local notary/POA) then court-registered. | verify-rest 2026-10: foundation is 'zaklada'; costs restated in EUR (HRK replaced 1 Jan 2023)</t>
+          <t>EU e-government decent; javno korisna (public-benefit) status is a separate Ministry of Interior step; many expats use a local legal/NGO-service provider. | Verified: Foreign founder allowed, no residency rule; deed of establishment must be notarized (via local notary/POA) then court-registered. | verify-rest 2026-10: foundation is 'zaklada'; costs restated in EUR (HRK replaced 1 Jan 2023)</t>
         </is>
       </c>
       <c r="H119" s="2" t="inlineStr">
@@ -12053,7 +12053,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Registration itself is cheap and fast, but active war, banking/sanctions friction for a foreign resident founder and currency risk make this a risky base; many Western expat charities run via local Ukrainian partners. | Confirm public organization/foundation; state duty ~2,000 UAH (~$50) plus translations/notary; registration itself fast as noted. | verify-rest 2026-10: no state duty for public-association registration; 'fundatsiia' replaced with blahodiinyi fond</t>
+          <t>Registration itself is cheap and fast, but active war, banking/sanctions friction for a foreign resident founder and currency risk make this a risky base; many Western expat charities run via local Ukrainian partners. | verify-rest 2026-10: no state duty for public-association registration; 'fundatsiia' replaced with blahodiinyi fond</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -12421,7 +12421,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>2019 law modernized foundations, but process is paper/notary-heavy, Greek language required, no meaningful online registry; use a local lawyer. | Association min 7 founders (not 5); general-benefit status is a separate application after court registry filing. Confirm prior fees/timeline. | verify-rest 2026-10: somateio needs 20 founders; registration via Magistrates' Court since 2016; Law 5259/2025 replaced 4182/2013</t>
+          <t>Paper/notary-heavy process, Greek language required, no meaningful online registry; foundations now under Law 5259/2025; use a local lawyer. | verify-rest 2026-10: somateio needs 20 founders; registration via Magistrates' Court since 2016; Law 5259/2025 replaced 4182/2013</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -12441,7 +12441,7 @@
       </c>
       <c r="K130" s="2" t="inlineStr">
         <is>
-          <t>2-4 months (notary + first-instance court filing; slower for remote founders)</t>
+          <t>2-4 months (notary + Magistrates' Court registration; slower for remote founders)</t>
         </is>
       </c>
       <c r="L130" s="2" t="inlineStr">
@@ -12508,12 +12508,12 @@
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
-          <t>Trust: ~500-2,000 EUR via solicitor, days; registered body: ~100-500 EUR, ~2-6 weeks</t>
+          <t>Trust: ~500-2,000 EUR via solicitor, days; society/institution: ~100-500 EUR, up to ~3 months (Registrar review)</t>
         </is>
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>English common-law jurisdiction — most expats set up a simple charitable trust with a Cypriot trustee; tax deductibility requires income-tax authority approval and a Cypriot public-benefit nexus; strong English-language professional services. | Registered body under s.250 Companies Law needs 7 members, not 3; trust route unchanged (unregistered, no govt fee). Confirm prior fees/timeline. | verify-rest 2026-10: society needs 20 founders under Law 104(I)/2017; Registrar may take up to 3 months</t>
+          <t>English common-law jurisdiction — most expats set up a simple charitable trust with a Cypriot trustee; tax deductibility requires income-tax authority approval and a Cypriot public-benefit nexus; strong English-language professional services. | verify-rest 2026-10: society needs 20 founders under Law 104(I)/2017; Registrar may take up to 3 months</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -12881,7 +12881,7 @@
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Documents in Icelandic; tax exemption (reykjafrjálsefni) must be applied for separately with the tax office; small bureaucracy but limited English support | verify-rest 2026-10: charitable foundations fall under Act 19/1988 (Act 33/1999 is for business foundations); third-sector Act 110/2021; RSK is now Skatturinn</t>
+          <t>Documents in Icelandic; tax-deductible status requires registration on Skatturinn's public-benefit register; small bureaucracy but limited English support | verify-rest 2026-10: charitable foundations fall under Act 19/1988 (Act 33/1999 is for business foundations); third-sector Act 110/2021; RSK is now Skatturinn</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr">
@@ -12906,7 +12906,7 @@
       </c>
       <c r="L135" s="2" t="inlineStr">
         <is>
-          <t>Deductible if the org is tax-exempt (reykjafrjálst), plus ~10% surtax deduction on the gift.</t>
+          <t>Deductible if the organisation is on Skatturinn's public-benefit register (almannaheillaskrá); individuals deduct ISK 10,000-350,000/yr, companies up to 1.5% of income.</t>
         </is>
       </c>
       <c r="M135" s="2" t="inlineStr">
@@ -13428,12 +13428,12 @@
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
-          <t>State fee about EUR 11-12; total EUR 30-100; 1-4 weeks. The 2014 Associations &amp; Foundations law removed the notary step. A Latvian-resident board and local address are required.</t>
+          <t>State fee EUR 11.38 (10% less online); total EUR 30-100; 1-4 weeks. E-filing with an e-signature avoids the notary step. A Latvian address is required.</t>
         </is>
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>The 2016 Nonprofit Organizations Law unified the forms; the notary step forces an in-person visit or a local representative, which is the main barrier for a foreign founder | NVO registers electronically via e-portals; no notary step needed. Real barriers: Latvian-resident board requirement plus local address and e-ID | verify-rest 2026-10: law date corrected to 2003/2004; no '2016 Nonprofit Organizations Law' exists; state fee EUR 11.38 (Cabinet Reg. 308)</t>
+          <t>Associations and foundations share one law (2003); e-filing with an EU e-signature avoids the notary, otherwise notarised signatures force an in-person visit or a local representative | NVO registers electronically via e-portals; no notary step needed. Real barriers: Latvian-resident board requirement plus local address and e-ID | verify-rest 2026-10: law date corrected to 2003/2004; no '2016 Nonprofit Organizations Law' exists; state fee EUR 11.38 (Cabinet Reg. 308)</t>
         </is>
       </c>
       <c r="H141" s="2" t="inlineStr">
@@ -13483,7 +13483,7 @@
       </c>
       <c r="Q141" s="2" t="inlineStr">
         <is>
-          <t>Registration automatic; PBO status is a separate VID application (2016 Law) - PBOs exempt from income tax. Donors: individuals 25.5% tax refund; corporate 5% of prior profit or CIT reduction.</t>
+          <t>Registration automatic; PBO status is a separate VID application (Public Benefit Organisation Law) - PBOs exempt from income tax. Donors: individuals 25.5% tax refund; corporate 5% of prior profit or CIT reduction.</t>
         </is>
       </c>
       <c r="R141" s="2" t="inlineStr">
@@ -13709,7 +13709,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>The most straightforward of the four for a foreign founder: no citizenship/residency requirement for the founder, and no fixed minimum capital. However, to be treated as an entity of public interest (required for tax-exempt status and grants) it needs an endowment and approval by the relevant authority. English filings are not routine; use a Portuguese lawyer. A local office can be provided by a law firm or registered agent, which is what keeps this at medium rather than easy. | confirm prior: no statutory minimum endowment, EUR 1,000-2,500, 1-2 months, medium difficulty all accurate. | verify-rest 2026-10: 'no statutory minimum endowment' corrected — Portaria 75/2013 sufficiency threshold applies; 'Instituto' is not a separate private form</t>
+          <t>The most straightforward of the four for a foreign founder: no citizenship/residency requirement for the founder, and no fixed minimum capital. However, to be treated as an entity of public interest (required for tax-exempt status and grants) it needs an endowment and approval by the relevant authority. English filings are not routine; use a Portuguese lawyer. A local office can be provided by a law firm or registered agent, which is what keeps this at medium rather than easy. | verify-rest 2026-10: 'no statutory minimum endowment' corrected — Portaria 75/2013 sufficiency threshold applies; 'Instituto' is not a separate private form</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr">
@@ -13801,7 +13801,7 @@
       </c>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>Foreign (including Australian) founders can legally establish a fondazione — explicitly no nationality or residency requirement — but the €150,000 fully-contributed endowment is the main barrier and makes it one of the costlier routes. Charitable status requires registration in RUNTS (Registro Unico Nazionale del Terzo Settore); the procedure is document-based and can be handled by a local lawyer with a representative, avoiding in-person steps. Italian-language filings are mandatory; English is not accepted for registry documents. The higher endowment and bureaucracy keep it at medium despite the permissive foreign-founder rule. | confirm prior: EUR 150,000 endowment, EUR 3,000-6,000 professional costs, 2-4 months, medium difficulty all accurate. | verify-rest 2026-10: minimum patrimony corrected to EUR 30,000 (foundations) / 15,000 (associations) per D.Lgs. 117/2017 art. 22</t>
+          <t>Foreign (including Australian) founders can legally establish a fondazione — explicitly no nationality or residency requirement — with a minimum EUR 30,000 patrimony (EUR 15,000 for associations) for legal personality via RUNTS (Registro Unico Nazionale del Terzo Settore); the procedure is document-based and can be handled by a local notary/lawyer with a representative, avoiding in-person steps. Italian-language filings are mandatory. | verify-rest 2026-10: minimum patrimony corrected to EUR 30,000 (foundations) / 15,000 (associations) per D.Lgs. 117/2017 art. 22</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr">
@@ -13811,7 +13811,7 @@
       </c>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>EUR 150,000 endowment fully paid at formation plus Italian registered office; foreign founders allowed with no residency rule.</t>
+          <t>EUR 30,000 patrimony for a fondazione (EUR 15,000 associazione) plus Italian registered office; foreign founders allowed with no residency rule.</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr">
@@ -14072,7 +14072,7 @@
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
-          <t>A$100-500 fees, 1-3 months (gated by finding 5+ Jordanian-citizen board members)</t>
+          <t>A$100-500 fees, 1-3 months (gated by finding 7+ Jordanian founders)</t>
         </is>
       </c>
       <c r="G148" s="2" t="inlineStr">
@@ -14107,7 +14107,7 @@
       </c>
       <c r="M148" s="2" t="inlineStr">
         <is>
-          <t>Foreign funding routed via registered local NGO; prior approval + detailed reporting to Ministry of Social Affairs</t>
+          <t>Foreign funding routed via registered local society; prior Council of Ministers approval + detailed reporting to the Ministry of Social Development</t>
         </is>
       </c>
       <c r="N148" s="2" t="inlineStr">
@@ -14127,7 +14127,7 @@
       </c>
       <c r="Q148" s="2" t="inlineStr">
         <is>
-          <t>Registration with the Ministry of Social Affairs confers legal personality; the income-tax law exempts income of registered associations/foundations pursuing public-benefit purposes, and donations to them are deductible.</t>
+          <t>Registration with the Ministry of Social Development confers legal personality; the income-tax law exempts income of registered societies pursuing public-benefit purposes, and donations to them are deductible.</t>
         </is>
       </c>
       <c r="R148" s="2" t="inlineStr">
@@ -14214,12 +14214,12 @@
       </c>
       <c r="P149" s="2" t="inlineStr">
         <is>
-          <t>Law 92/1909 is a simple declaration regime; detailed annual filing duties are unpublished, but the law prohibits undeclared associations and lets the government refuse a declaration and dissolve one.</t>
+          <t>Ottoman Law of Associations (1909) declaration regime; detailed annual filing duties are unpublished, but undeclared associations are prohibited and the government can dissolve one.</t>
         </is>
       </c>
       <c r="Q149" s="2" t="inlineStr">
         <is>
-          <t>Associations are valid by declaration to the local court (Law 92/1909); the income-tax code exempts income of public-benefit associations and institutions — no separate application; no donor-deduction regime.</t>
+          <t>Associations are valid by declaration to the Ministry of Interior (1909 Law); the income-tax code exempts income of public-benefit associations and institutions — no separate application; no donor-deduction regime.</t>
         </is>
       </c>
       <c r="R149" s="2" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>Civil-society registration resumed after 2025 transition (586 NGOs registered by Feb 2025) but framework unstable; sanctions exposure for foreign founders and their banks; English support effectively unavailable; advise against direct formation | Confirm prior: post-2025 regime unstable (586 NGOs registered by Feb 2025), funding-approval restrictions persist | verify-rest 2026-10: no new associations law enacted — Law 93/1958 still governs</t>
+          <t>Civil-society registration resumed after 2025 transition (586 NGOs registered by Feb 2025) but framework unstable; sanctions exposure for foreign founders and their banks; English support effectively unavailable; advise against direct formation | verify-rest 2026-10: no new associations law enacted — Law 93/1958 still governs</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
@@ -14398,12 +14398,12 @@
       </c>
       <c r="P151" s="2" t="inlineStr">
         <is>
-          <t>NGO Law 12/2010 Art. 15: each NGO sends the NGO Directorate (Interior Ministry) a financial report on fund sources and transactions plus an activity report, for the prior year by 31 March; Directorate can sanction.</t>
+          <t>NGO Law 12/2010 Art. 15: each NGO sends the NGOs Department (Council of Ministers Secretariat) a financial report on fund sources and transactions plus an activity report, for the prior year by 31 March; the Department can sanction.</t>
         </is>
       </c>
       <c r="Q151" s="2" t="inlineStr">
         <is>
-          <t>NGOs registered with the NGO Directorate, Interior Ministry: if classified as public utility, art. 17 of Law 12/2010 automatically exempts income tax, VAT, customs and sales tax; no separate application.</t>
+          <t>NGOs registered with the NGOs Department: if classified as public utility, art. 17 of Law 12/2010 automatically exempts income tax, VAT, customs and sales tax; no separate application.</t>
         </is>
       </c>
       <c r="R151" s="2" t="inlineStr">
@@ -14445,7 +14445,7 @@
       </c>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>New 2024 law (Royal Decree M/111) modernized the regime but kept the Saudi-citizenship floor; the only realistic foreign route is a program partnership with a Saudi charity or a representative office for an existing foreign NGO; English widely used in government dealings | Confirm prior: 2024 law kept Saudi-citizenship floor, 10 citizens, partnership/rep-office the only routes | verify-rest 2026-10: no '2024 Civil Society Law (M/111)' exists — the 2015/16 Royal Decree M/8 law governs</t>
+          <t>The 2016 Law of Associations and Foundations (RD M/8) keeps a Saudi-citizenship floor; the only realistic foreign route is a program partnership with a Saudi charity or a representative office for an existing foreign NGO; English widely used in government dealings | Confirm prior: 2024 law kept Saudi-citizenship floor, 10 citizens, partnership/rep-office the only routes | verify-rest 2026-10: no '2024 Civil Society Law (M/111)' exists — the 2015/16 Royal Decree M/8 law governs</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr">
@@ -14475,7 +14475,7 @@
       </c>
       <c r="M152" s="2" t="inlineStr">
         <is>
-          <t>Foreign funding only via approved partnership with Saudi entity; 2024 Civil Society Law (M/111) strengthens oversight</t>
+          <t>Foreign funding only via approved partnership with Saudi entity; Law of Associations and Foundations (RD M/8, 2016) requires approval and oversight</t>
         </is>
       </c>
       <c r="N152" s="2" t="inlineStr">
@@ -14629,7 +14629,7 @@
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>2023 philanthropy law tightened state oversight of foreign-funded work; standard foreign route is a partnership with Qatar Charity or an established Doha NGO, or a representative office approved by the relevant ministry | Confirm prior: foreigners cannot found standalone charity; partnership with Qatar Charity/Doha NGO is standard | verify-rest 2026-10: no '2023 philanthropy law' — Decree-Law 21/2020 + Law 15/2014 govern</t>
+          <t>State oversight of foreign-funded charitable work runs through RACA (Law 15/2014); standard foreign route is a partnership with Qatar Charity or an established Doha NGO, or a representative office approved by the relevant ministry | Confirm prior: foreigners cannot found standalone charity; partnership with Qatar Charity/Doha NGO is standard | verify-rest 2026-10: no '2023 philanthropy law' — Decree-Law 21/2020 + Law 15/2014 govern</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
@@ -14721,7 +14721,7 @@
       </c>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>Most accessible Gulf option for a foreign founder: a UAE private foundation can be 100% foreign-held and run charitable activities; Dubai Charities (DCC) also registers existing international charities; the association route is blocked for all-foreign boards by the 70% nationality rule; strong English-language support | Confirm prior: 100% foreign-owned private foundation is the viable route (AED 30k-75k all-in, 4-8 weeks); DCC also registers foreign charities. | verify-rest 2026-10: FL 2/2008 was repealed (not amended) by FDL 50/2023; the old 70% UAE-national board rule came from the repealed law</t>
+          <t>Most accessible Gulf option for a foreign founder: a DIFC/ADGM foundation can be 100% foreign-held and run charitable activities; Dubai's IACAD/DCC also registers existing international charities; federal NPOs follow FDL 50/2023 approval rules; strong English-language support | Confirm prior: 100% foreign-owned private foundation is the viable route (AED 30k-75k all-in, 4-8 weeks); DCC also registers foreign charities. | verify-rest 2026-10: FL 2/2008 was repealed (not amended) by FDL 50/2023; the old 70% UAE-national board rule came from the repealed law</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr">
@@ -14731,7 +14731,7 @@
       </c>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>Local service provider + UAE office required; associations need 70% UAE nationals, foreign-only boards excluded.</t>
+          <t>Local service provider + UAE office required; federal NPOs subject to FDL 50/2023 nationality and approval rules, so foreign founders typically use a DIFC/ADGM foundation.</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
@@ -14858,7 +14858,7 @@
       </c>
       <c r="P156" s="2" t="inlineStr">
         <is>
-          <t>Civil Associations Law (RD 14/2000, as amended): ministry supervision includes inspection of annual account audit reports and verification of compliance with the constitution; records must be kept and available.</t>
+          <t>Civil Society Institutions Law (RD 64/2026): ministry supervision includes inspection of annual audited accounts and verification of compliance with the constitution; executive regulations pending.</t>
         </is>
       </c>
       <c r="Q156" s="2" t="inlineStr">
@@ -14905,7 +14905,7 @@
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>Bahrain is the most English-friendly and transparent NGO administration in the Gulf, but the nationality floor on founders/board keeps foreign formation out of reach; standard route is a partnership with an existing Bahraini NGO; government relations are comparatively accessible | Confirm prior: nationality floor (20 Bahraini founders, 2/3 board) keeps foreign formation out of reach; partnership route is standard. | verify-rest 2026-10: founder minimum corrected to ~10; 'Law 19/2006' founder-rule reference removed</t>
+          <t>Bahrain is the most English-friendly and transparent NGO administration in the Gulf, but the nationality floor on founders/board keeps foreign formation out of reach; standard route is a partnership with an existing Bahraini NGO; government relations are comparatively accessible | verify-rest 2026-10: founder minimum corrected to ~10; 'Law 19/2006' founder-rule reference removed</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
@@ -14950,7 +14950,7 @@
       </c>
       <c r="P157" s="2" t="inlineStr">
         <is>
-          <t>NGO Law 19/2006: each association keeps an annual budget; where revenues or expenses exceed BHD 10,000 the board must present final accounts to a licensed accounting firm; the Ministry supervises and can sanction.</t>
+          <t>Decree-Law 21/1989: each association keeps an annual budget; where revenues or expenses exceed BHD 10,000 the board must present final accounts audited by a licensed firm; the Ministry supervises and can sanction.</t>
         </is>
       </c>
       <c r="Q157" s="2" t="inlineStr">
@@ -15226,7 +15226,7 @@
       </c>
       <c r="P160" s="2" t="inlineStr">
         <is>
-          <t>Law 70/2017: associations file an annual activity report and financial statements with the supervising ministry (Social Affairs or Interior) by 31 March; larger ones must have accounts audited; risks suspension.</t>
+          <t>Law 149/2019: associations file an annual activity report and financial statements with the Ministry of Social Solidarity; larger ones must have accounts audited; risks suspension.</t>
         </is>
       </c>
       <c r="Q160" s="2" t="inlineStr">
@@ -15365,7 +15365,7 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Fragmented dual-government structure, militia influence, no workable foreign-formation path; foreign NGOs operate via UN/embassy channels only. | Confirm prior, with correction: current framework is NGO Law No. 19 of 2001 (and 2013 circulars), not Law 12/1989 as sole basis | verify-rest 2026-10: '2013 circulars' replaced by the 2023 HJC opinion and PM Circular 7 re-imposing Law 19/2001</t>
+          <t>Fragmented dual-government structure, militia influence, no workable foreign-formation path; foreign NGOs operate via UN/embassy channels only. | verify-rest 2026-10: '2013 circulars' replaced by the 2023 HJC opinion and PM Circular 7 re-imposing Law 19/2001</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr">
@@ -15549,7 +15549,7 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>Most open civil-society law in the region; declaration-based, so registration is fast; post-2022 political centralisation adds compliance risk. | Confirm prior; governing text is Decree-Law 59-154 of 1959; only 2 founders needed; members 13+, must accept bylaws in writing | verify-rest 2026-10: governing text is Décret-loi 2011-88 (which repealed Law 59-154 of 1959); founders must be 16+ (13 is the member age floor); 2023 replacement bill still pending in the ARP</t>
+          <t>Most open civil-society law in the region; declaration-based, so registration is fast; post-2022 political centralisation adds compliance risk. | verify-rest 2026-10: governing text is Décret-loi 2011-88 (which repealed Law 59-154 of 1959); founders must be 16+ (13 is the member age floor); 2023 replacement bill still pending in the ARP</t>
         </is>
       </c>
       <c r="H164" s="2" t="inlineStr">
@@ -15917,7 +15917,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>2021 reform liberalised funding and registration, but foreigners cannot directly form a domestic charity; security clearance applies; Amharic/English documents. | Confirm prior: 2021 CSO Proclamation (1259/2021) keeps foreign founders out of domestic entities; cost 3-6 months via partner is reasonable. | verify-rest 2026-10: registrar is ACSO; resident foreigners may co-found local CSOs, non-residents cannot</t>
+          <t>2021 reform liberalised funding and registration, but foreigners cannot directly form a domestic charity; security clearance applies; Amharic/English documents. | verify-rest 2026-10: registrar is ACSO; resident foreigners may co-found local CSOs, non-residents cannot</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -16238,7 +16238,7 @@
       </c>
       <c r="P171" s="2" t="inlineStr">
         <is>
-          <t>NGO Act 2019 Art. 17: annual financial and narrative reports, including the audit report, are due to the NGO Coordination Office by 31 May; the certificate is valid 2 years and must be renewed (Art. 16).</t>
+          <t>Federal registration (MoPIED) requires annual financial and narrative reports including audit; registration renewal periodically; draft federal NGO Bill (2019) would formalise duties.</t>
         </is>
       </c>
       <c r="Q171" s="2" t="inlineStr">
@@ -16330,7 +16330,7 @@
       </c>
       <c r="P172" s="2" t="inlineStr">
         <is>
-          <t>Decree 82/11 (2010): the certificate is renewed annually (fee ~USD 60) and end-of-year NGO reports are assessed by the Consultative Committee; NGOs that suspend or fail to renew are struck off the General Register.</t>
+          <t>Law 43/2010: the certificate is renewed periodically with the Ministry of National Planning and Development and annual NGO reports are assessed; NGOs that fail to renew are struck off the register.</t>
         </is>
       </c>
       <c r="Q172" s="2" t="inlineStr">
@@ -16469,7 +16469,7 @@
       </c>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>English-language, simple, offshore-friendly regime; popular with foreign founders; a Seychelles charity gains no local tax-exempt status without local operations. | Confirm prior: NPO Act 2013 for local NPOs; the practical foreign route is the Seychelles Foundation Act 2009 (SIBA, $200 gov fee); prior $1,500-3,000 is agent-inclusive. | Verified: No local presence required; foreign founder may be a councillor; FSA registration fee ~US$200 plus ~US$200 annual. | Verified 2026: NPO Act Cap. 741 (Seychelles NPO Act 2013) is the current local regime; no amendment changing the route found; the foreign-foundation route (Foundation Act 2009) remains the practical path for non-residents. | verify-rest 2026-10: local regime is the Associations Act 2022 (Act 8/2022, in force 14 Aug 2023, repealing Cap 201) — the 'NPO Act Cap. 741' claim is unsupported; Foundations Act 2009 route unaffected</t>
+          <t>English-language, simple, offshore-friendly regime; popular with foreign founders; a Seychelles charity gains no local tax-exempt status without local operations. | Verified: No local presence required; foreign founder may be a councillor; FSA registration fee ~US$200 plus ~US$200 annual. | verify-rest 2026-10: local regime is the Associations Act 2022 (Act 8/2022, in force 14 Aug 2023, repealing Cap 201) — the 'NPO Act Cap. 741' claim is unsupported; Foundations Act 2009 route unaffected</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr">
@@ -16755,7 +16755,7 @@
       </c>
       <c r="I177" s="2" t="inlineStr">
         <is>
-          <t>Resident Pakistani director/secretary (Sec 21) or trustee required; FBR tax-exempt status is a separate application.</t>
+          <t>Resident Pakistani director/secretary (Section 42 company) or trustee required; SECP licence then FBR tax-exempt status as separate steps.</t>
         </is>
       </c>
       <c r="J177" s="2" t="inlineStr">
@@ -16882,7 +16882,7 @@
       </c>
       <c r="P178" s="2" t="inlineStr">
         <is>
-          <t>BIDA: the certificate is valid five years and must be renewed before expiry; the NGO files an annual report on donation receipt and utilisation; non-compliance can lead to suspension or deregistration.</t>
+          <t>NGO Affairs Bureau: registration valid ten years under FDRA 2016 and must be renewed; foreign-funded projects need prior approval; annual reports on donation receipt and utilisation; non-compliance can lead to suspension or deregistration.</t>
         </is>
       </c>
       <c r="Q178" s="2" t="inlineStr">
@@ -17021,7 +17021,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>The trust route is the simplest expat pathway (no citizen-quota for trust deed). Foreign funding requires Social Welfare Council approval, which adds time and discretion. | confirm prior - Trust Act 2064 (2007) route confirmed for foreigners; NGO route needs 5 of 7 Nepali-citizen board. | verify-rest 2026-10: no general 'Trust Act 2000' — Civil Code 2017 governs trusts; foreign-settlor trust carries a US$1M threshold; NGO needs 7 Nepali founders</t>
+          <t>The trust route is the simplest expat pathway (no citizen-quota for trust deed). Foreign funding requires Social Welfare Council approval, which adds time and discretion. | verify-rest 2026-10: no general 'Trust Act 2000' — Civil Code 2017 governs trusts; foreign-settlor trust carries a US$1M threshold; NGO needs 7 Nepali founders</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -17250,12 +17250,12 @@
       </c>
       <c r="P182" s="2" t="inlineStr">
         <is>
-          <t>NGOs file an annual activity report to the Ministry of Economy (Law on NGOs 2005, art. 31); associations file reports within 3 months of fiscal year end; non-filing risks sanctions or deregistration.</t>
+          <t>NGOs file annual activity and financial reports to the Ministry of Economy (NGO Directorate); non-filing risks sanctions or deregistration.</t>
         </is>
       </c>
       <c r="Q182" s="2" t="inlineStr">
         <is>
-          <t>NGO registered with NGO Registration Committee (Law on NGOs 2005); NOT automatic - apply to Revenue Authority for tax-exemption certificate (income tax + business receipt tax); no donor deduction; ~30-90 days.</t>
+          <t>NGO registered with the Ministry of Economy; NOT automatic - apply to the Revenue Authority for a tax-exemption certificate (income tax + business receipt tax); no donor deduction; ~30-90 days.</t>
         </is>
       </c>
       <c r="R182" s="2" t="inlineStr">
@@ -17389,7 +17389,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>Most structured path in West Africa but multi-layered; NCMM registration and ORC are the foreigner bottlenecks; English language; strong expat NGO sector in Lagos/Abuja | verify-rest 2026-10: 'NCMM' and 'Operational Readiness Certificate' layers unverifiable — replaced by SCUML + NPC; Foreign Aid Regulation Bill 2026 (SB.1034) is pending, not law</t>
+          <t>Most structured path in West Africa but multi-layered; CAC incorporation, SCUML and (for INGOs) National Planning Commission registration are the foreigner bottlenecks; English language; strong expat NGO sector in Lagos/Abuja | verify-rest 2026-10: 'NCMM' and 'Operational Readiness Certificate' layers unverifiable — replaced by SCUML + NPC; Foreign Aid Regulation Bill 2026 (SB.1034) is pending, not law</t>
         </is>
       </c>
       <c r="H184" s="2" t="inlineStr">
@@ -17399,7 +17399,7 @@
       </c>
       <c r="I184" s="2" t="inlineStr">
         <is>
-          <t>CAC incorporation (CLBG) then NCMM/NGO Bureau registration; foreign NGOs also need SCUML and an Interior ORC</t>
+          <t>CAC incorporation (incorporated trustees or CLG), then SCUML registration before banking; international NGOs also register with the National Planning Commission</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -17419,7 +17419,7 @@
       </c>
       <c r="M184" s="2" t="inlineStr">
         <is>
-          <t>Foreign NGOs need NCMM registration; SCUML registration mandatory; Interior Ministry ORC for foreign-funded NGOs</t>
+          <t>SCUML (EFCC) registration mandatory; international NGOs register with the National Planning Commission; a Foreign Aid Regulation Bill (2026) is pending</t>
         </is>
       </c>
       <c r="N184" s="2" t="inlineStr">
@@ -17434,12 +17434,12 @@
       </c>
       <c r="P184" s="2" t="inlineStr">
         <is>
-          <t>CAC annual returns + annual report for NGOs (CAMA 2020) due within 6 months of fiscal year end (commonly Jun 30); NCMM annual reports; non-compliance risks fines and deregistration.</t>
+          <t>CAC annual returns + annual report for incorporated trustees (CAMA 2020) due within 6 months of fiscal year end; SCUML reporting; non-compliance risks fines and deregistration.</t>
         </is>
       </c>
       <c r="Q184" s="2" t="inlineStr">
         <is>
-          <t>Incorporated trustee registered with CAC (NGO listed with NCMM); tax exemption under CITA 1999 (non-profit organization) via separate FIRS application; no general donor income-tax deduction; time unpublished.</t>
+          <t>Incorporated trustee registered with CAC; tax exemption under CITA (non-profit organization) via separate FIRS application; no general donor income-tax deduction; time unpublished.</t>
         </is>
       </c>
       <c r="R184" s="2" t="inlineStr">
@@ -17476,12 +17476,12 @@
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
-          <t>ORC statutory fee ~GHS 490 (~$40, 2025) plus non-refundable licensing bank draft to Dept. of Social Welfare; provisional license 3 months, official time unpublished.</t>
+          <t>ORC statutory fee ~GHS 490 (~$40, 2025) plus non-refundable licensing fee to the NPO Secretariat; provisional licence 3 months, official time unpublished.</t>
         </is>
       </c>
       <c r="G185" s="2" t="inlineStr">
         <is>
-          <t>Most foreigner-friendly framework in the list: no local-national director requirement under the Companies Act 2019 (Act 992); Charities Commission registration has been operational since ~2021; English language | verify-rest 2026-10: there is no Ghana Charities Commission/Charities Act — licensing is by the NPO Secretariat; NPO Bill still pending</t>
+          <t>Most foreigner-friendly framework in the region: no local-national director requirement under the Companies Act 2019 (Act 992); NPO licensing by the NPO Secretariat (NPO Bill pending); English language | verify-rest 2026-10: there is no Ghana Charities Commission/Charities Act — licensing is by the NPO Secretariat; NPO Bill still pending</t>
         </is>
       </c>
       <c r="H185" s="2" t="inlineStr">
@@ -17491,7 +17491,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>Two-stage: ORC incorporation under Companies Act 992, then NPOS operating license (Charities Act 1035 regime)</t>
+          <t>Two-stage: ORC incorporation under Companies Act 992, then NPO Secretariat operating licence (NPOs Policy/Directive 2020)</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -17695,7 +17695,7 @@
       </c>
       <c r="M187" s="2" t="inlineStr">
         <is>
-          <t>Foreign NGOs need authorization under Law 2015-04/PRB + Decree 2025-636 (Oct 2025) to establish or act in Benin</t>
+          <t>Foreign NGOs need authorization under Loi 2025-19 + Decree 2025-636 (Oct 2025) to establish or act in Benin</t>
         </is>
       </c>
       <c r="N187" s="2" t="inlineStr">
@@ -17849,7 +17849,7 @@
       </c>
       <c r="G189" s="2" t="inlineStr">
         <is>
-          <t>High political risk: 2018 constitutional ban on foreign-funded NGOs, 2022–2025 military rule, repeated suspensions of international NGOs (e.g. 2023–24 expulsions); effectively impractical for a foreign-funded charity | Association law replaced by Law n° 011-2025/ALT (17 July 2025, promulgated 23 July 2025); prior Law 014/1997 superseded | verify-rest 2026-10: Loi 064-2015 replaced by Loi 011-2025/ALT; unsupported '2018 constitutional amendment' claim removed</t>
+          <t>High political risk: military rule since 2022, repeated suspensions of international NGOs (e.g. 2023–24 expulsions) and mass dissolutions under Loi 011-2025/ALT; effectively impractical for a foreign-funded charity | Association law replaced by Law n° 011-2025/ALT (17 July 2025, promulgated 23 July 2025); prior Law 014/1997 superseded | verify-rest 2026-10: Loi 064-2015 replaced by Loi 011-2025/ALT; unsupported '2018 constitutional amendment' claim removed</t>
         </is>
       </c>
       <c r="H189" s="2" t="inlineStr">
@@ -17894,12 +17894,12 @@
       </c>
       <c r="P189" s="2" t="inlineStr">
         <is>
-          <t>Associations declared at préfecture; ONGs need ministry-of-finance authorization (loi 064-2015); ongoing oversight, non-compliance risks administrative dissolution (118 CSOs dissolved in 2025).</t>
+          <t>Associations under Loi 011-2025/ALT; ONGs need ministry authorization; ongoing oversight, non-compliance risks administrative dissolution (118 organisations dissolved, 1,056 suspended in Apr 2026).</t>
         </is>
       </c>
       <c r="Q189" s="2" t="inlineStr">
         <is>
-          <t>Association declared with prefecture (loi 064-2015); public-utility recognition by decree adds full tax benefits; association income tax-exempt when applied to its purposes; no donor deduction; time unpublished.</t>
+          <t>Association registered under Loi 011-2025/ALT; public-utility recognition by decree adds full tax benefits; association income tax-exempt when applied to its purposes; no donor deduction; time unpublished.</t>
         </is>
       </c>
       <c r="R189" s="2" t="inlineStr">
@@ -18125,7 +18125,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>Repeated military coups (7 since independence), fragile state capacity, weak enforcement of registrations; Portuguese (not French) documents; practical operations very difficult | Prior cited Lei n. 5/VI/96 (1996) is superseded: Loi L/005/013/AN (2013) is the operative association law (repealed 1986 NGO decree) | [verified] Requires a physical public deed in Portuguese at the Serviços Notariais (Bissau only) plus 10+ founding members; no remote channel for foreign founders (Constitution art. 44d grants the right to citizens; IMVF 2021 study s4.2, s4.2.4). | Correction: Mechanism: notarial registration under the Código Civil (Decreto 23/92 opinion route inoperative); cited 2013 law unverified; fees per 2021 IMVF study (~93k-300k CFA). | verify-rest 2026-10: misattributed 'Lei 5/VI/96' (Cape Verde numbering) and Guinea-Conakry 'L/005/013/AN' references removed</t>
+          <t>Repeated military coups (7 since independence), fragile state capacity, weak enforcement of registrations; Portuguese (not French) documents; practical operations very difficult | [verified] Requires a physical public deed in Portuguese at the Serviços Notariais (Bissau only) plus 10+ founding members; no remote channel for foreign founders (Constitution art. 44d grants the right to citizens; IMVF 2021 study s4.2, s4.2.4). | Correction: Mechanism: notarial registration under the Código Civil (Decreto 23/92 opinion route inoperative); cited 2013 law unverified; fees per 2021 IMVF study (~93k-300k CFA). | verify-rest 2026-10: misattributed 'Lei 5/VI/96' (Cape Verde numbering) and Guinea-Conakry 'L/005/013/AN' references removed</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -18267,7 +18267,7 @@
       </c>
       <c r="Q193" s="2" t="inlineStr">
         <is>
-          <t>Association declared with prefecture (loi 71-604); income tax exemption automatic under CGI art.5(7) (since 2019) for non-profit entities without commercial activity; donors deduct gifts to public-utility orgs, cap 0.5%.</t>
+          <t>Association declared to the administrative authority (COCC arts. 811 ff.); income tax exemption automatic under CGI art.5(7) (since 2019) for non-profit entities without commercial activity; donors deduct gifts to public-utility orgs, cap 0.5%.</t>
         </is>
       </c>
       <c r="R193" s="2" t="inlineStr">
@@ -18309,7 +18309,7 @@
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>English language, stable democracy; 2022 NGO Bill has been in draft years without enactment, so the old 1972 Societies Act still applies; Banjul filings manageable with a local agent | Confirm prior: Societies Act 1972 (Act No. 19 of 1972) still operative; NGO Bill still unenacted | verify-rest 2026-10: NGO Decree is No. 81 of 1996 (not 1993); Companies Act 2013 replaced the 1955 Act</t>
+          <t>English language, stable democracy; 2022 NGO Bill has been in draft years without enactment, so the old 1972 Societies Act still applies; Banjul filings manageable with a local agent | verify-rest 2026-10: NGO Decree is No. 81 of 1996 (not 1993); Companies Act 2013 replaced the 1955 Act</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
@@ -18401,7 +18401,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>English language; 2022 NGO Bill pending, so existing NGO/charitable-society registration practices continue; Freetown has expat-friendly law firms; registry throughput is slower than Ghana | Confirm prior: Companies Act 2013 CLG route; NGO Bill 2022 still pending | verify-rest 2026-10: Companies Act is 2009 (Act No. 5, am. 2014), not 2013; separate NGO registration (~US$500/yr) added</t>
+          <t>English language; 2022 NGO Bill pending, so existing NGO/charitable-society registration practices continue; Freetown has expat-friendly law firms; registry throughput is slower than Ghana | verify-rest 2026-10: Companies Act is 2009 (Act No. 5, am. 2014), not 2013; separate NGO registration (~US$500/yr) added</t>
         </is>
       </c>
       <c r="H195" s="2" t="inlineStr">
@@ -18493,7 +18493,7 @@
       </c>
       <c r="G196" s="2" t="inlineStr">
         <is>
-          <t>English language; the 2015 Act is the operative law (it replaced the older NGO Bill regime); permits must be renewed every 3 years; local principal officer requirement is the main hurdle for a fully foreign board | Confirm prior: NGO Act 2015 operative, US$150 fee, 3-year renewal, local principal officer | verify-rest 2026-10: unverifiable 'NGO Act 2015' removed — accreditation is under the National Aid &amp; NGO Policy (MFDP NGO Unit)</t>
+          <t>English language; the 2015 Act is the operative law (it replaced the older NGO Bill regime); permits must be renewed every 3 years; local principal officer requirement is the main hurdle for a fully foreign board | verify-rest 2026-10: unverifiable 'NGO Act 2015' removed — accreditation is under the National Aid &amp; NGO Policy (MFDP NGO Unit)</t>
         </is>
       </c>
       <c r="H196" s="2" t="inlineStr">
@@ -18503,7 +18503,7 @@
       </c>
       <c r="I196" s="2" t="inlineStr">
         <is>
-          <t>Liberian-national principal officer required to sign filings; local office; 3-year permit renewal cycle</t>
+          <t>Liberian principal officer required to sign filings; local office; MFA endorsement plus MFDP NGO Unit accreditation with annual fees</t>
         </is>
       </c>
       <c r="J196" s="2" t="inlineStr">
@@ -18585,7 +18585,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>Military rule since 2023; security situation in the north (Sahel conflict); Niamey filings are French-only; some discretionary elements in approvals | Confirm prior: Law 93-010 association regime; 2022-182 decree adds explicit prior-authorization layer; military rule since 2023 confirmed | verify-rest 2026-10: unverifiable 'Law 93-010' removed; 2025-26 crackdown added</t>
+          <t>Military rule since 2023; security situation in the north (Sahel conflict); Niamey filings are French-only; some discretionary elements in approvals | verify-rest 2026-10: unverifiable 'Law 93-010' removed; 2025-26 crackdown added</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Apply follow-up corrections A/C: 11 items, 49 cells; rebuild xlsx + webapp
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -2393,7 +2393,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>International ONGDs must register in the Registro Público de ONGD; moderate bureaucracy; all filings in Spanish. | verify-rest 2026-10: granting body is SGJD/DIRRSAC (not the Judiciary/Chancillería)</t>
+          <t>International ONGDs must register in the Registro Público de ONGD; moderate bureaucracy; all filings in Spanish. | verify-rest 2026-10: granting body is SGJD/DIRRSAC (not the Judiciary/Chancillería) | verify-followup 2026-10 (confirmed): Government acuerdos published in La Gaceta (incl.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>https://www.sgjd.gob.hn/institucion/dependencias/subsecretaria-de-justicia/direccion-de-regulacion-registro-y-seguimiento-de-asociaciones-civiles-dirrsac; https://diref.gob.hn/; https://consortiumlegal.com/2022/09/21/que-se-debe-tener-en-consideracion-si-desea-constituir-o-incorporar-una-ongd-en-honduras/; https://sgjd.gob.hn/servicios-y-gestiones-web/requisitos/servicios-de-atencion-al-ciudadano/personalidad-juridica/fundaciones</t>
+          <t>https://www.sgjd.gob.hn/institucion/dependencias/subsecretaria-de-justicia/direccion-de-regulacion-registro-y-seguimiento-de-asociaciones-civiles-dirrsac; https://diref.gob.hn/; https://consortiumlegal.com/2022/09/21/que-se-debe-tener-en-consideracion-si-desea-constituir-o-incorporar-una-ongd-en-honduras/; https://sgjd.gob.hn/servicios-y-gestiones-web/requisitos/servicios-de-atencion-al-ciudadano/personalidad-juridica/fundaciones; https://portalunico.iaip.gob.hn/ver_archivo/MTY2MTM1NA==; https://www.leybook.com/doc/29461/pdf</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2465,7 +2465,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Asociación or fundación under Ley 1115 (Ley General de Regulación y Control de Organismos sin Fines de Lucro, 2022; reformed by Ley 1127/2022 and Ley 1212/2024), registered with the Ministerio de Gobernación; fideicomiso (Ley 741/2010).</t>
+          <t>Asociación or fundación under Ley 1115 (Ley General de Regulación y Control de Organismos sin Fines de Lucro, 2022, which repealed Ley 147/1992; reformed by Ley 1127/2022 and Ley 1212/2024), registered with the Dirección General de Registro y Control de OSFL (now under the Ministerio del Interior, formerly Gobernación); fideicomiso (Ley 741/2010).</t>
         </is>
       </c>
       <c r="D22" s="6" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Spanish articles, local address, registration with the Ministerio de Gobernación (Dirección General de Registro y Control de OSFL), which now grants and cancels legal status directly; Ley 1040/2020 (Agentes Extranjeros) applies to foreign-funded entities.</t>
+          <t>Spanish articles, local address, registration with the Dirección General de Registro y Control de OSFL (Ministerio del Interior, formerly Gobernación), which grants and cancels legal status directly; foreign members of an asociación capped at 25% and must hold current Nicaraguan residence (Ley 1115 art. 12); foreign founders must file apostilled criminal records and a residence card; foreign OSFLs need a resident Apoderado Generalísimo; programmes only via state 'alianzas' (Ley 1212/2024, Decreto 13-2024); Ley 1040/2020 (Agentes Extranjeros) applies to foreign-funded entities.</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -2485,17 +2485,17 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Avoid: government has dissolved 5,700+ NGO legal personalities since 2018, including foreign-funded ones; laws target foreign-financed civil society, so an Australian-founded charity faces extreme cancellation/political risk. | confirm prior 'very hard'; add Ley 1115 (2022) as the controlling OSFL regulation; mass cancellations by Ministry of Governance decrees continue | verify-rest 2026-10: Ley 1115 (2022, reformed 2022/2024) is now the controlling law; legal personality granted by Gobernación, not the National Assembly</t>
+          <t>Avoid: government has dissolved 5,700+ NGO legal personalities since 2018, including foreign-funded ones; laws target foreign-financed civil society, so an Australian-founded charity faces extreme cancellation/political risk. | confirm prior 'very hard'; add Ley 1115 (2022) as the controlling OSFL regulation; mass cancellations by Ministry of Governance decrees continue | verify-rest 2026-10: Ley 1115 (2022, reformed 2022/2024) is now the controlling law; legal personality granted by Gobernación, not the National Assembly | verify-followup 2026-10 (corrected): Ley 1115 (approved 31 Mar 2022, La Gaceta No.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>no</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>Extreme political risk: 5,700+ NGO legal personalities cancelled since 2018; state controls authorization and registry of OSFLs.</t>
+          <t>Effectively closed: foreign members/founders must hold Nicaraguan residence (Ley 1115 art. 12, 25% cap on foreign members of associations), programmes require a state alliance, and 5,700+ NGO legal personalities have been cancelled since 2018 (cancellations continuing in 2025).</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2525,7 +2525,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>http://legislacion.asamblea.gob.ni/normaweb.nsf/09cf45d6fc893868062572650059911e/bfed6e3afb3d8fbf06258ae10075cd64; https://www.icnl.org/wp-content/uploads/Nicaragua_perjurid.pdf; http://legislacion.asamblea.gob.ni/normaweb.nsf/($All)/1A61F4734310A53406258A5400520EC1?OpenDocument=; https://nicaragua.justia.com/nacionales/decretos-ley/ley-sobre-asociaciones-y-registro-central-de-personas-juridicas-nov-21-1983/gdoc/; https://www.ey.com/es_ce/technical/tax/tax-alerts/nicaragua-entran-en-vigencia-reformas-al-marco-normativo-sobre-organismos</t>
+          <t>http://legislacion.asamblea.gob.ni/normaweb.nsf/09cf45d6fc893868062572650059911e/bfed6e3afb3d8fbf06258ae10075cd64; https://www.icnl.org/wp-content/uploads/Nicaragua_perjurid.pdf; http://legislacion.asamblea.gob.ni/normaweb.nsf/($All)/1A61F4734310A53406258A5400520EC1?OpenDocument=; https://nicaragua.justia.com/nacionales/decretos-ley/ley-sobre-asociaciones-y-registro-central-de-personas-juridicas-nov-21-1983/gdoc/; https://www.ey.com/es_ce/technical/tax/tax-alerts/nicaragua-entran-en-vigencia-reformas-al-marco-normativo-sobre-organismos; https://www.leybook.com/doc/27738; https://www.gchnicaragua.com/constitucion-y-operacion-de-osfl-en-nicaragua-ley-1115/; https://www.leybook.com/doc/33754/pdf</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2649,7 +2649,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Fundación de interés privado (Ley 25/1995; min endowment US$10,000); asociación sin fines de lucro (personería jurídica from the Ministerio de Gobierno); fideicomiso (Ley 21 of 10 May 2017, replacing Ley 1/1984).</t>
+          <t>Fundación de interés privado (Ley 25/1995; min endowment US$10,000); asociación sin fines de lucro (personería jurídica from the Ministerio de Gobierno); fideicomiso (Ley 1 of 5 January 1984, as amended by Ley 21 of 10 May 2017, which regulates trustees and repealed Decreto Ejecutivo 16/1984).</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>The FIP (Ley No. 8 de 2000) is the most popular expat foundation vehicle in Latin America; IFPF is a specialized fast registry; strong English-language support. | correct prior: FIP is governed by Ley 25 de 1995 (not 'Ley 8 de 2000'); registered in Registro Publico de la Propiedad, not 'IFPF' | Verified: Personero legal extranjero debe residir en Panamá; acta protocolizada en notaría y Tasa Única B/.400 | verify-rest 2026-10: trust law is Ley 21/2017; FIP needs a Panamanian resident agent and a council of 3 natural persons or 1 legal entity</t>
+          <t>The FIP (Ley No. 8 de 2000) is the most popular expat foundation vehicle in Latin America; IFPF is a specialized fast registry; strong English-language support. | correct prior: FIP is governed by Ley 25 de 1995 (not 'Ley 8 de 2000'); registered in Registro Publico de la Propiedad, not 'IFPF' | Verified: Personero legal extranjero debe residir en Panamá; acta protocolizada en notaría y Tasa Única B/.400 | verify-rest 2026-10: fideicomiso law is Ley 1/1984 as amended by Ley 21/2017 (trustee regulation); FIP needs a Panamanian resident agent and a council of 3 natural persons or 1 legal entity | verify-followup 2026-10 (corrected): Ley 21 of 10 May 2017 (Gaceta Oficial 28277 of 12 May 2017) sets the rules for regulating and supervising trustees (fiduciarios) and the trust business.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2709,7 +2709,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>https://www.organojudicial.gob.pa/uploads/wp_repo/blogs.dir/cendoj/CIVIL/ley_25_de_1995_fundaciones_de_interes_privado.pdf; https://laglex.net/nuestros-servicios/fundaciones-de-interes-privado/; https://www.rglawfirmpa.com/fundaciones-privadas-en-panama; https://www.gacetaoficial.gob.pa/; https://docs.panama.justia.com/federales/leyes/25-de-1995-jun-14-1995.pdf</t>
+          <t>https://www.organojudicial.gob.pa/uploads/wp_repo/blogs.dir/cendoj/CIVIL/ley_25_de_1995_fundaciones_de_interes_privado.pdf; https://laglex.net/nuestros-servicios/fundaciones-de-interes-privado/; https://www.rglawfirmpa.com/fundaciones-privadas-en-panama; https://www.gacetaoficial.gob.pa/; https://docs.panama.justia.com/federales/leyes/25-de-1995-jun-14-1995.pdf; https://www.superbancos.gob.pa/documentos/leyes_y_regulaciones/circulares/2017/circular-068-2017.pdf; https://morimor.com/es/?p=24509</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2756,12 +2756,12 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>US$300–600 incl. lawyer; 2–6 weeks at Cámara de Comercio. Notary for the deed ~US$50–150; official timelines unpublished.</t>
+          <t>US$300–600 incl. lawyer; 2–6 weeks at Cámara de Comercio. Notary signature recognition (or optional public deed) ~US$50–150; official timelines unpublished.</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Most expat-friendly in the region; foreigners can be president/directors; Bogotá has strong English-speaking legal market; donation tax deductions require separate DIAN certification; 2023 NGO-law reforms (Ley 2287/2022) added transparency reporting for foreign-funded entities. | Prior context confirmed; deduction is a separate DIAN certification step, not automatic; Ley 2287/2022 adds transparency duties | Verified: Constitution deed must be signed before a Colombian notary; remote founders need an apostilled poder especial | verify-rest 2026-10: Civil Code articles corrected to 633-652; private document suffices for ESAL constitution</t>
+          <t>Most expat-friendly in the region; foreigners can be president/directors; Bogotá has strong English-speaking legal market; donation tax deductions require separate DIAN certification; 2023 NGO-law reforms (Ley 2287/2022) added transparency reporting for foreign-funded entities. | Prior context confirmed; deduction is a separate DIAN certification step, not automatic; Ley 2287/2022 adds transparency duties | Verified: Constitution deed must be signed before a Colombian notary; remote founders need an apostilled poder especial | verify-rest 2026-10: Civil Code articles corrected to 633-652; private document suffices for ESAL constitution | verify-followup 2026-10 (corrected): Código Civil Libro I Título XXXVI 'De las personas jurídicas' runs from art.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>Colombian registered address + local lawyer for public deed &amp; Cámara de Comercio registration; Spanish filings</t>
+          <t>Colombian registered address + local lawyer for Cámara de Comercio registration; constitution by escritura pública or documento privado reconocido (signatures recognized before a notary, or via apostilled poder); Spanish filings</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>https://www.ccb.org.co; https://neo-project.github.io/global-blockchain-compliance-hub/colombia/colombia-registry-requirements.html; https://www.whydonate.com; https://www.minjusticia.gov.co/programas-co/LegalApp/Paginas/Que-debo-hacer-para-constituir-una-fundacion.aspx; https://www.ccb.org.co/processes-and-consultations/about-registrations/registration-non-profit-entities/non-profit-entities-common-regime; https://www.ccb.org.co/servicios/registros-publicos/registro-de-entidades-sin-animo-de-lucro</t>
+          <t>https://www.ccb.org.co; https://neo-project.github.io/global-blockchain-compliance-hub/colombia/colombia-registry-requirements.html; https://www.whydonate.com; https://www.minjusticia.gov.co/programas-co/LegalApp/Paginas/Que-debo-hacer-para-constituir-una-fundacion.aspx; https://www.ccb.org.co/processes-and-consultations/about-registrations/registration-non-profit-entities/non-profit-entities-common-regime; https://www.ccb.org.co/servicios/registros-publicos/registro-de-entidades-sin-animo-de-lucro; https://encolombia.com/derecho/codigos/civil-colombiano/codcivillibro1-t36/; https://normas.cra.gov.co/Gestor/Docs/decreto_0427_1996.htm</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>No nationality requirement; foreign founders allowed; tax exemption (exoneración) from SUNAT is separate, discretionary and needs annual reporting; Lima is the practical hub; English not official. | Prior context confirmed; deduction cap is 10% of net taxable income (PwC); SUNAT tax exemption is separate and discretionary | verify-rest 2026-10: Civil Code article numbers corrected; SUNARP fee is modest — the larger figure is notary/lawyer cost</t>
+          <t>No nationality requirement; foreign founders allowed; tax exemption (exoneración) from SUNAT is separate, discretionary and needs annual reporting; Lima is the practical hub; English not official. | Prior context confirmed; deduction cap is 10% of net taxable income (PwC); SUNAT tax exemption is separate and discretionary | verify-rest 2026-10: Civil Code article numbers corrected; SUNARP fee is modest — the larger figure is notary/lawyer cost | verify-followup 2026-10 (confirmed): The Código Civil (Libro I, Sección Segunda) places Asociación in Título II (arts.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -3077,7 +3077,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>https://taxsummaries.pwc.com/peru/corporate/deductions; https://nvcabogados.com/how-to-start-an-ngo-in-peru/; https://peru.iom.int/sites/g/files/tmzbdl951/files/documents/2024-01/guia-practica-asociaciones-sin-fines-de-lucro.pdf; https://www.gob.pe/institucion/sunarp</t>
+          <t>https://taxsummaries.pwc.com/peru/corporate/deductions; https://nvcabogados.com/how-to-start-an-ngo-in-peru/; https://peru.iom.int/sites/g/files/tmzbdl951/files/documents/2024-01/guia-practica-asociaciones-sin-fines-de-lucro.pdf; https://www.gob.pe/institucion/sunarp; https://www.icnl.org/research/library/peru_civil/; https://cdn.www.gob.pe/uploads/document/file/1532870/DECRETO%20SUPREMO%20N%C2%B0%2003-94-JUS%20REGLAMENTO%20DEL%20CONSEJO%20DE%20SUPERVIGILANCIA%20DE%20FUNDACIONES.pdf.pdf</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -3957,7 +3957,7 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>The fastest expat path is the non-profit general incorporated association (can register in as little as two weeks); Specified-NPO status adds tax-deductible donation treatment but a longer, prefecture-run certification. All documents in Japanese; English support is limited. | confirm prior: no nationality bar for founders/directors; fees ~YEN 30k-50k; 2-4 weeks for nonprofit general incorporated association | verify-rest 2026-10: government cost corrected to registration licence tax ¥60,000 + notary</t>
+          <t>The fastest expat path is the non-profit general incorporated association (can register in as little as two weeks); Specified-NPO status adds tax-deductible donation treatment but a longer, prefecture-run certification. All documents in Japanese; English support is limited. | confirm prior: no nationality bar for founders/directors; fees ~YEN 30k-50k; 2-4 weeks for nonprofit general incorporated association | verify-rest 2026-10: government cost corrected to registration licence tax ¥60,000 + notary | verify-followup 2026-10 (confirmed): Under Registration and Licence Tax Act Appended Table 1 item 24, incorporation registration of a general incorporated association (一般社団法人) carries a flat registration licence tax of JPY 60,000.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
@@ -3997,7 +3997,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>https://www.jnpoc.ne.jp/en/nonprofits-in-japan/about-npo-law/; https://cof.org/country-notes/nonprofit-law-japan; https://isvd.or.jp/en/guides/nonprofit-association-setup-complete-guide; https://www.moj.go.jp/MINJI/minji06_00106.html</t>
+          <t>https://www.jnpoc.ne.jp/en/nonprofits-in-japan/about-npo-law/; https://cof.org/country-notes/nonprofit-law-japan; https://isvd.or.jp/en/guides/nonprofit-association-setup-complete-guide; https://www.moj.go.jp/MINJI/minji06_00106.html; https://biz.moneyforward.com/establish/basic/86338/; https://shiodome.co.jp/js/blog/13252; https://www.zeiken.co.jp/yougo/</t>
         </is>
       </c>
       <c r="P38" s="2" t="inlineStr">
@@ -4039,7 +4039,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Foreigners may establish non-profit corporations (Civil Act arts. 32-33; permission of the competent ministry), then register at the court registry within 3 weeks; needs a local office address and Korean-language constitution; foundations face a ministry-guideline endowment (often ~KRW 100M+, no statutory minimum).</t>
+          <t>Foreigners may establish non-profit corporations (Civil Act art. 32 permission of the competent ministry; art. 33), then register at the court registry within 3 weeks of the permit arriving (arts. 49, 53); needs a local office address and Korean-language constitution; no statutory minimum endowment, but foundations face ministry/agency guideline endowments that vary by field (often several hundred million KRW or more).</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -4049,7 +4049,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Confirmed viable for expats (KOTRA/Invest Korea and formation guides both confirm foreigners can register foundations and NGOs); Korean-language paperwork is the main burden; popular expat-charity route is the 재단 법인 for grantmaking. | confirm prior: foreigners may establish foundations and NGOs (KOTRA/Invest Korea FAQ confirms); Korean-language docs main burden | verify-rest 2026-10: legal basis is Civil Act arts. 32-33 with court-registry registration; KRW 100M endowment is an administrative guideline, not statutory</t>
+          <t>Confirmed viable for expats (KOTRA/Invest Korea and formation guides both confirm foreigners can register foundations and NGOs); Korean-language paperwork is the main burden; popular expat-charity route is the 재단 법인 for grantmaking. | confirm prior: foreigners may establish foundations and NGOs (KOTRA/Invest Korea FAQ confirms); Korean-language docs main burden | verify-rest 2026-10: legal basis is Civil Act arts. 32-33 with court-registry registration; KRW 100M endowment is an administrative guideline, not statutory | verify-followup 2026-10 (corrected): Civil Act art.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -4089,7 +4089,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>https://www.investkorea.org/upload/kotraexpress/2021/12/images/FAQ.pdf; https://elaw.klri.re.kr/eng_service/lawView.do?lang=ENG&amp;hseq=18330; https://taxsummaries.pwc.com/republic-of-korea/individual/deductions; https://www.law.go.kr/</t>
+          <t>https://www.investkorea.org/upload/kotraexpress/2021/12/images/FAQ.pdf; https://elaw.klri.re.kr/eng_service/lawView.do?lang=ENG&amp;hseq=18330; https://taxsummaries.pwc.com/republic-of-korea/individual/deductions; https://www.law.go.kr/; https://korea.legal/wiki/%eb%af%bc%eb%b2%95-%ec%a0%9c49%ec%a1%b0/; https://www.botoai.co/posts/재단법인-설립-자본금</t>
         </is>
       </c>
       <c r="P39" s="2" t="inlineStr">
@@ -4136,12 +4136,12 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>Several months to over a year including the 2-year operational-pilot requirement and approvals; official fees low, agent/legal costs significant.</t>
+          <t>Several months to over a year for approvals; public-fundraising qualification only after 1 year of registration (cut from 2 years by the 2023 Charity Law amendment, in force 5 Sep 2024); official fees low, agent/legal costs significant.</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Direct foreign formation is effectively barred without a local Chinese partner organization; foreign-funded groups must register under the Foreign NGO Law (2+ years of overseas track record) or operate through a local partner — heavy political/supervision risk, no English-language process. | confirm prior: direct foreign formation effectively barred; Foreign NGO Law route needs 2+ yrs track record; heavy political supervision | verify-rest 2026-10: foundation minimum funds corrected per Regulations on the Management of Foundations (2004) art. 8</t>
+          <t>Direct foreign formation is effectively barred without a local Chinese partner organization; foreign-funded groups must register under the Foreign NGO Law (2+ years of overseas track record) or operate through a local partner — heavy political/supervision risk, no English-language process. | confirm prior: direct foreign formation effectively barred; Foreign NGO Law route needs 2+ yrs track record; heavy political supervision | verify-rest 2026-10: foundation minimum funds corrected per Regulations on the Management of Foundations (2004) art. 8 | verify-followup 2026-10 (corrected): Art.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>Foreign individuals cannot form a foundation directly; needs Chinese supervising unit, RMB 2m/800k fund, Foreign NGO Law</t>
+          <t>Foreign individuals cannot form a foundation directly; needs Chinese supervising unit, RMB 2M–8M paid-in original fund (2004 Foundation Regulations art. 8), Foreign NGO Law</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>https://www.chinalawtranslate.com/en/foundations-regulations-draft/; https://www.svcf.org/sites/default/files/documents/csr/SVCF_ChinaForeignNGOLaw_web.pdf; https://taxsummaries.pwc.com/peoples-republic-of-china/individual/deductions</t>
+          <t>https://www.chinalawtranslate.com/en/foundations-regulations-draft/; https://www.svcf.org/sites/default/files/documents/csr/SVCF_ChinaForeignNGOLaw_web.pdf; https://taxsummaries.pwc.com/peoples-republic-of-china/individual/deductions; https://www.gov.cn/zhengce/content/2008-03/28/content_6434.htm; https://www.gov.cn/zhengce/202409/content_6972648.htm</t>
         </is>
       </c>
       <c r="P40" s="2" t="inlineStr">
@@ -8353,7 +8353,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>National NGO (Law N°04/2012) or international NGO (Law N°05/2012), registered with the Rwanda Governance Board (RGB) - certificate of legal personality; a consolidated NGO bill was tabled in 2024.</t>
+          <t>National NGO or international NGO under Law N°058/2024 of 20/06/2024 governing Non-Governmental Organisations (gazetted 17/07/2024; repealed Laws N°04/2012 and N°05/2012), registered with the Rwanda Governance Board (RGB) - certificate of legal personality.</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
@@ -8373,7 +8373,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Strict, well-enforced 2016 NGO Act; English/French/Kinyarwanda; many expats operate through Rwandan partners rather than foreign registration. | verify-rest 2026-10: no 'Law 01/2016' — NGOs governed by Laws 04/2012 and 05/2012; 300,000 RWF ≈ US$210 (not ~$24)</t>
+          <t>Strict, well-enforced 2016 NGO Act; English/French/Kinyarwanda; many expats operate through Rwandan partners rather than foreign registration. | verify-rest 2026-10: no 'Law 01/2016' — NGOs governed by Laws 04/2012 and 05/2012; 300,000 RWF ≈ US$210 (not ~$24) | verify-followup 2026-10 (corrected): The bill tabled 18 April 2024 was enacted as Law N°058/2024 of 20/06/2024 governing Non-Governmental Organisations, gazetted 17 July 2024;</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr">
@@ -8413,7 +8413,7 @@
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
-          <t>https://www.rgb.rw/1/civil-society-faith-based-and-political-organisations/non-governmental-organisations</t>
+          <t>https://www.rgb.rw/1/civil-society-faith-based-and-political-organisations/non-governmental-organisations; https://www.mondaq.com/corporate-and-company-law/1534440/ens-rwanda-in-brief; https://www.icnl.org/resources/civic-freedom-monitor/rwanda</t>
         </is>
       </c>
       <c r="P86" s="2" t="inlineStr">
@@ -14517,7 +14517,7 @@
       </c>
       <c r="C153" s="2" t="inlineStr">
         <is>
-          <t>Association (jam'iyya) under Law 24/1962 on Clubs and Public Welfare Societies (Ministry of Social Affairs; 2025 Ministerial Decision 90 cut charitable-association founders to 10 Kuwaitis); representative office of foreign NGO</t>
+          <t>Association (jam'iyya) under Law 24/1962 on Clubs and Public Welfare Societies (Ministry of Social Affairs; 2025 Ministerial Decision 90 cut charitable-association founders from 50 to 10, board members 30+ with a degree); charitable sector now also governed by Decree-Law No. 87 of 2026 (National Center for Charitable and Humanitarian Work; fundraising needs prior ministry approval); representative office of foreign NGO</t>
         </is>
       </c>
       <c r="D153" s="6" t="inlineStr">
@@ -14537,7 +14537,7 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>Closed to foreign formation; foreigners work through established Kuwaiti charities (e.g. Kuwait Foundation for the Disabled, local societies) or a government-approved representative office; English usable informally, filings in Arabic | Confirm prior; new rules (10 Kuwaiti founders, KWD 10k deposit) re-confirm closed regime | verify-rest 2026-10: governing law Law 24/1962 cited; 2025 founder rule added</t>
+          <t>Closed to foreign formation; foreigners work through established Kuwaiti charities (e.g. Kuwait Foundation for the Disabled, local societies) or a government-approved representative office; English usable informally, filings in Arabic | Confirm prior; new rules (10 Kuwaiti founders, KWD 10k deposit) re-confirm closed regime | verify-rest 2026-10: governing law Law 24/1962 cited; 2025 founder rule added | verify-followup 2026-10 (corrected): Both exist per Kuwait Times (KUNA): Decree-Law No.</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr">
@@ -14577,7 +14577,7 @@
       </c>
       <c r="O153" s="2" t="inlineStr">
         <is>
-          <t>https://www.asarlegal.com/kuwait-reshapes-regulations-for-charitable-organisations/; https://www.icnl.org/research/library/kuwait_24-62-en/; https://alsubaielawfirm.com/en/establishing-non-profit-companies-in-kuwait/</t>
+          <t>https://www.asarlegal.com/kuwait-reshapes-regulations-for-charitable-organisations/; https://www.icnl.org/research/library/kuwait_24-62-en/; https://alsubaielawfirm.com/en/establishing-non-profit-companies-in-kuwait/; https://kuwaittimes.com/article/49666/kuwait/social-affairs-min-new-charity-law-boosts-governance-transparency/; https://kuwaittimes.com/article/31446/kuwait/other-news/new-law-makes-it-harder-to-mismanage-charity-organizations-in-kuwait/</t>
         </is>
       </c>
       <c r="P153" s="2" t="inlineStr">
@@ -14895,17 +14895,17 @@
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>Founders must be Bahraini citizens (min. ~10 adults under Decree-Law 21/1989 as amended); Bahraini-controlled board; local address; Arabic filings</t>
+          <t>Min. 10 adult natural-person founders (Decree-Law 21/1989 Art. 4; nationality declared in the articles, no statutory Bahraini quota found); main seat in Bahrain; Ministry of Social Development registration with publication in the Official Gazette; Arabic filings</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
-          <t>Registration is effectively out of reach for foreigners: Decree-Law 21/1989 requires Bahraini founders (~10 minimum). Official processing time unpublished.</t>
+          <t>Registration is effectively out of reach for a remote foreigner: Decree-Law 21/1989 requires at least 10 founders, a seat in Bahrain and ministry approval. Official processing time unpublished.</t>
         </is>
       </c>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>Bahrain is the most English-friendly and transparent NGO administration in the Gulf, but the nationality floor on founders/board keeps foreign formation out of reach; standard route is a partnership with an existing Bahraini NGO; government relations are comparatively accessible | verify-rest 2026-10: founder minimum corrected to ~10; 'Law 19/2006' founder-rule reference removed</t>
+          <t>Bahrain is the most English-friendly and transparent NGO administration in the Gulf, but the nationality floor on founders/board keeps foreign formation out of reach; standard route is a partnership with an existing Bahraini NGO; government relations are comparatively accessible | verify-rest 2026-10: founder minimum corrected to ~10; 'Law 19/2006' founder-rule reference removed | verify-followup 2026-10 (corrected): The official LLOC English consolidated text of Legislative Decree 21/1989 (published May 2024) sets the minimum at ten founders where founders are natural persons (Art.</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr">
@@ -14915,7 +14915,7 @@
       </c>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>20+ Bahraini-citizen founders and 2/3 Bahraini board required; foreigners cannot form an association alone.</t>
+          <t>At least 10 natural-person founders (Decree-Law 21/1989 Art. 4) with the association's seat in Bahrain and Ministry approval; statute sets no nationality quota but founders' nationality must be declared and in practice a foreign non-resident cannot form an association alone.</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Round-2 re-verification of 113 rows; add Palau, Kosovo, Cabo Verde, Greenland
Round 2 re-checked every medium-confidence row against official sources
(verify-rest-out/r2/result_01..10): 56 corrected, 53 confirmed, 4
unverifiable. apply_followups.py now ingests r2 results alongside the
follow-ups, validates enum columns, and carries a reviewed CELL_FIX sweep
of 23 superseded claims left in other columns (e.g. Mongolia law name,
Ethiopia regulator, Taiwan endowment). Review overrides: Tajikistan
remote founding -> no (residence permit required), Tuvalu -> hard.

Coverage: Palau, Kosovo, Cabo Verde (the sovereign states missing from
the map) and Greenland (self-governing, own legislature and tax system)
researched from primary sources and merged via add_countries.py from
research/new_countries/. Dataset is now 202 rows; GfN 185 of 202.
build_xlsx.py counts are computed from the data. Top-10 unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Methodology" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master'!$A$1:$R$199</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Master'!$A$1:$R$203</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R199"/>
+  <dimension ref="A1:R203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -901,7 +901,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee (Companies Act 2004, Form 1B); charitable status via Recognized Charitable Organisation under the Charities Act 2013 (Companies Office of Jamaica).</t>
+          <t>Company limited by guarantee (Companies Act 2004, Form 1B, Companies Office of Jamaica); charitable status via registration as a charitable organisation under the Charities Act 2013 with the DCFS (Charities Authority).</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -916,12 +916,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Registration JMD 27,000 (~USD 150) + name search JMD 500 / reservation JMD 3,000; ~1-2 weeks; a local registered office and agent are required, adding ~USD 1,000-2,000 agent fees.</t>
+          <t>Incorporation ~J$27,500 (~USD 175) + optional name search J$500 / reservation J$3,000; ~1-2 weeks; a local registered office and agent are required, adding ~USD 1,000-2,000 agent fees.</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>No formal charity status, regulator, or donation tax-deductibility regime; most foreign founders use a company limited by guarantee + local manager. | prior claim of 'no charity regulator/tax-deduction regime' is outdated: Charities Act 2013 registration (RCOs) exists with tax-deductible status</t>
+          <t>No formal charity status, regulator, or donation tax-deductibility regime; most foreign founders use a company limited by guarantee + local manager. | prior claim of 'no charity regulator/tax-deduction regime' is outdated: Charities Act 2013 registration (RCOs) exists with tax-deductible status | verify-r2 2026-10 (corrected): Under the Charities Act 2013 the Department of Co-operatives and Friendly Societies (DCFS) is the Charities Authority with which organisations register to obtain charitable status, separate from Companies Office incorporation.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>~$150 (J$25,000 Companies Office filing; agent fees separate)</t>
+          <t>~$175 (J$27,500 Companies Office filing; agent fees separate)</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>https://www.jamaicatax.gov.jm/charitable-donations; https://www.orcjamaica.com/Services.aspx; https://dcfs.gov.jm/docs/Charities/DCFS_CharitiesPolicy.pdf; https://www.miic.gov.jm/register-your-business/</t>
+          <t>https://www.jamaicatax.gov.jm/charitable-donations; https://www.orcjamaica.com/Services.aspx; https://dcfs.gov.jm/docs/Charities/DCFS_CharitiesPolicy.pdf; https://www.miic.gov.jm/register-your-business/; https://jis.gov.jm/charities-must-register-benefit-tax-exemptions/; https://jamaicaobserver.com/2024/05/01/minding-business-start-company; https://bjdc.mfaft.gov.jm/pdf/COMP_OF_JAM.pdf</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee (Companies Act, Chapter 308 (1992, as am.)); domestic company incorporated at the Registrar General's Department; charitable deduction status applied for with IRD.</t>
+          <t>Company limited by guarantee (Companies Act, Chapter 308 (1992, as am.)) incorporated at the Registrar General's Department; must also register as an NPO under the Non-Profit Organisations Act 2019 (no income tax, so no deduction status).</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -1003,7 +1003,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Bahamas registered office and licensed registered agent; no residency requirement for directors; English.</t>
+          <t>Bahamas registered office and licensed registered agent; NPO Act 2019 registration (controller ID, board structure, KYC); no residency requirement for directors; English.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -1013,7 +1013,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Strong offshore-agent ecosystem; no income tax so no tax-exempt registration is needed; donations are not tax-deductible for donors. | confirm prior - Companies Act, Ch. 308 (1992) CLBG via Corporate Business Registry with licensed agent; no charity tax regime</t>
+          <t>Strong offshore-agent ecosystem; no income tax so no tax-exempt registration is needed; donations are not tax-deductible for donors. | confirm prior - Companies Act, Ch. 308 (1992) CLBG via Corporate Business Registry with licensed agent; no charity tax regime | verify-r2 2026-10 (corrected): The Bahamas Non-Profit Organisations Act 2019 (Act No.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -1053,7 +1053,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>https://rgd.gov.bs/service/foreign-registration-of-companies; https://www.bahamas.gov.bs/corporate-registry; https://www.expanship.com/bs/blog/how-much-does-it-cost-to-incorporate-a-company-in-bahamas; https://www.rgd.gov.bs/service/incorporation-of-a-regular-company</t>
+          <t>https://rgd.gov.bs/service/foreign-registration-of-companies; https://www.bahamas.gov.bs/corporate-registry; https://www.expanship.com/bs/blog/how-much-does-it-cost-to-incorporate-a-company-in-bahamas; https://www.rgd.gov.bs/service/incorporation-of-a-regular-company; https://webiis10.mondaq.com/financial-services/980182/the-non-profit-organisations-act-2019-act-no-25-of-2019-the-non-profit-organisations-amendment-act-2019-act-no-28-of-2019-the-npo-act; https://thenassauguardian.com/non-profits-have-two-week-grace-period-before-facing-hefty-fines/</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee (Companies Act, Cap. 308 (1982, as am.), CAIPO); tax-deductible charitable status under the Income Tax Act; foreign entities register as external companies (Form 28).</t>
+          <t>Non-profit company (Companies Act, Cap. 308, Part III; Minister's prior approval of articles, min. 3 directors; CAIPO); charity registration under the Charities Act, Cap. 243 (Registrar of Charities, CAIPO); foreign entities register as external companies.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -1100,12 +1100,12 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Registry incorporation fee ~BBD 250-500 (~USD 125-250); 2-4 weeks at CAIPO; a local registered office and Barbadian agent are mandatory - all-in with agent ~USD 2,500-3,000 first year.</t>
+          <t>Non-profit company filing BDS 150 + name reservation BDS 30 (~USD 90); charity registration nil fee; 2-4 weeks at CAIPO plus ministerial approval; a local registered office is required - all-in with agent ~USD 2,500-3,000 first year.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>No dedicated charity regulator; standard expat path is a company limited by guarantee with a local secretary. | confirm prior - Companies Act, Cap. 308 (1982) CLBG via Business Barbados (CAIPO) with local agent; standard expat path</t>
+          <t>No dedicated charity regulator; standard expat path is a company limited by guarantee with a local secretary. | confirm prior - Companies Act, Cap. 308 (1982) CLBG via Business Barbados (CAIPO) with local agent; standard expat path | verify-r2 2026-10 (corrected): CAIPO (Business Barbados) incorporates non-profit companies on Form 2 for BDS 150 (plus BDS 30 name reservation), with articles pre-approved by the Minister under s.314(1) and at least three directors.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1115,12 +1115,12 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Local registered office + agent required; no dedicated charity regulator, so deductible status is limited.</t>
+          <t>Ministerial approval of non-profit articles and local registered office/agent required; separate Charities Act registration needed for charitable status.</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>~$300-800 incl. agent</t>
+          <t>~$90 (gov, BDS 180 incl. name); agent/attorney fees extra</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>https://caipo.gov.bb/corporate-affairs/incorporation/; https://caipo.gov.bb/corporate-affairs/registered-agent/; https://www.expanship.com/bb/blog/how-much-does-it-cost-to-incorporate-a-company-in-barbados</t>
+          <t>https://caipo.gov.bb/corporate-affairs/incorporation/; https://caipo.gov.bb/corporate-affairs/registered-agent/; https://www.expanship.com/bb/blog/how-much-does-it-cost-to-incorporate-a-company-in-barbados; https://caipo.gov.bb/corporate-affairs/incorporation-non-profit/; https://caipo.gov.bb/fees/; https://caipo.gov.bb/corporate-affairs/registration-charity/; https://caipo.gov.bb/wp-content/uploads/2021/09/11.-CharitiesCAP243.pdf</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1177,7 +1177,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee (Companies Act Chap. 81:01, Companies Registry); NPO registration under the Non-Profit Organisations Act 2019 (Act No. 7 of 2019); charitable/tax-exempt status by Ministry of Finance approval under the Income Tax Act Chap. 75:01.</t>
+          <t>Non-profit company (Companies Act Chap. 81:01, Companies Registry); NPO registration under the Non-Profit Organisations Act 2019 (Act No. 7 of 2019); charitable/tax-exempt status by Ministry of Finance approval under the Income Tax Act Chap. 75:01.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -1197,7 +1197,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Gifts to approved charitable organizations are income-tax deductible (T&amp;T Income Tax Act); no formal charity status beyond government approval. | confirm prior - Companies Act 2019 CLBG plus separate charitable-status application under Income Tax Act s.76(3)(d) | verify-rest 2026-10: law refs corrected (Companies Act Chap. 81:01, Income Tax Act Chap. 75:01; no 'Charities Act' — NPO Act 2019 registration applies)</t>
+          <t>Gifts to approved charitable organizations are income-tax deductible (T&amp;T Income Tax Act); no formal charity status beyond government approval. | confirm prior - Companies Act 2019 CLBG plus separate charitable-status application under Income Tax Act s.76(3)(d) | verify-rest 2026-10: law refs corrected (Companies Act Chap. 81:01, Income Tax Act Chap. 75:01; no 'Charities Act' — NPO Act 2019 registration applies) | verify-r2 2026-10 (corrected): The T&amp;T government portal lists incorporation of a 'Profit or Non-Profit Company' under the Companies Act Chap.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>https://www.finance.gov.tt/services/licenses/application-for-charitable-status/; https://www.ird.gov.tt/approvals-deeds-of-covenants; https://rgd.legalaffairs.gov.tt/laws2/Alphabetical_List/lawspdfs/75.01.pdf; https://legalaffairs.gov.tt/faqs.php; https://fiu.gov.tt/wp-content/uploads/Non-Profit-Organisations-Act-2019.pdf</t>
+          <t>https://www.finance.gov.tt/services/licenses/application-for-charitable-status/; https://www.ird.gov.tt/approvals-deeds-of-covenants; https://rgd.legalaffairs.gov.tt/laws2/Alphabetical_List/lawspdfs/75.01.pdf; https://legalaffairs.gov.tt/faqs.php; https://fiu.gov.tt/wp-content/uploads/Non-Profit-Organisations-Act-2019.pdf; https://ttconnect.gov.tt/?p=558</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1269,7 +1269,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee (Companies Act 1995 (Act 18/1995), ABIPCO); domestic company; no separate charity registry - charitable purpose stated in the objects; IBCs only via a licensed agent.</t>
+          <t>Non-profit company (Companies Act 1995 (Act 18/1995), ABIPCO); domestic company; no separate charity registry - charitable purpose stated in the objects; IBCs only via a licensed agent.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Established offshore-agent services make remote formation straightforward; no charity tax regime. | confirm prior - Companies Act 1995 CLBG via ABIPCO with licensed agent; remote formation straightforward</t>
+          <t>Established offshore-agent services make remote formation straightforward; no charity tax regime. | confirm prior - Companies Act 1995 CLBG via ABIPCO with licensed agent; remote formation straightforward | verify-r2 2026-10 (corrected): Antigua's Companies Act 1995 (amended most recently in 2025) provides a distinct non-profit company category for patriotic, religious, philanthropic, charitable, educational and similar objects, registered at ABIPCO, which is the charitabl…</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>https://abipco.gov.ag/companies/; https://laws.gov.ag/wp-content/uploads/2018/08/a1995-18.pdf; https://www.expanship.com/ag/blog/incorporation-requirements-in-antigua-and-barbuda</t>
+          <t>https://abipco.gov.ag/companies/; https://laws.gov.ag/wp-content/uploads/2018/08/a1995-18.pdf; https://www.expanship.com/ag/blog/incorporation-requirements-in-antigua-and-barbuda; https://bizlatinhub.com/how-to-form-a-company-in-antigua-barbuda</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Strong offshore-agent infrastructure; remote formation in English is practical. | confirm prior: CLBG/ordinary company EC$270 (~US$100) official fee, no resident-director rule, fast with local agent</t>
+          <t>Strong offshore-agent infrastructure; remote formation in English is practical. | confirm prior: CLBG/ordinary company EC$270 (~US$100) official fee, no resident-director rule, fast with local agent | verify-r2 2026-10 (confirmed): The St Kitts Companies Act 1996 (Cap.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1513,7 +1513,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>https://www.efiling.fsrc.kn/2015-11-19-14-16-32/237-company-registry-brochure-1/file; https://www.prenticeandco.com/guide-part-5; https://exploreskn.co/downloads/business/ProcedureforIncorporatingaCompany-1.pdf; https://efiling.fsrc.kn</t>
+          <t>https://www.efiling.fsrc.kn/2015-11-19-14-16-32/237-company-registry-brochure-1/file; https://www.prenticeandco.com/guide-part-5; https://exploreskn.co/downloads/business/ProcedureforIncorporatingaCompany-1.pdf; https://efiling.fsrc.kn; https://vlex.com/vid/st-kitts-international-financial-centre-29350567</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee (Companies Act, Chapter 13.01 (1996), Commercial Registry Agency); domestic company; charitable status via Inland Revenue. (IBCs exist under the International Business Companies Act Cap. 12.14, but are not a charity vehicle.)</t>
+          <t>Non-profit company (Companies Act, Chapter 13.01 (1996), Part III; Attorney General's prior approval; Commercial Registry Agency); charitable status via Inland Revenue. (IBCs exist under the International Business Companies Act Cap. 12.14, but are not a charity vehicle.)</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1560,12 +1560,12 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Government incorporation fee ~US$100-400; 2-5 days at the CRA; a local registered office and licensed agent are required - all-in with agent ~USD 1,500-2,500 first year.</t>
+          <t>Non-profit certificate of incorporation EC$150 (~US$55) + name reservation EC$25; AG approval adds time; a local registered office and licensed agent are required - all-in with agent ~USD 1,500-2,500 first year.</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Agent services available; no charity regulator; English-language filings. | confirm prior structure; official certificate of incorporation fee is EC$750 under Companies Act Part 9, higher than implied | verify-rest 2026-10: removed claim that IBCs are prohibited — IBC Act Cap. 12.14 remains in force (IBCs resident/taxable regime since 1 July 2021)</t>
+          <t>Agent services available; no charity regulator; English-language filings. | confirm prior structure; official certificate of incorporation fee is EC$750 under Companies Act Part 9, higher than implied | verify-rest 2026-10: removed claim that IBCs are prohibited — IBC Act Cap. 12.14 remains in force (IBCs resident/taxable regime since 1 July 2021) | verify-r2 2026-10 (corrected): Saint Lucia's Companies Regulations (Part 9 fees) set the certificate of incorporation at EC$150 for a non-profit company versus EC$750 for a profit company, with EC$25 for name search/reservation.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1575,12 +1575,12 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Registered office/agent required and a local attorney must make the statutory declaration; higher official fee</t>
+          <t>Attorney General's prior approval of non-profit articles; registered office/agent required and a local attorney must make the statutory declaration</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>~$100-400 (gov); ~$1,500-2,500 all-in w/ local agent</t>
+          <t>~$55 (gov, EC$150 non-profit); ~$1,500-2,500 all-in w/ local agent</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1605,7 +1605,7 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>https://www.lexadin.nl/wlg/legis/nofr/oeur/arch/stl/int_trust.pdf; http://attorneygeneralchambers.com/laws-of-saint-lucia/international-business-companies-act/section-39; https://esaintlucia.com/pricing; https://www.cra.gov.lc; https://saintluciaifc.com/legislative-update-july-2021</t>
+          <t>https://www.lexadin.nl/wlg/legis/nofr/oeur/arch/stl/int_trust.pdf; http://attorneygeneralchambers.com/laws-of-saint-lucia/international-business-companies-act/section-39; https://esaintlucia.com/pricing; https://www.cra.gov.lc; https://saintluciaifc.com/legislative-update-july-2021; https://www.attorneygeneralchambers.com/laws-of-saint-lucia/companies-act/part-9-fees; https://www.attorneygeneralchambers.com/laws-of-saint-lucia/companies-act/section-328; https://www.govt.lc/media.govt.lc/www/resources/forms/CompanyArticlesNonProfit.pdf</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Domestic company limited by guarantee (Companies Act No. 8 of 1994, CIPO); business companies only via a licensed VFA agent; charitable status via Inland Revenue.</t>
+          <t>Domestic non-profit company (Companies Act No. 8 of 1994, CIPO; Attorney General's written approval under s.328(1), min. 3 directors); business companies only via a licensed VFA agent; charitable status via Inland Revenue.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1652,12 +1652,12 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Domestic incorporation fee EC$950 (~US$350) + EC$25 per consent notice; ~2-5 days; a local registered office and agent are mandatory - agent fees add ~USD 1,500-2,000/year.</t>
+          <t>Non-profit fees are 20% of profit-company fees (incorporation ~EC$190, ~US$70; name reservation EC$5); ~2-5 days after AG approval; a local registered office and agent are mandatory - agent fees add ~USD 1,500-2,000/year.</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Agent services in English; minimal charity-specific legislation; company limited by guarantee is the standard form. | confirm prior; CIPO official fees: EC$950 incorporation + EC$190 non-profit fee, so official fee higher than ~$300-800 suggests</t>
+          <t>Agent services in English; minimal charity-specific legislation; company limited by guarantee is the standard form. | confirm prior; CIPO official fees: EC$950 incorporation + EC$190 non-profit fee, so official fee higher than ~$300-800 suggests | verify-r2 2026-10 (corrected): CIPO's non-profit company guide requires written Attorney General approval under s.328(1) of the Companies Act and at least three directors, and states that all non-profit company fees are 20% of profit-company fees.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1667,12 +1667,12 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Local registered office/agent and attorney's statutory declaration required to file with CIPO</t>
+          <t>Attorney General approval of non-profit articles; local registered office/agent and attorney's statutory declaration required to file with CIPO</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>~$350 (gov, EC$950); ~$1,500+ all-in w/ agent</t>
+          <t>~$70 (gov, EC$190 non-profit); ~$1,500+ all-in w/ agent</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>https://cipo.gov.vc/index.php/domestic-companies-items/54-incorporation; https://fsasvg.com/fees/; https://fsasvg.com/business-companies/</t>
+          <t>https://cipo.gov.vc/index.php/domestic-companies-items/54-incorporation; https://fsasvg.com/fees/; https://fsasvg.com/business-companies/; https://cipo.gov.vc/images/pdf/brochures/non-profit.pdf; https://cipo.gov.vc/images/pdf/brochures/companies_formalities_forms_fees.pdf</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Domestic company limited by guarantee (Companies Act, Act No. 10 of 1995 (CIPO)); IBC registration prohibited since 1 Jan 2022; charitable status via Inland Revenue.</t>
+          <t>Non-profit company (Companies Act, Act No. 10 of 1995 (CIPO); Minister's prior approval); IBC registration prohibited since 1 Jan 2022; charitable status via Inland Revenue.</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -1744,12 +1744,12 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Incorporation fee EC$750 (~US$277) at CIPO; 1-3 days; annual government fee ~US$550; a local registered office and licensed agent are required - agent fees ~USD 1,500-2,500/year.</t>
+          <t>Non-profit incorporation fee EC$150 (~US$55) + name reservation EC$25 at CIPO; Minister's prior approval adds time; annual government fee ~US$550; a local registered office and licensed agent are required - agent fees ~USD 1,500-2,500/year.</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Offshore-agent ecosystem; English; no formal charity status. | confirm prior: CLBG standard vehicle; official registration fee low (~EC$150), US$300-800 total is mostly agent cost</t>
+          <t>Offshore-agent ecosystem; English; no formal charity status. | confirm prior: CLBG standard vehicle; official registration fee low (~EC$150), US$300-800 total is mostly agent cost | verify-r2 2026-10 (corrected): Dominica's CIPO fee schedule sets the certificate of incorporation at EC$150 for a non-profit company (EC$750 for an ordinary company) and EC$25 for name reservation.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1759,12 +1759,12 @@
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Local registered office/agent needed; small registry, filings in person or via agent in English</t>
+          <t>Minister's prior approval for non-profit company; local registered office/agent needed; filings in person or via agent in English</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>~$100</t>
+          <t>~$55 (gov, EC$150 non-profit)</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>https://investdominica.com/doing-business/start-a-business/; https://cipo.gov.dm/businesses-and-companies/companies; https://www.expanship.com/dm/blog/company-limited-by-guarantee-in-dominica; https://www.cipodominica.com</t>
+          <t>https://investdominica.com/doing-business/start-a-business/; https://cipo.gov.dm/businesses-and-companies/companies; https://www.expanship.com/dm/blog/company-limited-by-guarantee-in-dominica; https://www.cipodominica.com; https://cipo.gov.dm/fees/companies</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>French-language notarial deed plus registration with the public prosecutor; a local partner is effectively required; high security/political risk. | confirm prior: Law 30 of 1943 association plus 1989 NGO decree (MPCE) govern; very hard for remote founder, local partner needed</t>
+          <t>French-language notarial deed plus registration with the public prosecutor; a local partner is effectively required; high security/political risk. | confirm prior: Law 30 of 1943 association plus 1989 NGO decree (MPCE) govern; very hard for remote founder, local partner needed | verify-r2 2026-10 (confirmed): The decree of 14 September 1989 (amending the law of 13 December 1982) remains the governing NGO framework, with recognition as an 'ONG d'aide au développement' processed by the MPCE's UCAONG and inscribed in its register.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1973,7 +1973,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>https://mpce.gouv.ht/registre-des-ong_/; https://centrengo.org/wp-content/uploads/2024/08/1989-Nonprofit-Decree-English-Translation.pdf; https://centrengo.org/wp-content/uploads/2024/08/Formalites-a-Remplir-pour-lobtention-du-statut-legal-dorganisation-Non-Governmentale-ONG-daide-au-developpement-1.pdf; https://mpce.gouv.ht/wp-content/uploads/2025/10/FORMALITES-A-REMPLIR-POUR-LOBTENTION-DU-STATUT-LEGAL-DORGANISATION-NON-GOUVERNEMENTALE.pdf</t>
+          <t>https://mpce.gouv.ht/registre-des-ong_/; https://centrengo.org/wp-content/uploads/2024/08/1989-Nonprofit-Decree-English-Translation.pdf; https://centrengo.org/wp-content/uploads/2024/08/Formalites-a-Remplir-pour-lobtention-du-statut-legal-dorganisation-Non-Governmentale-ONG-daide-au-developpement-1.pdf; https://mpce.gouv.ht/wp-content/uploads/2025/10/FORMALITES-A-REMPLIR-POUR-LOBTENTION-DU-STATUT-LEGAL-DORGANISATION-NON-GOUVERNEMENTALE.pdf; https://cliohaiti.net/media/documents/decret-du-14-septembre-1989-modifiant-la-loi-du-13-decembre-1982-regissant-les-ong.pdf</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -2107,7 +2107,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Notarized Spanish articles, Guatemalan legal address, Registro de Comercio filing; foreign founders permitted.</t>
+          <t>Notarized Spanish deed (escritura pública), Guatemalan seat (utility bill), local bank account in the entity's name, REPEJU registration; foreign founders permitted.</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -2117,7 +2117,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>No dedicated charity registry or donor tax-benefit regime; notary and registry processes are slow; everything in Spanish. | correct prior: there IS a dedicated NGO registry (Ley 94-95, MRE) and a donor deduction via SAT tax-exempt status</t>
+          <t>No dedicated charity registry or donor tax-benefit regime; notary and registry processes are slow; everything in Spanish. | correct prior: there IS a dedicated NGO registry (Ley 94-95, MRE) and a donor deduction via SAT tax-exempt status | verify-r2 2026-10 (corrected): MINGOB's REPEJU checklist sets the NGO registration arancel at Q150 and requires a public deed, a utility bill proving the Guatemalan seat, and a bank account in the NGO's name;</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>~$100-200 (government); notary/attorney extra</t>
+          <t>~$20 (REPEJU arancel Q150); notary/attorney extra</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -2157,7 +2157,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>https://cof.org/country-notes/nonprofit-law-guatemala; https://www.asesoriaglobal.com.gt/blog/civil-association-foundation-ngo-guatemala.html; https://www.bizlatinhub.com/how-to-form-ngo-guatemala/; https://repeju.gob.gt/requisitos-y-documentos/ongs/</t>
+          <t>https://cof.org/country-notes/nonprofit-law-guatemala; https://www.asesoriaglobal.com.gt/blog/civil-association-foundation-ngo-guatemala.html; https://www.bizlatinhub.com/how-to-form-ngo-guatemala/; https://repeju.gob.gt/requisitos-y-documentos/ongs/; https://mingob.gob.gt/mingobsites/repeju/wp-content/uploads/sites/2/2024/05/Requisitos-de-inscripcion-de-Organizaciones-no-Gubernamentales-ONG.pdf; https://www.deloitte.com/content/dam/Deloitte/gt/Documents/tax/notas-fiscales/280220%20-Tax%20Alert%2003.pdf; https://www.icnl.org/wp-content/uploads/ListasVerificacion_Guatemala.pdf</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>NGO = company limited by guarantee (Companies Act No. 11 of 2022) with NGO status under NGO Act Cap. 315 RE 2020; domestic company at BCCAR.</t>
+          <t>NGO = company limited by guarantee (Belize Companies Act 2022) registered as an NGO under NGO Act Cap. 315 RE 2020 and as an NPO under the NPO Act No. 14 of 2023; both registers are kept by the FSC Registrar via BCCAR.</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -2204,12 +2204,12 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>BZ$100 (~USD 8) NGO application + incorporation ~BZ$250-400 (~USD 20-30); 1-4 weeks; a licensed local agent/registered office is required - agent fees add ~USD 750-1,500/year.</t>
+          <t>Company incorporation ~US$292 (BZ$584) at BCCAR; NGO registration (Cap. 315) via BCCAR OBRS has no fee; NPO registration BZ$100 (~USD 50); 1-4 weeks; a licensed local registered agent is required - agent fees add ~USD 750-1,500/year.</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>English-speaking, simple Companies Registry; most expats form the non-profit company first and add charity registration later; local service providers handle everything. | confirm prior; standard vehicle is company limited by guarantee (Companies Act Ch. 250); charity status is a later AG licensing step | Verified: NPO status must be separately registered with the Attorney General's Ministry after incorporation</t>
+          <t>English-speaking, simple Companies Registry; most expats form the non-profit company first and add charity registration later; local service providers handle everything. | confirm prior; standard vehicle is company limited by guarantee (Companies Act Ch. 250); NGO/NPO registration with the FSC Registrar is a later step | NPO status must be separately registered (FSC Registrar) after incorporation | verify-r2 2026-10 (corrected): The Belize FSC's 2024 NGO/NPO webinar states that the FSC Director General is Registrar of both NGOs (NGO Act Cap.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2219,12 +2219,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>Local registered office and company secretary via Belizean agent; NGO license (AG's Office) for foreign-funded work.</t>
+          <t>Licensed Belizean registered agent/registered office required (Companies Act 2022); NGO/NPO registration with the FSC Registrar via BCCAR (not the AG's Office), with ongoing AML-style NPO reporting.</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>200</t>
+          <t>~340 (incorporation ~US$292 + NPO BZ$100)</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -2239,7 +2239,7 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>NGOs receiving foreign contributions need an Attorney General NGO license (Non-Governmental Organizations Act)</t>
+          <t>NGOs receiving foreign contributions must be registered as an NGO with the FSC Registrar (NGO Act Cap. 315)</t>
         </is>
       </c>
       <c r="N19" s="2" t="inlineStr">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>https://beltraide.bz/belize-invest/doing-business-in-belize/company-incorporation/; https://bccar.bz/services/non-governmental-organisations/; https://www.facebook.com/BelizeCompaniesRegistry/posts/frequently-asked-questionswhat-type-of-legal-vehicle-should-a-not-for-profit-org/191133726554188/; https://www.belizefsc.org.bz/wp-content/uploads/2025/04/FSC_BCCAR-NPO-Webinar_23-04-2024.pdf</t>
+          <t>https://beltraide.bz/belize-invest/doing-business-in-belize/company-incorporation/; https://bccar.bz/services/non-governmental-organisations/; https://www.facebook.com/BelizeCompaniesRegistry/posts/frequently-asked-questionswhat-type-of-legal-vehicle-should-a-not-for-profit-org/191133726554188/; https://www.belizefsc.org.bz/wp-content/uploads/2025/04/FSC_BCCAR-NPO-Webinar_23-04-2024.pdf; https://www.belizefsc.org.bz/wp-content/uploads/2024/10/Webinar-Presentation-Mastering-NGOs-and-NPOs-Final.pdf; https://www.belizefsc.org.bz/wp-content/uploads/2023/05/Act-No-14-of-2023-Non-Profit-Organization.pdf; https://beltraide.bz/?p=5380</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -2281,7 +2281,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Asociación sin fines de lucro (Ley de ONG's No. 894 + Reglamento, Registro de Asociaciones y Fundaciones, Ministerio de Gobernación); fundación; tax benefits via the MEF.</t>
+          <t>Asociación or fundación sin fines de lucro (Ley de Asociaciones y Fundaciones sin Fines de Lucro, D.L. 894/1996 + Reglamento D.E. 78/1997), Registro de Asociaciones y Fundaciones, Ministerio de Gobernación y Desarrollo Territorial; tax benefits via the Ministerio de Hacienda.</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Spanish-language articles, local address, registry filing under the 2011 Associations and Foundations Law; foreign founders permitted.</t>
+          <t>Spanish-language articles, local address, registry filing under the 1996 Associations and Foundations Law (D.L. 894); foreign-funded entities must also register in the RAEX (2025 Foreign Agents Law); foreign founders permitted.</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2301,7 +2301,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Donor tax benefits are limited; NGOs receiving international funds should also register in the Ministry of Foreign Affairs NGO directory. | confirm prior; fundacion (Ley 2011) can be formed by one foreign founder via local counsel; donor donations are deductible, not 'limited'</t>
+          <t>Donor tax benefits are limited; NGOs receiving international funds should also register in the Ministry of Foreign Affairs NGO directory. | confirm prior; fundacion (D.L. 894/1996) can be formed by one foreign founder via local counsel; donor donations are deductible, not 'limited' | verify-r2 2026-10 (corrected): El Salvador's non-profit law is the Ley de Asociaciones y Fundaciones sin Fines de Lucro, Decreto Legislativo 894 of 21 Nov 1996 (regulated by D.E.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Spanish filings + local address; associations need resident members, foundations allow a single foreign founder via local POA.</t>
+          <t>Spanish filings + local address; foundations allow a single foreign founder via local POA; foreign-funded NPOs must register with RAEX and face a 30% levy on foreign funds (Ley de Agentes Extranjeros 2025) unless exempted.</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>http://www.oas.org/juridico/spanish/mesicic3_slv_funciones.pdf; https://www.taiia.gob.sv/wp-content/uploads/2020/11/LAS-ORGANIZACIONES-SIN-FINES-DE-LUCRO-SU-TRATAMIENTO-TRIBUTARIO.pdf; https://consortiumlegal.com/wp-content/uploads/Tratamiento-fiscal-de-las-donaciones-en-Centroamerica.pdf; https://www.gobernacion.gob.sv/preguntas-frecuentes/</t>
+          <t>http://www.oas.org/juridico/spanish/mesicic3_slv_funciones.pdf; https://www.taiia.gob.sv/wp-content/uploads/2020/11/LAS-ORGANIZACIONES-SIN-FINES-DE-LUCRO-SU-TRATAMIENTO-TRIBUTARIO.pdf; https://consortiumlegal.com/wp-content/uploads/Tratamiento-fiscal-de-las-donaciones-en-Centroamerica.pdf; https://www.gobernacion.gob.sv/preguntas-frecuentes/; https://www.icnl.org/research/library/el-salvador_found/; https://diario.elmundo.sv/politica/asamblea-aprueba-ley-de-agentes-extranjeros-que-crea-un-registro-de-ong-y-un-impuesto-del-30; https://lexlatin.com/opinion/ley-agentes-extranjeros-el-salvador-efectos-un-ano-vigencia</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>International ONGDs must register in the Registro Público de ONGD; moderate bureaucracy; all filings in Spanish. | verify-rest 2026-10: granting body is SGJD/DIRRSAC (not the Judiciary/Chancillería) | verify-followup 2026-10 (confirmed): Government acuerdos published in La Gaceta (incl.</t>
+          <t>International ONGDs must register in the Registro Público de ONGD; moderate bureaucracy; all filings in Spanish. | verify-rest 2026-10: granting body is SGJD/DIRRSAC (not the Judiciary/Chancillería) | verify-followup 2026-10 (confirmed): Government acuerdos published in La Gaceta (incl. | verify-r2 2026-10 (confirmed): A January 2023 acuerdo in La Gaceta confirms the Secretaría de Gobernación, Justicia y Descentralización grants, registers and supervises legal personality of civil associations through DIRRSAC, citing the ONGD law (Decreto 32-2011).</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2433,7 +2433,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>https://www.sgjd.gob.hn/institucion/dependencias/subsecretaria-de-justicia/direccion-de-regulacion-registro-y-seguimiento-de-asociaciones-civiles-dirrsac; https://diref.gob.hn/; https://consortiumlegal.com/2022/09/21/que-se-debe-tener-en-consideracion-si-desea-constituir-o-incorporar-una-ongd-en-honduras/; https://sgjd.gob.hn/servicios-y-gestiones-web/requisitos/servicios-de-atencion-al-ciudadano/personalidad-juridica/fundaciones; https://portalunico.iaip.gob.hn/ver_archivo/MTY2MTM1NA==; https://www.leybook.com/doc/29461/pdf</t>
+          <t>https://www.sgjd.gob.hn/institucion/dependencias/subsecretaria-de-justicia/direccion-de-regulacion-registro-y-seguimiento-de-asociaciones-civiles-dirrsac; https://diref.gob.hn/; https://consortiumlegal.com/2022/09/21/que-se-debe-tener-en-consideracion-si-desea-constituir-o-incorporar-una-ongd-en-honduras/; https://sgjd.gob.hn/servicios-y-gestiones-web/requisitos/servicios-de-atencion-al-ciudadano/personalidad-juridica/fundaciones; https://portalunico.iaip.gob.hn/ver_archivo/MTY2MTM1NA==; https://www.leybook.com/doc/29461/pdf; https://www.icnl.org/research/library/honduras_national/; https://www.icnl.org/wp-content/uploads/Honduras_leyong.pdf</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2567,7 +2567,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Notarized Spanish articles, local registered office, Registro de Personas Jurídicas; 3+ members for an asociación; a fundación's Junta Administrativa must include one member appointed by the Executive and one by the cantonal municipality.</t>
+          <t>Notarized Spanish articles, local registered office, Registro de Personas Jurídicas; 10+ founders for an asociación (Ley 218 art. 18) with a 5+ member board (art. 10); a fundación's Junta Administrativa must include one member appointed by the Executive and one by the cantonal municipality.</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Stable, professional services widely available in English; donor tax exemption requires separate Ministry of Finance (MINFIN) approval. | correct prior: asociacion requires 5+ founders (Ley 218), not 3+; donor deduction needs the interes publico decree, MINFIN covers entity exemption | verify-rest 2026-10: foundations governed by Ley 5338; registry is the Registro de Personas Jurídicas (not commercial registry/Education Ministry)</t>
+          <t>Stable, professional services widely available in English; donor tax exemption requires separate Ministry of Finance (MINFIN) approval. | correct prior: asociacion requires 10+ founders (Ley 218 art. 18) and a 5+ member board; donor deduction needs the interes publico decree, MINFIN covers entity exemption | verify-rest 2026-10: foundations governed by Ley 5338; registry is the Registro de Personas Jurídicas (not commercial registry/Education Ministry) | verify-r2 2026-10 (corrected): Ley de Asociaciones No.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Public deed before a CR notary + local office; asociaciones need 5+ members, so a fundacion (single founder) is the practical path.</t>
+          <t>Public deed before a CR notary + local office; asociaciones need 10+ founders, so a fundacion (single founder) is the practical path.</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Most expat-friendly in the region; foreigners can be president/directors; Bogotá has strong English-speaking legal market; donation tax deductions require separate DIAN certification; 2023 NGO-law reforms (Ley 2287/2022) added transparency reporting for foreign-funded entities. | Prior context confirmed; deduction is a separate DIAN certification step, not automatic; Ley 2287/2022 adds transparency duties | Verified: Constitution deed must be signed before a Colombian notary; remote founders need an apostilled poder especial | verify-rest 2026-10: Civil Code articles corrected to 633-652; private document suffices for ESAL constitution | verify-followup 2026-10 (corrected): Código Civil Libro I Título XXXVI 'De las personas jurídicas' runs from art.</t>
+          <t>Most expat-friendly in the region; foreigners can be president/directors; Bogotá has strong English-speaking legal market; donation tax deductions require separate DIAN certification; 2023 NGO-law reforms (Ley 2287/2022) added transparency reporting for foreign-funded entities. | Prior context confirmed; deduction is a separate DIAN certification step, not automatic; Ley 2287/2022 adds transparency duties | Verified: Constitution deed must be signed before a Colombian notary; remote founders need an apostilled poder especial | verify-rest 2026-10: Civil Code articles corrected to 633-652; private document suffices for ESAL constitution | verify-followup 2026-10 (corrected): Código Civil Libro I Título XXXVI 'De las personas jurídicas' runs from art. | verify-r2 2026-10 (confirmed): Chambers of Commerce still administer the Registro de Entidades sin Ánimo de Lucro under Decreto 2150/1995 and Decreto 427/1996, with 2026 registry fees set in UVB (COP 12,110 per UVB) by the same tariff table as the Registro Mercantil.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2801,7 +2801,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>https://www.ccb.org.co; https://neo-project.github.io/global-blockchain-compliance-hub/colombia/colombia-registry-requirements.html; https://www.whydonate.com; https://www.minjusticia.gov.co/programas-co/LegalApp/Paginas/Que-debo-hacer-para-constituir-una-fundacion.aspx; https://www.ccb.org.co/processes-and-consultations/about-registrations/registration-non-profit-entities/non-profit-entities-common-regime; https://www.ccb.org.co/servicios/registros-publicos/registro-de-entidades-sin-animo-de-lucro; https://encolombia.com/derecho/codigos/civil-colombiano/codcivillibro1-t36/; https://normas.cra.gov.co/Gestor/Docs/decreto_0427_1996.htm</t>
+          <t>https://www.ccb.org.co; https://neo-project.github.io/global-blockchain-compliance-hub/colombia/colombia-registry-requirements.html; https://www.whydonate.com; https://www.minjusticia.gov.co/programas-co/LegalApp/Paginas/Que-debo-hacer-para-constituir-una-fundacion.aspx; https://www.ccb.org.co/processes-and-consultations/about-registrations/registration-non-profit-entities/non-profit-entities-common-regime; https://www.ccb.org.co/servicios/registros-publicos/registro-de-entidades-sin-animo-de-lucro; https://encolombia.com/derecho/codigos/civil-colombiano/codcivillibro1-t36/; https://normas.cra.gov.co/Gestor/Docs/decreto_0427_1996.htm; https://cccartagena.org.co/sites/default/files/media/tarifas/1231-Cf-Memorando-Interno-Tablas-de-Tarifas-Registros-Publicos-2026.pdf</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Fundación (1+ founders) or corporación (5+ members) under Decreto Ejecutivo 193/2017 (Reglamento para el Otorgamiento de Personalidad Jurídica a las Organizaciones Sociales), registered in SUIOS via the competent ministry</t>
+          <t>Fundación or corporación under the Ley Orgánica de Transparencia Social (R.O. 3S-112, 28 Aug 2025) and its Reglamento General (Decreto Ejecutivo 191, Oct 2025, which repealed Decreto 193/2017); legal personality via the competent ministry and registration in the unified OSSFL information system</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Foreign founders permitted as members/board; Spanish-language documents; IUP status adds time and a public-benefit declaration; banking and tax (SRI) onboarding is slow. | Prior context confirmed; 2025 Social Transparency Organic Law adds registration + foreign-funding controls (30% tax, suspension) | verify-rest 2026-10: Decreto 193/2017 governs; unverifiable 'Ley 2023-13/COEP' removed; ministerial grant carries no government fee</t>
+          <t>Foreign founders permitted as members/board; Spanish-language documents; IUP status adds time and a public-benefit declaration; banking and tax (SRI) onboarding is slow. | Prior context confirmed; 2025 Social Transparency Organic Law adds registration + foreign-funding controls (30% tax, suspension) | verify-rest 2026-10: Decreto 193/2017 then governed (repealed by Decreto 191/2025); unverifiable 'Ley 2023-13/COEP' removed; ministerial grant carries no government fee | verify-r2 2026-10 (corrected): Decreto Ejecutivo 191 (Registro Oficial Supl.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>https://www.upi.com/Top_News/World-News/2025-08-01/ecuador-NGO-funding-bill-legislature/1921754058618/; https://www.icnl.org/post/analysis/five-things-to-know-ecuadors-2025-organic-law-on-social-transparency; https://www.gob.ec/sites/default/files/regulations/2018-10/Documento_Reglamento-Otorgamiento-Personalidad-Jur%C3%ADdica-Organizaciones-Sociales.pdf; https://www.gob.ec/regulaciones/193-expidese-reglamento-otorgamiento-personalidad-juridica-organizaciones-sociales</t>
+          <t>https://www.upi.com/Top_News/World-News/2025-08-01/ecuador-NGO-funding-bill-legislature/1921754058618/; https://www.icnl.org/post/analysis/five-things-to-know-ecuadors-2025-organic-law-on-social-transparency; https://www.gob.ec/sites/default/files/regulations/2018-10/Documento_Reglamento-Otorgamiento-Personalidad-Jur%C3%ADdica-Organizaciones-Sociales.pdf; https://www.gob.ec/regulaciones/193-expidese-reglamento-otorgamiento-personalidad-juridica-organizaciones-sociales; https://www.primicias.ec/politica/noboa-decreto191-reglamento-ley-transparencia-social-fundaciones-108206/; https://www.gob.ec/regulaciones/reglamento-general-ley-organica-transparencia-social</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -3037,7 +3037,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>No nationality requirement; foreign founders allowed; tax exemption (exoneración) from SUNAT is separate, discretionary and needs annual reporting; Lima is the practical hub; English not official. | Prior context confirmed; deduction cap is 10% of net taxable income (PwC); SUNAT tax exemption is separate and discretionary | verify-rest 2026-10: Civil Code article numbers corrected; SUNARP fee is modest — the larger figure is notary/lawyer cost | verify-followup 2026-10 (confirmed): The Código Civil (Libro I, Sección Segunda) places Asociación in Título II (arts.</t>
+          <t>No nationality requirement; foreign founders allowed; tax exemption (exoneración) from SUNAT is separate, discretionary and needs annual reporting; Lima is the practical hub; English not official. | Prior context confirmed; deduction cap is 10% of net taxable income (PwC); SUNAT tax exemption is separate and discretionary | verify-rest 2026-10: Civil Code article numbers corrected; SUNARP fee is modest — the larger figure is notary/lawyer cost | verify-followup 2026-10 (confirmed): The Código Civil (Libro I, Sección Segunda) places Asociación in Título II (arts. | verify-r2 2026-10 (confirmed): The Peruvian Civil Code (arts.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Foreign NGOs must register with the Ministry of Foreign Affairs (Cancillería); 2023 law caps foreign government funding for certain activities and tightens oversight; heavy Spanish-language bureaucracy; few English speakers. | verify-rest 2026-10: registering authority corrected (not a 'Superintendencia de Compañías'); unverifiable 'Ley 1417/1475' references removed</t>
+          <t>Foreign NGOs must register with the Ministry of Foreign Affairs (Cancillería); 2023 law caps foreign government funding for certain activities and tightens oversight; heavy Spanish-language bureaucracy; few English speakers. | verify-rest 2026-10: registering authority corrected (not a 'Superintendencia de Compañías'); unverifiable 'Ley 1417/1475' references removed | verify-r2 2026-10 (confirmed): Ley 351/2013 and DS 1597/2013 remain the framework for NGOs, foundations and civil non-profits operating in more than one department, processed by the Viceministerio de Autonomías under the Ministerio de la Presidencia, while single-depart…</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -3169,7 +3169,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>https://www.bizlatinhub.com/how-to-form-ngo-bolivia/; https://www.rigobertoparedes.com/en/legal-requirements-to-establish-an-ngo-in-bolivia/; https://www.lexivox.org/norms/BO-L-N351.html; https://va.presidencia.gob.bo/images/personalidadesJuridicas/Normativa/1-ley-351_de_otorgacion_de_personalidades_jurdicas.pdf</t>
+          <t>https://www.bizlatinhub.com/how-to-form-ngo-bolivia/; https://www.rigobertoparedes.com/en/legal-requirements-to-establish-an-ngo-in-bolivia/; https://www.lexivox.org/norms/BO-L-N351.html; https://va.presidencia.gob.bo/images/personalidadesJuridicas/Normativa/1-ley-351_de_otorgacion_de_personalidades_jurdicas.pdf; https://va.presidencia.gob.bo/images/personalidadesJuridicas/Normativa/2-ds_1597_reglamentacion_parcial_a_la_ley_351.pdf; https://bolivia.infoleyes.com/norma/4373/ley-de-otorgaci%C3%B3n-de-personalidades-jur%C3%ADdicas-351</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -3293,7 +3293,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Stichting (privaat nut) — Dutch-style foundation by notarial deed under the Stichtingenwet of 19 July 1968; also vereniging (association) and coöperatie.</t>
+          <t>Stichting — foundation under Book 2 of the new Burgerlijk Wetboek (S.B. 2024 no. 164, in force 1 May 2025, replacing the Stichtingenwet 1968); also vereniging (association) and coöperatie.</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -3303,17 +3303,17 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Surinamese notary (deeds in Dutch), local board/office in practice; 2013 Dutch-style Civil Code permits stichting with foreign elements but a local notary and presence are required in practice; Dutch language barrier.</t>
+          <t>Surinamese notary (deeds in Dutch), local board/office in practice; new Civil Code Book 2 (in force 1 May 2025) also allows a government model deed with KKF-legalized signatures, though none issued yet; Dutch language barrier.</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Official fees unpublished (as of 2026); register fees set by staatsbesluit (Besluit Stichtingenregister G.B. 1970 no. 126, as amended). KKF excerpt SRD 300. Notary ~US$200–500, total ~US$500–1,500; 1–3 months (unofficial estimates).</t>
+          <t>Official fees unpublished (as of 2026); registration in the KKF Handelsregister (new Handelsregisterwet in force 1 May 2025). KKF excerpt SRD 300. Notary ~US$200–500, total ~US$500–1,500; 1–3 months (unofficial estimates).</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Dutch is the working language — the main barrier; small legal market; banking requires a local presence; few English-speaking professionals; new Civil Code (in force 2013) modernized foundation law but practice is conservative. | Prior context confirmed; 2013 Civil Code modernized foundation law; notary deed + local presence required in practice | [verified] Stichtingenwet 1968 has no nationality/residence requirement for founder or board, and the seat is the place designated in the articles; but creation requires a notarial deed by a Surinamese notary, so a remote founder needs a notarized power of attorney; banking and practice favor local presence.</t>
+          <t>Dutch is the working language — the main barrier; small legal market; banking requires a local presence; few English-speaking professionals; new Civil Code Book 2 (in force 1 May 2025) modernized foundation law but practice is conservative. | Prior context confirmed; 2013 Civil Code modernized foundation law; notary deed + local presence required in practice | [verified, pre-2025 law] Stichtingenwet 1968 had no nationality/residence requirement for founder or board, and the seat is the place designated in the articles; but creation requires a notarial deed by a Surinamese notary, so a remote founder needs a notarized power of attorney; banking and practice favor local presence. | verify-r2 2026-10 (corrected): Suriname's new Burgerlijk Wetboek (S.B.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3353,7 +3353,7 @@
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>https://www.offshorecompany.com/company/suriname-private-foundation-spf/; https://www.icnl.org/wp-content/uploads/Suriname_suriname-Muskiet_T.pdf; https://www.doingbusinessdutchcaribbean.com/suriname/structures-for-doing-business-sur/the-foundation-sur/; https://www.notariaatmannes.sr/ondernemen-stichtingen-verenigingen/stichting/; https://www.dna.sr/media/twjew2do/wet_op_stichtingen.pdf</t>
+          <t>https://www.offshorecompany.com/company/suriname-private-foundation-spf/; https://www.icnl.org/wp-content/uploads/Suriname_suriname-Muskiet_T.pdf; https://www.doingbusinessdutchcaribbean.com/suriname/structures-for-doing-business-sur/the-foundation-sur/; https://www.notariaatmannes.sr/ondernemen-stichtingen-verenigingen/stichting/; https://www.dna.sr/media/twjew2do/wet_op_stichtingen.pdf; https://www.curacao-law.com/wp-content/uploads/2026/07/Frielink-Nieuw-Boek-2-BW-Suriname-MvO-april-2026.pdf; https://www.dna.sr/media/avzdei43/s-b-_2024_no-_164__boek_2.pdf; https://sris.sr/wp-content/uploads/2025/01/S.B.-2024-no.-165-Overgangswet-aanpassingswetgeving-nieuw-Burgerlijk-Wetboek.pdf</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Minimum 2 members (association) or 1 founder (foundation); Brazilian CNPJ and local address; notarial deed registered with a cartório; foreign founder may join the board; filings in Portuguese.</t>
+          <t>Association: founding minutes + lawyer-signed statutes registered at the RCPJ cartório (no notarial deed needed); foundation: escritura pública or will (CC art. 62) + Ministério Público statute approval; CNPJ and local address; foreign founder may join the board; Portuguese filings.</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3405,7 +3405,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Heavy red tape (famous bureaucracy); main hurdles are getting a CPF and a bank account (foreign-inflow/câmbio rules); OSCIP certification gives donation tax deductions; 'instituição de utilidade pública' (federal/municipal) is a long, discretionary extra step. | Prior context confirmed; deduction is 6% individual / 2% corporate; OSCIP certification required for donor deductions</t>
+          <t>Heavy red tape (famous bureaucracy); main hurdles are getting a CPF and a bank account (foreign-inflow/câmbio rules); OSCIP certification gives donation tax deductions; 'instituição de utilidade pública' (federal/municipal) is a long, discretionary extra step. | Prior context confirmed; deduction is 6% individual / 2% corporate; OSCIP certification required for donor deductions | verify-r2 2026-10 (corrected): Under Código Civil art.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>https://brazilfoundation.org/en/get-involved/foundations-and-companies/; https://www.gbflaw.com.br/imposto-de-renda-2025-pague-menos-imposto-fazendo-doacoes/; https://taxsummaries.pwc.com/brazil/corporate/deductions; https://www.planalto.gov.br/ccivil_03/leis/l9790.htm</t>
+          <t>https://brazilfoundation.org/en/get-involved/foundations-and-companies/; https://www.gbflaw.com.br/imposto-de-renda-2025-pague-menos-imposto-fazendo-doacoes/; https://taxsummaries.pwc.com/brazil/corporate/deductions; https://www.planalto.gov.br/ccivil_03/leis/l9790.htm; https://www.ufmg.br/proex/cpinfo/saberesplurais/wp-content/uploads/2015/09/9-Documentação-Necessária-Registro-Associação-Estatuto.pdf; https://modeloinicial.com.br/lei/CC/fundacoes-@_GERAL_I_II_III</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Under-regulated and relatively tolerant of foreign founders, but the legal market is small and Spanish-only; tax exemption requires separate certification; fewer English-speaking lawyers than neighboring countries; slower administration than Chile/Argentina. | Confirm prior; foundation route needs US$400 min. capital in a capital-integration account; NGO route via Min. Interior fee. | verify-rest 2026-10: unverifiable 'Ley 5833/2017' removed; Ley 7363/2024 control/transparency regime added</t>
+          <t>Under-regulated and relatively tolerant of foreign founders, but the legal market is small and Spanish-only; tax exemption requires separate certification; fewer English-speaking lawyers than neighboring countries; slower administration than Chile/Argentina. | Confirm prior; foundation route needs US$400 min. capital in a capital-integration account; NGO route via Min. Interior fee. | verify-rest 2026-10: unverifiable 'Ley 5833/2017' removed; Ley 7363/2024 control/transparency regime added | verify-r2 2026-10 (confirmed): Decreto 4806/2025 (23 Oct 2025) regulates Ley 7363/2024 on control, transparency and accountability of non-profits, with the MEF running the mandatory registry (SIARA) and semi-annual reporting.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -3537,7 +3537,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>https://www.latribuna.com.py/destacado/200761-costo-de-crear-una-ong-en-paraguay-requisitos-y-financiamiento/; https://www.dnit.gov.py/documents/20123/218007/IRP-RSP-Tratamiento+Impositivo+donaciones_Abril.2021.pdf; https://informacionpublica.paraguay.gov.py/public/651218-requisitosIPDF-requisitosI.PDF; https://www.mef.gov.py/es/dependencias/direcciones/direccion-general-personas-estructuras-juridicas-beneficiarios-finales/pf; https://www.lanacion.com.py/politica/2024/11/15/pena-promulgo-ley-de-control-y-transparencia-de-ong/</t>
+          <t>https://www.latribuna.com.py/destacado/200761-costo-de-crear-una-ong-en-paraguay-requisitos-y-financiamiento/; https://www.dnit.gov.py/documents/20123/218007/IRP-RSP-Tratamiento+Impositivo+donaciones_Abril.2021.pdf; https://informacionpublica.paraguay.gov.py/public/651218-requisitosIPDF-requisitosI.PDF; https://www.mef.gov.py/es/dependencias/direcciones/direccion-general-personas-estructuras-juridicas-beneficiarios-finales/pf; https://www.lanacion.com.py/politica/2024/11/15/pena-promulgo-ley-de-control-y-transparencia-de-ong/; https://impuestospy.com/impuestos/decreto-n-4806-2025/; https://eusee.hivos.org/?p=3518; https://www.icnl.org/post/news/paraguay-non-profit-checklist</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -3589,7 +3589,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Very stable, low political risk; foundations enjoy tax incentives (50% exemption on qualifying income); English reasonably available in Montevideo business circles; 'declaración de utilidad pública' optional. | Confirm prior (association from 3 members; foundation needs local rep; foundations enjoy tax incentives). | verify-rest 2026-10: recognition is by the MEC (not the DGR); Ley 17.163 also governs foundations</t>
+          <t>Very stable, low political risk; foundations enjoy tax incentives (50% exemption on qualifying income); English reasonably available in Montevideo business circles; 'declaración de utilidad pública' optional. | Confirm prior (association from 3 members; foundation needs local rep; foundations enjoy tax incentives). | verify-rest 2026-10: recognition is by the MEC (not the DGR); Ley 17.163 also governs foundations | verify-r2 2026-10 (corrected): The official gub.uy procedure page shows MEC recognition of asociaciones civiles and fundaciones carries a tasa de inscripción of UYU 2,530 (about US$63), above the US$10-30 previously stated.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>low (~US$10-30, MEC recognition + registry)</t>
+          <t>low (~US$65: MEC inscription fee UYU 2,530, subject to update; plus DGR registry fee)</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Private foundation (хувийн сан); Association (нийгмийн эвлэл); NGO under the Law on Associations (1997) + Civil Code (2002)</t>
+          <t>Private foundation (хувийн сан); Association (нийгмийн эвлэл); NGO under the Law on Non-Governmental Organizations (1997, foundations chapter 2002) + Civil Code (2002)</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -3855,7 +3855,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>As a Mongolian citizen you register with the Legal Entity Registration Office (LERO, Justice ministry) with a Mongolian-language notarized charter, a local registered address, and a governing board (minimum 5 members for non-membership NGOs); a foundation requires an endowment adequate to its stated purpose.</t>
+          <t>As a Mongolian citizen (or legally resident foreigner) you register with the General Authority for State Registration with a Mongolian-language notarized charter, a local registered address, and a governing board (minimum 5 members for non-membership NGOs); a foundation requires an endowment adequate to its stated purpose; foreign NGO branches register with the Immigration Agency.</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -3865,7 +3865,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Scored on the local-citizen route, which is straightforward — no foreign-founder bar. The pure foreign-founder route is much harder: a foreigner must usually form a foreign-invested legal entity (LLC, ~$100,000 minimum investment per investor) and rely on a local agent, with in-person Mongolian-language steps and limited English support. | confirm prior: local-citizen route straightforward; pure foreign route requires FIE (~$100k) or rep office; no new NGO-law bar</t>
+          <t>Scored on the local-citizen route, which is straightforward — no foreign-founder bar. The pure foreign-founder route is much harder: a foreigner must usually form a foreign-invested legal entity (LLC, ~$100,000 minimum investment per investor) and rely on a local agent, with in-person Mongolian-language steps and limited English support. | confirm prior: local-citizen route straightforward; pure foreign route requires FIE (~$100k) or rep office; no new NGO-law bar | verify-r2 2026-10 (corrected): ICNL's Civic Freedom Monitor (updated 15 May 2026) shows the governing statute is the 1997 Law on Non-Governmental Organizations, not a 'Law on Associations';</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -3905,12 +3905,12 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>https://www.icnl.org/resources/civic-freedom-monitor/mongolia; https://taxsummaries.pwc.com/mongolia/corporate/deductions; https://immigration.gov.mn/en/non-government/</t>
+          <t>https://www.icnl.org/resources/civic-freedom-monitor/mongolia; https://taxsummaries.pwc.com/mongolia/corporate/deductions; https://immigration.gov.mn/en/non-government/; https://www.icnl.org/research/library/mongolia_ngo/</t>
         </is>
       </c>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>NGOs under the Law on Associations (1997) file annual reports with financial statements to the Civil Affairs Department; non-reporting can lead to suspension. Private foundations and associations register with civil affairs.</t>
+          <t>NGOs under the Law on Non-Governmental Organizations (1997) file annual reports with financial statements to the Civil Affairs Department; non-reporting can lead to suspension. Private foundations and associations register with civil affairs.</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
@@ -4233,7 +4233,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>The 財團法人 (foundation) is the standard expat charitable vehicle; formation guides confirm foreign founders are accepted and foreign staff may be hired; Chinese-language bureaucracy, no direct foreign-ownership ban. | confirm prior: foreign founders accepted; NT$15m (local) / NT$30m (central) minimum capital; 4-12 weeks with legal help | verify-rest 2026-10: endowment minimum varies by competent authority (no uniform NT$15M/30M tiers); court registration follows permission</t>
+          <t>The 財團法人 (foundation) is the standard expat charitable vehicle; formation guides confirm foreign founders are accepted and foreign staff may be hired; Chinese-language bureaucracy, no direct foreign-ownership ban. | confirm prior: foreign founders accepted; minimum endowment set per competent authority (e.g. Taipei social-welfare foundations NT$10m cash); 4-12 weeks with legal help | verify-rest 2026-10: endowment minimum varies by competent authority (no uniform NT$15M/30M tiers); court registration follows permission | verify-r2 2026-10 (corrected): Taipei City rules set a NT$10 million cash minimum for social welfare foundations, and MOFA guidance shows thresholds vary by competent authority (e.g.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Local office, deposited capital (NT$15m local / NT$30m central), Chinese-language docs and local counsel</t>
+          <t>Local office, endowment set by each competent authority (e.g. Taipei NT$10m cash), Chinese-language docs, court registration and local counsel</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>https://btlaw.com.tw/h/newsinfo?key=2719736319&amp;cont=414464; https://startabusinessintaiwan.tw/book/faqs/setting-up-a-business/is-there-a-minimum-capital-requirement-for-setting-up-a-business-in-taiwan/; https://laws.gov.taipei/Law/LawSearch/LawArticleContent/FL043047</t>
+          <t>https://btlaw.com.tw/h/newsinfo?key=2719736319&amp;cont=414464; https://startabusinessintaiwan.tw/book/faqs/setting-up-a-business/is-there-a-minimum-capital-requirement-for-setting-up-a-business-in-taiwan/; https://laws.gov.taipei/Law/LawSearch/LawArticleContent/FL043047; https://taiwanngo.tw/Post/79997</t>
         </is>
       </c>
       <c r="P41" s="2" t="inlineStr">
@@ -4417,7 +4417,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Formation under Law 2/99/M and the Civil Code (arts. 140-172) via DSI registration; a new associations law was in public consultation in 2026; documents in Chinese or Portuguese — English support is limited. | verify-rest 2026-10: Civil Code articles and procedure corrected — registration runs through the DSI</t>
+          <t>Formation under Law 2/99/M and the Civil Code (arts. 140-172) via DSI registration; a new associations law was in public consultation in 2026; documents in Chinese or Portuguese — English support is limited. | verify-rest 2026-10: Civil Code articles and procedure corrected — registration runs through the DSI | verify-r2 2026-10 (confirmed): The Macau government portal confirms the procedure: DSI name-availability certificate, notarised constitution at a public notary, publication in the Boletim Oficial, then DSI registration number issued.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -4457,7 +4457,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.mo/en/services/ps-1069/; https://www.bo.dsaj.gov.mo/cn/entities/assoc</t>
+          <t>https://www.gov.mo/en/services/ps-1069/; https://www.bo.dsaj.gov.mo/cn/entities/assoc; https://macaubusiness.com/winding-down-dormant-associations-helps-clean-up-macaus-image-sonia-chan/</t>
         </is>
       </c>
       <c r="P43" s="2" t="inlineStr">
@@ -4785,7 +4785,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Most foreigners establish a foundation with all-Thai board and act as funder/advisor; high political sensitivity (NGO rules, lèse-majesté) — avoid politically active purposes. | Confirm foundation min assets THB 500k (250k cash); official fee only ~THB 210 — prior THB 30k–100k figure is counsel cost | verify-rest 2026-10: no 'Foundation Act B.E. 2550' — CCC governs; registrar is the Ministry of Interior, not Justice</t>
+          <t>Most foreigners establish a foundation with all-Thai board and act as funder/advisor; high political sensitivity (NGO rules, lèse-majesté) — avoid politically active purposes. | Confirm foundation min assets THB 500k (250k cash); official fee only ~THB 210 — prior THB 30k–100k figure is counsel cost | verify-rest 2026-10: no 'Foundation Act B.E. 2550' — CCC governs; registrar is the Ministry of Interior, not Justice | verify-r2 2026-10 (confirmed): Law-firm sources confirm foundations are registered under the Civil and Commercial Code with the Ministry of Interior registrar (district office in Bangkok, Provincial Governor elsewhere), with THB 500,000 assets (or 250,000 for public-cha…</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -5133,7 +5133,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Association under Decree on Associations No. 238/GOV (2017); foundation under the foundations decree; INGO under Decree No. 126/GOV of 25 May 2026 (in force 15 Jul 2026, replacing PM Decree 013/2010)</t>
+          <t>Association under Decree on Associations No. 536 (2025, replacing Decree 238/GOV of 2017); foundation under the foundations decree; INGO under Decree No. 126/GOV of 25 May 2026 (in force 15 Jul 2026, replacing PM Decree 013/2010)</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
@@ -5153,7 +5153,7 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Heavily state-controlled civil society; Lao language required; INGOs operate only through approved local partners and MFA authorisation. | Confirm state-controlled model; 2023 decree on associations: resident foreigners may join as members, chair must be Lao national | verify-rest 2026-10: no 'Law on Social Organisations and NGOs' — Decree 238/2017 governs associations; new INGO Decree 126/GOV (2026) requires prior MOFA approval for cooperation</t>
+          <t>Heavily state-controlled civil society; Lao language required; INGOs operate only through approved local partners and MFA authorisation. | Confirm state-controlled model; 2023 decree on associations: resident foreigners may join as members, chair must be Lao national | verify-rest 2026-10: no 'Law on Social Organisations and NGOs' — Decree 238/2017 then governed associations (since replaced by Decree 536/2025); new INGO Decree 126/GOV (2026) requires prior MOFA approval for cooperation | verify-r2 2026-10 (corrected): CIVICUS Monitor (June 2026), citing the UN Special Rapporteur's February 2026 report, states that Decree No.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -5193,7 +5193,7 @@
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
-          <t>https://ilawasia.com/blogs/setting-up-ngo-in-lao-pdr; https://www.icj.org/resource/lao-pdr-the-icj-criticizes-new-decree-on-associations/; https://www.wto.org/english/thewto_e/acc_e/lao_e/wtacclao38_leg_1.pdf; https://www.rajahtannasia.com/viewpoints/ingos-regulations-amended/</t>
+          <t>https://ilawasia.com/blogs/setting-up-ngo-in-lao-pdr; https://www.icj.org/resource/lao-pdr-the-icj-criticizes-new-decree-on-associations/; https://www.wto.org/english/thewto_e/acc_e/lao_e/wtacclao38_leg_1.pdf; https://www.rajahtannasia.com/viewpoints/ingos-regulations-amended/; https://monitor.civicus.org/explore/laos-dissident-found-dead-as-un-expert-highlights-strict-restriction-on-freedoms-and-reprisals-against-activists/; https://vdb-loi.com/laos_publication/laos-updates-ingo-regulatory-framework/</t>
         </is>
       </c>
       <c r="P51" s="2" t="inlineStr">
@@ -5245,7 +5245,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>High political risk (civil war, sanctions, unstable NCA); most foreign charities operate via international partners or pre-2021 registered bodies only. | 2022 Organization Registration Law (Notification 46/2022) repeals the 2014 ARL cited in context; foreign founder route is effectively closed, INGO route only. | verify-rest 2026-10: registration body is the Union Registration Board under the 2022 law (no 'National Registration Bureau')</t>
+          <t>High political risk (civil war, sanctions, unstable NCA); most foreign charities operate via international partners or pre-2021 registered bodies only. | 2022 Organization Registration Law (Notification 46/2022) repeals the 2014 ARL cited in context; foreign founder route is effectively closed, INGO route only. | verify-rest 2026-10: registration body is the Union Registration Board under the 2022 law (no 'National Registration Bureau') | verify-r2 2026-10 (confirmed): DFDL and Allen &amp; Gledhill confirm the SAC's Organization Registration Law (Notification 46/2022, 28 Oct 2022) repealed the 2014 Association Registration Law, with MOHA issuing certificates after review by the Union/Region/State Registratio…</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
-          <t>https://www.icj.org/wp-content/uploads/2022/11/Myanmar-ORL-final.pdf; https://asiacentre.org/the-law-on-organisation-registration/; https://www.dfdl.com/insights/legal-and-tax-updates/myanmar-new-organization-registration-law-enacted/</t>
+          <t>https://www.icj.org/wp-content/uploads/2022/11/Myanmar-ORL-final.pdf; https://asiacentre.org/the-law-on-organisation-registration/; https://www.dfdl.com/insights/legal-and-tax-updates/myanmar-new-organization-registration-law-enacted/; https://www.allenandgledhill.com/perspectives/articles/22817/mmkh-new-myanmar-registration-of-associations-law-imposes-additional-requirements-on-non-governmental-organisations</t>
         </is>
       </c>
       <c r="P52" s="2" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Very small, closed registration culture aimed at locals; English is official so language is fine, but foreign-led charities are rare — most operate through existing local bodies. | confirm prior (very hard, local majority/resident officers, in-person); society is deemed established only if an office-bearer/member resides in Brunei (s.6(1) 2005 gazette).</t>
+          <t>Very small, closed registration culture aimed at locals; English is official so language is fine, but foreign-led charities are rare — most operate through existing local bodies. | confirm prior (very hard, local majority/resident officers, in-person); society is deemed established only if an office-bearer/member resides in Brunei (s.6(1) 2005 gazette). | verify-r2 2026-10 (confirmed): The Royal Brunei Police Force site confirms societies register under the Societies Act (Chapter 203) with the Registrar of Societies, a unit of the police Criminal Intelligence Department at Police HQ Gadong, contactable in person or by em…</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -5429,7 +5429,7 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Foreign members are permitted under the 2009 law and INGOs do register here; bureaucracy is slow and requires a local agent; less predictable than Singapore/Malaysia. | governing instrument is Decree-Law No. 5/2005 (non-profit corporate bodies), not a 2009 Law on Associations; foreign corporate bodies may register if they prove legal existence and have a permanent local representative. | verify-rest 2026-10: registration handled by the National Directorate for Registration and Notarial Services (DNRN), Ministry of Justice</t>
+          <t>Foreign members are permitted under the 2009 law and INGOs do register here; bureaucracy is slow and requires a local agent; less predictable than Singapore/Malaysia. | governing instrument is Decree-Law No. 5/2005 (non-profit corporate bodies), not a 2009 Law on Associations; foreign corporate bodies may register if they prove legal existence and have a permanent local representative. | verify-rest 2026-10: registration handled by the National Directorate for Registration and Notarial Services (DNRN), Ministry of Justice | verify-r2 2026-10 (confirmed): Decree-Law No.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
@@ -5787,17 +5787,17 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Resident company secretary in PNG; 7+ members with 3+ PNG residents for non-commercial company; local registered office</t>
+          <t>Company: resident company secretary in PNG and local registered office. Association (2023 Act): committee of 3+ and public officer, each with at least one PNG-ordinarily-resident person; PNG registered office; newspaper notice of intent.</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Incorporation fees in the low hundreds of USD (in PNGK); a few weeks; an associations pathway arrives mid-2026; foreign participation in charities is restricted in practice.</t>
+          <t>Incorporation fees in the low hundreds of USD (in PNGK); a few weeks for companies; new associations regime in force since 1 July 2026 adds a 60-day public objection period; foreign participation restricted in practice.</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Bureaucracy heavy, English official language but processes slow; most international NGOs register via a PNG partner or use an Australian-registered entity operating cross-border | verify-rest 2026-10: Associations Incorporation Act 2023 itself commenced 1 July 2026</t>
+          <t>Bureaucracy heavy, English official language but processes slow; most international NGOs register via a PNG partner or use an Australian-registered entity operating cross-border | verify-rest 2026-10: Associations Incorporation Act 2023 itself commenced 1 July 2026 | verify-r2 2026-10 (corrected): IPA guidance confirms the Associations Incorporation Act 2023 commenced 1 July 2026, with free re-registration of existing associations due by 30 June 2027.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
@@ -5837,7 +5837,7 @@
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
-          <t>https://www.ipa.gov.pg/public/help.aspx?cn=NewAssociationsAct; https://www.ipa.gov.pg/corp/index.aspx; https://www.ipa.gov.pg/Documentation/PG/ActsAndRegulations/Associations%20Incorporation%20Act%202023.pdf</t>
+          <t>https://www.ipa.gov.pg/public/help.aspx?cn=NewAssociationsAct; https://www.ipa.gov.pg/corp/index.aspx; https://www.ipa.gov.pg/Documentation/PG/ActsAndRegulations/Associations%20Incorporation%20Act%202023.pdf; https://www.ipa.gov.pg/Documentation/PG/IPA-Associations-Information-Eng.pdf</t>
         </is>
       </c>
       <c r="P58" s="2" t="inlineStr">
@@ -5971,7 +5971,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Resident trustee/director and local office; registration with Ministry of Justice/trust registry</t>
+          <t>Resident service agent and local registered office for companies (2014 Regs); charitable trusts incorporate as a Board with the Registrar of Charitable Trusts (= Registrar of Incorporated Societies, MCCTIL); foreign investor certification if overseas shareholders</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -5981,7 +5981,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Small, insular bureaucracy; limited precedent for foreign-registered charities; political sensitivity around foreign NGOs - community consent often expected | confirm prior: resident service agent requirement verified in Companies (Amendment) Regulations 2014 | verify-rest 2026-10: amendments to the Charitable Trusts Act 1993 under consultation (MCCTIL memo 21 July 2026), incl. trustee disclosure requirements</t>
+          <t>Small, insular bureaucracy; limited precedent for foreign-registered charities; political sensitivity around foreign NGOs - community consent often expected | confirm prior: resident service agent requirement verified in Companies (Amendment) Regulations 2014 | verify-rest 2026-10: amendments to the Charitable Trusts Act 1993 under consultation (MCCTIL memo 21 July 2026), incl. trustee disclosure requirements | verify-r2 2026-10 (corrected): The Charitable Trusts Act 1993 defines the Registrar as the Registrar of Incorporated Societies, administered by MCCTIL's Business Registries Office, not a Ministry of Justice trust registry;</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -6021,7 +6021,7 @@
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
-          <t>https://businessregistries.gov.to/public/howto.aspx?cn=RegisterCompany&amp;ctk=CompanyHowTo; https://businessregistries.gov.to/Documentation/TO/CompaniesAmendmentRegulations2014_Eng_final.pdf; https://www.revenue.gov.to/company-partnership-corporative-society-trust; https://ago.gov.to/cms/images/LEGISLATION/PRINCIPAL/1993/1993-0014/CharitableTrustsAct1993_2.pdf; https://businessregistries.gov.to/Documentation/TO/Consultation_Memo_Proposed_Amendments_CharitableTrustsAct_July_21_2026.pdf</t>
+          <t>https://businessregistries.gov.to/public/howto.aspx?cn=RegisterCompany&amp;ctk=CompanyHowTo; https://businessregistries.gov.to/Documentation/TO/CompaniesAmendmentRegulations2014_Eng_final.pdf; https://www.revenue.gov.to/company-partnership-corporative-society-trust; https://ago.gov.to/cms/images/LEGISLATION/PRINCIPAL/1993/1993-0014/CharitableTrustsAct1993_2.pdf; https://businessregistries.gov.to/Documentation/TO/Consultation_Memo_Proposed_Amendments_CharitableTrustsAct_July_21_2026.pdf; https://lpr.adb.org/sites/default/files/resource/%5Bnid%5D/tonga-charitable-trusts-act-english.pdf</t>
         </is>
       </c>
       <c r="P60" s="2" t="inlineStr">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee under the Companies Act 2012, registered with the Financial Services Commission, the main charitable form; trusts registered under trustee regulations.</t>
+          <t>Charitable association (committee incorporated under the Charitable Associations (Incorporation) Act [Cap 140]) or community company under the Companies Act 2012, both registered with the Vanuatu Financial Services Commission; the 2012 Act has no company-limited-by-guarantee form.</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -6063,17 +6063,17 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>CLBG needs local registered office/agent; 1+ resident director recommended; English widely used</t>
+          <t>Registered office and postal address in Vanuatu required (Companies Act 2012 s17); no statutory resident-director requirement; community-company shareholders must be members of the community served</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>Registration fee VT35,000 (~USD 330) via the online registry; processing a few days to weeks; a Vanuatu resident officeholder is required, so a non-resident founder must appoint a local director.</t>
+          <t>Company registration fee VT35,000 (~USD 300) via the VFSC online registry; processing a few days to weeks; the Companies Act 2012 sets no resident-director rule, but a registered office and postal address in Vanuatu are mandatory.</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Relatively permissive offshore-friendly registry; post-2021 coup political risk noted by some aid donors | correct prior: verified registration fee is VUV 35,000 (VFSC fee schedule), not VUV 5,000-20,000; 1+ resident director required</t>
+          <t>Relatively permissive offshore-friendly registry; post-2021 coup political risk noted by some aid donors | correct prior: verified registration fee is VUV 35,000 (VFSC fee schedule), not VUV 5,000-20,000; no resident-director rule in the Companies Act 2012 (registered office required) | verify-r2 2026-10 (corrected): The VFSC fee schedule confirms a VT35,000 fee to register a company under s6 of the Companies Act 2012.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
@@ -6083,7 +6083,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>Companies Act 2012 requires at least one Vanuatu-resident director and a local registered office.</t>
+          <t>Mandatory Vanuatu registered office and postal address (s17), usually via a local agent; community-company shareholders must belong to the community, so local participants are needed.</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
@@ -6113,7 +6113,7 @@
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
-          <t>https://www.vfsc.vu/companies-fees-and-penalties/; https://www.vfsc.vu/registering/; https://tradeportal.gov.vu/procedure/711/step/224</t>
+          <t>https://www.vfsc.vu/companies-fees-and-penalties/; https://www.vfsc.vu/registering/; https://tradeportal.gov.vu/procedure/711/step/224; https://tradeportal.gov.vu/media/Companies-Act-2012-Official-Gazetted-Version.pdf; https://www.vfsc.vu/wp-content/uploads/2015/08/140-Charitable-Associations-Incorporation-Act.pdf</t>
         </is>
       </c>
       <c r="P61" s="2" t="inlineStr">
@@ -6145,7 +6145,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Company limited by guarantee under the Companies Act 2009 with the Solomon Islands Business Registry; charitable trusts under trustee rules; a company limited by guarantee is the standard NGO form.</t>
+          <t>Charitable trust board incorporated under the Charitable Trusts Act (Cap 55) by the Registrar of Companies (Company Haus); community company under the Companies Act 2009 (no limited-by-guarantee form).</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -6160,12 +6160,12 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>Incorporation fee roughly USD 50-150, paid at the Treasury counter after online application; a few weeks; a resident company secretary is required, so a local agent is needed.</t>
+          <t>No fee to incorporate a charitable trust board or register a community company at Company Haus; a local private company costs SBD 1,250 (published schedule), paid at the Treasury counter; trust incorporation is described as quite fast.</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>English official, cooperative registry; foreign charitable trusts common (many Pacific-worker charities registered here); political instability occasional | confirm prior: Companies Act 2009 regime, online Company Haus registration plus Treasury fee payment | verify-rest 2026-10: foreign founders can incorporate via a local agent/resident secretary (SBD 1,500 fee, Company Haus) — presence downgraded no-&gt;partial</t>
+          <t>English official, cooperative registry; foreign charitable trusts common (many Pacific-worker charities registered here); political instability occasional | confirm prior: Companies Act 2009 regime, online Company Haus registration plus Treasury fee payment | verify-rest 2026-10: foreign founders can incorporate via a local agent/resident secretary (SBD 1,500 fee, Company Haus) — presence downgraded no-&gt;partial | verify-r2 2026-10 (corrected): The Solomon Islands Business Registry states there is no fee to set up a charitable trust and that it is quite fast, and that community companies register free at Company Haus.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>~$180 (SBD 1,500 incorporation)</t>
+          <t>none (charitable trust/community company); ~$150 (SBD 1,250) local company</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -6205,7 +6205,7 @@
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
-          <t>https://www.solomonbusinessregistry.gov.sb/companies/how-to-register-a-company/; https://www.solomonbusinessregistry.gov.sb/companies/how-to-update-a-company/restore-a-company/companies_act_2009-gazettal-as-an-act-18-mar09-2/; https://www.investsolomons.gov.sb/step-by-step-guide-to-starting-a-business/step-2-incorporate-the-enterprise-with-company-haus</t>
+          <t>https://www.solomonbusinessregistry.gov.sb/companies/how-to-register-a-company/; https://www.solomonbusinessregistry.gov.sb/companies/how-to-update-a-company/restore-a-company/companies_act_2009-gazettal-as-an-act-18-mar09-2/; https://www.investsolomons.gov.sb/step-by-step-guide-to-starting-a-business/step-2-incorporate-the-enterprise-with-company-haus; https://www.solomonbusinessregistry.gov.sb/companies/how-to-register-a-company/what-are-community-companies/additional-important-information/; https://www.solomonbusinessregistry.gov.sb/wp-content/uploads/2016/11/Schedule-of-fees-and-penalties-for-the-Company-Haus-and-InvestSolomons.pdf; https://pacliirms.austlii.edu.au/sb/legis/consol_act/cta201</t>
         </is>
       </c>
       <c r="P62" s="2" t="inlineStr">
@@ -6424,9 +6424,9 @@
           <t>Company under the Companies Act (Cap 40.08) and the Companies and Business Registration Act, administered by the Ministry of Finance; international companies under a 2009 Act.</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>very hard</t>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>hard</t>
         </is>
       </c>
       <c r="E65" s="2" t="inlineStr">
@@ -6436,12 +6436,12 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>Fees are set by regulation and unpublished; registration is effectively reserved to Tuvaluan nationals and local business - practically barred for a foreign founder without a resident partner.</t>
+          <t>Company registration fee $100 (AUD/TVD) paid at the Government Cashier under the Companies Act 2008, plus a Kaupule operating licence; non-citizens/foreign-based applicants must first contact business@gov.tv; a few weeks.</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
         <is>
-          <t>Explicit non-citizen registration restrictions; no practical foreign charity pathway; use a partner in Fiji/NZ instead | confirm prior (citizen-restricted local registration); adds TVD 100 local fee per Ministry of Finance; 2009 International Companies Act allows offshore IBC | verify-rest 2026-10: Ministry of Finance states non-citizens/foreign-based businesses may register after contacting business@gov.tv (no-&gt;partial)</t>
+          <t>Explicit non-citizen registration restrictions; no practical foreign charity pathway; use a partner in Fiji/NZ instead | confirm prior (citizen-restricted local registration); adds TVD 100 local fee per Ministry of Finance; 2009 International Companies Act allows offshore IBC | verify-rest 2026-10: Ministry of Finance states non-citizens/foreign-based businesses may register after contacting business@gov.tv (no-&gt;partial) | verify-r2 2026-10 (corrected): The Ministry of Finance business page sets a $100 company registration fee under the Companies Act 2008, payable at the Government Cashier, followed by a Kaupule operating licence, and directs non-citizens or businesses based outside Tuval…</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
@@ -6451,7 +6451,7 @@
       </c>
       <c r="I65" s="2" t="inlineStr">
         <is>
-          <t>Local business/company registration effectively restricted to Tuvaluan citizens/residents; only offshore IBC (2009 ICA) open to foreigners</t>
+          <t>Non-citizen/foreign-based registrations handled case by case via the Ministry of Finance (business@gov.tv); no NGO/charity incorporation statute, so a company plus Kaupule licence is the main local vehicle</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
-          <t>https://finance.gov.tv/business/; https://tuvalu-legislation.tv/cms/images/LEGISLATION/PRINCIPAL/2009/2009-0014/2009-0014_2.pdf; https://www.offshorecompany.com/company/tuvalu-ibc/</t>
+          <t>https://finance.gov.tv/business/; https://tuvalu-legislation.tv/cms/images/LEGISLATION/PRINCIPAL/2009/2009-0014/2009-0014_2.pdf; https://www.offshorecompany.com/company/tuvalu-ibc/; https://www.icnl.org/resources/research/ijnl/consultations-toward-legal-reform-in-tuvalu</t>
         </is>
       </c>
       <c r="P65" s="2" t="inlineStr">
@@ -6605,7 +6605,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Corporations and non-profit associations under the FSM Corporations Act (FSMC Title 36), registered with the FSM Registrar of Corporations; state-level registration for local business.</t>
+          <t>Non-profit corporation under FSM Code Title 36 ch. 7 (P.L. 23-130, Nov 2024), registered with the FSM Registrar of Corporations (DOJ, Palikir); state-level corporations/registration for local business.</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -6620,12 +6620,12 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>Filing fee roughly USD 50-200, unpublished in detail; a few weeks; foreign founders may incorporate without local presence, with a registered agent in Pohnpei serving filings.</t>
+          <t>Filing fees set under the P.L. 23-130 fee structure, amounts not published online; a few weeks; foreign founders may incorporate without local presence, with a registered agent in Pohnpei serving filings.</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>Small registries, English official; registered-agent services available; charitable framework informal - trust deed is the usual vehicle | confirm prior (medium, USD 200-600, 2-6 weeks); 100% foreign ownership and state-level LLC regime confirmed</t>
+          <t>Small registries, English official; registered-agent services available; charitable framework informal - trust deed is the usual vehicle | confirm prior (medium, USD 200-600, 2-6 weeks); 100% foreign ownership and state-level LLC regime confirmed | verify-r2 2026-10 (corrected): FSM Public Law 23-130 (Congressional Act 23-135, signed November 2024) added a new Chapter 7 to Title 36 establishing incorporation requirements, a filing-fee structure, record-keeping and annual reporting to the Registrar of Corporations…</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -6635,12 +6635,12 @@
       </c>
       <c r="I67" s="2" t="inlineStr">
         <is>
-          <t>No charitable register; must register LLC/corporation in one of 4 states (or federally) with a local registered agent/office</t>
+          <t>New national non-profit corporation regime (P.L. 23-130, 2024) with fees and implementing rules not yet published online; local registered agent needed in practice; annual reports to the Registrar</t>
         </is>
       </c>
       <c r="J67" s="2" t="inlineStr">
         <is>
-          <t>~$300</t>
+          <t>unpublished (P.L. 23-130 fee schedule)</t>
         </is>
       </c>
       <c r="K67" s="2" t="inlineStr">
@@ -6665,7 +6665,7 @@
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
-          <t>https://www.offshorecompany.com/company/micronesia-llc/; https://www.expanship.com/fm/blog/types-of-companies-in-micronesia; https://chandrawatpartners.com/micronesia-limited-liability-company-llc-key-insights-for-investors/; https://roc.doj.gov.fm/</t>
+          <t>https://www.offshorecompany.com/company/micronesia-llc/; https://www.expanship.com/fm/blog/types-of-companies-in-micronesia; https://chandrawatpartners.com/micronesia-limited-liability-company-llc-key-insights-for-investors/; https://roc.doj.gov.fm/; https://habeleinstitute.org/wiki/Zotero_reference:L6T4AK7A; https://www.cfsm.gov.fm/?p=16379; https://fsmlaw.org/fsm/code/title36/T36_Ch01_2014.html</t>
         </is>
       </c>
       <c r="P67" s="2" t="inlineStr">
@@ -6697,7 +6697,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Foundation (vakif) under the Foundations Law No. 5736 (2008), requiring legal and factual reciprocity for foreigners; association (dernek) under the Associations Law No. 5253 (2004), registered with the provincial governor.</t>
+          <t>Foundation (vakif) under the Foundations Law No. 5737 (2008), requiring legal and factual reciprocity for foreigners; association (dernek) under the Associations Law No. 5253 (2004), registered with the provincial governor.</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -6712,12 +6712,12 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>Foundation registration fee around USD 70-140 plus notary and translation, a few weeks to months; an association costs little; foreign founders are allowed for vakif where reciprocity applies.</t>
+          <t>Vakif needs a minimum endowment of TRY 5,000,000 (~USD 115k) for 2026 (Foundations Council decision 819/790), registered by the civil court; a few weeks to months; a dernek costs little but foreign founders need Turkish residence.</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>Vakıflar Genel Müdürlüğü (Foundation Directorate) handles vakıfs; dernek registration is cheaper and simpler (province governor's office, ~1 month). English paperwork accepted with sworn Turkish translation. Political/currency risk (lira volatility) is the main practical concern, not formation law. | Confirm entity types and difficulty; state fees are nominal (no US$500-1,500 official fee — that is legal service cost); add dernek 1-3 month timeline</t>
+          <t>Vakıflar Genel Müdürlüğü (Foundation Directorate) handles vakıfs; dernek registration is cheaper and simpler (province governor's office, ~1 month). English paperwork accepted with sworn Turkish translation. Political/currency risk (lira volatility) is the main practical concern, not formation law. | Confirm entity types and difficulty; state fees are nominal (no US$500-1,500 official fee — that is legal service cost); add dernek 1-3 month timeline | verify-r2 2026-10 (corrected): Turkey's Foundations Law is No.</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr">
@@ -6757,7 +6757,7 @@
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
-          <t>https://lawyer-turkey.com/set-up-a-foundation-in-turkey/; https://istanbullawyerfirm.com/blog/legal-requirements-foreign-ngos-operating-turkey; https://a-m.com.tr/non-profit-organization-in-turkey/; https://www.vgm.gov.tr/foundations-in-turkiye/foundations-in-turkiye/how-foreigners-establish-foundation-in-turkiye</t>
+          <t>https://lawyer-turkey.com/set-up-a-foundation-in-turkey/; https://istanbullawyerfirm.com/blog/legal-requirements-foreign-ngos-operating-turkey; https://a-m.com.tr/non-profit-organization-in-turkey/; https://www.vgm.gov.tr/foundations-in-turkiye/foundations-in-turkiye/how-foreigners-establish-foundation-in-turkiye; https://www.ffkpartnerhukuk.com.tr/turkiyede-vakif-kurmak-isteyen-yabancilar-icin-hukuki-rehber-2026-guncel-rehber/; https://www.tahanci.av.tr/vakif-nedir-nasil-kurulur/</t>
         </is>
       </c>
       <c r="P68" s="2" t="inlineStr">
@@ -6896,12 +6896,12 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>Minimal state fee (~600 AMD, under US$2), ~10–15 business days</t>
+          <t>State duty 10,000 AMD (~US$25) for a public organization or foundation; ~10–15 business days</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Registration via public services (e-gov) system; apostille/translation of foreign documents needed. Post-2020 South Caucasus realignment has not tightened NGO law; Armenia is one of the more open CIS-adjacent jurisdictions for foreigners. | Correct fee: state duty is 10,000 AMD (~$25), not ~600 AMD (&lt;$2); NGOs need 2+ founders, foundation 1; 10-15 business days confirmed</t>
+          <t>Registration via public services (e-gov) system; apostille/translation of foreign documents needed. Post-2020 South Caucasus realignment has not tightened NGO law; Armenia is one of the more open CIS-adjacent jurisdictions for foreigners. | Correct fee: state duty is 10,000 AMD (~$25), not ~600 AMD (&lt;$2); NGOs need 2+ founders, foundation 1; 10-15 business days confirmed | verify-r2 2026-10 (corrected): Armenian legal guidance states the state registration duty is 10,000 AMD (~USD 25) for both public organizations and foundations under the Law on State Duty, matching the fee column but contradicting the ~600 AMD figure in the cost cell.</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr">
@@ -6941,7 +6941,7 @@
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
-          <t>https://armenian-lawyer.com/business-immigration/register-nonprofit-organization-armenia/; https://www.am.business/foundation; https://lawzana.com/legal-questions/armenia/how-do-i-register-a-charity-in-armenia-and-legally-accept-foreign-donations-3799</t>
+          <t>https://armenian-lawyer.com/business-immigration/register-nonprofit-organization-armenia/; https://www.am.business/foundation; https://lawzana.com/legal-questions/armenia/how-do-i-register-a-charity-in-armenia-and-legally-accept-foreign-donations-3799; https://www.e-register.am/en/docs/213</t>
         </is>
       </c>
       <c r="P70" s="2" t="inlineStr">
@@ -7085,7 +7085,7 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Registration with the Justice Committee/region. Kazakhstan's 2023 NGO reform simplified formation, but annual reporting and foreign-funding reporting obligations are strict. A Mongolian dual citizen faces no special preference — treated as a foreign founder. | Confirm prior; small/none state fee, 5-10 business days via single window confirmed; foreign natural persons can be founders, foreign legal persons generally cannot | verify-rest 2026-10: NPO registration fee is 6.5 MCI; foreign founders realistic only via a foundation (public associations closed to foreigners)</t>
+          <t>Registration with the Justice Committee/region. Kazakhstan's 2023 NGO reform simplified formation, but annual reporting and foreign-funding reporting obligations are strict. A Mongolian dual citizen faces no special preference — treated as a foreign founder. | Confirm prior; small/none state fee, 5-10 business days via single window confirmed; foreign natural persons can be founders, foreign legal persons generally cannot | verify-rest 2026-10: NPO registration fee is 6.5 MCI; foreign founders realistic only via a foundation (public associations closed to foreigners) | verify-r2 2026-10 (confirmed): The 2026 MCI is KZT 4,325, so a 6.5 MCI state fee is about KZT 28,100 (~USD 55), consistent with the row.</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr">
@@ -7125,7 +7125,7 @@
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.kz/services/3932?lang=en; https://crd.org/2023/10/19/kazakhstan-abolish-the-foreign-funding-register/; https://www.icnl.org/resources/civic-freedom-monitor/kazakhstan</t>
+          <t>https://www.gov.kz/services/3932?lang=en; https://crd.org/2023/10/19/kazakhstan-abolish-the-foreign-funding-register/; https://www.icnl.org/resources/civic-freedom-monitor/kazakhstan; https://finratings.kz/news/10442-skolko-mrp-v-2026-godu-v-kazakhstane-novyi-raschet-nalogov-shtrafov-i-posobii/</t>
         </is>
       </c>
       <c r="P72" s="2" t="inlineStr">
@@ -7172,12 +7172,12 @@
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
-          <t>Near-zero state fee, ~5 business days via one-stop window (2023 reform)</t>
+          <t>State fee 1 BCV (regional NNO) to 3 BCV (republican), territorial NNOs 50% since 2021; Ministry of Justice review within one month by law, often extended by 'expert evaluation'.</t>
         </is>
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>The 2023 Presidential Decree modernized NGO registration (simplified one-stop process, e-filing), making formation the easiest phase; ongoing supervision and foreign-funding disclosure remain tight. Use a local partner or registered agent; Russian widely accepted in business practice. | Confirm medium difficulty; 2023 reform (Presidential Decree UP-111) streamlined one-stop-shop registration; fee nominal; time 4-10 weeks prior estimate is realistic end-to-end</t>
+          <t>The 2023 Presidential Decree modernized NGO registration (e-filing), but Ministry of Justice registration takes a legal month, often extended; ongoing supervision and foreign-funding disclosure remain tight. Use a local partner or registered agent; Russian widely accepted in business practice. | Confirm medium difficulty; 2023 reform (Presidential Decree UP-111) streamlined one-stop-shop registration; fee nominal; time 4-10 weeks prior estimate is realistic end-to-end | verify-r2 2026-10 (corrected): ICNL reports NNOs register with the Ministry of Justice (also via e-ngo.uz) under the 1999 NNO Law, with a one-month legal review period that is often extended by referral for 'expert evaluation', not a ~5-day one-stop window.</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr">
@@ -7192,12 +7192,12 @@
       </c>
       <c r="J73" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>~$15-110 (0.5-3 BCV)</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
         <is>
-          <t>2-6 weeks with a local agent</t>
+          <t>1-3 months (one-month legal term, often extended)</t>
         </is>
       </c>
       <c r="L73" s="2" t="inlineStr">
@@ -7217,7 +7217,7 @@
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
-          <t>https://investmentpolicy.unctad.org/investment-policy-monitor/measures/4559/uzbekistan-introduces-one-stop-shop-and-other-services-to-assist-investors-; https://itpark-uzb.de/en/posts/how-to-register-a-business-in-uzbekistan-a-complete-guide-fo</t>
+          <t>https://investmentpolicy.unctad.org/investment-policy-monitor/measures/4559/uzbekistan-introduces-one-stop-shop-and-other-services-to-assist-investors-; https://itpark-uzb.de/en/posts/how-to-register-a-business-in-uzbekistan-a-complete-guide-fo; https://www.icnl.org/resources/civic-freedom-monitor/uzbekistan; https://www.uzbekembassy.in/?p=27650</t>
         </is>
       </c>
       <c r="P73" s="2" t="inlineStr">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Turkmenistan effectively has a state monopoly on civil society; no functioning independent charity sector, no English-language process, and no published cost/time. Not a viable jurisdiction for this founder; do not invest time here. | Escalate difficulty from medium to very hard: prior context understates the closed nature of Turkmenistan's NGO sector; no realistic foreign registration path | [verified] Law No. 70-V Art. 1: public associations are formed by citizens of Turkmenistan only; no foreign-founder route; foreign aid/programs need state registration (2013 presidential resolution). | Correction: Sources column cites ICNL's Tajikistan page; the Turkmenistan report URL is icnl.org/resources/civic-freedom-monitor/turkmenistan.</t>
+          <t>Turkmenistan effectively has a state monopoly on civil society; no functioning independent charity sector, no English-language process, and no published cost/time. Not a viable jurisdiction for this founder; do not invest time here. | Escalate difficulty from medium to very hard: prior context understates the closed nature of Turkmenistan's NGO sector; no realistic foreign registration path | [verified] Law No. 70-V Art. 1: public associations are formed by citizens of Turkmenistan only; no foreign-founder route; foreign aid/programs need state registration (2013 presidential resolution). | Correction: Sources column cites ICNL's Tajikistan page; the Turkmenistan report URL is icnl.org/resources/civic-freedom-monitor/turkmenistan. | verify-r2 2026-10 (confirmed): ICNL confirms the Law on Public Associations of 3 May 2014, registration by the Ministry of Adalat (Justice), and fees of about USD 86/143/571 for local/national/international associations, with a 25-day decision deadline.</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr">
@@ -7351,22 +7351,22 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>Foreign citizens may be founders, but registration is in-person in Dushanbe (Ministry of Justice), requires Tajik/Russian-language documents, a local legal address, and notarized/apostilled paperwork.</t>
+          <t>Foreign citizens may be PA founders only with a valid residence permit/legal domicile in Tajikistan; in-person MoJ registration in Dushanbe with Tajik/Russian documents, a local legal address and notarized/apostilled paperwork.</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>Registration fee set by government decree, amount unpublished; Ministry of Justice processing time unpublished; foreign founders face extra authorization.</t>
+          <t>State fee 10 calculation units (~USD 80) for a local PA, 20 (~USD 160) republican, 200 (~USD 1,600) international since late 2025; Ministry of Justice processing is bureaucratic and its timeline unpublished.</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Bureaucratic, Russian/Tajik-heavy process with no e-filing; NGOs operate under a restrictive environment (post-2024 crackdowns on civil society, 'foreign agent'-style pressure). Realistic only with a local law firm handling the file; political risk is significant. | Confirm hard difficulty; state fee nominal, but prior 6-10 week timeline is optimistic — 4-12+ weeks more realistic given co-founder and approval hurdles</t>
+          <t>Bureaucratic, Russian/Tajik-heavy process with no e-filing; NGOs operate under a restrictive environment (post-2024 crackdowns on civil society, 'foreign agent'-style pressure). Realistic only with a local law firm handling the file; political risk is significant. | Confirm hard difficulty; state fee nominal, but prior 6-10 week timeline is optimistic — 4-12+ weeks more realistic given co-founder and approval hurdles | verify-r2 2026-10 (corrected): ICNL reports Tajik public associations register with the Ministry of Justice under the 2003 Law on Public Associations (amended 2022), with fees raised in late 2025 to 10/20/200 calculation units (78 somoni each) for local/republican/inter…</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>no</t>
         </is>
       </c>
       <c r="I75" s="2" t="inlineStr">
@@ -7376,7 +7376,7 @@
       </c>
       <c r="J75" s="2" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>~$80 (10 calc. units, local PA)</t>
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr">
@@ -7729,7 +7729,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Conflict-affected with weak administration; security risk for on-ground work; few foreign NGOs operate legally. | Confirm prior. FAOLEX law text (caf213189) confirms the ONG statut is conferred by ministerial arrêté to authorized associations</t>
+          <t>Conflict-affected with weak administration; security risk for on-ground work; few foreign NGOs operate legally. | Confirm prior. FAOLEX law text (caf213189) confirms the ONG statut is conferred by ministerial arrêté to authorized associations | verify-r2 2026-10 (confirmed): The FAOLEX/LEAP text is the CAR law governing national and international ONGs (Loi n°19.002 of 16 January 2019), supplemented by implementing Décret n°24.098 of 23 April 2024;</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr">
@@ -7769,7 +7769,7 @@
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
-          <t>https://faolex.fao.org/docs/pdf/caf213189.pdf; https://freedomhouse.org/country/central-african-republic/freedom-world/2024</t>
+          <t>https://faolex.fao.org/docs/pdf/caf213189.pdf; https://freedomhouse.org/country/central-african-republic/freedom-world/2024; https://leap.unep.org/en/countries/cf/national-legislation/loi-regissant-les-organisations-non-gouvernementales-ong-en; https://institut.ifjd.org/wp-content/uploads/2025/09/25.09.09_GK_Brochure_4.1_Cadre-legal_SQ.pdf</t>
         </is>
       </c>
       <c r="P79" s="2" t="inlineStr">
@@ -7821,7 +7821,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>2017 NGO law replaced the 1967 framework; political instability since 2020; approval is slow and discretionary. | Confirm prior. FAOLEX association law plus Amnesty legal review confirm the authorization regime and regular renewal</t>
+          <t>2017 NGO law replaced the 1967 framework; political instability since 2020; approval is slow and discretionary. | Confirm prior. FAOLEX association law plus Amnesty legal review confirm the authorization regime and regular renewal | verify-r2 2026-10 (confirmed): Ordinance 023/PR/2018 verified in full official text (FAOLEX) as the governing association law: authorization regime, 3-month ministerial decision (art.</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr">
@@ -7913,7 +7913,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>French-language bureaucracy; accreditation is discretionary; stable enough for a registered agent/representative to work. | Confirm prior. JO 2017 issuances show active association declaration regime; prior context thin on specific legal citations | [verified] no statutory bar on foreign founders, but the filing needs a legalized local legal seat and national ID copies for every executive-body member, so a remote founder requires a local office and Congolese executive/representative; filings in French. | Correction: Mechanism confirmed officially (1901 law; prefectural recépissés in JO through 2026); fee 15,000 FCFA per local guide, time unpublished; confidence med.</t>
+          <t>French-language bureaucracy; accreditation is discretionary; stable enough for a registered agent/representative to work. | Confirm prior. JO 2017 issuances show active association declaration regime; prior context thin on specific legal citations | [verified] no statutory bar on foreign founders, but the filing needs a legalized local legal seat and national ID copies for every executive-body member, so a remote founder requires a local office and Congolese executive/representative; filings in French. | Correction: Mechanism confirmed officially (1901 law; prefectural recépissés in JO through 2026); fee 15,000 FCFA per local guide, time unpublished; confidence med. | verify-r2 2026-10 (confirmed): Official 2017 Journal Officiel shows the Interior Ministry citing the 1 July 1901 law as in force (with loi 19-60/1960 declaration regime) and confirms the fee schedule: 15,000 FCFA per association declaration.</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr">
@@ -7995,7 +7995,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Congolese national legal representative is mandatory; foreign NGO approval from Ministry of Interior; local office.</t>
+          <t>Foreign NGO: presidential authorization (decree) motioned by Justice Ministry, line-ministry approval, local representation in DRC, framework agreement with Planning Ministry; local office.</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Slow and heavily scrutinized; security risk in the east; most expats work through an established local partner. | Confirm prior. ICNL and OHCHR sources confirm Justice-ministry registration under the 2002 NGO law framework</t>
+          <t>Slow and heavily scrutinized; security risk in the east; most expats work through an established local partner. | Confirm prior. ICNL and OHCHR sources confirm Justice-ministry registration under the 2002 NGO law framework | verify-r2 2026-10 (corrected): Law 004/2001 (official text) sets the statutory fee at 500 CDF lodging + 250 CDF publication (~$1), not $100-300, and foreign NGOs need presidential authorization (decree) motioned by the Justice Ministry plus a framework agreement with th…</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr">
@@ -8015,12 +8015,12 @@
       </c>
       <c r="I82" s="2" t="inlineStr">
         <is>
-          <t>Congolese-national legal rep mandatory, Justice ministry registration plus line-ministry approval, local office</t>
+          <t>Presidential decree authorization for foreign NGO, local representation, framework agreement with Planning Ministry, local office</t>
         </is>
       </c>
       <c r="J82" s="2" t="inlineStr">
         <is>
-          <t>~$100-300</t>
+          <t>500 CDF filing + 250 CDF publication (~$1); notary costs extra</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
@@ -8097,7 +8097,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>French-language process; post-2023 political transition adds uncertainty to approvals. | verify-rest 2026-10: Law 35/62 still governs associations ('loi 001/2011' unsupported); NGO bill adopted by the National Assembly 16 May 2025, Senate vote/promulgation pending</t>
+          <t>French-language process; post-2023 political transition adds uncertainty to approvals. | verify-rest 2026-10: Law 35/62 still governs associations ('loi 001/2011' unsupported); NGO bill adopted by the National Assembly 16 May 2025, Senate vote/promulgation pending | verify-r2 2026-10 (confirmed): Law 35/62 full text confirms the declaration regime and that foreign associations require presidential authorization on the report of the Interior Minister (arts.</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr">
@@ -8281,7 +8281,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Verified against Lei n.º 8/2012 full text (DAN05-IIS, 28-05-2012, 41 articles). Prior 'declaration' framing was wrong: art. 3.1 requires escritura pública; no prior 'agrement' exists in the law. Registry entry by Minister of Justice despacho (15-day statutory window). Foreign founders face no nationality bar (art. 6.3), but must provide home-country gazette extract of the constitutive act (art. 9.3) or a certified constitutive act where no such publication exists (art. 9.4). Very small, under-resourced administration; Portuguese filings. | few public sources, details thin</t>
+          <t>Verified against Lei n.º 8/2012 full text (DAN05-IIS, 28-05-2012, 41 articles). Prior 'declaration' framing was wrong: art. 3.1 requires escritura pública; no prior 'agrement' exists in the law. Registry entry by Minister of Justice despacho (15-day statutory window). Foreign founders face no nationality bar (art. 6.3), but must provide home-country gazette extract of the constitutive act (art. 9.3) or a certified constitutive act where no such publication exists (art. 9.4). Very small, under-resourced administration; Portuguese filings. | few public sources, details thin | verify-r2 2026-10 (confirmed): Full text of Lei 8/2012 (National Assembly gazette, 28 May 2012) confirms every cited article: escritura pública (art.</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Multiple foreign NGOs have been expelled; very high political risk; approvals are discretionary and often denied. | Governing law is Law 02/2017 on associations (plus 2017 ministerial ordinances); confirms very hard and politically risky | verify-rest 2026-10: foreign-NGO route is governed by Law 1/01 of 2017</t>
+          <t>Multiple foreign NGOs have been expelled; very high political risk; approvals are discretionary and often denied. | Governing law is Law 02/2017 on associations (plus 2017 ministerial ordinances); confirms very hard and politically risky | verify-rest 2026-10: foreign-NGO route is governed by Law 1/01 of 2017 | verify-r2 2026-10 (confirmed): The official presidential website hosts the 2017 associations law (loi-02-2017, 23 pages) and ICNL's legal library holds the separate 2017 law regulating foreign NGOs in Burundi, confirming the 2017 dual framework;</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr">
@@ -8505,7 +8505,7 @@
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
-          <t>https://presidence.gov.bi/wp-content/uploads/2017/04/loi-02-2017.pdf; https://www.iwacu-burundi.org/englishnews/over-eighty-foreign-ngos-re-registered/</t>
+          <t>https://presidence.gov.bi/wp-content/uploads/2017/04/loi-02-2017.pdf; https://www.iwacu-burundi.org/englishnews/over-eighty-foreign-ngos-re-registered/; https://www.icnl.org/research/library/burundi_burundi/</t>
         </is>
       </c>
       <c r="P87" s="2" t="inlineStr">
@@ -8649,7 +8649,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Foreign-funding disclosure and local-content expectations apply; English/Swahili; NGO Registrar oversight is strict. | verify-rest 2026-10: NGO Act is No. 24 of 2002 (am. 2019); INGO fee USD 350; founder rules corrected</t>
+          <t>Foreign-funding disclosure and local-content expectations apply; English/Swahili; NGO Registrar oversight is strict. | verify-rest 2026-10: NGO Act is No. 24 of 2002 (am. 2019); INGO fee USD 350; founder rules corrected | verify-r2 2026-10 (confirmed): NGO Act No 24 of 2002 (revised 2005, 2019) confirmed as governing law;</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr">
@@ -8833,7 +8833,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Small islands, limited administrative capacity; political instability (2018 coup, 2024 elections); French required. | Main legal basis is Law 86-006/AF (1986) art. 9 plus Decree 20-101/PR of 31 July 2020 on NGO agrément; prior '2019 NGO law' reference is inaccurate</t>
+          <t>Small islands, limited administrative capacity; political instability (2018 coup, 2024 elections); French required. | Main legal basis is Law 86-006/AF (1986) art. 9 plus Decree 20-101/PR of 31 July 2020 on NGO agrément; prior '2019 NGO law' reference is inaccurate | verify-r2 2026-10 (confirmed): Law 86-006/AF of 30 May 1986 verified in full on the official Ministry of Justice site: declaration with 15-day récépissé (art.</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr">
@@ -8915,7 +8915,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>Foreign NGOs accredited via Ministry of Foreign Affairs with a local legal representative and local office; filings in French.</t>
+          <t>Foreign ONG: prior Interior Ministry authorization after MFA opinion (art. 37, Law 96-030); local legal representative and office; filings in French.</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -8925,7 +8925,7 @@
       </c>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>No local-citizenship board rule; political instability since 2023; French-language process, local agent usable. | Confirm prior; core law is Law 96-030 (1996) + Decree 98-711; MFA accord de siege route confirmed by French diplomatic services page</t>
+          <t>No local-citizenship board rule; political instability since 2023; French-language process, local agent usable. | Confirm prior; core law is Law 96-030 (1996) + Decree 98-711; MFA accord de siege route confirmed by French diplomatic services page | verify-r2 2026-10 (corrected): Law 96-030 (official MFA text) shows foreign ONGs need prior authorization from the Minister of the Interior after opinion of the Minister of Foreign Affairs (art.</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr">
@@ -8935,7 +8935,7 @@
       </c>
       <c r="I92" s="2" t="inlineStr">
         <is>
-          <t>Foreign NGOs need an 'accord de siege' (headquarters authorization) from the Ministry of Foreign Affairs plus local representative/office</t>
+          <t>Prior Interior-Ministry authorization (after MFA opinion) for foreign ONG plus local representative/office; discretionary</t>
         </is>
       </c>
       <c r="J92" s="2" t="inlineStr">
@@ -9099,7 +9099,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Local NGOs need a Malawian majority (two-thirds) board; local office; English filings.</t>
+          <t>&gt;=2 Malawian-citizen directors/trustees (s.20(2) NGO Act); local office; English filings; int'l NGOs need line-ministry approval letter/MoU.</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -9109,7 +9109,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>English-language, moderate bureaucracy; receiving foreign funds requires NGO registration. | Corrected: two-thirds Malawian board is not the rule - the Act requires &gt;=2 Malawian-citizen directors/trustees; NGORA fee MK 35k + CONGOMA MK 55k; 2-8 weeks realistic</t>
+          <t>English-language, moderate bureaucracy; receiving foreign funds requires NGO registration. | Corrected: two-thirds Malawian board is not the rule - the Act requires &gt;=2 Malawian-citizen directors/trustees; NGORA fee MK 35k + CONGOMA MK 55k; 2-8 weeks realistic | verify-r2 2026-10 (corrected): NGORA's official site confirms the NGO (Amendment) Act 2022, the one-off MK 250,000 registration fee (~$145, not $50-100) and the &gt;=2 Malawian-citizen directors/trustees rule (s.20(2));</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr">
@@ -9119,12 +9119,12 @@
       </c>
       <c r="I94" s="2" t="inlineStr">
         <is>
-          <t>&gt;=2 Malawian-citizen directors/trustees required; local office plus NGORA and CONGOMA filings</t>
+          <t>&gt;=2 Malawian-citizen directors/trustees; mandatory partnership with a local NGO for international NGOs (2024 Regulations, NGORA guidelines 2026); line-ministry MoU</t>
         </is>
       </c>
       <c r="J94" s="2" t="inlineStr">
         <is>
-          <t>~$50-100</t>
+          <t>MK 250,000 (~$145) one-off NGORA fee + incorporation costs</t>
         </is>
       </c>
       <c r="K94" s="2" t="inlineStr">
@@ -9181,7 +9181,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Associations (Lei 8/91); Foundations (Lei 16/2018); Foreign NGO authorization (Decreto 55/98 via Ministry of Foreign Affairs); 2022 NGO law proposal (Lei OSFL) still pending</t>
+          <t>Associations (Lei 8/91); Foundations (Lei 16/2018); Foreign NGO authorization (Decreto 55/98 via Ministry of Foreign Affairs); 2022 NGO law (OSFL) dropped from Parliament's agenda Apr 2023</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -9201,7 +9201,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Portuguese-language process; a hired local manager can serve as legal representative. | verify-rest 2026-10: 'Lei 31/2002' unsupported — Lei 8/91 + Decreto 55/98 remain operative; the 2022 OSFL bill was dropped from Parliament's agenda in Apr 2023</t>
+          <t>Portuguese-language process; a hired local manager can serve as legal representative. | verify-rest 2026-10: 'Lei 31/2002' unsupported — Lei 8/91 + Decreto 55/98 remain operative; the 2022 OSFL bill was dropped from Parliament's agenda in Apr 2023 | verify-r2 2026-10 (corrected): Lei 8/91, Lei 16/2018 and Decreto 55/98 (13 Oct, foreign-NGO authorization framework under Lei 8/91 art.</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr">
@@ -9293,7 +9293,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Slow Portuguese-language bureaucracy; cautious approach needed for sensitive activities; few foreign charities register directly. | Confirm hard/3-12 months; note Lei do Estatuto das ONG (Law 2/26) now requires prior authorization for all NGOs; AOA 100k-500k = ~$100-500 | verify-rest 2026-10: Lei 14/91 replaced by Lei 6/12; Lei 2/26 (2 Mar 2026) replaced PD 74/15 for NGOs — existing NGOs adapt by Sept 2026</t>
+          <t>Slow Portuguese-language bureaucracy; cautious approach needed for sensitive activities; few foreign charities register directly. | Confirm hard/3-12 months; note Lei do Estatuto das ONG (Law 2/26) now requires prior authorization for all NGOs; AOA 100k-500k = ~$100-500 | verify-rest 2026-10: Lei 14/91 replaced by Lei 6/12; Lei 2/26 (2 Mar 2026) replaced PD 74/15 for NGOs — existing NGOs adapt by Sept 2026 | verify-r2 2026-10 (confirmed): Lei 2/26 (NGO law, approved 22 Jan 2026, promulgated 19 Feb 2026, D.R.</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr">
@@ -9380,12 +9380,12 @@
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
-          <t>USD ~20-60 (society, P500-1,500) to ~190 (CLG, P4,600); no official processing time (unpublished), plan 4-8 weeks; foreigners may register but 2/3 of society office-bearers must reside in Botswana</t>
+          <t>USD ~18-37 (society, P250-500) to ~190 (CLG, P4,600); no official processing time (unpublished), plan 4-8 weeks; foreigners may register but 2/3 of society office-bearers must reside in Botswana</t>
         </is>
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Stable, English-language; straightforward but small-bureaucracy processing times. | Mostly confirm; common route is Societies Act (20+ members) or company limited by guarantee; resident director needed; P 500-1,500 = ~$25-75; 4-8 weeks | verify-rest 2026-10: Societies Act 2022 two-thirds resident office-bearer rule</t>
+          <t>Stable, English-language; straightforward but small-bureaucracy processing times. | Mostly confirm; common route is Societies Act (20+ members) or company limited by guarantee; resident director needed; P 500-1,500 = ~$25-75; 4-8 weeks | verify-rest 2026-10: Societies Act 2022 two-thirds resident office-bearer rule | verify-r2 2026-10 (corrected): The Government of Botswana societies-registration service page sets a non-refundable fee of BWP 500 for associations and churches and BWP 250 for all other societies (20+ members), not P500-1,500.</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr">
@@ -9400,7 +9400,7 @@
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>~$25-75</t>
+          <t>~$18-37 (BWP 250-500 society fee)</t>
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr">
@@ -9472,12 +9472,12 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>BIPA statutory fees ~N$500-1,000 (~USD 35-70) plus Namibian notary for MOI; local office + registered agent required, no local-director rule, foreigners OK; 2-4 weeks to incorporate</t>
+          <t>BIPA statutory fees ~N$150-225 (~USD 10-15: name reservation N$50-75 + CM4 N$100-150) plus Namibian notary for MOI; local office + registered agent required, no local-director rule, foreigners OK; 2-4 weeks to incorporate</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>English, registered agents widely available; a popular route for SADC-based charities; low regulatory burden. | Confirm prior; common route is Section 21 company via BIPA; local office + agent, no local director; NAD 300-1,000 = ~$20-70; 2-6 weeks | Verified: Documents must be notarized by a Namibian notary; non-resident directors allowed, a local agent can sign | verify-rest 2026-10: trusts register with the Master under the Trust Administration Act 11 of 2023 (not the Deeds Registries Act)</t>
+          <t>English, registered agents widely available; a popular route for SADC-based charities; low regulatory burden. | Confirm prior; common route is Section 21 company via BIPA; local office + agent, no local director; NAD 300-1,000 = ~$20-70; 2-6 weeks | Verified: Documents must be notarized by a Namibian notary; non-resident directors allowed, a local agent can sign | verify-rest 2026-10: trusts register with the Master under the Trust Administration Act 11 of 2023 (not the Deeds Registries Act) | verify-r2 2026-10 (corrected): BIPA's published fee schedule lists N$50-75 for name reservation (CM5) and N$100-150 for registering the memorandum and articles of a company without share capital (CM4), i.e.</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr">
@@ -9492,7 +9492,7 @@
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>~$10-15</t>
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr">
@@ -9517,7 +9517,7 @@
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
-          <t>https://www.bipa.na/business-registration/companies/section-21ngo/; https://www.civic264.org.na/images/pdf/2024/6/CIVIC_264_Guide_to_Setting_Up_CSOs_in_Namibia_e-_240625_121553.pdf; https://www.icnl.org/resources/research/ijnl/the-legal-and-regulatory-framework-for-civic-organizations-in-namibia; https://www.bipa.na/business-registration/application-fees/; https://www.lac.org.na/laws/annoSTAT/Trust%20Administration%20Act%2011%20of%202023.pdf</t>
+          <t>https://www.bipa.na/business-registration/companies/section-21ngo/; https://www.civic264.org.na/images/pdf/2024/6/CIVIC_264_Guide_to_Setting_Up_CSOs_in_Namibia_e-_240625_121553.pdf; https://www.icnl.org/resources/research/ijnl/the-legal-and-regulatory-framework-for-civic-organizations-in-namibia; https://www.bipa.na/business-registration/application-fees/; https://www.lac.org.na/laws/annoSTAT/Trust%20Administration%20Act%2011%20of%202023.pdf; https://globallawexperts.com/section-21-company-namibia/</t>
         </is>
       </c>
       <c r="P98" s="2" t="inlineStr">
@@ -9569,7 +9569,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Political risk and restrictions on donor funding for certain activities; English language; many NGOs operate via local partnerships. | Corrected: governing law is the PVO Act [Ch 17:05], not an 'NGO Act 2005'; 2/3 Zimbabwean board for local PVO; US$100-500 and 1-4 months realistic | verify-rest 2026-10: PVO (General) Regulations 2026 (SI 97/2026) set fees and a 90-day decision deadline; international PVOs need an authorised local agent</t>
+          <t>Political risk and restrictions on donor funding for certain activities; English language; many NGOs operate via local partnerships. | Corrected: governing law is the PVO Act [Ch 17:05], not an 'NGO Act 2005'; 2/3 Zimbabwean board for local PVO; US$100-500 and 1-4 months realistic | verify-rest 2026-10: PVO (General) Regulations 2026 (SI 97/2026) set fees and a 90-day decision deadline; international PVOs need an authorised local agent | verify-r2 2026-10 (confirmed): Statutory Instrument 82 of 2025 (gazetted 29 Aug 2025) set PVO registration fees at US$250 for international and US$150 for local organisations, matching the current cells.</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr">
@@ -9609,7 +9609,7 @@
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
-          <t>https://hrlibrary.umn.edu/research/Zimbabwe-NGO%20laws.pdf; https://www.nangozim.org/wp-content/uploads/2025/07/NANGO-PVO-Registration-Advisory-Note-2025.pdf; https://zimlii.org/akn/zw/act/1966/63; https://www.mmmlawfirm.co.zw/the-private-voluntary-organisations-board-and-general-regulations-2026-a-guide-to-registration-governance-and-regulatory-oversight/</t>
+          <t>https://hrlibrary.umn.edu/research/Zimbabwe-NGO%20laws.pdf; https://www.nangozim.org/wp-content/uploads/2025/07/NANGO-PVO-Registration-Advisory-Note-2025.pdf; https://zimlii.org/akn/zw/act/1966/63; https://www.mmmlawfirm.co.zw/the-private-voluntary-organisations-board-and-general-regulations-2026-a-guide-to-registration-governance-and-regulatory-oversight/; https://eusee.hivos.org/alert/zimbabwe-gazettes-new-registration-fees-for-private-voluntary-organisations/; https://www.icnl.org/post/tools/practical-guide-to-zimbabwes-pvo-act-2025-amendments</t>
         </is>
       </c>
       <c r="P99" s="2" t="inlineStr">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>Local office; registration with the Registrar of Societies plus NGO unit registration to receive foreign funds; English filings.</t>
+          <t>Local office; registration with the Registrar of Companies (s17 Companies Act 2009) plus NGO unit registration to receive foreign funds; English filings.</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -9661,7 +9661,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Small, English-speaking; no local-director requirement; moderate small-country bureaucracy. | Corrected: NPOs currently registered under s17 Companies Act 8/2009, not a Societies Act; 2024 NPO Bill pending; SZL 500-2,000 = ~$25-90; 4-12 weeks</t>
+          <t>Small, English-speaking; no local-director requirement; moderate small-country bureaucracy. | Corrected: NPOs currently registered under s17 Companies Act 8/2009, not a Societies Act; 2024 NPO Bill pending; SZL 500-2,000 = ~$25-90; 4-12 weeks | verify-r2 2026-10 (corrected): The September 2024 analysis of the Non-Profit Organisations Bill for CANGO states that non-profits are currently registered under section 17 of the Companies Act 8 of 2009 with the Registrar of Companies, so the reference to a Registrar of…</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr">
@@ -9701,7 +9701,7 @@
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
-          <t>https://www.icj.org/wp-content/uploads/2025/02/ANALYSIS-OF-THE-NGO-BILL-Prepared-for-CANGO.pdf; https://africanphilanthropy.org/wp-content/uploads/2023/03/Understanding-the-Legal-Framework-for-Philanthropy-in-Southern-Africa-eSwatini-Report-Jan-2023.pdf; https://eusee.hivos.org/assets/2025/10/Final-CFR_Eswatini_JW-9.pdf; https://eswatinilii.org/akn/sz/act/2009/8/eng@1998-12-01</t>
+          <t>https://www.icj.org/wp-content/uploads/2025/02/ANALYSIS-OF-THE-NGO-BILL-Prepared-for-CANGO.pdf; https://africanphilanthropy.org/wp-content/uploads/2023/03/Understanding-the-Legal-Framework-for-Philanthropy-in-Southern-Africa-eSwatini-Report-Jan-2023.pdf; https://eusee.hivos.org/assets/2025/10/Final-CFR_Eswatini_JW-9.pdf; https://eswatinilii.org/akn/sz/act/2009/8/eng@1998-12-01; https://www.gov.sz/index.php/services-sp-310196855/60-business/business/377-company-registration</t>
         </is>
       </c>
       <c r="P100" s="2" t="inlineStr">
@@ -9743,7 +9743,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Local office; registration with the Ministry of Justice; English filings.</t>
+          <t>Registered office in Lesotho; non-profit company (2+ members, 2+ directors) registers via OBFC/Registrar of Companies, societies with the Law Office; business permit if foreign members hold 30%+; English filings.</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -9753,7 +9753,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Small, English-speaking; no local-director requirement; slow small-bureaucracy processing. | Confirm prior; routes: Societies Act, Companies Act 18/2011, Trusts Act; practitioners call registration easy; LSL 500-2,000 = ~$25-90</t>
+          <t>Small, English-speaking; no local-director requirement; slow small-bureaucracy processing. | Confirm prior; routes: Societies Act, Companies Act 18/2011, Trusts Act; practitioners call registration easy; LSL 500-2,000 = ~$25-90 | verify-r2 2026-10 (corrected): Lesotho's official business-registration portal shows non-profit companies are registered online through the One-Stop Business Facilitation Centre under the Companies Act 2011, requiring at least 2 members, 2 directors and a registered off…</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr">
@@ -10029,7 +10029,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>ASBL is the standard vehicle and easy via a local registered-office provider; AIT tax-exempt status is a separate application; French-speaking practice dominates; no in-person steps required | Verified: Authentic notarial deed required; remote founders act through an apostilled notarial power of attorney | verify-rest 2026-10: ASBL needs 2+ founders (no 2024 one-founder reform); private deed suffices for an ASBL; no EUR 25,000 legal minimum for foundations</t>
+          <t>ASBL is the standard vehicle and easy via a local registered-office provider; AIT tax-exempt status is a separate application; French-speaking practice dominates; no in-person steps required | Verified: Authentic notarial deed required; remote founders act through an apostilled notarial power of attorney | verify-rest 2026-10: ASBL needs 2+ founders (no 2024 one-founder reform); private deed suffices for an ASBL; no EUR 25,000 legal minimum for foundations | verify-r2 2026-10 (confirmed): The official Moniteur belge tariff for publishing an ASBL constitution was EUR 168.31 incl.</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr">
@@ -10069,7 +10069,7 @@
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
-          <t>https://www.lexology.com/library/detail.aspx?g=5603c18f-02f9-4b06-b538-a9e49aab19cf; https://philea.eu/wp-content/uploads/2024/11/Belgium-Philea-2024-Legal-Environment-for-Philanthropy-in-Europe.pdf; https://www.aam-solutions.com/en/company-formation/asbl/; https://justice.belgium.be/fr/themes_et_dossiers/societes_associations_et_fondations/associations/asbl</t>
+          <t>https://www.lexology.com/library/detail.aspx?g=5603c18f-02f9-4b06-b538-a9e49aab19cf; https://philea.eu/wp-content/uploads/2024/11/Belgium-Philea-2024-Legal-Environment-for-Philanthropy-in-Europe.pdf; https://www.aam-solutions.com/en/company-formation/asbl/; https://justice.belgium.be/fr/themes_et_dossiers/societes_associations_et_fondations/associations/asbl; https://ejustice.just.fgov.be/img_2024/pdf/2024_asbl.pdf; https://www.xerius.be/fr-be/devenir-independant/se-lancer/constituer-asbl</t>
         </is>
       </c>
       <c r="P104" s="2" t="inlineStr">
@@ -10116,12 +10116,12 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>EUR 200-600 for association, 1-4 weeks; foundation several months (Tribunal authorisation)</t>
+          <t>EUR 200-600 for association, 1-4 weeks; foundation several months (Ministry of Justice authorisation)</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Most English-friendly EU jurisdiction; charitable income exempt from tax; foundation route is capital-heavy, association is the practical expat choice | mostly confirm; 2025 new NPA law (foundation regime mandatory) keeps EUR 100,000 endowment for new foundations | verify-rest 2026-10: 1928 law repealed and replaced by the Law of 7 Aug 2023; ASBL minimum is 2 founders</t>
+          <t>Most English-friendly EU jurisdiction; charitable income exempt from tax; foundation route is capital-heavy, association is the practical expat choice | mostly confirm; 2025 new NPA law (foundation regime mandatory) keeps EUR 100,000 endowment for new foundations | verify-rest 2026-10: 1928 law repealed and replaced by the Law of 7 Aug 2023; ASBL minimum is 2 founders | verify-r2 2026-10 (corrected): The Law of 7 August 2023 (in force 23 Sept 2023) set a EUR 100,000 initial foundation endowment (reduced from EUR 250,000 in the bill, net assets to stay above EUR 50,000), with applications processed by the Ministry of Justice after an op…</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr">
@@ -10131,7 +10131,7 @@
       </c>
       <c r="I105" s="2" t="inlineStr">
         <is>
-          <t>Luxembourg registered office and local management presence; new NPA law 2025 raised foundation endowment</t>
+          <t>Luxembourg registered office and local management presence; foundation needs EUR 100,000 endowment and ministerial authorisation (2023 law)</t>
         </is>
       </c>
       <c r="J105" s="2" t="inlineStr">
@@ -10161,7 +10161,7 @@
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
-          <t>https://philea.eu/wp-content/uploads/2024/11/Luxembourg-Philea-2024-Legal-Environment-for-Philanthropy-in-Europe.pdf; https://kleyrgrasso.com/news/new-law-on-non-profit-associations-and-foundations-the-new-npa-law/; https://molitorlegal.lu/23-september-2025-new-regime-governing-foundations-becomes-mandatory/; https://gouvernement.lu/dam-assets/documents/actualites/2023/10-octobre/18-myasbl/flyer-myasbl.pdf</t>
+          <t>https://philea.eu/wp-content/uploads/2024/11/Luxembourg-Philea-2024-Legal-Environment-for-Philanthropy-in-Europe.pdf; https://kleyrgrasso.com/news/new-law-on-non-profit-associations-and-foundations-the-new-npa-law/; https://molitorlegal.lu/23-september-2025-new-regime-governing-foundations-becomes-mandatory/; https://gouvernement.lu/dam-assets/documents/actualites/2023/10-octobre/18-myasbl/flyer-myasbl.pdf; https://gouvernement.lu/en/dossiers.gouv2024_mj%2Ben%2Bdossiers%2B2021%2Breforme-asbl-fondations.html</t>
         </is>
       </c>
       <c r="P105" s="2" t="inlineStr">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>Verein needs 3+ founders, Austrian seat (local address), Austrian-language articles; no citizenship requirement for founders or board</t>
+          <t>Verein needs 2+ founders, Austrian seat (local address), German-language statutes; no citizenship requirement for founders or board</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -10397,7 +10397,7 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Verein is the practical vehicle; foundation laws are state-by-state (Landesrecht) with endowments from ~EUR 30,000-75,000; German required; charity tax recognition via Finanzamt | confirm prior; two-step process (errichtung then Genehmigung), 3 founders, no citizenship rule | Verified: No citizenship or residency requirement; district authority reviews within 4 weeks, extendable to 6 | verify-rest 2026-10: foundation law citations corrected (BStFG 2015 for charitable foundations; PSG 1993 for private foundations)</t>
+          <t>Verein is the practical vehicle; foundation laws are state-by-state (Landesrecht) with endowments from ~EUR 30,000-75,000; German required; charity tax recognition via Finanzamt | confirm prior; two-step process (errichtung then Genehmigung), 2 founders, no citizenship rule | Verified: No citizenship or residency requirement; district authority reviews within 4 weeks, extendable to 6 | verify-rest 2026-10: foundation law citations corrected (BStFG 2015 for charitable foundations; PSG 1993 for private foundations) | verify-r2 2026-10 (corrected): The official oesterreich.gv.at Verein page states at least two (natural or legal) persons are needed to found a Verein, statutes must be in German, and founders need not be Austrian citizens.</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr">
@@ -10407,7 +10407,7 @@
       </c>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>Austrian seat (local address) + German-language articles; 3+ founders</t>
+          <t>Austrian seat (local address) + German-language statutes; 2+ founders</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr">
@@ -10581,7 +10581,7 @@
       </c>
       <c r="G110" s="2" t="inlineStr">
         <is>
-          <t>Small, stable, English-tolerant jurisdiction; local board presence makes it impractical without a local agent; no formal charity register; often paired with Swiss structures | confirm prior; CHF/EUR/USD 30,000 minimum endowment, founder may be any nationality, 0.1% annual charge (min CHF 1,000) | verify-rest 2026-10: foundation-law revision dated 2008/2009 (not 2002)</t>
+          <t>Small, stable, English-tolerant jurisdiction; local board presence makes it impractical without a local agent; no formal charity register; often paired with Swiss structures | confirm prior; CHF/EUR/USD 30,000 minimum endowment, founder may be any nationality, 0.1% annual charge (min CHF 1,000) | verify-rest 2026-10: foundation-law revision dated 2008/2009 (not 2002) | verify-r2 2026-10 (confirmed): Practitioner guidance confirms a CHF 30,000 (or EUR/USD equivalent) minimum foundation capital certified by a Liechtenstein bank, a CHF 700 commercial-register entry fee for common-benefit foundations, and confirmation of the filing by a L…</t>
         </is>
       </c>
       <c r="H110" s="2" t="inlineStr">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
-          <t>https://www.grantthornton.ch/en/insights/overview-liechtenstein-foundation-stiftung; https://globallawexperts.com/liechtenstein-foundation-taxation; https://incorporations.io/liechtenstein/foundation/li1i; https://www.grantthornton.ch/en/insights/overview-liechtenstein-foundation-stiftung/</t>
+          <t>https://www.grantthornton.ch/en/insights/overview-liechtenstein-foundation-stiftung; https://globallawexperts.com/liechtenstein-foundation-taxation; https://incorporations.io/liechtenstein/foundation/li1i; https://www.grantthornton.ch/en/insights/overview-liechtenstein-foundation-stiftung/; https://www.mondaq.com/contracts-and-commercial-law/1353206/establishment-of-a-foundation-respectively-filing-of-a-notice-of-formation-in-liechtenstein; https://www.liechtenstein-business.li/en/economic-area/Founding-a-company/Legal-forms/Foundations</t>
         </is>
       </c>
       <c r="P110" s="2" t="inlineStr">
@@ -11133,7 +11133,7 @@
       </c>
       <c r="G116" s="2" t="inlineStr">
         <is>
-          <t>VPO public-benefit status is a separate Ministry of Interior procedure; Slovak language barrier; paperwork moderate. | confirm prior; court registration fee ~150 EUR plus notary, so total ~200-600 EUR as noted | verify-rest 2026-10: civic association needs 3 founders, EUR 66 fee, ~10-15 days; Act 213/1997 amended by Act 109/2025 (Constitutional Court ruling PL. ÚS 11/2025)</t>
+          <t>VPO public-benefit status is a separate Ministry of Interior procedure; Slovak language barrier; paperwork moderate. | confirm prior; court registration fee ~150 EUR plus notary, so total ~200-600 EUR as noted | verify-rest 2026-10: civic association needs 3 founders, EUR 66 fee, ~10-15 days; Act 213/1997 amended by Act 109/2025 (Constitutional Court ruling PL. ÚS 11/2025) | verify-r2 2026-10 (confirmed): Ministry of Interior guidance confirms a EUR 66 administrative fee for registering a civic association, halved to EUR 33 for electronic filing.</t>
         </is>
       </c>
       <c r="H116" s="2" t="inlineStr">
@@ -11173,7 +11173,7 @@
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
-          <t>https://cof.org/country-notes/nonprofit-law-slovakia; https://www.slovensko.sk/en/life-situation/life-situation/_setting-up-a-company; https://www.lexmundi.com/guides/social-enterprise-law-surveys/jurisdictions/europe/slovak-republic/; https://www.justice.gov.sk/sluzby/obchodny-register/najcastejsie-otazky/; https://static.slov-lex.sk/static/SK/ZZ/2025/109/20260204.html</t>
+          <t>https://cof.org/country-notes/nonprofit-law-slovakia; https://www.slovensko.sk/en/life-situation/life-situation/_setting-up-a-company; https://www.lexmundi.com/guides/social-enterprise-law-surveys/jurisdictions/europe/slovak-republic/; https://www.justice.gov.sk/sluzby/obchodny-register/najcastejsie-otazky/; https://static.slov-lex.sk/static/SK/ZZ/2025/109/20260204.html; https://minv.sk/swift_data/source/miestna_statna_sprava/okres_zilina/ovvs/spravne/ZZPO.pdf; https://www.podnikajte.sk/zdruzenie/obcianske-zdruzenie-zalozenie-a-podnikanie</t>
         </is>
       </c>
       <c r="P116" s="2" t="inlineStr">
@@ -11312,12 +11312,12 @@
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
-          <t>Association ~200-500 EUR, ~1-2 months; foundation ~1,000-3,000 EUR, ~1-3 months</t>
+          <t>Association: EUR 31.72 admin fee at upravna enota, ~1-2 months; foundation ~1,000-3,000 EUR incl. notary, ~1-3 months</t>
         </is>
       </c>
       <c r="G118" s="2" t="inlineStr">
         <is>
-          <t>Public-benefit (javno koristno) status is a separate procedure with membership-base criteria; English support limited outside Ljubljana. | confirm prior; association ~200-500 EUR and foundation ~1,000-3,000 EUR incl. notary; javno koristno status separate</t>
+          <t>Public-benefit (javno koristno) status is a separate procedure with membership-base criteria; English support limited outside Ljubljana. | confirm prior; association ~200-500 EUR and foundation ~1,000-3,000 EUR incl. notary; javno koristno status separate | verify-r2 2026-10 (corrected): The official SPOT portal states a društvo is founded by at least three legally capable persons and registered at the upravna enota of its seat for an administrative fee (upravna taksa) of EUR 31.72, far below the ~EUR 200-500 / ~$300 in th…</t>
         </is>
       </c>
       <c r="H118" s="2" t="inlineStr">
@@ -11332,7 +11332,7 @@
       </c>
       <c r="J118" s="2" t="inlineStr">
         <is>
-          <t>~$300</t>
+          <t>~$37 (EUR 31.72 association admin fee)</t>
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr">
@@ -11357,7 +11357,7 @@
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
-          <t>https://e-uprava.gov.si/en/podrocja/state-and-society/societies-public-events-and-gatherings/registration-of-a-society-branch-of-foreign-society-and-associations-of-societies.html; https://companyformationslovenia.com/open-foundation-in-slovenia/</t>
+          <t>https://e-uprava.gov.si/en/podrocja/state-and-society/societies-public-events-and-gatherings/registration-of-a-society-branch-of-foreign-society-and-associations-of-societies.html; https://companyformationslovenia.com/open-foundation-in-slovenia/; https://spot.gov.si/sl/teme/drustvo</t>
         </is>
       </c>
       <c r="P118" s="2" t="inlineStr">
@@ -11491,7 +11491,7 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>3+ founders, local office, charter in local language; registration happens at entity level (Republika Srpska vs Federation of BiH), sometimes municipal, so structure depends on where the office is.</t>
+          <t>3+ founders (state-level law limits association founders to BiH citizens/residents or BiH-registered entities; RS law treats foreigners equally), local office, local-language charter; register at state level (BiH Ministry of Justice) or entity level (FBiH, RS, Brcko), so structure depends on scope and office location.</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -11501,7 +11501,7 @@
       </c>
       <c r="G120" s="2" t="inlineStr">
         <is>
-          <t>Three-layer state/entity system creates duplicated paperwork; no online registry; English support rare; foreign founders allowed but bureaucracy heavy. | confirm prior; fees ~100-300 BAM per tier; timeline can stretch to months in practice due to duplicated paperwork</t>
+          <t>Three-layer state/entity system creates duplicated paperwork; no online registry; English support rare; foreign founders allowed but bureaucracy heavy. | confirm prior; fees ~100-300 BAM per tier; timeline can stretch to months in practice due to duplicated paperwork | verify-r2 2026-10 (corrected): The BiH Ministry of Justice registers associations and foundations at state level under the Law on Associations and Foundations of BiH (OG 32/01, amended 2003, 2008, 2011), alongside separate FBiH, RS and Brcko registers, so registration i…</t>
         </is>
       </c>
       <c r="H120" s="2" t="inlineStr">
@@ -11541,7 +11541,7 @@
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
-          <t>https://www.ohchr.org/en/press-releases/2025/02/bosnia-and-herzegovina-bill-registering-ngos-will-increase-government; https://documents.worldbank.org/en/publication/documents-reports/documentdetail/664631468743400463/how-to-establish-and-register-business-association-in-bosnia-and-herzegovina</t>
+          <t>https://www.ohchr.org/en/press-releases/2025/02/bosnia-and-herzegovina-bill-registering-ngos-will-increase-government; https://documents.worldbank.org/en/publication/documents-reports/documentdetail/664631468743400463/how-to-establish-and-register-business-association-in-bosnia-and-herzegovina; https://mpr.gov.ba/en/registracija-pravnih-lica-koje-osnivaju-institucije-bosne-i-hercegovine; https://philea.eu/wp-content/uploads/2021/12/BosniaAndHerzegovina_2020LegalEnvironmentPhilanthropy.pdf; https://www.icnl.org/post/in-the-news/republic-of-srpska-adopts-a-new-law-on-associations-and-foundations</t>
         </is>
       </c>
       <c r="P120" s="2" t="inlineStr">
@@ -11588,12 +11588,12 @@
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
-          <t>~2,000-5,000 RSD fees + translations/apostille; ~1-2 months (statutory 30 days)</t>
+          <t>RSD 6,500 APR registration fee + translations/apostille; ~1-2 months (statutory 30 days)</t>
         </is>
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>Non-EU; English support limited; cheap registration; foreign founders routinely register (many Serbian diaspora do this); apostille for foreign ID documents. | confirm prior; difficulty better rated medium (not easy) given translation/apostille work; fees ~2,000-5,000 RSD plus docs | verify-rest 2026-10: Law on Associations requires a Serbia-resident founder and agent (yes-&gt;partial); APR fee RSD 6,500</t>
+          <t>Non-EU; English support limited; cheap registration; foreign founders routinely register (many Serbian diaspora do this); apostille for foreign ID documents. | confirm prior; difficulty better rated medium (not easy) given translation/apostille work; APR fee RSD 6,500 plus docs | verify-rest 2026-10: Law on Associations requires a Serbia-resident founder and agent (yes-&gt;partial); APR fee RSD 6,500 | verify-r2 2026-10 (corrected): APR states the fee for registering the formation of an association is RSD 6,500, which contradicts the '~2,000-5,000 RSD fees' in the cost cell.</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
@@ -11633,7 +11633,7 @@
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
-          <t>https://welcometoserbia.gov.rs/initiate-the-registration-process; https://globallawexperts.com/how-to-register-a-company-in-serbia-step-by-step-tier-2-guide/; https://apr.gov.rs/registers/associations/fees.1628.html</t>
+          <t>https://welcometoserbia.gov.rs/initiate-the-registration-process; https://globallawexperts.com/how-to-register-a-company-in-serbia-step-by-step-tier-2-guide/; https://apr.gov.rs/registers/associations/fees.1628.html; https://mduls.gov.rs/wp-content/uploads/vodic-za-primenu-zakona-o-udruzenjima.pdf</t>
         </is>
       </c>
       <c r="P121" s="2" t="inlineStr">
@@ -11685,7 +11685,7 @@
       </c>
       <c r="G122" s="2" t="inlineStr">
         <is>
-          <t>Slow bureaucracy, documents in Montenegrin, minimal English support; EU-candidate so framework is straightforward in principle. | Confirm association/foundation forms and 1-3 months; official gov.me page says registration is free, so prior 50-200 EUR is overestimated.</t>
+          <t>Slow bureaucracy, documents in Montenegrin, minimal English support; EU-candidate so framework is straightforward in principle. | Confirm association/foundation forms and 1-3 months; official gov.me page says registration is free, so prior 50-200 EUR is overestimated. | verify-r2 2026-10 (confirmed): Montenegro's Law on NGOs (SL CG 39/11, 37/17) Art.</t>
         </is>
       </c>
       <c r="H122" s="2" t="inlineStr">
@@ -11725,7 +11725,7 @@
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>https://www.gov.me/en/article/cooperation-between-the-government-of-montenegro-and-ngos; https://cof.org/country-notes/nonprofit-law-montenegro; https://saaccounting.me/blog/ngo-accounting-montenegro; https://ngo.gov.me/Udruzenje</t>
+          <t>https://www.gov.me/en/article/cooperation-between-the-government-of-montenegro-and-ngos; https://cof.org/country-notes/nonprofit-law-montenegro; https://saaccounting.me/blog/ngo-accounting-montenegro; https://ngo.gov.me/Udruzenje; https://www.icnl.org/research/library/montenegro_zakon-o-nevladinim-organizacijama-2011/; https://www.paragraf.me/propisi-crnegore/zakon-o-nevladinim-organizacijama.html</t>
         </is>
       </c>
       <c r="P122" s="2" t="inlineStr">
@@ -11777,7 +11777,7 @@
       </c>
       <c r="G123" s="2" t="inlineStr">
         <is>
-          <t>EU candidate, cheap and low-bureaucracy; language barrier for a resident-in-Australia founder means using a local agent/lawyer. | Confirm association/foundation and 1-2 months; state registration fee is nominal (~$0-50), prior 100-300 EUR overstates official cost. | verify-rest 2026-10: founder rule corrected to 5 (3 local); foundation endowment EUR 10,000</t>
+          <t>EU candidate, cheap and low-bureaucracy; language barrier for a resident-in-Australia founder means using a local agent/lawyer. | Confirm association/foundation and 1-2 months; state registration fee is nominal (~$0-50), prior 100-300 EUR overstates official cost. | verify-rest 2026-10: founder rule corrected to 5 (3 local); foundation endowment EUR 10,000 | verify-r2 2026-10 (confirmed): Philea's 2025 profile confirms that North Macedonian foundations need an initial asset pool of at least EUR 10,000 and register with the Central Register, filing within 30 days of the founding act.</t>
         </is>
       </c>
       <c r="H123" s="2" t="inlineStr">
@@ -11817,7 +11817,7 @@
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
-          <t>https://www.opengovpartnership.org/members/north-macedonia/commitments/MK0148/; https://ngobase.org/c/MK/north-macedonia-ngos-charities; https://www.crm.com.mk/en/services/perform-a-registration-or-complete-a-task/establish-a-new-entity/independent-registration-of-an-entity; https://www.ecoi.net/en/file/local/2076161/62e160a24.pdf; https://www.icnl.org/wp-content/uploads/Macedonia_zakon.pdf</t>
+          <t>https://www.opengovpartnership.org/members/north-macedonia/commitments/MK0148/; https://ngobase.org/c/MK/north-macedonia-ngos-charities; https://www.crm.com.mk/en/services/perform-a-registration-or-complete-a-task/establish-a-new-entity/independent-registration-of-an-entity; https://www.ecoi.net/en/file/local/2076161/62e160a24.pdf; https://www.icnl.org/wp-content/uploads/Macedonia_zakon.pdf; https://philea.eu/wp-content/uploads/2025/11/North-Macedonia-Philea-2025-Legal-Environment-for-Philanthropy-in-Europe.pdf; https://www.icnl.org/research/library/macedonia_assocs_founds_eng/</t>
         </is>
       </c>
       <c r="P123" s="2" t="inlineStr">
@@ -11869,7 +11869,7 @@
       </c>
       <c r="G124" s="2" t="inlineStr">
         <is>
-          <t>2021 NPO registration law modernized the register; English support limited; foreign-founded NGOs common, often with local partners. | Confirm association/foundation and 2021 electronic register; total all-in cost ~$300-550 incl. notary is consistent with prior. | verify-rest 2026-10: founder minimum is 5 natural/2 legal persons; register is held by the Tirana court, not the National Registration Center</t>
+          <t>2021 NPO registration law modernized the register; English support limited; foreign-founded NGOs common, often with local partners. | Confirm association/foundation and 2021 electronic register; total all-in cost ~$300-550 incl. notary is consistent with prior. | verify-rest 2026-10: founder minimum is 5 natural/2 legal persons; register is held by the Tirana court, not the National Registration Center | verify-r2 2026-10 (corrected): Under Law 80/2021, as partly struck down by Constitutional Court Decision No.</t>
         </is>
       </c>
       <c r="H124" s="2" t="inlineStr">
@@ -11879,7 +11879,7 @@
       </c>
       <c r="I124" s="2" t="inlineStr">
         <is>
-          <t>Albanian-language documents + local office; QKB electronic filing via courier, limited English support.</t>
+          <t>Albanian-language documents + local office; filing with the Tirana court NPO register (post/courier accepted), limited English support.</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
@@ -11909,7 +11909,7 @@
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
-          <t>https://jbc.al/registration-of-non-profit-organizations-in-albania/; https://sherbimekontabiliteti.al/en/albania-ngo-nonprofit-tax/; https://resourcecentre.al/frequently-asked-questions/; https://www.partnersalbania.org/wp-content/uploads/2019/01/ligj_nr.802021_24.6.2021.pdf; https://www.tatime.gov.al/eng/shkarko.php?id=5278</t>
+          <t>https://jbc.al/registration-of-non-profit-organizations-in-albania/; https://sherbimekontabiliteti.al/en/albania-ngo-nonprofit-tax/; https://resourcecentre.al/frequently-asked-questions/; https://www.partnersalbania.org/wp-content/uploads/2019/01/ligj_nr.802021_24.6.2021.pdf; https://www.tatime.gov.al/eng/shkarko.php?id=5278; https://ahc.org.al/en/the-constitutional-court-partially-abolishes-some-of-the-provisions-of-law-no-80-2021-for-the-registration-of-non-profit-organizations/</t>
         </is>
       </c>
       <c r="P124" s="2" t="inlineStr">
@@ -11961,7 +11961,7 @@
       </c>
       <c r="G125" s="2" t="inlineStr">
         <is>
-          <t>Cheap; EU candidate; political/economic volatility and weak enforcement; banking for foreign directors can be fiddly. | Confirm association/foundation and 2-6 weeks; no state registration fee (Lex Mundi guide), prior 100-300 EUR was notary/legal only. | verify-rest 2026-10: Law 86/2020 allows 2 founders; registration free with a 15-day statutory term</t>
+          <t>Cheap; EU candidate; political/economic volatility and weak enforcement; banking for foreign directors can be fiddly. | Confirm association/foundation and 2-6 weeks; no state registration fee (Lex Mundi guide), prior 100-300 EUR was notary/legal only. | verify-rest 2026-10: Law 86/2020 allows 2 founders; registration free with a 15-day statutory term | verify-r2 2026-10 (confirmed): Moldova's Law 86/2020 on Non-commercial Organisations governs associations, foundations and private institutions, and registration with the Public Services Agency is free.</t>
         </is>
       </c>
       <c r="H125" s="2" t="inlineStr">
@@ -12001,7 +12001,7 @@
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
-          <t>https://www.lexmundi.com/media/oyajwdaw/registering-ngos-moldova.pdf; https://ong.legal/articles/how-to-register-an-ngo-in-moldova.html; https://www.icnl.org/resources/research/ijnl/legislation-for-non-profit-organizations-in-the-republic-of-moldova; https://csometer.info/updates/moldova-new-progressive-law-non-commercial-organisations; https://asp.gov.md/en/intrebari-frecvente/persoane-juridice/0041</t>
+          <t>https://www.lexmundi.com/media/oyajwdaw/registering-ngos-moldova.pdf; https://ong.legal/articles/how-to-register-an-ngo-in-moldova.html; https://www.icnl.org/resources/research/ijnl/legislation-for-non-profit-organizations-in-the-republic-of-moldova; https://csometer.info/updates/moldova-new-progressive-law-non-commercial-organisations; https://asp.gov.md/en/intrebari-frecvente/persoane-juridice/0041; https://csometer.info/moldova-new-progressive-law-on-non-commercial-organisations/; https://archive.lexmundi.com/common/Uploaded%20files/LM/Corporate%20Counsel%20Toolkit/Ukraine%20Crisis%20Resource%20Center/Guide-Lex-Mundi-NGOs-Moldova-GP180322.pdf</t>
         </is>
       </c>
       <c r="P125" s="2" t="inlineStr">
@@ -12053,7 +12053,7 @@
       </c>
       <c r="G126" s="2" t="inlineStr">
         <is>
-          <t>Registration itself is cheap and fast, but active war, banking/sanctions friction for a foreign resident founder and currency risk make this a risky base; many Western expat charities run via local Ukrainian partners. | verify-rest 2026-10: no state duty for public-association registration; 'fundatsiia' replaced with blahodiinyi fond</t>
+          <t>Registration itself is cheap and fast, but active war, banking/sanctions friction for a foreign resident founder and currency risk make this a risky base; many Western expat charities run via local Ukrainian partners. | verify-rest 2026-10: no state duty for public-association registration; 'fundatsiia' replaced with blahodiinyi fond | verify-r2 2026-10 (confirmed): The existing Ukraine cells are consistent with Law 4572-VI on Public Associations and Law 5073-VI on Charitable Activities.</t>
         </is>
       </c>
       <c r="H126" s="2" t="inlineStr">
@@ -12227,7 +12227,7 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>Association 3+ founders (foreigners allowed), local office, Romanian-language statute; foundation 1 founder, endowment per charter, notary deed.</t>
+          <t>Association 3+ founders (foreigners allowed), local office, Romanian-language statute; foundation 1+ founder with initial assets of at least 100x the gross minimum wage (OG 26/2000 Art. 15), notary deed.</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -12237,7 +12237,7 @@
       </c>
       <c r="G128" s="2" t="inlineStr">
         <is>
-          <t>EU member; moderate bureaucracy; 'de utilitate publică' (public-benefit) tax status is a separate, stricter procedure; English support OK in Bucharest/Cluj. | Confirm association/foundation and separate public-utility status; state fee ~300 RON (~$70), prior 500 RON overstated.</t>
+          <t>EU member; moderate bureaucracy; 'de utilitate publică' (public-benefit) tax status is a separate, stricter procedure; English support OK in Bucharest/Cluj. | Confirm association/foundation and separate public-utility status; state fee ~300 RON (~$70), prior 500 RON overstated. | verify-r2 2026-10 (corrected): Article 15 of OG 26/2000 requires a Romanian foundation's initial assets to be worth at least 100 times the gross minimum wage at the date of incorporation (20 times for pure fund-raising foundations), so 'endowment per charter' was wrong.</t>
         </is>
       </c>
       <c r="H128" s="2" t="inlineStr">
@@ -12277,7 +12277,7 @@
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
-          <t>https://cof.org/country-notes/nonprofit-law-romania; https://www.romania-company.com/set-up-ngo-romania/; https://romanianlawoffice.com/non-profit-foundation-association-romania.htm</t>
+          <t>https://cof.org/country-notes/nonprofit-law-romania; https://www.romania-company.com/set-up-ngo-romania/; https://romanianlawoffice.com/non-profit-foundation-association-romania.htm; https://notari.pro/ordonanta-26-2000-asociatii-fundatii/art-15-infiintarea-asociatiilor-si-a-fundatiilor; https://contabilul.manager.ro/a/17807/noi-modificari-in-ordonanta-nr-262000-cu-privire-la-asociatii-si-fundatii.html</t>
         </is>
       </c>
       <c r="P128" s="2" t="inlineStr">
@@ -12329,7 +12329,7 @@
       </c>
       <c r="G129" s="2" t="inlineStr">
         <is>
-          <t>EU member; the 1-founder NPL form is the simplest for a lone foreign founder; good English support in Sofia; cheap to operate. | Confirm 1-founder NPL as simplest route; fees ~150-300 BGN plus notary; 30-day statutory limit as prior. | verify-rest 2026-10: association founder minimum is 3; Registry Agency fee ~EUR 25</t>
+          <t>EU member; the 1-founder NPL form is the simplest for a lone foreign founder; good English support in Sofia; cheap to operate. | Confirm 1-founder NPL as simplest route; fees ~150-300 BGN plus notary; 30-day statutory limit as prior. | verify-rest 2026-10: association founder minimum is 3; Registry Agency fee ~EUR 25 | verify-r2 2026-10 (confirmed): Initial registration of a Bulgarian NPLE in the Registry Agency costs BGN 50 (EUR 25.56) on paper or half that if filed electronically.</t>
         </is>
       </c>
       <c r="H129" s="2" t="inlineStr">
@@ -12369,7 +12369,7 @@
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
-          <t>https://www.lexmundi.com/media/wzqlyumt/guidance-for-ngos-operating-out-of-bulgaria.pdf; https://www.icnl.org/wp-content/uploads/Bulgarian-Non-Profit-Legal-Entities-Act-of-2000.pdf; https://globallawexperts.com/how-to-form-a-company-in-bulgaria/; https://portal.registryagency.bg/en/page/136; https://bcnl.org/en/category_legislation/basic-information</t>
+          <t>https://www.lexmundi.com/media/wzqlyumt/guidance-for-ngos-operating-out-of-bulgaria.pdf; https://www.icnl.org/wp-content/uploads/Bulgarian-Non-Profit-Legal-Entities-Act-of-2000.pdf; https://globallawexperts.com/how-to-form-a-company-in-bulgaria/; https://portal.registryagency.bg/en/page/136; https://bcnl.org/en/category_legislation/basic-information; https://www.innovires.com/en/blog/registracia-fondacia.html</t>
         </is>
       </c>
       <c r="P129" s="2" t="inlineStr">
@@ -12401,7 +12401,7 @@
       </c>
       <c r="C130" s="2" t="inlineStr">
         <is>
-          <t>Associations (somateio, min. 20 founders, Civil Code art. 78); foundations (Civil Code arts. 108-121 + Law 5259/2025, which repealed Law 4182/2013); general-benefit status via separate application.</t>
+          <t>Associations (somateio, min. 20 founders, Civil Code art. 78); foundations (Civil Code arts. 108-121 + Law 4182/2013, to be largely repealed by Law 5259/2025 once its Unit I takes effect); general-benefit status via separate application.</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
@@ -12421,7 +12421,7 @@
       </c>
       <c r="G130" s="2" t="inlineStr">
         <is>
-          <t>Paper/notary-heavy process, Greek language required, no meaningful online registry; foundations now under Law 5259/2025; use a local lawyer. | verify-rest 2026-10: somateio needs 20 founders; registration via Magistrates' Court since 2016; Law 5259/2025 replaced 4182/2013</t>
+          <t>Paper/notary-heavy process, Greek language required, no meaningful online registry; foundations now under Law 5259/2025; use a local lawyer. | verify-rest 2026-10: somateio needs 20 founders; registration via Magistrates' Court since 2016; Law 5259/2025 replaced 4182/2013 | verify-r2 2026-10 (corrected): Article 131 of Greece's Law 5259/2025 repeals arts.</t>
         </is>
       </c>
       <c r="H130" s="2" t="inlineStr">
@@ -12461,7 +12461,7 @@
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
-          <t>https://philea.eu/wp-content/uploads/2024/11/Greece-Philea-2024-Legal-Environment-for-Philanthropy-in-Europe.pdf; https://companyformationgreece.com/set-up-a-foundation-in-greece/; https://globallawexperts.com/how-to-start-a-business-in-greece-as-a-foreigner/; https://fra.europa.eu/sites/default/files/fra_uploads/greece-civil-space_en.pdf; https://www.e-nomothesia.gr/kat-oikonomia/nomos-5259-2025.html</t>
+          <t>https://philea.eu/wp-content/uploads/2024/11/Greece-Philea-2024-Legal-Environment-for-Philanthropy-in-Europe.pdf; https://companyformationgreece.com/set-up-a-foundation-in-greece/; https://globallawexperts.com/how-to-start-a-business-in-greece-as-a-foreigner/; https://fra.europa.eu/sites/default/files/fra_uploads/greece-civil-space_en.pdf; https://www.e-nomothesia.gr/kat-oikonomia/nomos-5259-2025.html; https://www.taxheaven.gr/law/5259/2025/arthro/131; https://mitos.gov.gr/index.php/%CE%94%CE%94:%CE%94%CE%B9%CE%B5%CE%BD%CE%AD%CF%81%CE%B3%CE%B5%CE%B9%CE%B1_%CE%B5%CE%B9%CE%B4%CE%B9%CE%BA%CF%8E%CE%BD_%CE%B4%CE%B7%CE%BC%CE%BF%CF%83%CE%B9%CE%BF%CE%BD%CE%BF%CE%BC%CE%B9%CE%BA%CF%8E%CE%BD_%CE%B5%CE%BB%CE%AD%CE%B3%CF%87%CF%89%CE%BD</t>
         </is>
       </c>
       <c r="P130" s="2" t="inlineStr">
@@ -12513,7 +12513,7 @@
       </c>
       <c r="G131" s="2" t="inlineStr">
         <is>
-          <t>English common-law jurisdiction — most expats set up a simple charitable trust with a Cypriot trustee; tax deductibility requires income-tax authority approval and a Cypriot public-benefit nexus; strong English-language professional services. | verify-rest 2026-10: society needs 20 founders under Law 104(I)/2017; Registrar may take up to 3 months</t>
+          <t>English common-law jurisdiction — most expats set up a simple charitable trust with a Cypriot trustee; tax deductibility requires income-tax authority approval and a Cypriot public-benefit nexus; strong English-language professional services. | verify-rest 2026-10: society needs 20 founders under Law 104(I)/2017; Registrar may take up to 3 months | verify-r2 2026-10 (corrected): Under Cyprus's Societies and Institutions Law 104(I)/2017, a society is an association of at least 20 persons registered by the District Officer acting as Registrar/Commissioner.</t>
         </is>
       </c>
       <c r="H131" s="2" t="inlineStr">
@@ -12523,7 +12523,7 @@
       </c>
       <c r="I131" s="2" t="inlineStr">
         <is>
-          <t>Trust unregistered (easiest); registered body needs Cypriot head office + 7 members + local agent for bank account</t>
+          <t>Trust unregistered (easiest); registered society needs Cypriot head office + 20 founding members + local agent for bank account</t>
         </is>
       </c>
       <c r="J131" s="2" t="inlineStr">
@@ -12553,7 +12553,7 @@
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
-          <t>https://www.companies.gov.cy/en/21-eservices/esearch-in-business-entity-s-registry; https://taxsummaries.pwc.com/cyprus/individual/deductions; https://whydonate.com/help/donate/what-are-the-tax-benefits-of-charitable-donations-in-different-countries; https://mondaq.co.uk/cyprus/directors-and-officers/1229390/registration-and-establishment-of-societies-in-the-republic-of-cyprus</t>
+          <t>https://www.companies.gov.cy/en/21-eservices/esearch-in-business-entity-s-registry; https://taxsummaries.pwc.com/cyprus/individual/deductions; https://whydonate.com/help/donate/what-are-the-tax-benefits-of-charitable-donations-in-different-countries; https://mondaq.co.uk/cyprus/directors-and-officers/1229390/registration-and-establishment-of-societies-in-the-republic-of-cyprus; https://ecnl.org/republic-cyprus-adopted-progressive-ngo-law/</t>
         </is>
       </c>
       <c r="P131" s="2" t="inlineStr">
@@ -12605,7 +12605,7 @@
       </c>
       <c r="G132" s="2" t="inlineStr">
         <is>
-          <t>English official language, streamlined 2021 framework; foundation is the stronger form for asset-holding; charitable trusts available under trust law without registration. | Association min 3 members + 3 administrators under Act V/2021; MBR online filing, English accepted. Confirm prior fees/timeline.</t>
+          <t>English official language, streamlined 2021 framework; foundation is the stronger form for asset-holding; charitable trusts available under trust law without registration. | Association min 3 members + 3 administrators under Act V/2021; MBR online filing, English accepted. Confirm prior fees/timeline. | verify-r2 2026-10 (confirmed): In Malta, the Foundations and Associations Unit of the Malta Business Registry registers legal organisations under the Second Schedule of the Civil Code.</t>
         </is>
       </c>
       <c r="H132" s="2" t="inlineStr">
@@ -12645,7 +12645,7 @@
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
-          <t>https://www.legislation.mt/eli/act/v/2021/eng; https://www.mbr.mt/website-pages/formation-and-registration; https://www.bmf.gv.at/dam/jcr:1da187f9-7f84-4c30-8b0b-f7c06244594d/Country-specific_Information_-_Malta_-_BMF_2021-07-22.pdf</t>
+          <t>https://www.legislation.mt/eli/act/v/2021/eng; https://www.mbr.mt/website-pages/formation-and-registration; https://www.bmf.gv.at/dam/jcr:1da187f9-7f84-4c30-8b0b-f7c06244594d/Country-specific_Information_-_Malta_-_BMF_2021-07-22.pdf; https://mbr.mt/foundations-and-associations; https://cvo.gov.mt/faqs</t>
         </is>
       </c>
       <c r="P132" s="2" t="inlineStr">
@@ -12697,7 +12697,7 @@
       </c>
       <c r="G133" s="2" t="inlineStr">
         <is>
-          <t>English-language, common-law system; no nationality requirement for trustees; most overseas founders set up a company limited by guarantee with a local registered-office agent, then register the charity | Confirm prior; regulator is the Charities Regulatory Authority (CRA), not the former 'Charity Commission for Ireland'. | verify-rest 2026-10: no EUR 50k registration threshold; regulator is the Charities Regulator; s.137 requires an EEA-resident director or bond</t>
+          <t>English-language, common-law system; no nationality requirement for trustees; most overseas founders set up a company limited by guarantee with a local registered-office agent, then register the charity | Confirm prior; regulator is the Charities Regulatory Authority (CRA), not the former 'Charity Commission for Ireland'. | verify-rest 2026-10: no EUR 50k registration threshold; regulator is the Charities Regulator; s.137 requires an EEA-resident director or bond | verify-r2 2026-10 (confirmed): The CRO fee leaflet lists EUR 100 to incorporate a new company on a paper Form A1 or EUR 50 online via CORE, consistent with the ~EUR 100 / ~$110 figures.</t>
         </is>
       </c>
       <c r="H133" s="2" t="inlineStr">
@@ -12737,7 +12737,7 @@
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
-          <t>https://www.charitiesregulatory.ie/; https://www.lexology.com/library/detail.aspx?g=68355ef2-1d01-4b55-8bee-7b145fb9cb5c; https://www.cro.ie/; https://www.charitiesregulator.ie/register-with-us/</t>
+          <t>https://www.charitiesregulatory.ie/; https://www.lexology.com/library/detail.aspx?g=68355ef2-1d01-4b55-8bee-7b145fb9cb5c; https://www.cro.ie/; https://www.charitiesregulator.ie/register-with-us/; https://cro.ie/wp-content/uploads/2024/04/Leaflet-4-v6.2.pdf</t>
         </is>
       </c>
       <c r="P133" s="2" t="inlineStr">
@@ -12871,17 +12871,17 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Icelandic registered address and local contact; association needs ~5 members; foundation requires ~ISK 3m endowment and Icelandic management</t>
+          <t>Icelandic registered address and local contact; association needs ~5 members; foundation needs ISK 1.75m minimum endowment (2026) and charter confirmation by the Westfjords District Commissioner</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
-          <t>Association registration about ISK 5,000-10,000; 2-4 weeks. Foundations require a minimum endowment of about ISK 1,000,000; foreigners may found.</t>
+          <t>Association registration ISK 30,000 (Skatturinn); 2-4 weeks. Non-business foundations need a minimum endowment of ISK 1,750,000 (2026) plus an ISK 14,000 charter-confirmation fee; foreigners may found.</t>
         </is>
       </c>
       <c r="G135" s="2" t="inlineStr">
         <is>
-          <t>Documents in Icelandic; tax-deductible status requires registration on Skatturinn's public-benefit register; small bureaucracy but limited English support | verify-rest 2026-10: charitable foundations fall under Act 19/1988 (Act 33/1999 is for business foundations); third-sector Act 110/2021; RSK is now Skatturinn</t>
+          <t>Documents in Icelandic; tax-deductible status requires registration on Skatturinn's public-benefit register; small bureaucracy but limited English support | verify-rest 2026-10: charitable foundations fall under Act 19/1988 (Act 33/1999 is for business foundations); third-sector Act 110/2021; RSK is now Skatturinn | verify-r2 2026-10 (corrected): Skatturinn's fee schedule lists ISK 30,000 to register an association or public-benefit association (félagasamtök / almannaheillafélag), not ISK 5,000-10,000.</t>
         </is>
       </c>
       <c r="H135" s="2" t="inlineStr">
@@ -12896,7 +12896,7 @@
       </c>
       <c r="J135" s="2" t="inlineStr">
         <is>
-          <t>~$50</t>
+          <t>~$240 (ISK 30,000 association registration)</t>
         </is>
       </c>
       <c r="K135" s="2" t="inlineStr">
@@ -12921,7 +12921,7 @@
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
-          <t>https://island.is/en/registration-of-a-philosophical-organisation; https://vlolawfirm.com/guides/how-to-register-a-company-in-iceland; https://www.government.is/library/04-Legislation/Act%20No%2033-1999.pdf; https://www.skatturinn.is/um-rsk/frettir-og-tilkynningar/almannaheillaskra</t>
+          <t>https://island.is/en/registration-of-a-philosophical-organisation; https://vlolawfirm.com/guides/how-to-register-a-company-in-iceland; https://www.government.is/library/04-Legislation/Act%20No%2033-1999.pdf; https://www.skatturinn.is/um-rsk/frettir-og-tilkynningar/almannaheillaskra; https://www.skatturinn.is/fyrirtaekjaskra/gjaldskra/; https://www.skatturinn.is/um-rsk/frettir-og-tilkynningar/skraningargjold-felagasamtaka-og-sambaerilegra-adila-breytast; https://island.is/umsokn-um-stadfestingu-skipulagsskrar-fyrir-nyjan-sjod-eda</t>
         </is>
       </c>
       <c r="P135" s="2" t="inlineStr">
@@ -13060,12 +13060,12 @@
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
-          <t>PRH registration fee about EUR 100; 1-3 months. Foreigners may be members; no residency requirement to found an association.</t>
+          <t>PRH association fee EUR 60 (guided online) or EUR 120 (other filings); 1-3 months. Foreigners may be members; no residency requirement to found an association.</t>
         </is>
       </c>
       <c r="G137" s="2" t="inlineStr">
         <is>
-          <t>Finnish-language requirement for documents and minutes; PRH bureaucracy is the main burden; foundations are hard for a foreign founder | confirm prior; PRH registration fee is about EUR 100. | verify-rest 2026-10: association needs 3 founders; foundation minimum capital EUR 50,000</t>
+          <t>Finnish-language requirement for documents and minutes; PRH bureaucracy is the main burden; foundations are hard for a foreign founder | confirm prior; PRH registration fee is about EUR 100. | verify-rest 2026-10: association needs 3 founders; foundation minimum capital EUR 50,000 | verify-r2 2026-10 (corrected): PRH's current price list charges EUR 60 for an association start-up notification filed through the guided online process and EUR 120 for other electronic or paper filings, not a flat ~EUR 100.</t>
         </is>
       </c>
       <c r="H137" s="2" t="inlineStr">
@@ -13080,7 +13080,7 @@
       </c>
       <c r="J137" s="2" t="inlineStr">
         <is>
-          <t>~$115</t>
+          <t>~$70-140</t>
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr">
@@ -13105,7 +13105,7 @@
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
-          <t>https://yhdistysrekisteri.prh.fi/?userLang=en; https://www.finlex.fi/fi/lainsaadanto/1989/503; https://www.prh.fi/en/price-lists/hinnasto/kasittelymaksut.html; https://www.prh.fi/en/companiesandorganisations/saatiorekisteri/establishmentandregistration.html</t>
+          <t>https://yhdistysrekisteri.prh.fi/?userLang=en; https://www.finlex.fi/fi/lainsaadanto/1989/503; https://www.prh.fi/en/price-lists/hinnasto/kasittelymaksut.html; https://www.prh.fi/en/companiesandorganisations/saatiorekisteri/establishmentandregistration.html; https://prh.fi/en/companiesandorganisations/yhdistysrekisteri/perustaminen/start-up_notification.html</t>
         </is>
       </c>
       <c r="P137" s="2" t="inlineStr">
@@ -13157,7 +13157,7 @@
       </c>
       <c r="G138" s="2" t="inlineStr">
         <is>
-          <t>Straightforward online registration with Bolagsverket, English widely understood; a Swedish bank account for the entity typically requires a personal/D-number for the signatory | verify-rest 2026-10: ideell förening gets its org. number from Skatteverket free; Bolagsverket fee applies only to economic associations</t>
+          <t>Straightforward online registration with Bolagsverket, English widely understood; a Swedish bank account for the entity typically requires a personal/D-number for the signatory | verify-rest 2026-10: ideell förening gets its org. number from Skatteverket free; Bolagsverket fee applies only to economic associations | verify-r2 2026-10 (confirmed): Registering an ekonomisk förening with Bolagsverket costs SEK 1,900 through the verksamt.se e-service (SEK 2,200 on paper) in 2026, matching the cell.</t>
         </is>
       </c>
       <c r="H138" s="2" t="inlineStr">
@@ -13197,7 +13197,7 @@
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
-          <t>https://bolagsverket.se/en/foretag/aktiebolag/startaaktiebolag.479.html; https://membly.app/en/blog/how-to-start-an-association; https://www.verksamt.se/en/setting-up/associations/economic-association; https://www.skatteverket.se/foreningar/driva/ideellforening/</t>
+          <t>https://bolagsverket.se/en/foretag/aktiebolag/startaaktiebolag.479.html; https://membly.app/en/blog/how-to-start-an-association; https://www.verksamt.se/en/setting-up/associations/economic-association; https://www.skatteverket.se/foreningar/driva/ideellforening/; https://www.skatteverket.se/foreningar/driva/ekonomiskforeningellerbostadsrattsforening/startaenekonomiskforening.4.6a6688231259309ff1f800028168.html; https://www.faronline.se/dokument/rb_ekonomiskforening/; https://www.lansstyrelsen.se/uppsala/samhalle/stiftelser/bilda-och-registrera-stiftelse.html</t>
         </is>
       </c>
       <c r="P138" s="2" t="inlineStr">
@@ -13249,7 +13249,7 @@
       </c>
       <c r="G139" s="2" t="inlineStr">
         <is>
-          <t>Association name and documents must be in Danish; CVR registration itself is easy; Danish-controlled foundation rules make the foundation route hard for a foreigner | verify-rest 2026-10: LB 938/2012 superseded by consolidated LBK nr. 2020 of 11/12/2020</t>
+          <t>Association name and documents must be in Danish; CVR registration itself is easy; Danish-controlled foundation rules make the foundation route hard for a foreigner | verify-rest 2026-10: LB 938/2012 superseded by consolidated LBK nr. 2020 of 11/12/2020 | verify-r2 2026-10 (corrected): Erhvervsstyrelsen guidance says registering a voluntary association (frivillig forening) for a CVR number via Virk is free, renewed every 3 years, and requires MitID, so the ~$20 fee was wrong.</t>
         </is>
       </c>
       <c r="H139" s="2" t="inlineStr">
@@ -13264,7 +13264,7 @@
       </c>
       <c r="J139" s="2" t="inlineStr">
         <is>
-          <t>~$20</t>
+          <t>$0 (CVR registration of a voluntary association is free)</t>
         </is>
       </c>
       <c r="K139" s="2" t="inlineStr">
@@ -13289,7 +13289,7 @@
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
-          <t>https://erhvervsstyrelsen.dk/vejledning-om-foreninger; https://businessindenmark.virk.dk/guidance/services-contact-point/Establish-a-business-in-Denmark/; https://virk.dk/myndigheder/stat/ERST/selvbetjening/Frivillige_foreninger/; https://www.retsinformation.dk/api/pdf/209400</t>
+          <t>https://erhvervsstyrelsen.dk/vejledning-om-foreninger; https://businessindenmark.virk.dk/guidance/services-contact-point/Establish-a-business-in-Denmark/; https://virk.dk/myndigheder/stat/ERST/selvbetjening/Frivillige_foreninger/; https://www.retsinformation.dk/api/pdf/209400; https://www.retsinformation.dk/eli/lta/2020/2020/pdf</t>
         </is>
       </c>
       <c r="P139" s="2" t="inlineStr">
@@ -13433,7 +13433,7 @@
       </c>
       <c r="G141" s="2" t="inlineStr">
         <is>
-          <t>Associations and foundations share one law (2003); e-filing with an EU e-signature avoids the notary, otherwise notarised signatures force an in-person visit or a local representative | NVO registers electronically via e-portals; no notary step needed. Real barriers: Latvian-resident board requirement plus local address and e-ID | verify-rest 2026-10: law date corrected to 2003/2004; no '2016 Nonprofit Organizations Law' exists; state fee EUR 11.38 (Cabinet Reg. 308)</t>
+          <t>Associations and foundations share one law (2003); e-filing with an EU e-signature avoids the notary, otherwise notarised signatures force an in-person visit or a local representative | NVO registers electronically via e-portals; no notary step needed. Real barriers: local address and e-ID (no board-residence rule in law) | verify-rest 2026-10: law date corrected to 2003/2004; no '2016 Nonprofit Organizations Law' exists; state fee EUR 11.38 (Cabinet Reg. 308) | verify-r2 2026-10 (corrected): Cabinet Regulation No.</t>
         </is>
       </c>
       <c r="H141" s="2" t="inlineStr">
@@ -13443,7 +13443,7 @@
       </c>
       <c r="I141" s="2" t="inlineStr">
         <is>
-          <t>Latvian address, Latvian-resident board, and Latvian e-ID for filing — a local representative is mandatory</t>
+          <t>Latvian address and Latvian-language documents; without a Latvian/EU e-signature, notarised signatures are needed, so a local representative is practical (no board residency rule)</t>
         </is>
       </c>
       <c r="J141" s="2" t="inlineStr">
@@ -13473,7 +13473,7 @@
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
-          <t>https://uronline.lv/en/membership/; https://cms.law/en/int/expert-guides/cms-expert-guide-on-taxation-of-charity-donations-for-eu/latvia; https://lexfinance.lv/en/blogs/company-registration-in-latvia-types-of-companies-registration-process-required-documents-; https://latvija.gov.lv/Services/46744; https://likumi.lv/ta/id/81050</t>
+          <t>https://uronline.lv/en/membership/; https://cms.law/en/int/expert-guides/cms-expert-guide-on-taxation-of-charity-donations-for-eu/latvia; https://lexfinance.lv/en/blogs/company-registration-in-latvia-types-of-companies-registration-process-required-documents-; https://latvija.gov.lv/Services/46744; https://likumi.lv/ta/id/81050; https://likumi.lv/ta/id/87233; https://likumi.lv/ta/en/en/id/81050-associations-and-foundations-law</t>
         </is>
       </c>
       <c r="P141" s="2" t="inlineStr">
@@ -13709,7 +13709,7 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>The most straightforward of the four for a foreign founder: no citizenship/residency requirement for the founder, and no fixed minimum capital. However, to be treated as an entity of public interest (required for tax-exempt status and grants) it needs an endowment and approval by the relevant authority. English filings are not routine; use a Portuguese lawyer. A local office can be provided by a law firm or registered agent, which is what keeps this at medium rather than easy. | verify-rest 2026-10: 'no statutory minimum endowment' corrected — Portaria 75/2013 sufficiency threshold applies; 'Instituto' is not a separate private form</t>
+          <t>The most straightforward of the four for a foreign founder: no citizenship/residency requirement for the founder, and no fixed minimum capital. However, to be treated as an entity of public interest (required for tax-exempt status and grants) it needs an endowment and approval by the relevant authority. English filings are not routine; use a Portuguese lawyer. A local office can be provided by a law firm or registered agent, which is what keeps this at medium rather than easy. | verify-rest 2026-10: 'no statutory minimum endowment' corrected — Portaria 75/2013 sufficiency threshold applies; 'Instituto' is not a separate private form | verify-r2 2026-10 (confirmed): Lei 24/2012 (Lei-Quadro das Fundações) remains in force as amended by Leis 150/2015, 36/2021 and 67/2021;</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr">
@@ -13749,7 +13749,7 @@
       </c>
       <c r="O144" s="2" t="inlineStr">
         <is>
-          <t>https://www.lvpadvogados.com/public-utility-status-in-portugal-what-it-is-who-can-apply-and-why-it-matters; https://imperiallegal.com/company-registration-portugal/; https://www.icnl.org/resources/research/ijnl/a-comparative-overview-of-public-benefit-status-in-europe-2; https://diariodarepublica.pt/dr/detalhe/portaria/75-2013-258694</t>
+          <t>https://www.lvpadvogados.com/public-utility-status-in-portugal-what-it-is-who-can-apply-and-why-it-matters; https://imperiallegal.com/company-registration-portugal/; https://www.icnl.org/resources/research/ijnl/a-comparative-overview-of-public-benefit-status-in-europe-2; https://diariodarepublica.pt/dr/detalhe/portaria/75-2013-258694; https://diariodarepublica.pt/dr/detalhe/lei/24-2012-179571; https://diariodarepublica.pt/dr/detalhe/lei/67-2021-170175410; https://diariodarepublica.pt/dr/detalhe/despacho/2820-2025-909307266</t>
         </is>
       </c>
       <c r="P144" s="2" t="inlineStr">
@@ -13893,7 +13893,7 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>The Vatican does not operate a conventional commercial-law or charity-registration framework open to foreign founders. There is no public registry an Australian-resident can simply file into. Charitable or philanthropic activity on Vatican territory is established by canonical/pontifical act (e.g., erection or recognition of a pontifical work), which requires a direct relationship with the appropriate Holy See authority and is typically reserved for Church-linked bodies. For a private foreign founder there is effectively no independent, self-service charitable-entity route; the realistic option is to establish the charity in Italy (or elsewhere) and, if relevant, seek a canonical relationship with the Holy See. | confirm prior: no ordinary charity registry, no fixed fee or timeline, very hard difficulty all accurate.</t>
+          <t>The Vatican does not operate a conventional commercial-law or charity-registration framework open to foreign founders. There is no public registry an Australian-resident can simply file into. Charitable or philanthropic activity on Vatican territory is established by canonical/pontifical act (e.g., erection or recognition of a pontifical work), which requires a direct relationship with the appropriate Holy See authority and is typically reserved for Church-linked bodies. For a private foreign founder there is effectively no independent, self-service charitable-entity route; the realistic option is to establish the charity in Italy (or elsewhere) and, if relevant, seek a canonical relationship with the Holy See. | confirm prior: no ordinary charity registry, no fixed fee or timeline, very hard difficulty all accurate. | verify-r2 2026-10 (confirmed): Vatican City State has no public charity or company registry open to private filers;</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr">
@@ -13933,7 +13933,7 @@
       </c>
       <c r="O146" s="2" t="inlineStr">
         <is>
-          <t>https://www.expanship.com/va/blog/types-of-companies-in-vatican-city; https://en.wikipedia.org/wiki/Holy_See</t>
+          <t>https://www.expanship.com/va/blog/types-of-companies-in-vatican-city; https://en.wikipedia.org/wiki/Holy_See; https://www.vatican.va/news_services/press/documentazione/documents/sp_ss_scv/informazione_generale/legge-fondamentale_en.html</t>
         </is>
       </c>
       <c r="P146" s="2" t="inlineStr">
@@ -14169,7 +14169,7 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>Legally one of the easiest for foreigners in the region, but heavy Arabic-only bureaucracy, bank-account opening friction, and macro instability (currency, banking) make practical setup harder; most internationals use a local registered partner or a foundation | Confirm prior: foreigners may found/direct, notification regime, 2-6 weeks; banking is the practical friction | verify-rest 2026-10: 'no nationality rule' softened — foreign-controlled associations may require authorization</t>
+          <t>Legally one of the easiest for foreigners in the region, but heavy Arabic-only bureaucracy, bank-account opening friction, and macro instability (currency, banking) make practical setup harder; most internationals use a local registered partner or a foundation | Confirm prior: foreigners may found/direct, notification regime, 2-6 weeks; banking is the practical friction | verify-rest 2026-10: 'no nationality rule' softened — foreign-controlled associations may require authorization | verify-r2 2026-10 (confirmed): Circular 10/AM/2006 confirms associations are formed by notification to the Ministry of Interior and Municipalities, which issues a receipt (ilm wa khabar) after reviewing bylaws, founder names and judicial records, and refers the associat…</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr">
@@ -14261,7 +14261,7 @@
       </c>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>Civil-society registration resumed after 2025 transition (586 NGOs registered by Feb 2025) but framework unstable; sanctions exposure for foreign founders and their banks; English support effectively unavailable; advise against direct formation | verify-rest 2026-10: no new associations law enacted — Law 93/1958 still governs</t>
+          <t>Civil-society registration resumed after 2025 transition (586 NGOs registered by Feb 2025) but framework unstable; sanctions exposure for foreign founders and their banks; English support effectively unavailable; advise against direct formation | verify-rest 2026-10: no new associations law enacted — Law 93/1958 still governs | verify-r2 2026-10 (confirmed): A September 2026 position paper says the Ministry of Social Affairs and Labor has only completed an initial draft of a law to replace Law 93 of 1958, which has not yet gone to the People's Assembly.</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr">
@@ -14301,7 +14301,7 @@
       </c>
       <c r="O150" s="2" t="inlineStr">
         <is>
-          <t>https://english.enabbaladi.net/archives/2025/10/syrian-ngos-oppose-restrictions-on-funding-approvals/; https://damascusinstitute.org/en/researches/syrian-organisations-and-associations-building-a-national-strategy-from-the-legacy-of-tyranny/; https://zd-consultation.com/en/licensing-international-ngos-syria-requirements/; https://stj-sy.org/wp-content/uploads/2026/09/From-State-Control-to-Safeguarding-Independence-Essential-Safeguards-for-Syrias-New-Law-on-Associations.pdf</t>
+          <t>https://english.enabbaladi.net/archives/2025/10/syrian-ngos-oppose-restrictions-on-funding-approvals/; https://damascusinstitute.org/en/researches/syrian-organisations-and-associations-building-a-national-strategy-from-the-legacy-of-tyranny/; https://zd-consultation.com/en/licensing-international-ngos-syria-requirements/; https://stj-sy.org/wp-content/uploads/2026/09/From-State-Control-to-Safeguarding-Independence-Essential-Safeguards-for-Syrias-New-Law-on-Associations.pdf; https://syriacpress.com/blog/2026/02/06/syriac-cultural-association-granted-nationwide-operating-license-in-syria/</t>
         </is>
       </c>
       <c r="P150" s="2" t="inlineStr">
@@ -14348,12 +14348,12 @@
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
-          <t>Fees low, but registration requires Iraqi-national or Iraq-resident founders, so non-resident foreigners cannot found directly. Official processing times unpublished.</t>
+          <t>No statutory fee (Law 12/2010 Art. 7 exempts applications from duties), but founders must be Iraqi nationals or Iraq residents, so non-resident foreigners cannot found directly. Statutory: 7-day decision on establishment, certificate within 30 days of a complete application.</t>
         </is>
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>Resident-expat route is the standard workaround (Iraqi-resident staff as founders); foreign funding rules restrict donor channels; English commonly understood in NGO sector but filings in Arabic; security considerations for in-person steps | Confirm prior: Law 12/2010 governs (new draft NGO law with 5 founders approved but 12/2010 still applied) | verify-rest 2026-10: registering body is the Council of Ministers Secretariat NGO Department; no 10-founder minimum (3 resident/national founders)</t>
+          <t>Resident-expat route is the standard workaround (Iraqi-resident staff as founders); foreign funding rules restrict donor channels; English commonly understood in NGO sector but filings in Arabic; security considerations for in-person steps | Confirm prior: Law 12/2010 governs (new draft NGO law with 5 founders approved but 12/2010 still applied) | verify-rest 2026-10: registering body is the Council of Ministers Secretariat NGO Department; no 10-founder minimum (3 resident/national founders) | verify-r2 2026-10 (corrected): Law 12 of 2010 requires an application signed by at least three founders who are Iraqi nationals or residents (Arts.</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr">
@@ -14363,12 +14363,12 @@
       </c>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>Founders must be Iraqi nationals (min 10), local board/address, Arabic filings, MoSAL activity approvals</t>
+          <t>Founders (min. 3) must be Iraqi nationals or Iraq residents; local address, Arabic filings with the Council of Ministers NGO Department</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr">
         <is>
-          <t>~$200-1,000</t>
+          <t>$0 statutory (Art. 7 exemption); legal/translation costs extra</t>
         </is>
       </c>
       <c r="K151" s="2" t="inlineStr">
@@ -14383,7 +14383,7 @@
       </c>
       <c r="M151" s="2" t="inlineStr">
         <is>
-          <t>Foreign funding channeled via registered Iraqi entity with MoSAL approvals; donor-channel restrictions apply</t>
+          <t>Foreign funding channeled via registered Iraqi entity with approvals from the Council of Ministers NGO Department; donor-channel restrictions apply</t>
         </is>
       </c>
       <c r="N151" s="2" t="inlineStr">
@@ -15631,7 +15631,7 @@
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Moroccan registered office, Arabic statutes, wilaya/provincial governor approval; foreign founders permitted.</t>
+          <t>Moroccan registered office, Arabic statutes; declaration filed with the local administrative authority (caïdat/pashalik), which issues a receipt; declaratory regime, not approval; foreign founders permitted.</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -15641,7 +15641,7 @@
       </c>
       <c r="G165" s="2" t="inlineStr">
         <is>
-          <t>Governor discretion can delay approvals; most expats register via a local address agent; Arabic mandatory. | Confirm prior with correction: governing text is Dahir 1-58-376 of 1958 (not 'Law 1956'); foreign founders permitted; 1-3 months realistic | verify-rest 2026-10: cooperatives governed by Law 112-12 (not 19-00)</t>
+          <t>Governor discretion can delay approvals; most expats register via a local address agent; Arabic mandatory. | Confirm prior with correction: governing text is Dahir 1-58-376 of 1958 (not 'Law 1956'); foreign founders permitted; 1-3 months realistic | verify-rest 2026-10: cooperatives governed by Law 112-12 (not 19-00) | verify-r2 2026-10 (corrected): Under Dahir 1-58-376 of 1958 as amended by Law 75-00, an association is formed by a declaration filed at the local administrative authority for its seat, which issues a stamped provisional receipt;</t>
         </is>
       </c>
       <c r="H165" s="2" t="inlineStr">
@@ -15651,7 +15651,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>Registered office + Arabic statutes; governor discretion can delay; local address agent usually needed</t>
+          <t>Registered office + Arabic statutes; local authorities can delay or withhold the declaration receipt; local address agent usually needed</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -15681,7 +15681,7 @@
       </c>
       <c r="O165" s="2" t="inlineStr">
         <is>
-          <t>https://9anonai.com/en/blog/ngo-establishment-law-morocco; https://www.lexmundi.com/guides/social-enterprise-law-surveys/jurisdictions/africa/morocco/; https://www.icnl.org/research/library/morocco_act-2002-en/; https://adala.justice.gov.ma/api/uploads/2024/04/09/Cooperatives-1712660938413.pdf</t>
+          <t>https://9anonai.com/en/blog/ngo-establishment-law-morocco; https://www.lexmundi.com/guides/social-enterprise-law-surveys/jurisdictions/africa/morocco/; https://www.icnl.org/research/library/morocco_act-2002-en/; https://adala.justice.gov.ma/api/uploads/2024/04/09/Cooperatives-1712660938413.pdf; https://www.hrw.org/reports/morocco1009frsumandrecs.pdf; https://capacity4dev.europa.eu/media/128043/download/0198162b-39bc-4350-b58b-05ff75271e2a_en</t>
         </is>
       </c>
       <c r="P165" s="2" t="inlineStr">
@@ -15917,7 +15917,7 @@
       </c>
       <c r="G168" s="2" t="inlineStr">
         <is>
-          <t>2021 reform liberalised funding and registration, but foreigners cannot directly form a domestic charity; security clearance applies; Amharic/English documents. | verify-rest 2026-10: registrar is ACSO; resident foreigners may co-found local CSOs, non-residents cannot</t>
+          <t>2021 reform liberalised funding and registration, but foreigners cannot directly form a domestic charity; security clearance applies; Amharic/English documents. | verify-rest 2026-10: registrar is ACSO; resident foreigners may co-found local CSOs, non-residents cannot | verify-r2 2026-10 (corrected): CSO Proclamation No.</t>
         </is>
       </c>
       <c r="H168" s="2" t="inlineStr">
@@ -15927,7 +15927,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>Domestic CSOs require Ethiopian-national founders/members; a foreign founder can only register a foreign NGO office, which needs a local entity and CSO Agency approval.</t>
+          <t>Local CSOs may be founded only by Ethiopians and/or Ethiopia-resident foreigners; a non-resident founder must use a partner or register a foreign CSO with ACSO, which needs local representation.</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -15947,7 +15947,7 @@
       </c>
       <c r="M168" s="2" t="inlineStr">
         <is>
-          <t>2021 reform allows foreign funding of registered CSOs, but funds must flow through the CSO Agency/ACSO channel; no direct foreign donor license.</t>
+          <t>2021 reform allows foreign funding of registered CSOs, but funds must flow through the ACSO (Authority for Civil Society Organizations) channel; no direct foreign donor license.</t>
         </is>
       </c>
       <c r="N168" s="2" t="inlineStr">
@@ -15957,12 +15957,12 @@
       </c>
       <c r="O168" s="2" t="inlineStr">
         <is>
-          <t>https://cof.org/country-notes/nonprofit-law-ethiopia; https://www.primelaw.law/insights/ngo-lawyer-ethiopia-cso-guide; https://www.icnl.org/resources/civic-freedom-monitor/ethiopia; https://www.csrc-et.org/resources/cso-registration-guide; https://www.jurist.org/news/2025/08/ethiopia-urged-to-abandon-proposed-changes-to-civil-society-organization-law</t>
+          <t>https://cof.org/country-notes/nonprofit-law-ethiopia; https://www.primelaw.law/insights/ngo-lawyer-ethiopia-cso-guide; https://www.icnl.org/resources/civic-freedom-monitor/ethiopia; https://www.csrc-et.org/resources/cso-registration-guide; https://www.jurist.org/news/2025/08/ethiopia-urged-to-abandon-proposed-changes-to-civil-society-organization-law; https://www.hrw.org/news/2025/07/29/ethiopia-proposed-legal-changes-threaten-civil-society</t>
         </is>
       </c>
       <c r="P168" s="2" t="inlineStr">
         <is>
-          <t>Proclamation 1113/2019 Arts. 72-73: annual performance and accounting report to the CSO Agency within 3 months of fiscal year-end, with certified audit in the same period; failure can lead to suspension or revocation.</t>
+          <t>Proclamation 1113/2019 Arts. 72-73: annual performance and accounting report to ACSO within 3 months of fiscal year-end, with certified audit in the same period; failure can lead to suspension or revocation.</t>
         </is>
       </c>
       <c r="Q168" s="2" t="inlineStr">
@@ -16101,7 +16101,7 @@
       </c>
       <c r="G170" s="2" t="inlineStr">
         <is>
-          <t>Tight, security-driven regulation in a small country; English sometimes tolerated in practice; foreign aid actors mostly work through local partners. | Confirm prior: association law requires local involvement; cost ~$100-300 and 1-3 months plausible.</t>
+          <t>Tight, security-driven regulation in a small country; English sometimes tolerated in practice; foreign aid actors mostly work through local partners. | Confirm prior: association law requires local involvement; cost ~$100-300 and 1-3 months plausible. | verify-r2 2026-10 (confirmed): US State Dept 2021 report confirms registration of foreign organizations sits with the Ministry of Interior, with extensive background checks and restrictions on foreign groups.</t>
         </is>
       </c>
       <c r="H170" s="2" t="inlineStr">
@@ -16141,7 +16141,7 @@
       </c>
       <c r="O170" s="2" t="inlineStr">
         <is>
-          <t>https://www.ecoi.net/en/countries/djibouti/national-laws/; https://2021-2025.state.gov/reports/2021-report-on-international-religious-freedom/djibouti/; https://www.womenconnect.org/web/djibouti/business-registration/-/asset_publisher/ObbONgnQXwfM/content/les-principaux-types-de-societe-enregistres-au-guichet-unique; https://www.nyulawglobal.org/globalex/djibouti1.html</t>
+          <t>https://www.ecoi.net/en/countries/djibouti/national-laws/; https://2021-2025.state.gov/reports/2021-report-on-international-religious-freedom/djibouti/; https://www.womenconnect.org/web/djibouti/business-registration/-/asset_publisher/ObbONgnQXwfM/content/les-principaux-types-de-societe-enregistres-au-guichet-unique; https://www.nyulawglobal.org/globalex/djibouti1.html; https://www.eci.net/world/ngos/journals/202105-djibouti.html</t>
         </is>
       </c>
       <c r="P170" s="2" t="inlineStr">
@@ -16173,7 +16173,7 @@
       </c>
       <c r="C171" s="2" t="inlineStr">
         <is>
-          <t>NGO registered administratively with the Ministry of Planning, Investment and Economic Development (federal NGO Bill 2019 still a draft); national and international NGOs; domestic associations under regional law</t>
+          <t>NGOs registered with the Ministry of Interior, Federal Affairs and Reconciliation (federal, Mogadishu); 2019 federal NGO Bill (cabinet-passed Dec 2019) still not enacted as of 2026; international NGOs; domestic associations under regional law (Puntland Law 3/2016, Somaliland Law 43/2010)</t>
         </is>
       </c>
       <c r="D171" s="6" t="inlineStr">
@@ -16193,7 +16193,7 @@
       </c>
       <c r="G171" s="2" t="inlineStr">
         <is>
-          <t>Severe insecurity and fragmented federal registries (Puntland, Somaliland, South West each have their own); foreign staff face high security risk. | Confirm prior: severe insecurity and fragmented registries; domestic charities need Somali founders; 3-6 months is optimistic, extend to 12. | verify-rest 2026-10: federal 'NGO Act 2019' is still a draft bill — registration is administrative via MoPIED</t>
+          <t>Severe insecurity and fragmented federal registries (Puntland, Somaliland, South West each have their own); foreign staff face high security risk. | Confirm prior: severe insecurity and fragmented registries; domestic charities need Somali founders; 3-6 months is optimistic, extend to 12. | verify-rest 2026-10: federal 'NGO Act 2019' is still a draft bill — registration is administrative via MoPIED | verify-r2 2026-10 (corrected): ICNL Civic Freedom Monitor (2026) shows NGO registration in Somalia is handled by the Ministry of Interior, Federal Affairs and Reconciliation, not the Ministry of Planning, Investment and Economic Development.</t>
         </is>
       </c>
       <c r="H171" s="2" t="inlineStr">
@@ -16285,7 +16285,7 @@
       </c>
       <c r="G172" s="2" t="inlineStr">
         <is>
-          <t>De facto state without international recognition: banking, sanctions-compliance and repatriation risk; the civil-society registry is relatively functional and stable. | Confirm prior: 2010 NGO law (not 2005) governs; registry is relatively functional; cost 1-3 months plausible. | verify-rest 2026-10: law is No. 43/2010 (not 'Decree 82/11'); registrar is the Ministry of National Planning and Development</t>
+          <t>De facto state without international recognition: banking, sanctions-compliance and repatriation risk; the civil-society registry is relatively functional and stable. | Confirm prior: 2010 NGO law (not 2005) governs; registry is relatively functional; cost 1-3 months plausible. | verify-rest 2026-10: law is No. 43/2010 (not 'Decree 82/11'); registrar is the Ministry of National Planning and Development | verify-r2 2026-10 (confirmed): ICNL confirms Somaliland's NGO Law No.</t>
         </is>
       </c>
       <c r="H172" s="2" t="inlineStr">
@@ -16325,7 +16325,7 @@
       </c>
       <c r="O172" s="2" t="inlineStr">
         <is>
-          <t>https://www.icnl.org/research/library/somalia_ngolaw/; https://www.icnl.org/research/library/somalia_ingos/; http://www.somalilandlaw.com/somaliland_ngos_law.html; https://slministryofplanning.org/documents/Manual-for-International-Org.pdf</t>
+          <t>https://www.icnl.org/research/library/somalia_ngolaw/; https://www.icnl.org/research/library/somalia_ingos/; http://www.somalilandlaw.com/somaliland_ngos_law.html; https://slministryofplanning.org/documents/Manual-for-International-Org.pdf; https://www.icnl.org/resources/civic-freedom-monitor/somalia</t>
         </is>
       </c>
       <c r="P172" s="2" t="inlineStr">
@@ -16377,7 +16377,7 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>Post-conflict, high security risk, weak institutions; most international actors work through established partners or missions. | Confirm prior, update: governing law is NGO Act 2016 (not 2009); 2023 amendment bill adds 80% local staff requirement; 6-12 months realistic. | verify-rest 2026-10: RRC fees — 2017: US$500 national / US$3,500 international; 2018 waiver left US$200/1,000 renewal fees</t>
+          <t>Post-conflict, high security risk, weak institutions; most international actors work through established partners or missions. | Confirm prior, update: governing law is NGO Act 2016 (not 2009); 2023 amendment bill adds 80% local staff requirement; 6-12 months realistic. | verify-rest 2026-10: RRC fees — 2017: US$500 national / US$3,500 international; 2018 waiver left US$200/1,000 renewal fees | verify-r2 2026-10 (confirmed): The NGO Forum coordination FAQ confirms the NGO Act 2016 and the RRC as the registration body.</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
@@ -17021,7 +17021,7 @@
       </c>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>The trust route is the simplest expat pathway (no citizen-quota for trust deed). Foreign funding requires Social Welfare Council approval, which adds time and discretion. | verify-rest 2026-10: no general 'Trust Act 2000' — Civil Code 2017 governs trusts; foreign-settlor trust carries a US$1M threshold; NGO needs 7 Nepali founders</t>
+          <t>The trust route is the simplest expat pathway (no citizen-quota for trust deed). Foreign funding requires Social Welfare Council approval, which adds time and discretion. | verify-rest 2026-10: no general 'Trust Act 2000' — Civil Code 2017 governs trusts; foreign-settlor trust carries a US$1M threshold; NGO needs 7 Nepali founders | verify-r2 2026-10 (confirmed): The SWC's official page confirms Social Welfare Council affiliation under the Social Welfare Act 2049 for INGOs.</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr">
@@ -17297,7 +17297,7 @@
       </c>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>Most expats use the MIRA-registered public trust with local resident trustees and a local manager. English used in filings; annual returns and audited accounts required by MIRA. | confirm prior - public trust registered with Ministry of Justice; MIRA approval (MIRA 103) is for tax exemption, not registration. | verify-rest 2026-10: Associations Act 3/2022 now governs; MIRA = Maldives Inland Revenue Authority (tax approval, not trust registration)</t>
+          <t>Most expats use the MIRA-registered public trust with local resident trustees and a local manager. English used in filings; annual returns and audited accounts required by MIRA. | confirm prior - public trust registered with Ministry of Justice; MIRA approval (MIRA 103) is for tax exemption, not registration. | verify-rest 2026-10: Associations Act 3/2022 now governs; MIRA = Maldives Inland Revenue Authority (tax approval, not trust registration) | verify-r2 2026-10 (confirmed): Associations Act No.</t>
         </is>
       </c>
       <c r="H183" s="2" t="inlineStr">
@@ -17389,7 +17389,7 @@
       </c>
       <c r="G184" s="2" t="inlineStr">
         <is>
-          <t>Most structured path in West Africa but multi-layered; CAC incorporation, SCUML and (for INGOs) National Planning Commission registration are the foreigner bottlenecks; English language; strong expat NGO sector in Lagos/Abuja | verify-rest 2026-10: 'NCMM' and 'Operational Readiness Certificate' layers unverifiable — replaced by SCUML + NPC; Foreign Aid Regulation Bill 2026 (SB.1034) is pending, not law</t>
+          <t>Most structured path in West Africa but multi-layered; CAC incorporation, SCUML and (for INGOs) National Planning Commission registration are the foreigner bottlenecks; English language; strong expat NGO sector in Lagos/Abuja | verify-rest 2026-10: 'NCMM' and 'Operational Readiness Certificate' layers unverifiable — replaced by SCUML + NPC; Foreign Aid Regulation Bill 2026 (SB.1034) is pending, not law | verify-r2 2026-10 (confirmed): The 2018 updated compliance manual for NGOs confirms CAC registration of incorporated trustees under the Companies and Allied Matters Act and states explicitly that SCUML registration is free.</t>
         </is>
       </c>
       <c r="H184" s="2" t="inlineStr">
@@ -17573,7 +17573,7 @@
       </c>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>2022 OSC law modernized the regime (declaration for associations, authorization for foreign-funded NGOs); French-only bureaucracy; Abidjan has active local law firms that handle expat NGO setups | OSC framework now Ordinance n° 2024-368 (12 June 2024) replacing Law 2022-443; eDA digital declaration portal live | verify-rest 2026-10: stale 'Law 2022-443' reference removed; Ordonnance 2024-368 ratified by National Assembly (Mar 2025) and Senate (Apr 2025)</t>
+          <t>2022 OSC law modernized the regime (declaration for associations, authorization for foreign-funded NGOs); French-only bureaucracy; Abidjan has active local law firms that handle expat NGO setups | OSC framework now Ordinance n° 2024-368 (12 June 2024) replacing Law 2022-443; eDA digital declaration portal live | verify-rest 2026-10: stale 'Law 2022-443' reference removed; Ordonnance 2024-368 ratified by National Assembly (Mar 2025) and Senate (Apr 2025) | verify-r2 2026-10 (confirmed): The official Journal Officiel text of Ordonnance n° 2024-368 du 12 juin 2024 confirms the declaration regime, filing at the Ministry of Territorial Administration/prefecture, a 2-month stand-down before activity, and the Foreign Affairs mi…</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr">
@@ -17665,7 +17665,7 @@
       </c>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>One of the more open, stable regimes in francophone West Africa; French-only; Cotonou has NGOs/lawyers familiar with expat filings | New Decree 2025-636 (8 Oct 2025) regulates foreign NGO authorization and compliance declarations via CatIS portal | verify-rest 2026-10: stale 'Law 2015-04' reference removed; declaration is now exclusively online under Décret 2025-575</t>
+          <t>One of the more open, stable regimes in francophone West Africa; French-only; Cotonou has NGOs/lawyers familiar with expat filings | New Decree 2025-636 (8 Oct 2025) regulates foreign NGO authorization and compliance declarations via CatIS portal | verify-rest 2026-10: stale 'Law 2015-04' reference removed; declaration is now exclusively online under Décret 2025-575 | verify-r2 2026-10 (confirmed): Benin's official government gazette confirms Law No.</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr">
@@ -17757,7 +17757,7 @@
       </c>
       <c r="G188" s="2" t="inlineStr">
         <is>
-          <t>Administrative practice varies by préfecture; some steps in practice require in-person filing at the Mairie or prefecture in Lomé; French-only | verify-rest 2026-10: unverifiable 'Law 2000-17' removed; Oct 2024 circular requires foreign NGOs to obtain recognition (6-month regularisation window)</t>
+          <t>Administrative practice varies by préfecture; some steps in practice require in-person filing at the Mairie or prefecture in Lomé; French-only | verify-rest 2026-10: unverifiable 'Law 2000-17' removed; Oct 2024 circular requires foreign NGOs to obtain recognition (6-month regularisation window) | verify-r2 2026-10 (confirmed): Décret 2022-002/PR (5 January 2022) and the 7 October 2024 circular are confirmed, with recognition now required before foreign associations can sign partnership agreements.</t>
         </is>
       </c>
       <c r="H188" s="2" t="inlineStr">
@@ -17941,7 +17941,7 @@
       </c>
       <c r="G190" s="2" t="inlineStr">
         <is>
-          <t>Political instability (2020–2024 coups, ongoing conflict); security situation in many regions makes on-ground operations difficult; Bamako filings are French-only | Current association law is n° 04-038/ANRM (5 Aug 2004), which repealed Law 01-019 (2001) cited in prior context | verify-rest 2026-10: repealed Law 2001-019 reference removed</t>
+          <t>Political instability (2020–2024 coups, ongoing conflict); security situation in many regions makes on-ground operations difficult; Bamako filings are French-only | Current association law is n° 04-038/ANRM (5 Aug 2004), which repealed Law 01-019 (2001) cited in prior context | verify-rest 2026-10: repealed Law 2001-019 reference removed | verify-r2 2026-10 (confirmed): ICNL confirms Loi n° 04-038/AN-RM du 5 août 2004 governs associations with a declaration regime, foreign associations require prior authorization from the Ministry of Local Government, and an accord-cadre (Arts.</t>
         </is>
       </c>
       <c r="H190" s="2" t="inlineStr">
@@ -18033,7 +18033,7 @@
       </c>
       <c r="G191" s="2" t="inlineStr">
         <is>
-          <t>2010 association law uses a declaration regime (more open than the old authorization system); French-only; military rule since 2021 adds some political risk but NGO sector remains active | Association regime rests on loi 013/05 (2005) + L013 NGO text; prior 'loi L/2010/004 (2010)' not confirmed | verify-rest 2026-10: 'Law L/2010/004' removed; Sept 2024 suspension of NGO agréments noted</t>
+          <t>2010 association law uses a declaration regime (more open than the old authorization system); French-only; military rule since 2021 adds some political risk but NGO sector remains active | Association regime rests on loi 013/05 (2005) + L013 NGO text; prior 'loi L/2010/004 (2010)' not confirmed | verify-rest 2026-10: 'Law L/2010/004' removed; Sept 2024 suspension of NGO agréments noted | verify-r2 2026-10 (confirmed): MATD's official site confirms loi 013/05 remains the law governing the association regime, with regional modernization workshops running in late 2025.</t>
         </is>
       </c>
       <c r="H191" s="2" t="inlineStr">
@@ -18073,7 +18073,7 @@
       </c>
       <c r="O191" s="2" t="inlineStr">
         <is>
-          <t>https://matd.gov.gn/dnarproma-ouverture-des-ateliers-regionaux-sur-lactualisation-de-la-loi-013-05-a-kindia-et-kankan/; https://guineelex.com/decrets-arretes/arrete-a-2022-3220-matd-cab-sgg; https://www.amnestyguinee.org/wp-content/uploads/2020/09/Loi-L013-ONG-Guinee.pdf; https://guineenews.org/2024/09/02/guinee-le-gouvernement-suspend-la-delivrance-des-agrements-aux-ongs-et-mouvements-associatifs-decision/</t>
+          <t>https://matd.gov.gn/dnarproma-ouverture-des-ateliers-regionaux-sur-lactualisation-de-la-loi-013-05-a-kindia-et-kankan/; https://guineelex.com/decrets-arretes/arrete-a-2022-3220-matd-cab-sgg; https://www.amnestyguinee.org/wp-content/uploads/2020/09/Loi-L013-ONG-Guinee.pdf; https://guineenews.org/2024/09/02/guinee-le-gouvernement-suspend-la-delivrance-des-agrements-aux-ongs-et-mouvements-associatifs-decision/; https://guineenews.org/2024-09-02/guinee-le-gouvernement-suspend-la-delivrance-des-agrements-aux-ongs-et-mouvements-associatifs-decision/</t>
         </is>
       </c>
       <c r="P191" s="2" t="inlineStr">
@@ -18125,7 +18125,7 @@
       </c>
       <c r="G192" s="2" t="inlineStr">
         <is>
-          <t>Repeated military coups (7 since independence), fragile state capacity, weak enforcement of registrations; Portuguese (not French) documents; practical operations very difficult | [verified] Requires a physical public deed in Portuguese at the Serviços Notariais (Bissau only) plus 10+ founding members; no remote channel for foreign founders (Constitution art. 44d grants the right to citizens; IMVF 2021 study s4.2, s4.2.4). | Correction: Mechanism: notarial registration under the Código Civil (Decreto 23/92 opinion route inoperative); cited 2013 law unverified; fees per 2021 IMVF study (~93k-300k CFA). | verify-rest 2026-10: misattributed 'Lei 5/VI/96' (Cape Verde numbering) and Guinea-Conakry 'L/005/013/AN' references removed</t>
+          <t>Repeated military coups (7 since independence), fragile state capacity, weak enforcement of registrations; Portuguese (not French) documents; practical operations very difficult | [verified] Requires a physical public deed in Portuguese at the Serviços Notariais (Bissau only) plus 10+ founding members; no remote channel for foreign founders (Constitution art. 44d grants the right to citizens; IMVF 2021 study s4.2, s4.2.4). | Correction: Mechanism: notarial registration under the Código Civil (Decreto 23/92 opinion route inoperative); cited 2013 law unverified; fees per 2021 IMVF study (~93k-300k CFA). | verify-rest 2026-10: misattributed 'Lei 5/VI/96' (Cape Verde numbering) and Guinea-Conakry 'L/005/013/AN' references removed | verify-r2 2026-10 (confirmed): No 2024-2026 reform of Guinea-Bissau's association or NGO framework was found;</t>
         </is>
       </c>
       <c r="H192" s="2" t="inlineStr">
@@ -18165,7 +18165,7 @@
       </c>
       <c r="O192" s="2" t="inlineStr">
         <is>
-          <t>https://natlex.ilo.org/dyn/natlex2/r/natlex/fe/details?p3_isn=73216; https://rimap.unhcr.org/node/61431; https://www.imvf.org/wp-content/uploads/2021/09/estudo-Quadro-legal-osc-guine-bissau-ianda-djuntu.pdf; https://www.imvf.org/wp-content/uploads/2021/09/estudo-quadro-legal-osc-guine-bissau-ianda-djuntu.pdf</t>
+          <t>https://natlex.ilo.org/dyn/natlex2/r/natlex/fe/details?p3_isn=73216; https://rimap.unhcr.org/node/61431; https://www.imvf.org/wp-content/uploads/2021/09/estudo-Quadro-legal-osc-guine-bissau-ianda-djuntu.pdf; https://www.imvf.org/wp-content/uploads/2021/09/estudo-quadro-legal-osc-guine-bissau-ianda-djuntu.pdf; https://monitor.civicus.org/explore/association-GuineaBissau/; https://capacity4dev.europa.eu/media/32664/download/a9cd4339-c5f9-4241-8847-d8769a420b05_en</t>
         </is>
       </c>
       <c r="P192" s="2" t="inlineStr">
@@ -18197,7 +18197,7 @@
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Association under the Code des obligations civiles et commerciales arts. 811 ff. (Loi 68-08 of 26 Mar 1968, am. Loi 79-02) and Décret 76-040 of 16 Jan 1976 (declaration + récépissé); ONG under décret n° 96-103 du 8 février 1996 as modified by décret n° 2010-1490 du 10 novembre 2010.</t>
+          <t>Association under the Code des obligations civiles et commerciales arts. 811 ff. (Loi 68-08 of 26 Mar 1968, am. Loi 79-02) and Décret 76-040 of 16 Jan 1976 (declaration + récépissé); ONG under décret n° 96-103 du 8 février 1996 as modified by décret n° 2010-1490 du 10 novembre 2010 and décret n° 2015-145 du 4 février 2015.</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
@@ -18207,7 +18207,7 @@
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>Declaration to the administrative authority (Ministry of Interior/préfecture), refusable only on legality grounds (COCC art. 812); local registered office; French-language documents</t>
+          <t>Declaration to the administrative authority (regional governor/préfet, forwarded to the Ministry of Interior), refusable only on legality grounds (COCC art. 812); local registered office; French-language documents</t>
         </is>
       </c>
       <c r="F193" s="2" t="inlineStr">
@@ -18217,7 +18217,7 @@
       </c>
       <c r="G193" s="2" t="inlineStr">
         <is>
-          <t>Stable, well-established association culture; declaration regime is the easiest in francophone West Africa; 2022/2023 framework on foreign-funded NGOs (OSC law) adds a reporting layer for foreign funders; French-only | Confirm prior: 1965 declaration regime (1901 model) stands; 2023 OSC framework confirmed as reporting layer, not a ban | verify-rest 2026-10: 'Loi 71-604' is not the associations law — COCC arts. 811 ff. + Décret 76-040 govern</t>
+          <t>Stable, well-established association culture; declaration regime is the easiest in francophone West Africa; 2022/2023 framework on foreign-funded NGOs (OSC law) adds a reporting layer for foreign funders; French-only | Confirm prior: 1965 declaration regime (1901 model) stands; 2023 OSC framework confirmed as reporting layer, not a ban | verify-rest 2026-10: 'Loi 71-604' is not the associations law — COCC arts. 811 ff. + Décret 76-040 govern | verify-r2 2026-10 (corrected): ICNL's Civic Freedom Monitor (updated Sept 2026) lists Senegal's NGO regime as Décret 96-103, amended by Décret 2010-1490 and further by Décret 2015-145 of 4 Feb 2015 (investment programmes, funding control), published in JO n°6842.</t>
         </is>
       </c>
       <c r="H193" s="2" t="inlineStr">
@@ -18257,7 +18257,7 @@
       </c>
       <c r="O193" s="2" t="inlineStr">
         <is>
-          <t>https://www.icnl.org/resources/civic-freedom-monitor/senegal; https://www.service-public.gouv.fr/particuliers/vosdroits/F426; https://dgsfc.gouv.sn/sites/default/files/2021-03/guide_pour_la%20constitution_ASSOCIATION_et_ONG.pdf; https://www.sports.gouv.sn/wp-content/uploads/2022/02/DECLARATION-ET-ENREGISTREMENT-DES-ASSOCIATIONS-SPORTIVES.pdf</t>
+          <t>https://www.icnl.org/resources/civic-freedom-monitor/senegal; https://www.service-public.gouv.fr/particuliers/vosdroits/F426; https://dgsfc.gouv.sn/sites/default/files/2021-03/guide_pour_la%20constitution_ASSOCIATION_et_ONG.pdf; https://www.sports.gouv.sn/wp-content/uploads/2022/02/DECLARATION-ET-ENREGISTREMENT-DES-ASSOCIATIONS-SPORTIVES.pdf; https://www.vie-publique.sn/documents/1467/JO-6842-du-04-avril-2015</t>
         </is>
       </c>
       <c r="P193" s="2" t="inlineStr">
@@ -18304,12 +18304,12 @@
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
-          <t>MoJ fees: business name 20,000 GMD, company 80,000-90,000 GMD (~$300-350); NGO annual fee ~$5; time unpublished. Non-residents need a resident agent or representative.</t>
+          <t>MoJ fees: name reservation D500, business registration D1,000, company limited by guarantee D5,000 (~$90-100 total); NGO annual fee ~$5; time unpublished. Non-residents need a resident agent or representative.</t>
         </is>
       </c>
       <c r="G194" s="2" t="inlineStr">
         <is>
-          <t>English language, stable democracy; 2022 NGO Bill has been in draft years without enactment, so the old 1972 Societies Act still applies; Banjul filings manageable with a local agent | verify-rest 2026-10: NGO Decree is No. 81 of 1996 (not 1993); Companies Act 2013 replaced the 1955 Act</t>
+          <t>English language, stable democracy; NGO Bill has been in draft for years without enactment, so the NGO Decree No. 81 of 1996 still applies; Banjul filings manageable with a local agent | verify-rest 2026-10: NGO Decree is No. 81 of 1996 (not 1993); Companies Act 2013 replaced the 1955 Act | verify-r2 2026-10 (corrected): The Ministry of Justice company-registration page lists D5,000 for a company limited by guarantee plus D500 name reservation and D1,000 business registration, and requires particulars of a Gambian agent for non-resident directors;</t>
         </is>
       </c>
       <c r="H194" s="2" t="inlineStr">
@@ -18319,7 +18319,7 @@
       </c>
       <c r="I194" s="2" t="inlineStr">
         <is>
-          <t>Local office and local representative needed; Societies Act filings in person in Banjul; NGO Bill not yet enacted</t>
+          <t>Local office and local representative needed; NGO Affairs Agency clearance and Registrar General filings in Banjul; NGO Bill not yet enacted</t>
         </is>
       </c>
       <c r="J194" s="2" t="inlineStr">
@@ -18339,7 +18339,7 @@
       </c>
       <c r="M194" s="2" t="inlineStr">
         <is>
-          <t>No FCRA-style licensing; 2022 NGO Bill pending, so 1972 Societies Act regime applies; no ban on foreign donations</t>
+          <t>No FCRA-style licensing; NGO Bill pending, so the NGO Decree No. 81 of 1996 regime applies; no ban on foreign donations</t>
         </is>
       </c>
       <c r="N194" s="2" t="inlineStr">
@@ -18349,7 +18349,7 @@
       </c>
       <c r="O194" s="2" t="inlineStr">
         <is>
-          <t>https://www.wipo.int/wipolex/en/legislation/details/10617; https://www.moj.gm/companies-division; https://www.icnl.org/research/library/gambia_ngodec</t>
+          <t>https://www.wipo.int/wipolex/en/legislation/details/10617; https://www.moj.gm/companies-division; https://www.icnl.org/research/library/gambia_ngodec; https://www.moj.gm/company-registration; https://thepoint.gm/africa/gambia/article/non-governmental-affairs-agency-clears-the-air</t>
         </is>
       </c>
       <c r="P194" s="2" t="inlineStr">
@@ -18401,7 +18401,7 @@
       </c>
       <c r="G195" s="2" t="inlineStr">
         <is>
-          <t>English language; 2022 NGO Bill pending, so existing NGO/charitable-society registration practices continue; Freetown has expat-friendly law firms; registry throughput is slower than Ghana | verify-rest 2026-10: Companies Act is 2009 (Act No. 5, am. 2014), not 2013; separate NGO registration (~US$500/yr) added</t>
+          <t>English language; 2022 NGO Bill pending, so existing NGO/charitable-society registration practices continue; Freetown has expat-friendly law firms; registry throughput is slower than Ghana | verify-rest 2026-10: Companies Act is 2009 (Act No. 5, am. 2014), not 2013; separate NGO registration (~US$500/yr) added | verify-r2 2026-10 (confirmed): Sierra Leone's Companies Act 2009 (amended 2014, including s.22 on companies limited by guarantee) remains the CAC's governing law;</t>
         </is>
       </c>
       <c r="H195" s="2" t="inlineStr">
@@ -18441,7 +18441,7 @@
       </c>
       <c r="O195" s="2" t="inlineStr">
         <is>
-          <t>https://nib.gov.sl/business-registration-corporate-affairs/; https://manwaadvocates.com/why-more-non-profits-are-choosing-companies-limited-by-guarantee-instead-of-ngos/; https://www.wipo.int/wipolex/en/legislation/details/9820; https://www.jica.go.jp/sierraleone/office/others/ngo.html</t>
+          <t>https://nib.gov.sl/business-registration-corporate-affairs/; https://manwaadvocates.com/why-more-non-profits-are-choosing-companies-limited-by-guarantee-instead-of-ngos/; https://www.wipo.int/wipolex/en/legislation/details/9820; https://www.jica.go.jp/sierraleone/office/others/ngo.html; https://old.sierralii.org/node/5047; https://www.parliament.gov.sl/uploads/acts/COMPANIES AMENDMNET ACT 2014.pdf; https://eusee.hivos.org/alert/ministry-of-planning-and-economic-development-moped-bans-ngos-over-regulatory-compliance/</t>
         </is>
       </c>
       <c r="P195" s="2" t="inlineStr">
@@ -18585,7 +18585,7 @@
       </c>
       <c r="G197" s="2" t="inlineStr">
         <is>
-          <t>Military rule since 2023; security situation in the north (Sahel conflict); Niamey filings are French-only; some discretionary elements in approvals | verify-rest 2026-10: unverifiable 'Law 93-010' removed; 2025-26 crackdown added</t>
+          <t>Military rule since 2023; security situation in the north (Sahel conflict); Niamey filings are French-only; some discretionary elements in approvals | verify-rest 2026-10: unverifiable 'Law 93-010' removed; 2025-26 crackdown added | verify-r2 2026-10 (confirmed): Press reports confirm Niger's Interior Ministry suspended NGOs lacking 2024 financial statements in the Journal officiel in Nov 2025 and dissolved non-compliant ones by arrêté of 7 Jan 2026, leaving 1,809 authorised (1,684 national, 125 in…</t>
         </is>
       </c>
       <c r="H197" s="2" t="inlineStr">
@@ -18625,7 +18625,7 @@
       </c>
       <c r="O197" s="2" t="inlineStr">
         <is>
-          <t>https://wacsi.org/wp-content/uploads/2022/06/DECRET-2022-182-SECTEUR-DES-ONG-3-1-1.pdf; https://www.omct.org/fr/ressources/appels-urgents/niger-suspension-des-activit%C3%A9s-des-ong-nayant-pas-publi%C3%A9-leurs-%C3%A9tats-financiers-au-journal-officiel-de-la-r%C3%A9publique-du-niger; https://www.icnl.org/resources/library/ordonnance-no-84-06-portant-regime-des-associations</t>
+          <t>https://wacsi.org/wp-content/uploads/2022/06/DECRET-2022-182-SECTEUR-DES-ONG-3-1-1.pdf; https://www.omct.org/fr/ressources/appels-urgents/niger-suspension-des-activit%C3%A9s-des-ong-nayant-pas-publi%C3%A9-leurs-%C3%A9tats-financiers-au-journal-officiel-de-la-r%C3%A9publique-du-niger; https://www.icnl.org/resources/library/ordonnance-no-84-06-portant-regime-des-associations; https://lanouvelletribune.info/2026/01/le-niger-dissout-pres-de-la-moitie-des-ong-operant-sur-son-territoire/; https://fr.allafrica.com/stories/202511180173.html; https://www.afrique-sur7.fr/niger-pres-de-3-000-ong-suspendues-en-2025</t>
         </is>
       </c>
       <c r="P197" s="2" t="inlineStr">
@@ -18828,8 +18828,376 @@
         </is>
       </c>
     </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Cabo Verde</t>
+        </is>
+      </c>
+      <c r="B200" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C200" s="2" t="inlineStr">
+        <is>
+          <t>Associação sem fins lucrativos and fundação under Lei n.º 25/VI/2003 de 21 de julho (with Código Civil arts. 157 ff., e.g. art. 185 for foundations), constituted/registered at the Conservatória dos Registos (Registo de Pessoas Coletivas, DGRNI, Ministério da Justiça) and published in the Boletim Oficial II Série (art. 9.1.b); optional OSCD status (organização da sociedade civil de desenvolvimento, Lei n.º 114/VIII/2016); foreign associations/foundations need a Ministry of Justice despacho de autorização before their local representation is registered; optional utilidade pública status (Decreto-Lei 59/2005 as amended by Lei 16/X/2022).</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>Registered seat (sede) in Cabo Verde; Portuguese-language estatutos and constitutive act (escritura or registo de constituição at the Conservatória); governing bodies (Assembleia Geral, Direção/Conselho Diretivo, Conselho Fiscal) - statutory founder minimum not confirmed in published sources; no nationality bar found (Constitution art. 51: association free without administrative authorisation); NIF tax number for the entity and for foreign directors; foreign founders can act via apostilled power of attorney to a local lawyer; branch of a foreign NGO requires Ministry of Justice authorisation plus a named local legal representative.</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="inlineStr">
+        <is>
+          <t>Registry/notary emolumentos (Decreto-Lei 70/2009 tariff) and Boletim Oficial publication fee: unpublished amounts, typically modest; local lawyer/representative + translations/apostille realistically CVE 100,000-250,000 (~USD 1,050-2,600, estimate); 1-3 months for a local association, 2-6 months for a foreign NGO representation (ministerial despacho first).</t>
+        </is>
+      </c>
+      <c r="G200" s="2" t="inlineStr">
+        <is>
+          <t>Lei n.º 25/VI/2003 (21 July 2003) remains in force: 2025-2026 Boletim Oficial extracts still cite art. 9.1.b for association and foundation constitutions | Foreign entities: 2026 BO extracts show a US (Delaware) non-profit and a foreign foundation registered as permanent representations only after a despacho de autorização do exercício de atividades em Cabo Verde (Ministry of Justice), criteria unpublished | Lei 114/VIII/2016 (OSCD statute) excludes religious, political, union and military bodies | Utilidade pública: Decreto-Lei 59/2005 (19 Sept), amended by Lei 16/X/2022 (30 Dec) + Despacho 41/2022; grants fiscal/fee benefits, annual report &amp; accounts to the Government | Casa do Cidadão handles 'empresa no dia' company formation, not associations | Portuguese only; CIVICUS reports registration refusals rare | CVE pegged to EUR (110.265 CVE/EUR), ~95 CVE/USD</t>
+        </is>
+      </c>
+      <c r="H200" s="2" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="I200" s="2" t="inlineStr">
+        <is>
+          <t>In-person Conservatória/notary formalities in Portuguese require a local lawyer under apostilled power of attorney (and, for a foreign-NGO branch, a prior Ministry of Justice authorisation with unpublished criteria), plus obtaining a NIF and opening a local bank account.</t>
+        </is>
+      </c>
+      <c r="J200" s="2" t="inlineStr">
+        <is>
+          <t>unpublished (Conservatória emolumentos under Decreto-Lei 70/2009 plus Boletim Oficial publication fee; amounts not published online)</t>
+        </is>
+      </c>
+      <c r="K200" s="2" t="inlineStr">
+        <is>
+          <t>1-3 months (local association); 2-6 months (foreign NGO representation)</t>
+        </is>
+      </c>
+      <c r="L200" s="2" t="inlineStr">
+        <is>
+          <t>Código dos Benefícios Fiscais (Lei 26/VIII/2013, amended Lei 102/VIII/2016) mecenato: companies deduct 130% of gifts up to 10/1000 of turnover (art. 31); individuals in organised accounting 130% as expense, others a tax credit of 30% of gifts capped at 15% of the IRPS liability (art. 32); only to beneficiaries in arts. 33/36-40 (e.g. IPSS and utilidade pública bodies for social mecenato), with project recognition by the line ministry (art. 34, tacit approval after 30 days).</t>
+        </is>
+      </c>
+      <c r="M200" s="2" t="inlineStr">
+        <is>
+          <t>None notable (no foreign-funding register or prior-approval rule found); foreign NGOs operating locally need Ministry of Justice authorisation of their representation.</t>
+        </is>
+      </c>
+      <c r="N200" s="2" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="O200" s="2" t="inlineStr">
+        <is>
+          <t>https://boe.incv.cv/Bulletins/DownloadAct?id=63647; https://boe.incv.cv/Bulletins/DownloadAct?id=101745; https://boe.incv.cv/Bulletins/DownloadAct?id=112398; https://boe.incv.cv/Bulletins/Download/2163; https://boe.incv.cv/Bulletins/Download/12753; https://boe.incv.cv/Bulletins/DownloadAct?id=90257; https://boe.incv.cv/Bulletins/Download/1957; https://www.camara.cv/wp-content/uploads/2016/07/Codigo-dos-Beneficios-Fiscais.pdf; https://monitor.civicus.org/explore/association-cape-verde/</t>
+        </is>
+      </c>
+      <c r="P200" s="2" t="inlineStr">
+        <is>
+          <t>No general NGO annual-filing regime published under Lei 25/VI/2003; statutory amendments/officer changes must be registered and published in the BO; utilidade pública bodies send annual report and accounts to the Chefia do Governo and must report statute changes (DL 59/2005), losing status if requirements lapse; entities with taxable income file IRPC returns with the DNRE.</t>
+        </is>
+      </c>
+      <c r="Q200" s="2" t="inlineStr">
+        <is>
+          <t>No automatic exemption for charities: Código do IRPC (Lei 82/VIII/2015) art. 13 exempts only religious bodies (cult income) and cultural, recreational, sporting and professional associations (subject to art. 5.2 conditions), excluding commercial/investment income; utilidade pública declaration (DL 59/2005/Lei 16/X/2022, by government despacho) brings tax exemptions and fee reductions; customs duty exemption on imports for mecenato-eligible non-profits (CBF art. 50); timing unpublished.</t>
+        </is>
+      </c>
+      <c r="R200" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: banks (Banco Comercial do Atlântico, Caixa Económica de Cabo Verde, Banco Interatlântico, BCN, BAI Cabo Verde) require the registered entity's certidão, NIF, BO publication and in-person KYC of signatories with passport; remote opening exists mainly for Cape Verdean emigrants via certified documents, not for foreign-founded NGOs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+      <c r="B201" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C201" s="2" t="inlineStr">
+        <is>
+          <t>NGOs under Law No. 06/L-043 on Freedom of Association in NGOs (2019, amended by Law No. 08/L-244, 2024): association (3+ founders), foundation (1+ founder, EUR 1,000 initial capital) and institute (1+ founder, non-membership) (Arts. 16-19); foreign/international NGOs register a Kosovo branch (Art. 24); all registered by the Department for Registration and Liaison with NGOs (DRLNGO), Ministry of Internal Affairs (MPB); optional public beneficiary status (Art. 37).</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E201" s="2" t="inlineStr">
+        <is>
+          <t>Foreign natural/legal persons may found an NGO (Art. 3(1.7)); association needs 3+ founders, foundation/institute 1+; foundation needs EUR 1,000 initial capital; authorized representative must be an adult resident of Kosovo (Arts. 3(1.8), 23(4)); Kosovo seat/address; documents: act of establishment, statute, ID copies of founders and representative, registration certificate for legal-person founders (Art. 22(4)); foreign branch: notarized proof of legal personality abroad, Kosovo branch address, head-office representative declaration (Art. 24); filings in Albanian or Serbian (official languages).</t>
+        </is>
+      </c>
+      <c r="F201" s="2" t="inlineStr">
+        <is>
+          <t>Government fee: none published (no fee in Law 06/L-043); realistic all-in EUR 300-1,000 (~USD 350-1,150) for translation/notarisation of foreign documents, statute drafting and a local representative/lawyer, plus EUR 1,000 capital for a foundation; statutory decision within 45 days (Art. 25(2) as amended by 08/L-244), 1-3 months end-to-end.</t>
+        </is>
+      </c>
+      <c r="G201" s="2" t="inlineStr">
+        <is>
+          <t>Law No. 06/L-043 (Official Gazette No. 11/2019, 24.04.2019) repealed Law No. 04/L-057; amended by Law No. 08/L-244 (Official Gazette 05.01.2024) which lengthened the registration decision period from 30 to 45 days and set a EUR 50 fine on the authorized representative for not reporting changes | implementing rules: Administrative Instruction (GRK) No. 12/2022 on registration and functioning of NGOs, amended by AI (GRK) No. 02/2025 (45-day review confirmed) | 2019 law removed the old bar on foreign residents as founders and added the 'institute' form | incomplete applications get 15 days to cure (Art. 25(4)-(5)) | foreign documents (e.g. a branch's proof of legal personality) need notarisation plus certified Albanian/Serbian translation | NGO department moved from the Ministry of Public Administration to the Ministry of Internal Affairs in the 2021 reorganisation.</t>
+        </is>
+      </c>
+      <c r="H201" s="2" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="I201" s="2" t="inlineStr">
+        <is>
+          <t>The NGO's authorized representative must be a Kosovo resident (Law 06/L-043 Arts. 3(1.8), 23(4)), so a remote Australian founder needs a trusted local representative.</t>
+        </is>
+      </c>
+      <c r="J201" s="2" t="inlineStr">
+        <is>
+          <t>none (no state fee in Law 06/L-043 or AI 12/2022; Global Philanthropy Environment Index reports USD 0)</t>
+        </is>
+      </c>
+      <c r="K201" s="2" t="inlineStr">
+        <is>
+          <t>6 weeks-3 months (45-day statutory decision period under Art. 25(2) as amended by Law 08/L-244)</t>
+        </is>
+      </c>
+      <c r="L201" s="2" t="inlineStr">
+        <is>
+          <t>Individuals (taxed on real-income basis) and companies may deduct donations/sponsorship for humanitarian, health, education, religious, scientific, cultural, environmental and sports purposes up to 10% of taxable income (CIT Law No. 06/L-105; PIT law), plus up to a further 10% for areas set by special laws; receipts signed and stamped by the beneficiary required; donations to public-beneficiary-status NGOs qualify.</t>
+        </is>
+      </c>
+      <c r="M201" s="2" t="inlineStr">
+        <is>
+          <t>None notable (no foreign-agent or foreign-funding register); AML rules limit NGO cash receipts/disbursements (EUR 500 per source per day, EUR 5,000 per source per year) and require suspicious-transaction reports to the Financial Intelligence Unit.</t>
+        </is>
+      </c>
+      <c r="N201" s="2" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="O201" s="2" t="inlineStr">
+        <is>
+          <t>https://gzk.rks-gov.net/ActDocumentDetail.aspx?ActID=19055; https://gzk.rks-gov.net/ActDetail.aspx?ActID=19055&amp;langid=2; https://kryeministri.rks-gov.net/wp-content/uploads/2023/06/Projektligji-per-Ndryshimin-dhe-Plotesimin-e-Ligjit-per-Lirine-e-Asociimit-ne-Organizata-Jo-qeveritare.pdf; https://kryeministri.rks-gov.net/wp-content/uploads/2025/03/UDHEZIM-ADMINISTRATIV-QRK-NR.-02-2025.pdf; https://cof.org/country-notes/nonprofit-law-kosovo; https://ecnl.org/news/kosovo-adopts-new-progressive-law-ngos; https://taxsummaries.pwc.com/kosovo/corporate/deductions; https://taxsummaries.pwc.com/kosovo/individual/deductions; https://globalindices.iupui.edu/environment-index/historical-data/regions/balkan/kosovo.html</t>
+        </is>
+      </c>
+      <c r="P201" s="2" t="inlineStr">
+        <is>
+          <t>Public-beneficiary-status NGOs file an annual report (management, activities, financial statements, auditor's report where required) by 31 March (Art. 38), extendable 30 days; independent audit if annual income/expenses exceed EUR 100,000 (Art. 38(8)); missing reports lead to suspension then revocation of status (Art. 39); all NGOs must report changes within 30 days (fines EUR 50-250 on the NGO/authorized representative under Art. 29 as amended); NGOs also file tax returns with the Tax Administration of Kosovo (ATK).</t>
+        </is>
+      </c>
+      <c r="Q201" s="2" t="inlineStr">
+        <is>
+          <t>Not automatic: public beneficiary status (Art. 37) is requested at registration or later for principal activities such as humanitarian aid, education, health, human rights; DRLNGO decides within 45 days; benefits are CIT exemption on income used for public-benefit purposes and tax/fiscal relief (e.g. immovable property tax); non-PBS NGOs pay 10% CIT on profits; revoked status can be re-sought only after 2 years.</t>
+        </is>
+      </c>
+      <c r="R201" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: Kosovo banks (ProCredit, Raiffeisen Bank Kosovo, TEB, NLB Prishtina) require account holders and authorised signatories to appear at a branch with valid ID and proof of address for KYC; a non-resident-founded NGO also presents its DRLNGO registration certificate and fiscal number, and banks apply enhanced AML due diligence to NGOs and foreign beneficial owners - a resident authorized representative can usually handle it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>Palau</t>
+        </is>
+      </c>
+      <c r="B202" s="3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C202" s="2" t="inlineStr">
+        <is>
+          <t>Nonprofit corporation (public-benefit, mutual-benefit or religious subtype) under the Corporations Act 2021 (RPPL 10-11, codified 12 PNCA Ch. 1), registered online with the Registrar of Corporations at the Financial Institutions Commission (FIC); corporations sole under separate ecclesiastical legislation.</t>
+        </is>
+      </c>
+      <c r="D202" s="4" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E202" s="2" t="inlineStr">
+        <is>
+          <t>At least 1 director must be a lawful resident of Palau (1 director minimum; 1 incorporator suffices); registered agent and registered office in Palau named in the Articles; directors upload passport/ID scans with name, residential address and nationality; beneficial-ownership info kept for the Registrar; English; no notarisation or presidential signature any more</t>
+        </is>
+      </c>
+      <c r="F202" s="2" t="inlineStr">
+        <is>
+          <t>Government fee USD 150 (Articles, nonprofit) plus resident-director/registered-agent arrangements (private quotes, unpublished) and optional legal fees, roughly USD 500-2,000 in year one; Registrar issues the certificate in 1-2 business days once the online account is approved, but finding a trustworthy Palau-resident director typically takes weeks.</t>
+        </is>
+      </c>
+      <c r="G202" s="2" t="inlineStr">
+        <is>
+          <t>RPPL 10-11 (signed 29 Sep 2021) repealed the old 12 PNC corporations law; online register live 20 Jan 2025 and registrar role moved from the Office of the Attorney General to the FIC (Executive Order No. 477) | old 3-incorporator, notarised, President-signed procedure abolished | public-benefit nonprofits must pass assets to another public-benefit nonprofit on dissolution | entities not re-registered by Jan 2026 were administratively dissolved | Foreign Investment Act (28 PNCA Ch. 1, as amended by RPPL 9-64) targets foreign-owned 'business enterprises' needing an FIB certificate; a nonprofit barred from business activity normally needs none, but the Corporations Act does not displace the FIA and the 2019 border-security EO subjects foreign nonprofit founders to background checks | front-company crackdown: false filings to the Registrar are a crime</t>
+        </is>
+      </c>
+      <c r="H202" s="2" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="I202" s="2" t="inlineStr">
+        <is>
+          <t>The Corporations Act requires at least one director who is a lawful resident of Palau, so an Australian founder must recruit a trusted local resident director (and registered agent) before the online filing can be lodged.</t>
+        </is>
+      </c>
+      <c r="J202" s="2" t="inlineStr">
+        <is>
+          <t>~$150 (USD 150 Articles of Incorporation, Palau nonprofit, code A-2; foreign nonprofit registration USD 500)</t>
+        </is>
+      </c>
+      <c r="K202" s="2" t="inlineStr">
+        <is>
+          <t>1-4 weeks</t>
+        </is>
+      </c>
+      <c r="L202" s="2" t="inlineStr">
+        <is>
+          <t>40 PNC § 1104 historically refunds/credits donations to Palau non-profit corporations up to 10% of the taxpayer's wages or gross revenue; survival and mechanics after the 2023 tax reform (RPPL 11-11: PGST + Business Profits Tax) are unconfirmed; check with the Bureau of Revenue and Taxation.</t>
+        </is>
+      </c>
+      <c r="M202" s="2" t="inlineStr">
+        <is>
+          <t>None notable; no foreign-funding register, though FIC AML/CFT rules (Money Laundering Act, 17 PNCA Ch. 33) and beneficial-ownership disclosure apply and nonprofits may not engage in business.</t>
+        </is>
+      </c>
+      <c r="N202" s="2" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="O202" s="2" t="inlineStr">
+        <is>
+          <t>https://palauregistries.pw/; https://palauregistries.pw/Documentation/PW/Corporations_Reform_Summary_January_20_2025.pdf; https://palauregistries.pw/public/howto.aspx?ctk=CompanyHowTo; https://islandtimes.org/palau-adopts-modern-corporations-law/; https://islandtimes.org/corporate-registry-launches-online-platform; https://www.palaugov.pw/taxreform/bpt/; https://pacliirms.austlii.edu.au/pw/legis/consol_act/fratt28291.pdf; https://islandtimes.org/eo-issuance-meant-to-boost-capacity-to-check-foreigners-background-remengesau/; https://islandtimes.org/hod-seeks-to-raise-of-tax-refundable-donations-2/; https://www.imf.org/-/media/files/publications/selected-issues-papers/2026/english/sipea2026010.pdf</t>
+        </is>
+      </c>
+      <c r="P202" s="2" t="inlineStr">
+        <is>
+          <t>Online annual report to the FIC Registrar (USD 100 for a Palau nonprofit, USD 200 if late); file changes of directors, officers or addresses (USD 15, USD 100 late); maintain beneficial-ownership records available to the Registrar on request; no public accounts filing or statutory audit; non-filing removes good standing and leads to administrative dissolution (reinstatement possible).</t>
+        </is>
+      </c>
+      <c r="Q202" s="2" t="inlineStr">
+        <is>
+          <t>Automatic in practice: Business Profits Tax rules list the income of a resident nonprofit corporation as exempt income (12% BPT otherwise); PGST (10%) registration only above USD 300,000 taxable supplies or for FIB certificate holders; no separate charity-status application found.</t>
+        </is>
+      </c>
+      <c r="R202" s="2" t="inlineStr">
+        <is>
+          <t>Needs a local visit: the three FDIC-insured US bank branches (Bank of Hawaii, Bank of Guam, BankPacific) hold ~98% of deposits and open accounts on paper with in-person KYC in Koror, requiring certified Articles, bylaws, a director list and signatories' IDs; non-resident signatories face enhanced due diligence, so the resident director usually has to be a signatory.</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>Greenland</t>
+        </is>
+      </c>
+      <c r="B203" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C203" s="2" t="inlineStr">
+        <is>
+          <t>Association (forening): no Greenlandic or Danish registration act for ordinary associations - it exists from its founding general meeting (freedom of association) and registers in the Danish-run CVR register under Inatsisartutlov nr. 33 of 28 Nov 2016 on registration in the Central Business Register (GER abolished 1 Jan 2018); foundation (fond): Danish Act on Foundations and Certain Associations applied by royal decree - Anordning nr. 917 of 15 Dec 1998 on entry into force for Greenland, as amended by Anordning nr. 2460 of 14 Dec 2021 (consolidated as LTA 2021 nr. 2702); fondsmyndighed = Danish Minister of Justice (Civilstyrelsen), with statutes also filed with Skattestyrelsen (Akileraartarnermut Aqutsisoqarfik), Nuuk</t>
+        </is>
+      </c>
+      <c r="D203" s="7" t="inlineStr">
+        <is>
+          <t>hard</t>
+        </is>
+      </c>
+      <c r="E203" s="2" t="inlineStr">
+        <is>
+          <t>Statutes must name a Greenlandic municipality as seat (hjemsted) and the CVR office requires a Greenlandic postal address; association: founding general meeting + board, no nationality rule or member minimum in statute; foundation (assets DKK 1m+): min. assets DKK 1,000,000 at founding (lower only with fondsmyndighed permission), board of at least 3, director(s) and at least half the board resident 'her i landet' unless the fondsmyndighed exempts, founder and family may not form a board majority without consent, statutes + board list to fondsmyndighed and municipal tax authority within 3 months; online CVR filing on virk.dk needs MitID (CPR) - others use paper forms sent to cvr@nanoq.gl; filings in Danish or Greenlandic (official language per Inatsisartutlov nr. 7 of 19 May 2010 on language policy), English guidance only</t>
+        </is>
+      </c>
+      <c r="F203" s="2" t="inlineStr">
+        <is>
+          <t>No government fee for CVR registration; local lawyer/accountant in Nuuk to draft Danish-language statutes and file roughly DKK 10,000-30,000 (~US$1,500-4,500, market estimate, unpublished); association 2-6 weeks to CVR number, plus 1-3 months for a tax-exemption decision; foundation also needs DKK 1m (~US$150,000) endowment and Civilstyrelsen dealings, 2-4 months</t>
+        </is>
+      </c>
+      <c r="G203" s="2" t="inlineStr">
+        <is>
+          <t>Greenland's own tax system (Skattestyrelsen, aka.gl) governs tax exemption; private-law fonde rules remain Danish law applied by royal decree (Anordning 917/1998, in force 1 Jan 1999; 2021 amendment added beneficial-owner registration in Erhvervsstyrelsen's IT system) | Foundations with assets under DKK 1m fall outside most of the act but still need statutes and beneficial-owner registration (s.1(6)) | Ordinary associations are not supervised; chapter 12 of the anordning only covers trade/employer associations | Associations may operate unregistered, but aka.gl warns that without a CVR number opening a bank account and receiving public funds is difficult | Greenland's CVR register merged into the Danish CVR on 1 Jan 2018 (Inatsisartutlov nr. 33/2016); Greenlandic guidance at aka.gl/sullissivik.gl | Feb 2025 Inatsisartut urgent law bans foreign donations to political parties - does not target charities</t>
+        </is>
+      </c>
+      <c r="H203" s="2" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="I203" s="2" t="inlineStr">
+        <is>
+          <t>Practical need for Greenland-resident board members - foundations must have at least half the board resident unless exempted, and banks verify each association board member with a Greenlandic residence certificate.</t>
+        </is>
+      </c>
+      <c r="J203" s="2" t="inlineStr">
+        <is>
+          <t>none (CVR registration of associations/foundations has no published government fee; Civilstyrelsen may levy administration charges on foundations under anordning s.36, amount unpublished)</t>
+        </is>
+      </c>
+      <c r="K203" s="2" t="inlineStr">
+        <is>
+          <t>2-6 weeks (association CVR number); 2-4 months for a foundation incl. fondsmyndighed filings and tax-exemption ruling</t>
+        </is>
+      </c>
+      <c r="L203" s="2" t="inlineStr">
+        <is>
+          <t>No general donor deduction: the consolidated Greenland income tax act (Landstingslov nr. 12 of 2 Nov 2006, Selvstyrets lovbekendtgørelse nr. 62 of 24 Sep 2025) contains no gift deduction for charities - the Danish Ligningsloven s.8 A deduction and Danish approved-charity list do not apply to Greenlandic taxpayers; businesses can deduct only genuine operating expenses (s.24, e.g. sponsorship as marketing).</t>
+        </is>
+      </c>
+      <c r="M203" s="2" t="inlineStr">
+        <is>
+          <t>None notable for charities; foundations must report significant donors/contributors to the fondsmyndighed within 4 weeks of receipt (anordning s.1(3)); the 2025 ban on foreign donations applies only to political parties and politicians.</t>
+        </is>
+      </c>
+      <c r="N203" s="2" t="inlineStr">
+        <is>
+          <t>med</t>
+        </is>
+      </c>
+      <c r="O203" s="2" t="inlineStr">
+        <is>
+          <t>https://www.retsinformation.dk/eli/lta/2021/2702; https://nalunaarutit.gl/groenlandsk-lovgivning/2025/selvstyrets-lovbekendtgoerelse-nr-62-af-24_09_2025; https://aka.gl/-/media/aka/erhverv/ger/inatsisartutlov-nr-33-af-28-november-2016-om-registrering-i-det-centrale-virksomhedsregister.pdf; https://aka.gl/en/erhverv/associations-and-foundations; https://aka.gl/en/erhverv/associations-and-foundations/registration-of-associations; https://aka.gl/en/erhverv/associations-and-foundations/exemption-from-tax-on-profits-associations; https://aka.gl/emner/erhverv/ny-virksomhed/registrering-af-afdeling-af-udenlandsk-selskab?sc_lang=en; https://www.banken.gl/en/private-customers/daily-economy/associations/</t>
+        </is>
+      </c>
+      <c r="P203" s="2" t="inlineStr">
+        <is>
+          <t>Associations and foundations file financial statements with Skattestyrelsen every year even when tax-exempt (aka.gl); foundations: accounts per good accounting practice signed within 6 months of year-end, mandatory audit (state-authorised/registered auditor if equity DKK 3m+, auditor resident unless exempted), auditor appointment notified within 3 months, beneficial owners (board) registered and reviewed annually; board changes reported with the tax return; fines for missed filings (anordning s.40, s.50).</t>
+        </is>
+      </c>
+      <c r="Q203" s="2" t="inlineStr">
+        <is>
+          <t>Non-commercial associations are taxable only on business income (income tax act s.1(1) nr.14, s.1(3)) and can apply by email to Skattestyrelsen for exemption if non-profit, non-distributing and democratic; foundations are fully taxable (s.1(1) nr.13) but may be wholly/partly exempted where statutory purpose is charitable/public-benefit (s.3(2), decision by Naalakkersuisut); self-owning educational/social/cultural institutions exempt (s.3(1) nr.6). No donor-deduction benefit attaches.</t>
+        </is>
+      </c>
+      <c r="R203" s="2" t="inlineStr">
+        <is>
+          <t>Effectively blocked: only two banks - GrønlandsBANKEN (BANK of Greenland) and the former BankNordik Greenland branch (Bankivik since 2025) - and GrønlandsBANKEN's association onboarding requires CVR documentation, board-signed statutes and founding-meeting minutes, and two IDs per board member including a Greenlandic residence certificate (bopælsattest) under 1 year old; non-resident boards need case-by-case approval under Danish/Greenlandic AML rules, so a Danish bank or EMI is the realistic fallback.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R199"/>
+  <autoFilter ref="A1:R203"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19424,22 +19792,22 @@
         </is>
       </c>
       <c r="B2" s="10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" s="10" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E2" s="10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F2" s="10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G2" s="10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" s="10" t="n">
         <v>1</v>
@@ -19620,16 +19988,16 @@
         </is>
       </c>
       <c r="B9" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>0</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>3</v>
@@ -19676,7 +20044,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>10</v>
@@ -19688,7 +20056,7 @@
         <v>6</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" s="10" t="n">
         <v>0</v>
@@ -19732,7 +20100,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>18</v>
@@ -19741,7 +20109,7 @@
         <v>5</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13" s="10" t="n">
         <v>2</v>
@@ -19955,7 +20323,7 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>198 jurisdictions researched via DSH subagent fan-out (16 regional batches, 196 countries + North Korea/Russia extras), then enrichment passes 2 (32 agents x ~6 countries), 2b (141 gap-filler deep-dives), 3 (annual compliance), 4 (tax-exemption) and 5 (bank-access feasibility) with fresh web research against official registries, tax authorities and NGO-law guides. All 198 rows reached high/med confidence (zero 'low' remaining). Costs in USD approximations; times are realistic end-to-end durations for a foreign founder.</t>
+          <t>202 jurisdictions researched via DSH subagent fan-out (16 regional batches, 196 countries + North Korea/Russia extras; Palau, Kosovo and Cabo Verde added Oct 2026), then enrichment passes 2 (32 agents x ~6 countries), 2b (141 gap-filler deep-dives), 3 (annual compliance), 4 (tax-exemption) and 5 (bank-access feasibility) with fresh web research against official registries, tax authorities and NGO-law guides. All rows reached high/med confidence (zero 'low' remaining). Costs in USD approximations; times are realistic end-to-end durations for a foreign founder.</t>
         </is>
       </c>
     </row>
@@ -19979,7 +20347,7 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>186 authoritative names tokenized from the Google for Nonprofits program list; 183 of 198 countries qualify. The 15 not on the list: Belarus, China, Cuba, Georgia, Iran, Liechtenstein, Myanmar, Nepal, North Korea, Russia, Somaliland, South Sudan, Sudan, Syria, Western Sahara.</t>
+          <t>186 authoritative names tokenized from the Google for Nonprofits program list; 185 of 202 countries qualify. The 17 not on the list: Belarus, China, Cuba, Georgia, Greenland, Iran, Kosovo, Liechtenstein, Myanmar, Nepal, North Korea, Russia, Somaliland, South Sudan, Sudan, Syria, Western Sahara.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mobile-responsive atlas, theme toggle, screenshots and a full README
Atlas (build_atlas.py -> webapp/atlas.html + docs/index.html):
- phones: filters fold behind a Filters button, map-colour tabs scroll
  horizontally, zoom controls move below the map, the ranking renders as
  cards, dossier sections collapse, benchmark labels stay pinned
- header links to GitHub, CSV and Excel; light/dark/auto theme toggle
- Open Graph / Twitter card tags on the GitHub Pages copy

make_screenshots.py renders docs/screenshots/{desktop-light,desktop-dark,
benchmark,mobile}.png with headless Chrome (phone view via a 390px iframe).

README rewritten: badges, screenshots, at-a-glance stats, top 10,
quick answers, usage guide, column reference, ranking formulas,
research passes, pipeline, layout, contributing.

Russia and North Korea moved from a catch-all region to Central &
E. Europe and East Asia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/charities_by_country_v2.xlsx
+++ b/charities_by_country_v2.xlsx
@@ -19730,7 +19730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19820,7 +19820,7 @@
         </is>
       </c>
       <c r="B3" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" s="10" t="n">
         <v>6</v>
@@ -19835,7 +19835,7 @@
         <v>0</v>
       </c>
       <c r="G3" s="10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" s="10" t="n">
         <v>0</v>
@@ -20100,7 +20100,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" s="10" t="n">
         <v>18</v>
@@ -20112,7 +20112,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G13" s="10" t="n">
         <v>1</v>
@@ -20230,34 +20230,6 @@
         <v>1</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>EXTRA</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="C18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="10" t="n">
-        <v>1</v>
-      </c>
-      <c r="H18" s="10" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>